<commit_message>
[monitoramento 14/09] Registro fecha em 23 avaliadas / 18 maturacao; proposta da linha do Controle Semanal
Registro de Alteracoes conferido apos os vereditos EC-003 e EC-004:
42 entradas, 23 EXECUTADA - AVALIADA, 18 EXECUTADA - EM MATURACAO,
1 BLOQUEADA - CONFERIR ESTADO. Contadores da linha 6 batem.

Proposta da linha 12 do Controle Semanal (14/09, janela 07-14/09),
apenas colunas A:H e N:P conforme a instrucao da propria aba.
Impressoes ficam em branco por ausencia de dado na janela correta.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -1178,12 +1178,6 @@
     <t>Última atividade em 31/08; ausente da Era a partir daí</t>
   </si>
   <si>
-    <t>Janela pós começa em 08/09. Até 09/09: PG2460 vendeu em 07/09 (R$ 223,88) e PXP vendeu 2 vezes em 08/09 (R$ 302,20 e R$ 151,10), todas com Melhor Oferta de −10%</t>
-  </si>
-  <si>
-    <t>Dias de execução dentro da semana de 07 a 13/09</t>
-  </si>
-  <si>
     <t>MANTIDA — a inelegibilidade persiste. Reativar somente com o anúncio liberado. Pausa por inelegibilidade, não conta como falha de desempenho (Playbook §30)</t>
   </si>
   <si>
@@ -1241,10 +1235,16 @@
     <t>EFETIVA — conserto da O4-006</t>
   </si>
   <si>
-    <t>NÃO AVALIÁVEL até 14/09. ACHADO JÁ CONFIRMADO: nos 3 pedidos o Ads registrou o valor COM desconto — a Melhor Oferta é atribuída ao PREÇO DA OFERTA. A atribuição a preço de tabela vale para a promoção de quantidade, que é outro mecanismo</t>
-  </si>
-  <si>
-    <t>NÃO AVALIÁVEL até 14/09</t>
+    <t>Evento encerrado em 13/09. Das 11 Melhores Ofertas, 3 venderam: PXP 3 un por R$ 453,30 (−10%), PXM 3 un por R$ 519,03 (−15%) e PG2460 1 un por R$ 223,88 (−10%). Total R$ 1.196,21 em 7 unidades e 174 visualizações somadas. As 8 restantes: zero venda.</t>
+  </si>
+  <si>
+    <t>Evento encerrado. As 5 Ofertas Relâmpago (07/09 ×2, 10/09 ×1, 11/09 ×2) terminaram com ZERO venda, ZERO unidade e 19 visualizações somadas nos cinco dias de exibição.</t>
+  </si>
+  <si>
+    <t>PARCIALMENTE POSITIVO — o formato converte, mas só na família de suporte de extintor e porta-guarda-chuva. NENHUMA LIXEIRA VENDEU COM OFERTA, e lixeira é o grosso do catálogo e do tráfego. Para o Vem de Amazon, 8 das 11 não pontuam (a regra exige ao menos 1 venda por oferta no trimestre). Achado colateral confirmado: a atribuição de Ads usa o PREÇO DA OFERTA — 5 pedidos, 3 SKUs, 4 campanhas, todos batendo ao centavo.</t>
+  </si>
+  <si>
+    <t>NEGATIVO — o formato não gerou nem tráfego. 19 visualizações em 5 deals não é falha de conversão, é falha de exibição: não houve amostra para converter. Nenhuma das 5 pontua no Vem de Amazon. NÃO REPETIR RELÂMPAGO (inclusive na Black Friday) antes de entender por que a exibição foi tão baixa — é a pergunta em aberto do evento.</t>
   </si>
 </sst>
 </file>
@@ -1625,78 +1625,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="21">
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9A3412"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFED7AA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF991B1B"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEE2E2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF374151"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF3F4F6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF166534"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDCFCE7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF3730A3"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE0E7FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF92400E"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEF3C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1E40AF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDBEAFE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="14">
     <dxf>
       <font>
         <b/>
@@ -2233,11 +2162,11 @@
       </c>
       <c r="E6" s="3">
         <f>COUNTIF(P11:P210,"EXECUTADA - EM MATURAÇÃO")</f>
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F6" s="4">
         <f>COUNTIF(P11:P210,"EXECUTADA - AVALIADA")</f>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="H6" s="47"/>
       <c r="I6" s="47"/>
@@ -2402,13 +2331,13 @@
       </c>
       <c r="R11" s="17">
         <f t="shared" ref="R11:R42" ca="1" si="1">IF(E11="","",TODAY()-E11)</f>
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="S11" t="s">
         <v>362</v>
       </c>
       <c r="T11" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="U11" s="6"/>
       <c r="V11" s="38" t="s">
@@ -2468,13 +2397,13 @@
       </c>
       <c r="R12" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="S12" t="s">
         <v>363</v>
       </c>
       <c r="T12" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="U12" s="7"/>
       <c r="V12" s="27" t="s">
@@ -2532,13 +2461,13 @@
       </c>
       <c r="R13" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="S13" t="s">
         <v>364</v>
       </c>
       <c r="T13" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="U13" s="7">
         <v>46273</v>
@@ -2600,13 +2529,13 @@
       </c>
       <c r="R14" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="S14" t="s">
         <v>365</v>
       </c>
       <c r="T14" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="U14" s="7">
         <v>46273</v>
@@ -2670,13 +2599,13 @@
       </c>
       <c r="R15" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="S15" t="s">
         <v>366</v>
       </c>
       <c r="T15" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="U15" s="7">
         <v>46273</v>
@@ -2740,13 +2669,13 @@
       </c>
       <c r="R16" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="S16" t="s">
         <v>367</v>
       </c>
       <c r="T16" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="U16" s="7">
         <v>46273</v>
@@ -2810,13 +2739,13 @@
       </c>
       <c r="R17" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="S17" t="s">
         <v>368</v>
       </c>
       <c r="T17" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="U17" s="7"/>
       <c r="V17" s="27" t="s">
@@ -2878,13 +2807,13 @@
       </c>
       <c r="R18" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="S18" t="s">
         <v>369</v>
       </c>
       <c r="T18" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="U18" s="7">
         <v>46273</v>
@@ -2948,13 +2877,13 @@
       </c>
       <c r="R19" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="S19" t="s">
         <v>370</v>
       </c>
       <c r="T19" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="U19" s="7">
         <v>46273</v>
@@ -3018,13 +2947,13 @@
       </c>
       <c r="R20" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="S20" t="s">
         <v>371</v>
       </c>
       <c r="T20" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="U20" s="7"/>
       <c r="V20" s="27" t="s">
@@ -3086,13 +3015,13 @@
       </c>
       <c r="R21" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="S21" t="s">
         <v>372</v>
       </c>
       <c r="T21" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="U21" s="7"/>
       <c r="V21" s="27"/>
@@ -3152,13 +3081,13 @@
       </c>
       <c r="R22" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="S22" t="s">
         <v>373</v>
       </c>
       <c r="T22" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="U22" s="7"/>
       <c r="V22" s="27"/>
@@ -3218,13 +3147,13 @@
       </c>
       <c r="R23" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="S23" t="s">
         <v>372</v>
       </c>
       <c r="T23" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="U23" s="7"/>
       <c r="V23" s="27"/>
@@ -3284,13 +3213,13 @@
       </c>
       <c r="R24" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="S24" t="s">
         <v>374</v>
       </c>
       <c r="T24" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="U24" s="7">
         <v>46273</v>
@@ -3354,13 +3283,13 @@
       </c>
       <c r="R25" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="S25" t="s">
         <v>375</v>
       </c>
       <c r="T25" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="U25" s="7"/>
       <c r="V25" s="27"/>
@@ -3420,13 +3349,13 @@
       </c>
       <c r="R26" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="S26" t="s">
         <v>376</v>
       </c>
       <c r="T26" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="U26" s="7">
         <v>46273</v>
@@ -3488,13 +3417,13 @@
       </c>
       <c r="R27" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="S27" t="s">
         <v>377</v>
       </c>
       <c r="T27" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="U27" s="7">
         <v>46273</v>
@@ -3558,13 +3487,13 @@
       </c>
       <c r="R28" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="S28" t="s">
         <v>378</v>
       </c>
       <c r="T28" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="U28" s="7">
         <v>46273</v>
@@ -3628,13 +3557,13 @@
       </c>
       <c r="R29" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="S29" t="s">
         <v>379</v>
       </c>
       <c r="T29" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="U29" s="7">
         <v>46273</v>
@@ -3698,13 +3627,13 @@
       </c>
       <c r="R30" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="S30" t="s">
         <v>380</v>
       </c>
       <c r="T30" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="U30" s="41">
         <v>46273</v>
@@ -3768,13 +3697,13 @@
       </c>
       <c r="R31" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="S31" t="s">
         <v>381</v>
       </c>
       <c r="T31" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="U31" s="41">
         <v>46273</v>
@@ -3829,8 +3758,8 @@
       <c r="O32" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="P32" s="11" t="s">
-        <v>47</v>
+      <c r="P32" s="9" t="s">
+        <v>51</v>
       </c>
       <c r="Q32" s="18">
         <f t="shared" si="0"/>
@@ -3838,16 +3767,16 @@
       </c>
       <c r="R32" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="S32" t="s">
-        <v>382</v>
+        <v>401</v>
       </c>
       <c r="T32" t="s">
         <v>403</v>
       </c>
-      <c r="U32" s="7">
-        <v>46279</v>
+      <c r="U32" s="41">
+        <v>46287</v>
       </c>
       <c r="V32" s="27"/>
     </row>
@@ -3897,8 +3826,8 @@
       <c r="O33" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="P33" s="11" t="s">
-        <v>47</v>
+      <c r="P33" s="9" t="s">
+        <v>51</v>
       </c>
       <c r="Q33" s="18">
         <f t="shared" si="0"/>
@@ -3906,16 +3835,16 @@
       </c>
       <c r="R33" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="S33" t="s">
-        <v>383</v>
+        <v>402</v>
       </c>
       <c r="T33" t="s">
         <v>404</v>
       </c>
-      <c r="U33" s="7">
-        <v>46279</v>
+      <c r="U33" s="41">
+        <v>46287</v>
       </c>
       <c r="V33" s="27"/>
     </row>
@@ -3973,7 +3902,7 @@
       </c>
       <c r="R34" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="S34" s="22"/>
       <c r="T34" s="22"/>
@@ -4038,7 +3967,7 @@
       </c>
       <c r="R35" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="S35" s="22"/>
       <c r="T35" s="22"/>
@@ -4103,7 +4032,7 @@
       </c>
       <c r="R36" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S36" s="22"/>
       <c r="T36" s="22"/>
@@ -4168,7 +4097,7 @@
       </c>
       <c r="R37" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S37" s="22"/>
       <c r="T37" s="22"/>
@@ -4233,7 +4162,7 @@
       </c>
       <c r="R38" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S38" s="22"/>
       <c r="T38" s="22"/>
@@ -4298,7 +4227,7 @@
       </c>
       <c r="R39" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S39" s="22"/>
       <c r="T39" s="22"/>
@@ -4363,7 +4292,7 @@
       </c>
       <c r="R40" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S40" s="22"/>
       <c r="T40" s="22"/>
@@ -4428,7 +4357,7 @@
       </c>
       <c r="R41" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S41" s="22"/>
       <c r="T41" s="22"/>
@@ -4493,7 +4422,7 @@
       </c>
       <c r="R42" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S42" s="22"/>
       <c r="T42" s="22"/>
@@ -4558,7 +4487,7 @@
       </c>
       <c r="R43" s="19">
         <f t="shared" ref="R43:R74" ca="1" si="2">IF(E43="","",TODAY()-E43)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S43" s="22"/>
       <c r="T43" s="22"/>
@@ -4623,7 +4552,7 @@
       </c>
       <c r="R44" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S44" s="22"/>
       <c r="T44" s="22"/>
@@ -4688,7 +4617,7 @@
       </c>
       <c r="R45" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S45" s="22"/>
       <c r="T45" s="22"/>
@@ -4753,7 +4682,7 @@
       </c>
       <c r="R46" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S46" s="22"/>
       <c r="T46" s="22"/>
@@ -4818,7 +4747,7 @@
       </c>
       <c r="R47" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S47" s="22"/>
       <c r="T47" s="22"/>
@@ -4942,7 +4871,7 @@
       </c>
       <c r="R49" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S49" s="22"/>
       <c r="T49" s="22"/>
@@ -5007,7 +4936,7 @@
       </c>
       <c r="R50" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S50" s="22"/>
       <c r="T50" s="22"/>
@@ -5072,7 +5001,7 @@
       </c>
       <c r="R51" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S51" s="22"/>
       <c r="T51" s="22"/>
@@ -5137,7 +5066,7 @@
       </c>
       <c r="R52" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="S52" s="22"/>
       <c r="T52" s="22"/>
@@ -9897,25 +9826,25 @@
     <mergeCell ref="A8:V8"/>
   </mergeCells>
   <conditionalFormatting sqref="P11:P210">
-    <cfRule type="expression" dxfId="20" priority="1">
+    <cfRule type="expression" dxfId="13" priority="1">
       <formula>P11="RECOMENDADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="19" priority="2">
+    <cfRule type="expression" dxfId="12" priority="2">
       <formula>P11="APROVADA - AGUARDANDO EXECUÇÃO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="3">
+    <cfRule type="expression" dxfId="11" priority="3">
       <formula>P11="EXECUTADA - EM MATURAÇÃO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="17" priority="4">
+    <cfRule type="expression" dxfId="10" priority="4">
       <formula>P11="EXECUTADA - AVALIADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="5">
+    <cfRule type="expression" dxfId="9" priority="5">
       <formula>P11="APROVADA - NÃO EXECUTADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="6">
+    <cfRule type="expression" dxfId="8" priority="6">
       <formula>P11="REJEITADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="7">
+    <cfRule type="expression" dxfId="7" priority="7">
       <formula>LEFT(P11,9)="BLOQUEADA"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
[EC 18/09] Registro fechado: 52 entradas, 25 avaliadas, 26 em maturacao, 1 bloqueada
Vereditos de EC-005 e EC-006 aplicados e formula de "Dias desde execucao"
restaurada nas linhas 53-62. Diff de exatamente 16 celulas contra o commit
anterior — 6 dos vereditos e 10 das formulas — sem nenhuma colateral.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="853" uniqueCount="460">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1659" uniqueCount="464">
   <si>
     <t>REGISTRO DE ALTERAÇÕES — AMAZON ADS | WINNET METAIS</t>
   </si>
@@ -1410,6 +1410,18 @@
   </si>
   <si>
     <t>Opcional — tráfego marginal (6 sessões/sem). Margem final 16,1% (SP Interior); custo por unidade vendida R$ 4,57. Critério: tráfego × margem ≥ 15%.</t>
+  </si>
+  <si>
+    <t>Janela 05–18/09 (14 dias): ZERO vendas de P2025 no Registro_Vendas. Cupom de 12% ativo o período inteiro, sem resgate.</t>
+  </si>
+  <si>
+    <t>Janela 05–18/09 (14 dias): ZERO vendas de EMB-05, EMB-05P e EMB-08 no Registro_Vendas, com cupom de 50% ativo. Nenhuma unidade escoada; espaço físico não liberado; perda de caixa zero (nada foi resgatado).</t>
+  </si>
+  <si>
+    <t>SEM EFEITO — 12% não moveu o P2025 em duas semanas. Recomendação: ENCERRAR o cupom. Não há ganho comprovado e há risco de empilhamento com a promo de quantidade (5+ → 19% de desconto, margem 7,2%) se um dia resgatar. Confiança MÉDIA.</t>
+  </si>
+  <si>
+    <t>NEGATIVO NO OBJETIVO — a liquidação não escoou uma unidade em 14 dias a metade do preço. Confirma a hipótese registrada em ciclos/EC-04-09.md e não acatada à época: o gargalo desses SKUs é TRÁFEGO, não preço (linha de base 0–3 sessões/semana). Desconto não resolve falta de visitante.</t>
   </si>
 </sst>
 </file>
@@ -1810,7 +1822,78 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="14">
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9A3412"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFED7AA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF991B1B"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF374151"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF3F4F6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF166534"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFDCFCE7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF3730A3"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFE0E7FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF92400E"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEF3C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1E40AF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFDBEAFE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -2276,11 +2359,11 @@
       </c>
       <c r="E6" s="3">
         <f>COUNTIF(P11:P210,"EXECUTADA - EM MATURAÇÃO")</f>
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F6" s="4">
         <f>COUNTIF(P11:P210,"EXECUTADA - AVALIADA")</f>
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H6" s="40"/>
       <c r="I6" s="40"/>
@@ -4009,7 +4092,7 @@
         <v>40</v>
       </c>
       <c r="P34" s="46" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="Q34" s="49">
         <v>46270</v>
@@ -4018,8 +4101,12 @@
         <f t="shared" ca="1" si="1"/>
         <v>14</v>
       </c>
-      <c r="S34" s="50"/>
-      <c r="T34" s="50"/>
+      <c r="S34" s="50" t="s">
+        <v>460</v>
+      </c>
+      <c r="T34" s="50" t="s">
+        <v>462</v>
+      </c>
       <c r="U34" s="49">
         <v>46283</v>
       </c>
@@ -4074,7 +4161,7 @@
         <v>40</v>
       </c>
       <c r="P35" s="46" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="Q35" s="49">
         <v>46270</v>
@@ -4083,8 +4170,12 @@
         <f t="shared" ca="1" si="1"/>
         <v>14</v>
       </c>
-      <c r="S35" s="50"/>
-      <c r="T35" s="50"/>
+      <c r="S35" s="50" t="s">
+        <v>461</v>
+      </c>
+      <c r="T35" s="50" t="s">
+        <v>463</v>
+      </c>
       <c r="U35" s="49">
         <v>46283</v>
       </c>
@@ -5245,8 +5336,9 @@
       <c r="Q53" s="54">
         <v>46287</v>
       </c>
-      <c r="R53" s="53" t="s">
-        <v>413</v>
+      <c r="R53" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="S53" s="53"/>
       <c r="T53" s="53"/>
@@ -5309,8 +5401,9 @@
       <c r="Q54" s="54">
         <v>46287</v>
       </c>
-      <c r="R54" s="53" t="s">
-        <v>413</v>
+      <c r="R54" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="S54" s="53"/>
       <c r="T54" s="53"/>
@@ -5373,8 +5466,9 @@
       <c r="Q55" s="54">
         <v>46287</v>
       </c>
-      <c r="R55" s="53" t="s">
-        <v>413</v>
+      <c r="R55" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="S55" s="53"/>
       <c r="T55" s="53"/>
@@ -5437,8 +5531,9 @@
       <c r="Q56" s="54">
         <v>46287</v>
       </c>
-      <c r="R56" s="53" t="s">
-        <v>413</v>
+      <c r="R56" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="S56" s="53"/>
       <c r="T56" s="53"/>
@@ -5501,8 +5596,9 @@
       <c r="Q57" s="54">
         <v>46287</v>
       </c>
-      <c r="R57" s="53" t="s">
-        <v>413</v>
+      <c r="R57" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="S57" s="53"/>
       <c r="T57" s="53"/>
@@ -5565,8 +5661,9 @@
       <c r="Q58" s="54">
         <v>46287</v>
       </c>
-      <c r="R58" s="53" t="s">
-        <v>413</v>
+      <c r="R58" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="S58" s="53"/>
       <c r="T58" s="53"/>
@@ -5629,8 +5726,9 @@
       <c r="Q59" s="54">
         <v>46287</v>
       </c>
-      <c r="R59" s="53" t="s">
-        <v>413</v>
+      <c r="R59" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="S59" s="53"/>
       <c r="T59" s="53"/>
@@ -5693,8 +5791,9 @@
       <c r="Q60" s="54">
         <v>46287</v>
       </c>
-      <c r="R60" s="53" t="s">
-        <v>413</v>
+      <c r="R60" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="S60" s="53"/>
       <c r="T60" s="53"/>
@@ -5757,8 +5856,9 @@
       <c r="Q61" s="54">
         <v>46287</v>
       </c>
-      <c r="R61" s="53" t="s">
-        <v>413</v>
+      <c r="R61" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="S61" s="53"/>
       <c r="T61" s="53"/>
@@ -5821,8 +5921,9 @@
       <c r="Q62" s="54">
         <v>46287</v>
       </c>
-      <c r="R62" s="53" t="s">
-        <v>413</v>
+      <c r="R62" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="S62" s="53"/>
       <c r="T62" s="53"/>
@@ -10282,25 +10383,25 @@
     <mergeCell ref="A8:V8"/>
   </mergeCells>
   <conditionalFormatting sqref="P11:P210">
-    <cfRule type="expression" dxfId="6" priority="1">
+    <cfRule type="expression" dxfId="13" priority="1">
       <formula>P11="RECOMENDADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="2">
+    <cfRule type="expression" dxfId="12" priority="2">
       <formula>P11="APROVADA - AGUARDANDO EXECUÇÃO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="3">
+    <cfRule type="expression" dxfId="11" priority="3">
       <formula>P11="EXECUTADA - EM MATURAÇÃO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="10" priority="4">
       <formula>P11="EXECUTADA - AVALIADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="5">
+    <cfRule type="expression" dxfId="9" priority="5">
       <formula>P11="APROVADA - NÃO EXECUTADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="6">
+    <cfRule type="expression" dxfId="8" priority="6">
       <formula>P11="REJEITADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="7">
+    <cfRule type="expression" dxfId="7" priority="7">
       <formula>LEFT(P11,9)="BLOQUEADA"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
[O6 22/09] Registro: data de execucao 22/09 e formulas Q/R nas 20 linhas O6 (status ainda AGUARDANDO EXECUCAO)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -3213,7 +3213,7 @@
         <v>51</v>
       </c>
       <c r="Q11" s="16">
-        <f t="shared" ref="Q11:Q33" si="0">IF(E11="","",E11+1)</f>
+        <f t="shared" ref="Q11:Q74" si="0">IF(E11="","",E11+1)</f>
         <v>46252</v>
       </c>
       <c r="R11" s="17">
@@ -4784,7 +4784,8 @@
       <c r="P34" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="Q34" s="42">
+      <c r="Q34" s="18">
+        <f t="shared" si="0"/>
         <v>46270</v>
       </c>
       <c r="R34" s="19">
@@ -4853,7 +4854,8 @@
       <c r="P35" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="Q35" s="42">
+      <c r="Q35" s="18">
+        <f t="shared" si="0"/>
         <v>46270</v>
       </c>
       <c r="R35" s="19">
@@ -4922,7 +4924,8 @@
       <c r="P36" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="Q36" s="42">
+      <c r="Q36" s="18">
+        <f t="shared" si="0"/>
         <v>46275</v>
       </c>
       <c r="R36" s="19">
@@ -4991,7 +4994,8 @@
       <c r="P37" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="Q37" s="42">
+      <c r="Q37" s="18">
+        <f t="shared" si="0"/>
         <v>46275</v>
       </c>
       <c r="R37" s="19">
@@ -5060,7 +5064,8 @@
       <c r="P38" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="Q38" s="42">
+      <c r="Q38" s="18">
+        <f t="shared" si="0"/>
         <v>46275</v>
       </c>
       <c r="R38" s="19">
@@ -5129,7 +5134,8 @@
       <c r="P39" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="Q39" s="42">
+      <c r="Q39" s="18">
+        <f t="shared" si="0"/>
         <v>46275</v>
       </c>
       <c r="R39" s="19">
@@ -5198,7 +5204,8 @@
       <c r="P40" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="Q40" s="42">
+      <c r="Q40" s="18">
+        <f t="shared" si="0"/>
         <v>46275</v>
       </c>
       <c r="R40" s="19">
@@ -5267,7 +5274,8 @@
       <c r="P41" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="Q41" s="42">
+      <c r="Q41" s="18">
+        <f t="shared" si="0"/>
         <v>46275</v>
       </c>
       <c r="R41" s="19">
@@ -5336,7 +5344,8 @@
       <c r="P42" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="Q42" s="42">
+      <c r="Q42" s="18">
+        <f t="shared" si="0"/>
         <v>46275</v>
       </c>
       <c r="R42" s="19">
@@ -5405,11 +5414,12 @@
       <c r="P43" s="39" t="s">
         <v>47</v>
       </c>
-      <c r="Q43" s="42">
+      <c r="Q43" s="18">
+        <f t="shared" si="0"/>
         <v>46275</v>
       </c>
       <c r="R43" s="19">
-        <f t="shared" ref="R43:R74" ca="1" si="2">IF(E43="","",TODAY()-E43)</f>
+        <f t="shared" ref="R43:R82" ca="1" si="2">IF(E43="","",TODAY()-E43)</f>
         <v>13</v>
       </c>
       <c r="S43" t="s">
@@ -5474,7 +5484,8 @@
       <c r="P44" s="39" t="s">
         <v>47</v>
       </c>
-      <c r="Q44" s="42">
+      <c r="Q44" s="18">
+        <f t="shared" si="0"/>
         <v>46275</v>
       </c>
       <c r="R44" s="19">
@@ -5543,7 +5554,8 @@
       <c r="P45" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="Q45" s="42">
+      <c r="Q45" s="18">
+        <f t="shared" si="0"/>
         <v>46275</v>
       </c>
       <c r="R45" s="19">
@@ -5612,7 +5624,8 @@
       <c r="P46" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="Q46" s="42">
+      <c r="Q46" s="18">
+        <f t="shared" si="0"/>
         <v>46275</v>
       </c>
       <c r="R46" s="19">
@@ -5681,7 +5694,8 @@
       <c r="P47" s="39" t="s">
         <v>47</v>
       </c>
-      <c r="Q47" s="42">
+      <c r="Q47" s="18">
+        <f t="shared" si="0"/>
         <v>46275</v>
       </c>
       <c r="R47" s="19">
@@ -5748,7 +5762,10 @@
       <c r="P48" s="39" t="s">
         <v>55</v>
       </c>
-      <c r="Q48" s="39"/>
+      <c r="Q48" s="18" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="R48" s="19" t="str">
         <f t="shared" ca="1" si="2"/>
         <v/>
@@ -5815,7 +5832,8 @@
       <c r="P49" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="Q49" s="42">
+      <c r="Q49" s="18">
+        <f t="shared" si="0"/>
         <v>46275</v>
       </c>
       <c r="R49" s="19">
@@ -5884,7 +5902,8 @@
       <c r="P50" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="Q50" s="42">
+      <c r="Q50" s="18">
+        <f t="shared" si="0"/>
         <v>46275</v>
       </c>
       <c r="R50" s="19">
@@ -5953,7 +5972,8 @@
       <c r="P51" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="Q51" s="42">
+      <c r="Q51" s="18">
+        <f t="shared" si="0"/>
         <v>46275</v>
       </c>
       <c r="R51" s="19">
@@ -6022,7 +6042,8 @@
       <c r="P52" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="Q52" s="42">
+      <c r="Q52" s="18">
+        <f t="shared" si="0"/>
         <v>46275</v>
       </c>
       <c r="R52" s="19">
@@ -6091,8 +6112,9 @@
       <c r="P53" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="Q53" s="47">
-        <v>46287</v>
+      <c r="Q53" s="18">
+        <f t="shared" si="0"/>
+        <v>46284</v>
       </c>
       <c r="R53" s="19">
         <f t="shared" ca="1" si="2"/>
@@ -6160,8 +6182,9 @@
       <c r="P54" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="Q54" s="47">
-        <v>46287</v>
+      <c r="Q54" s="18">
+        <f t="shared" si="0"/>
+        <v>46284</v>
       </c>
       <c r="R54" s="19">
         <f t="shared" ca="1" si="2"/>
@@ -6229,8 +6252,9 @@
       <c r="P55" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="Q55" s="47">
-        <v>46287</v>
+      <c r="Q55" s="18">
+        <f t="shared" si="0"/>
+        <v>46284</v>
       </c>
       <c r="R55" s="19">
         <f t="shared" ca="1" si="2"/>
@@ -6298,8 +6322,9 @@
       <c r="P56" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="Q56" s="47">
-        <v>46287</v>
+      <c r="Q56" s="18">
+        <f t="shared" si="0"/>
+        <v>46284</v>
       </c>
       <c r="R56" s="19">
         <f t="shared" ca="1" si="2"/>
@@ -6367,8 +6392,9 @@
       <c r="P57" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="Q57" s="47">
-        <v>46287</v>
+      <c r="Q57" s="18">
+        <f t="shared" si="0"/>
+        <v>46284</v>
       </c>
       <c r="R57" s="19">
         <f t="shared" ca="1" si="2"/>
@@ -6436,8 +6462,9 @@
       <c r="P58" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="Q58" s="47">
-        <v>46287</v>
+      <c r="Q58" s="18">
+        <f t="shared" si="0"/>
+        <v>46284</v>
       </c>
       <c r="R58" s="19">
         <f t="shared" ca="1" si="2"/>
@@ -6505,8 +6532,9 @@
       <c r="P59" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="Q59" s="47">
-        <v>46287</v>
+      <c r="Q59" s="18">
+        <f t="shared" si="0"/>
+        <v>46284</v>
       </c>
       <c r="R59" s="19">
         <f t="shared" ca="1" si="2"/>
@@ -6574,8 +6602,9 @@
       <c r="P60" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="Q60" s="47">
-        <v>46287</v>
+      <c r="Q60" s="18">
+        <f t="shared" si="0"/>
+        <v>46284</v>
       </c>
       <c r="R60" s="19">
         <f t="shared" ca="1" si="2"/>
@@ -6643,8 +6672,9 @@
       <c r="P61" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="Q61" s="47">
-        <v>46287</v>
+      <c r="Q61" s="18">
+        <f t="shared" si="0"/>
+        <v>46284</v>
       </c>
       <c r="R61" s="19">
         <f t="shared" ca="1" si="2"/>
@@ -6712,8 +6742,9 @@
       <c r="P62" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="Q62" s="47">
-        <v>46287</v>
+      <c r="Q62" s="18">
+        <f t="shared" si="0"/>
+        <v>46284</v>
       </c>
       <c r="R62" s="19">
         <f t="shared" ca="1" si="2"/>
@@ -6745,6 +6776,9 @@
       <c r="D63" s="55">
         <v>46287</v>
       </c>
+      <c r="E63" s="55">
+        <v>46287</v>
+      </c>
       <c r="F63" t="s">
         <v>465</v>
       </c>
@@ -6777,6 +6811,14 @@
       </c>
       <c r="P63" t="s">
         <v>43</v>
+      </c>
+      <c r="Q63" s="18">
+        <f t="shared" si="0"/>
+        <v>46288</v>
+      </c>
+      <c r="R63" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="U63" t="s">
         <v>469</v>
@@ -6798,6 +6840,9 @@
       <c r="D64" s="55">
         <v>46287</v>
       </c>
+      <c r="E64" s="55">
+        <v>46287</v>
+      </c>
       <c r="F64" t="s">
         <v>110</v>
       </c>
@@ -6830,6 +6875,14 @@
       </c>
       <c r="P64" t="s">
         <v>43</v>
+      </c>
+      <c r="Q64" s="18">
+        <f t="shared" si="0"/>
+        <v>46288</v>
+      </c>
+      <c r="R64" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="U64" t="s">
         <v>474</v>
@@ -6851,6 +6904,9 @@
       <c r="D65" s="55">
         <v>46287</v>
       </c>
+      <c r="E65" s="55">
+        <v>46287</v>
+      </c>
       <c r="F65" t="s">
         <v>270</v>
       </c>
@@ -6883,6 +6939,14 @@
       </c>
       <c r="P65" t="s">
         <v>43</v>
+      </c>
+      <c r="Q65" s="18">
+        <f t="shared" si="0"/>
+        <v>46288</v>
+      </c>
+      <c r="R65" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="U65" t="s">
         <v>146</v>
@@ -6904,6 +6968,9 @@
       <c r="D66" s="55">
         <v>46287</v>
       </c>
+      <c r="E66" s="55">
+        <v>46287</v>
+      </c>
       <c r="F66" t="s">
         <v>270</v>
       </c>
@@ -6936,6 +7003,14 @@
       </c>
       <c r="P66" t="s">
         <v>43</v>
+      </c>
+      <c r="Q66" s="18">
+        <f t="shared" si="0"/>
+        <v>46288</v>
+      </c>
+      <c r="R66" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="U66" t="s">
         <v>469</v>
@@ -6957,6 +7032,9 @@
       <c r="D67" s="55">
         <v>46287</v>
       </c>
+      <c r="E67" s="55">
+        <v>46287</v>
+      </c>
       <c r="F67" t="s">
         <v>264</v>
       </c>
@@ -6989,6 +7067,14 @@
       </c>
       <c r="P67" t="s">
         <v>43</v>
+      </c>
+      <c r="Q67" s="18">
+        <f t="shared" si="0"/>
+        <v>46288</v>
+      </c>
+      <c r="R67" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="U67" t="s">
         <v>469</v>
@@ -7010,6 +7096,9 @@
       <c r="D68" s="55">
         <v>46287</v>
       </c>
+      <c r="E68" s="55">
+        <v>46287</v>
+      </c>
       <c r="F68" t="s">
         <v>264</v>
       </c>
@@ -7042,6 +7131,14 @@
       </c>
       <c r="P68" t="s">
         <v>43</v>
+      </c>
+      <c r="Q68" s="18">
+        <f t="shared" si="0"/>
+        <v>46288</v>
+      </c>
+      <c r="R68" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="U68" s="57">
         <v>46293</v>
@@ -7063,6 +7160,9 @@
       <c r="D69" s="55">
         <v>46287</v>
       </c>
+      <c r="E69" s="55">
+        <v>46287</v>
+      </c>
       <c r="F69" t="s">
         <v>112</v>
       </c>
@@ -7095,6 +7195,14 @@
       </c>
       <c r="P69" t="s">
         <v>43</v>
+      </c>
+      <c r="Q69" s="18">
+        <f t="shared" si="0"/>
+        <v>46288</v>
+      </c>
+      <c r="R69" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="U69" t="s">
         <v>146</v>
@@ -7116,6 +7224,9 @@
       <c r="D70" s="55">
         <v>46287</v>
       </c>
+      <c r="E70" s="55">
+        <v>46287</v>
+      </c>
       <c r="F70" t="s">
         <v>112</v>
       </c>
@@ -7148,6 +7259,14 @@
       </c>
       <c r="P70" t="s">
         <v>43</v>
+      </c>
+      <c r="Q70" s="18">
+        <f t="shared" si="0"/>
+        <v>46288</v>
+      </c>
+      <c r="R70" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="U70" t="s">
         <v>469</v>
@@ -7169,6 +7288,9 @@
       <c r="D71" s="55">
         <v>46287</v>
       </c>
+      <c r="E71" s="55">
+        <v>46287</v>
+      </c>
       <c r="F71" t="s">
         <v>112</v>
       </c>
@@ -7201,6 +7323,14 @@
       </c>
       <c r="P71" t="s">
         <v>43</v>
+      </c>
+      <c r="Q71" s="18">
+        <f t="shared" si="0"/>
+        <v>46288</v>
+      </c>
+      <c r="R71" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="U71" t="s">
         <v>146</v>
@@ -7222,6 +7352,9 @@
       <c r="D72" s="55">
         <v>46287</v>
       </c>
+      <c r="E72" s="55">
+        <v>46287</v>
+      </c>
       <c r="F72" t="s">
         <v>519</v>
       </c>
@@ -7254,6 +7387,14 @@
       </c>
       <c r="P72" t="s">
         <v>43</v>
+      </c>
+      <c r="Q72" s="18">
+        <f t="shared" si="0"/>
+        <v>46288</v>
+      </c>
+      <c r="R72" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="U72" t="s">
         <v>469</v>
@@ -7275,6 +7416,9 @@
       <c r="D73" s="55">
         <v>46287</v>
       </c>
+      <c r="E73" s="55">
+        <v>46287</v>
+      </c>
       <c r="F73" t="s">
         <v>527</v>
       </c>
@@ -7307,6 +7451,14 @@
       </c>
       <c r="P73" t="s">
         <v>43</v>
+      </c>
+      <c r="Q73" s="18">
+        <f t="shared" si="0"/>
+        <v>46288</v>
+      </c>
+      <c r="R73" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="U73" s="57">
         <v>46308</v>
@@ -7328,6 +7480,9 @@
       <c r="D74" s="55">
         <v>46287</v>
       </c>
+      <c r="E74" s="55">
+        <v>46287</v>
+      </c>
       <c r="F74" t="s">
         <v>527</v>
       </c>
@@ -7360,6 +7515,14 @@
       </c>
       <c r="P74" t="s">
         <v>43</v>
+      </c>
+      <c r="Q74" s="18">
+        <f t="shared" si="0"/>
+        <v>46288</v>
+      </c>
+      <c r="R74" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="U74" s="57">
         <v>46308</v>
@@ -7378,6 +7541,9 @@
       <c r="D75" s="55">
         <v>46287</v>
       </c>
+      <c r="E75" s="55">
+        <v>46287</v>
+      </c>
       <c r="F75" t="s">
         <v>527</v>
       </c>
@@ -7410,6 +7576,14 @@
       </c>
       <c r="P75" t="s">
         <v>43</v>
+      </c>
+      <c r="Q75" s="18">
+        <f t="shared" ref="Q75:Q82" si="3">IF(E75="","",E75+1)</f>
+        <v>46288</v>
+      </c>
+      <c r="R75" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="U75" s="57">
         <v>46308</v>
@@ -7431,6 +7605,9 @@
       <c r="D76" s="55">
         <v>46287</v>
       </c>
+      <c r="E76" s="55">
+        <v>46287</v>
+      </c>
       <c r="F76" t="s">
         <v>527</v>
       </c>
@@ -7463,6 +7640,14 @@
       </c>
       <c r="P76" t="s">
         <v>43</v>
+      </c>
+      <c r="Q76" s="18">
+        <f t="shared" si="3"/>
+        <v>46288</v>
+      </c>
+      <c r="R76" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="U76" s="57">
         <v>46308</v>
@@ -7481,6 +7666,9 @@
       <c r="D77" s="55">
         <v>46287</v>
       </c>
+      <c r="E77" s="55">
+        <v>46287</v>
+      </c>
       <c r="F77" t="s">
         <v>527</v>
       </c>
@@ -7513,6 +7701,14 @@
       </c>
       <c r="P77" t="s">
         <v>43</v>
+      </c>
+      <c r="Q77" s="18">
+        <f t="shared" si="3"/>
+        <v>46288</v>
+      </c>
+      <c r="R77" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="U77" s="57">
         <v>46308</v>
@@ -7534,6 +7730,9 @@
       <c r="D78" s="55">
         <v>46287</v>
       </c>
+      <c r="E78" s="55">
+        <v>46287</v>
+      </c>
       <c r="F78" t="s">
         <v>527</v>
       </c>
@@ -7566,6 +7765,14 @@
       </c>
       <c r="P78" t="s">
         <v>43</v>
+      </c>
+      <c r="Q78" s="18">
+        <f t="shared" si="3"/>
+        <v>46288</v>
+      </c>
+      <c r="R78" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="U78" s="57">
         <v>46308</v>
@@ -7587,6 +7794,9 @@
       <c r="D79" s="55">
         <v>46287</v>
       </c>
+      <c r="E79" s="55">
+        <v>46287</v>
+      </c>
       <c r="F79" t="s">
         <v>527</v>
       </c>
@@ -7619,6 +7829,14 @@
       </c>
       <c r="P79" t="s">
         <v>43</v>
+      </c>
+      <c r="Q79" s="18">
+        <f t="shared" si="3"/>
+        <v>46288</v>
+      </c>
+      <c r="R79" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="U79" s="57">
         <v>46308</v>
@@ -7640,6 +7858,9 @@
       <c r="D80" s="55">
         <v>46287</v>
       </c>
+      <c r="E80" s="55">
+        <v>46287</v>
+      </c>
       <c r="F80" t="s">
         <v>569</v>
       </c>
@@ -7672,6 +7893,14 @@
       </c>
       <c r="P80" t="s">
         <v>43</v>
+      </c>
+      <c r="Q80" s="18">
+        <f t="shared" si="3"/>
+        <v>46288</v>
+      </c>
+      <c r="R80" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="U80" t="s">
         <v>469</v>
@@ -7693,6 +7922,9 @@
       <c r="D81" s="55">
         <v>46287</v>
       </c>
+      <c r="E81" s="55">
+        <v>46287</v>
+      </c>
       <c r="F81" t="s">
         <v>264</v>
       </c>
@@ -7725,6 +7957,14 @@
       </c>
       <c r="P81" t="s">
         <v>43</v>
+      </c>
+      <c r="Q81" s="18">
+        <f t="shared" si="3"/>
+        <v>46288</v>
+      </c>
+      <c r="R81" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="U81" t="s">
         <v>469</v>
@@ -7746,6 +7986,9 @@
       <c r="D82" s="55">
         <v>46287</v>
       </c>
+      <c r="E82" s="55">
+        <v>46287</v>
+      </c>
       <c r="F82" t="s">
         <v>583</v>
       </c>
@@ -7778,6 +8021,14 @@
       </c>
       <c r="P82" t="s">
         <v>43</v>
+      </c>
+      <c r="Q82" s="18">
+        <f t="shared" si="3"/>
+        <v>46288</v>
+      </c>
+      <c r="R82" s="19">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
       </c>
       <c r="U82" t="s">
         <v>469</v>
@@ -7804,11 +8055,11 @@
       <c r="O83" s="11"/>
       <c r="P83" s="11"/>
       <c r="Q83" s="18" t="str">
-        <f t="shared" ref="Q75:Q106" si="3">IF(E83="","",E83+1)</f>
+        <f t="shared" ref="Q75:Q106" si="4">IF(E83="","",E83+1)</f>
         <v/>
       </c>
       <c r="R83" s="19" t="str">
-        <f t="shared" ref="R75:R106" ca="1" si="4">IF(E83="","",TODAY()-E83)</f>
+        <f t="shared" ref="R75:R106" ca="1" si="5">IF(E83="","",TODAY()-E83)</f>
         <v/>
       </c>
       <c r="S83" s="43"/>
@@ -7834,11 +8085,11 @@
       <c r="O84" s="11"/>
       <c r="P84" s="11"/>
       <c r="Q84" s="18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="R84" s="19" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
       <c r="S84" s="43"/>
@@ -7864,11 +8115,11 @@
       <c r="O85" s="11"/>
       <c r="P85" s="11"/>
       <c r="Q85" s="18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="R85" s="19" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
       <c r="S85" s="43"/>
@@ -7894,11 +8145,11 @@
       <c r="O86" s="11"/>
       <c r="P86" s="11"/>
       <c r="Q86" s="18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="R86" s="19" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
       <c r="S86" s="43"/>
@@ -7924,11 +8175,11 @@
       <c r="O87" s="11"/>
       <c r="P87" s="11"/>
       <c r="Q87" s="18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="R87" s="19" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
       <c r="S87" s="43"/>
@@ -7954,11 +8205,11 @@
       <c r="O88" s="11"/>
       <c r="P88" s="11"/>
       <c r="Q88" s="18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="R88" s="19" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
       <c r="S88" s="43"/>
@@ -7984,11 +8235,11 @@
       <c r="O89" s="11"/>
       <c r="P89" s="11"/>
       <c r="Q89" s="18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="R89" s="19" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
       <c r="S89" s="43"/>
@@ -8014,11 +8265,11 @@
       <c r="O90" s="11"/>
       <c r="P90" s="11"/>
       <c r="Q90" s="18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="R90" s="19" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
       <c r="S90" s="43"/>
@@ -8044,11 +8295,11 @@
       <c r="O91" s="11"/>
       <c r="P91" s="11"/>
       <c r="Q91" s="18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="R91" s="19" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
       <c r="S91" s="43"/>
@@ -8074,11 +8325,11 @@
       <c r="O92" s="11"/>
       <c r="P92" s="11"/>
       <c r="Q92" s="18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="R92" s="19" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
       <c r="S92" s="43"/>
@@ -8104,11 +8355,11 @@
       <c r="O93" s="11"/>
       <c r="P93" s="11"/>
       <c r="Q93" s="18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="R93" s="19" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
       <c r="S93" s="43"/>
@@ -8134,11 +8385,11 @@
       <c r="O94" s="11"/>
       <c r="P94" s="11"/>
       <c r="Q94" s="18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="R94" s="19" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
       <c r="S94" s="43"/>
@@ -8164,11 +8415,11 @@
       <c r="O95" s="11"/>
       <c r="P95" s="11"/>
       <c r="Q95" s="18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="R95" s="19" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
       <c r="S95" s="43"/>
@@ -8194,11 +8445,11 @@
       <c r="O96" s="11"/>
       <c r="P96" s="11"/>
       <c r="Q96" s="18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="R96" s="19" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
       <c r="S96" s="43"/>
@@ -8224,11 +8475,11 @@
       <c r="O97" s="11"/>
       <c r="P97" s="11"/>
       <c r="Q97" s="18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="R97" s="19" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
       <c r="S97" s="43"/>
@@ -8254,11 +8505,11 @@
       <c r="O98" s="11"/>
       <c r="P98" s="11"/>
       <c r="Q98" s="18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="R98" s="19" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
       <c r="S98" s="43"/>
@@ -8284,11 +8535,11 @@
       <c r="O99" s="11"/>
       <c r="P99" s="11"/>
       <c r="Q99" s="18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="R99" s="19" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
       <c r="S99" s="43"/>
@@ -8314,11 +8565,11 @@
       <c r="O100" s="11"/>
       <c r="P100" s="11"/>
       <c r="Q100" s="18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="R100" s="19" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
       <c r="S100" s="43"/>
@@ -8344,11 +8595,11 @@
       <c r="O101" s="11"/>
       <c r="P101" s="11"/>
       <c r="Q101" s="18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="R101" s="19" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
       <c r="S101" s="43"/>
@@ -8374,11 +8625,11 @@
       <c r="O102" s="11"/>
       <c r="P102" s="11"/>
       <c r="Q102" s="18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="R102" s="19" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
       <c r="S102" s="43"/>
@@ -8404,11 +8655,11 @@
       <c r="O103" s="11"/>
       <c r="P103" s="11"/>
       <c r="Q103" s="18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="R103" s="19" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
       <c r="S103" s="43"/>
@@ -8434,11 +8685,11 @@
       <c r="O104" s="11"/>
       <c r="P104" s="11"/>
       <c r="Q104" s="18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="R104" s="19" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
       <c r="S104" s="43"/>
@@ -8464,11 +8715,11 @@
       <c r="O105" s="11"/>
       <c r="P105" s="11"/>
       <c r="Q105" s="18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="R105" s="19" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
       <c r="S105" s="43"/>
@@ -8494,11 +8745,11 @@
       <c r="O106" s="11"/>
       <c r="P106" s="11"/>
       <c r="Q106" s="18" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="R106" s="19" t="str">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
       <c r="S106" s="43"/>
@@ -8524,11 +8775,11 @@
       <c r="O107" s="11"/>
       <c r="P107" s="11"/>
       <c r="Q107" s="18" t="str">
-        <f t="shared" ref="Q107:Q138" si="5">IF(E107="","",E107+1)</f>
+        <f t="shared" ref="Q107:Q138" si="6">IF(E107="","",E107+1)</f>
         <v/>
       </c>
       <c r="R107" s="19" t="str">
-        <f t="shared" ref="R107:R138" ca="1" si="6">IF(E107="","",TODAY()-E107)</f>
+        <f t="shared" ref="R107:R138" ca="1" si="7">IF(E107="","",TODAY()-E107)</f>
         <v/>
       </c>
       <c r="S107" s="43"/>
@@ -8554,11 +8805,11 @@
       <c r="O108" s="11"/>
       <c r="P108" s="11"/>
       <c r="Q108" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R108" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S108" s="43"/>
@@ -8584,11 +8835,11 @@
       <c r="O109" s="11"/>
       <c r="P109" s="11"/>
       <c r="Q109" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R109" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S109" s="43"/>
@@ -8614,11 +8865,11 @@
       <c r="O110" s="11"/>
       <c r="P110" s="11"/>
       <c r="Q110" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R110" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S110" s="43"/>
@@ -8644,11 +8895,11 @@
       <c r="O111" s="11"/>
       <c r="P111" s="11"/>
       <c r="Q111" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R111" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S111" s="43"/>
@@ -8674,11 +8925,11 @@
       <c r="O112" s="11"/>
       <c r="P112" s="11"/>
       <c r="Q112" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R112" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S112" s="43"/>
@@ -8704,11 +8955,11 @@
       <c r="O113" s="11"/>
       <c r="P113" s="11"/>
       <c r="Q113" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R113" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S113" s="43"/>
@@ -8734,11 +8985,11 @@
       <c r="O114" s="11"/>
       <c r="P114" s="11"/>
       <c r="Q114" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R114" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S114" s="43"/>
@@ -8764,11 +9015,11 @@
       <c r="O115" s="11"/>
       <c r="P115" s="11"/>
       <c r="Q115" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R115" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S115" s="43"/>
@@ -8794,11 +9045,11 @@
       <c r="O116" s="11"/>
       <c r="P116" s="11"/>
       <c r="Q116" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R116" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S116" s="43"/>
@@ -8824,11 +9075,11 @@
       <c r="O117" s="11"/>
       <c r="P117" s="11"/>
       <c r="Q117" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R117" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S117" s="43"/>
@@ -8854,11 +9105,11 @@
       <c r="O118" s="11"/>
       <c r="P118" s="11"/>
       <c r="Q118" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R118" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S118" s="43"/>
@@ -8884,11 +9135,11 @@
       <c r="O119" s="11"/>
       <c r="P119" s="11"/>
       <c r="Q119" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R119" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S119" s="43"/>
@@ -8914,11 +9165,11 @@
       <c r="O120" s="11"/>
       <c r="P120" s="11"/>
       <c r="Q120" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R120" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S120" s="43"/>
@@ -8944,11 +9195,11 @@
       <c r="O121" s="11"/>
       <c r="P121" s="11"/>
       <c r="Q121" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R121" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S121" s="43"/>
@@ -8974,11 +9225,11 @@
       <c r="O122" s="11"/>
       <c r="P122" s="11"/>
       <c r="Q122" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R122" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S122" s="43"/>
@@ -9004,11 +9255,11 @@
       <c r="O123" s="11"/>
       <c r="P123" s="11"/>
       <c r="Q123" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R123" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S123" s="43"/>
@@ -9034,11 +9285,11 @@
       <c r="O124" s="11"/>
       <c r="P124" s="11"/>
       <c r="Q124" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R124" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S124" s="43"/>
@@ -9064,11 +9315,11 @@
       <c r="O125" s="11"/>
       <c r="P125" s="11"/>
       <c r="Q125" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R125" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S125" s="43"/>
@@ -9094,11 +9345,11 @@
       <c r="O126" s="11"/>
       <c r="P126" s="11"/>
       <c r="Q126" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R126" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S126" s="43"/>
@@ -9124,11 +9375,11 @@
       <c r="O127" s="11"/>
       <c r="P127" s="11"/>
       <c r="Q127" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R127" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S127" s="43"/>
@@ -9154,11 +9405,11 @@
       <c r="O128" s="11"/>
       <c r="P128" s="11"/>
       <c r="Q128" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R128" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S128" s="43"/>
@@ -9184,11 +9435,11 @@
       <c r="O129" s="11"/>
       <c r="P129" s="11"/>
       <c r="Q129" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R129" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S129" s="43"/>
@@ -9214,11 +9465,11 @@
       <c r="O130" s="11"/>
       <c r="P130" s="11"/>
       <c r="Q130" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R130" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S130" s="43"/>
@@ -9244,11 +9495,11 @@
       <c r="O131" s="11"/>
       <c r="P131" s="11"/>
       <c r="Q131" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R131" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S131" s="43"/>
@@ -9274,11 +9525,11 @@
       <c r="O132" s="11"/>
       <c r="P132" s="11"/>
       <c r="Q132" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R132" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S132" s="43"/>
@@ -9304,11 +9555,11 @@
       <c r="O133" s="11"/>
       <c r="P133" s="11"/>
       <c r="Q133" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R133" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S133" s="43"/>
@@ -9334,11 +9585,11 @@
       <c r="O134" s="11"/>
       <c r="P134" s="11"/>
       <c r="Q134" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R134" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S134" s="43"/>
@@ -9364,11 +9615,11 @@
       <c r="O135" s="11"/>
       <c r="P135" s="11"/>
       <c r="Q135" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R135" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S135" s="43"/>
@@ -9394,11 +9645,11 @@
       <c r="O136" s="11"/>
       <c r="P136" s="11"/>
       <c r="Q136" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R136" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S136" s="43"/>
@@ -9424,11 +9675,11 @@
       <c r="O137" s="11"/>
       <c r="P137" s="11"/>
       <c r="Q137" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R137" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S137" s="43"/>
@@ -9454,11 +9705,11 @@
       <c r="O138" s="11"/>
       <c r="P138" s="11"/>
       <c r="Q138" s="18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R138" s="19" t="str">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S138" s="43"/>
@@ -9484,11 +9735,11 @@
       <c r="O139" s="11"/>
       <c r="P139" s="11"/>
       <c r="Q139" s="18" t="str">
-        <f t="shared" ref="Q139:Q170" si="7">IF(E139="","",E139+1)</f>
+        <f t="shared" ref="Q139:Q170" si="8">IF(E139="","",E139+1)</f>
         <v/>
       </c>
       <c r="R139" s="19" t="str">
-        <f t="shared" ref="R139:R170" ca="1" si="8">IF(E139="","",TODAY()-E139)</f>
+        <f t="shared" ref="R139:R170" ca="1" si="9">IF(E139="","",TODAY()-E139)</f>
         <v/>
       </c>
       <c r="S139" s="43"/>
@@ -9514,11 +9765,11 @@
       <c r="O140" s="11"/>
       <c r="P140" s="11"/>
       <c r="Q140" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R140" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S140" s="43"/>
@@ -9544,11 +9795,11 @@
       <c r="O141" s="11"/>
       <c r="P141" s="11"/>
       <c r="Q141" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R141" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S141" s="43"/>
@@ -9574,11 +9825,11 @@
       <c r="O142" s="11"/>
       <c r="P142" s="11"/>
       <c r="Q142" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R142" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S142" s="43"/>
@@ -9604,11 +9855,11 @@
       <c r="O143" s="11"/>
       <c r="P143" s="11"/>
       <c r="Q143" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R143" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S143" s="43"/>
@@ -9634,11 +9885,11 @@
       <c r="O144" s="11"/>
       <c r="P144" s="11"/>
       <c r="Q144" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R144" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S144" s="43"/>
@@ -9664,11 +9915,11 @@
       <c r="O145" s="11"/>
       <c r="P145" s="11"/>
       <c r="Q145" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R145" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S145" s="43"/>
@@ -9694,11 +9945,11 @@
       <c r="O146" s="11"/>
       <c r="P146" s="11"/>
       <c r="Q146" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R146" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S146" s="43"/>
@@ -9724,11 +9975,11 @@
       <c r="O147" s="11"/>
       <c r="P147" s="11"/>
       <c r="Q147" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R147" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S147" s="43"/>
@@ -9754,11 +10005,11 @@
       <c r="O148" s="11"/>
       <c r="P148" s="11"/>
       <c r="Q148" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R148" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S148" s="43"/>
@@ -9784,11 +10035,11 @@
       <c r="O149" s="11"/>
       <c r="P149" s="11"/>
       <c r="Q149" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R149" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S149" s="43"/>
@@ -9814,11 +10065,11 @@
       <c r="O150" s="11"/>
       <c r="P150" s="11"/>
       <c r="Q150" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R150" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S150" s="43"/>
@@ -9844,11 +10095,11 @@
       <c r="O151" s="11"/>
       <c r="P151" s="11"/>
       <c r="Q151" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R151" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S151" s="43"/>
@@ -9874,11 +10125,11 @@
       <c r="O152" s="11"/>
       <c r="P152" s="11"/>
       <c r="Q152" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R152" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S152" s="43"/>
@@ -9904,11 +10155,11 @@
       <c r="O153" s="11"/>
       <c r="P153" s="11"/>
       <c r="Q153" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R153" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S153" s="43"/>
@@ -9934,11 +10185,11 @@
       <c r="O154" s="11"/>
       <c r="P154" s="11"/>
       <c r="Q154" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R154" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S154" s="43"/>
@@ -9964,11 +10215,11 @@
       <c r="O155" s="11"/>
       <c r="P155" s="11"/>
       <c r="Q155" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R155" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S155" s="43"/>
@@ -9994,11 +10245,11 @@
       <c r="O156" s="11"/>
       <c r="P156" s="11"/>
       <c r="Q156" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R156" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S156" s="43"/>
@@ -10024,11 +10275,11 @@
       <c r="O157" s="11"/>
       <c r="P157" s="11"/>
       <c r="Q157" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R157" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S157" s="43"/>
@@ -10054,11 +10305,11 @@
       <c r="O158" s="11"/>
       <c r="P158" s="11"/>
       <c r="Q158" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R158" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S158" s="43"/>
@@ -10084,11 +10335,11 @@
       <c r="O159" s="11"/>
       <c r="P159" s="11"/>
       <c r="Q159" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R159" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S159" s="43"/>
@@ -10114,11 +10365,11 @@
       <c r="O160" s="11"/>
       <c r="P160" s="11"/>
       <c r="Q160" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R160" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S160" s="22"/>
@@ -10144,11 +10395,11 @@
       <c r="O161" s="11"/>
       <c r="P161" s="11"/>
       <c r="Q161" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R161" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S161" s="22"/>
@@ -10174,11 +10425,11 @@
       <c r="O162" s="11"/>
       <c r="P162" s="11"/>
       <c r="Q162" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R162" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S162" s="22"/>
@@ -10204,11 +10455,11 @@
       <c r="O163" s="11"/>
       <c r="P163" s="11"/>
       <c r="Q163" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R163" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S163" s="22"/>
@@ -10234,11 +10485,11 @@
       <c r="O164" s="11"/>
       <c r="P164" s="11"/>
       <c r="Q164" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R164" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S164" s="22"/>
@@ -10264,11 +10515,11 @@
       <c r="O165" s="11"/>
       <c r="P165" s="11"/>
       <c r="Q165" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R165" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S165" s="22"/>
@@ -10294,11 +10545,11 @@
       <c r="O166" s="11"/>
       <c r="P166" s="11"/>
       <c r="Q166" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R166" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S166" s="22"/>
@@ -10324,11 +10575,11 @@
       <c r="O167" s="11"/>
       <c r="P167" s="11"/>
       <c r="Q167" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R167" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S167" s="22"/>
@@ -10354,11 +10605,11 @@
       <c r="O168" s="11"/>
       <c r="P168" s="11"/>
       <c r="Q168" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R168" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S168" s="22"/>
@@ -10384,11 +10635,11 @@
       <c r="O169" s="11"/>
       <c r="P169" s="11"/>
       <c r="Q169" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R169" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S169" s="22"/>
@@ -10414,11 +10665,11 @@
       <c r="O170" s="11"/>
       <c r="P170" s="11"/>
       <c r="Q170" s="18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R170" s="19" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S170" s="22"/>
@@ -10444,11 +10695,11 @@
       <c r="O171" s="11"/>
       <c r="P171" s="11"/>
       <c r="Q171" s="18" t="str">
-        <f t="shared" ref="Q171:Q202" si="9">IF(E171="","",E171+1)</f>
+        <f t="shared" ref="Q171:Q202" si="10">IF(E171="","",E171+1)</f>
         <v/>
       </c>
       <c r="R171" s="19" t="str">
-        <f t="shared" ref="R171:R202" ca="1" si="10">IF(E171="","",TODAY()-E171)</f>
+        <f t="shared" ref="R171:R202" ca="1" si="11">IF(E171="","",TODAY()-E171)</f>
         <v/>
       </c>
       <c r="S171" s="22"/>
@@ -10474,11 +10725,11 @@
       <c r="O172" s="11"/>
       <c r="P172" s="11"/>
       <c r="Q172" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R172" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S172" s="22"/>
@@ -10504,11 +10755,11 @@
       <c r="O173" s="11"/>
       <c r="P173" s="11"/>
       <c r="Q173" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R173" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S173" s="22"/>
@@ -10534,11 +10785,11 @@
       <c r="O174" s="11"/>
       <c r="P174" s="11"/>
       <c r="Q174" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R174" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S174" s="22"/>
@@ -10564,11 +10815,11 @@
       <c r="O175" s="11"/>
       <c r="P175" s="11"/>
       <c r="Q175" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R175" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S175" s="22"/>
@@ -10594,11 +10845,11 @@
       <c r="O176" s="11"/>
       <c r="P176" s="11"/>
       <c r="Q176" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R176" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S176" s="22"/>
@@ -10624,11 +10875,11 @@
       <c r="O177" s="11"/>
       <c r="P177" s="11"/>
       <c r="Q177" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R177" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S177" s="22"/>
@@ -10654,11 +10905,11 @@
       <c r="O178" s="11"/>
       <c r="P178" s="11"/>
       <c r="Q178" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R178" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S178" s="22"/>
@@ -10684,11 +10935,11 @@
       <c r="O179" s="11"/>
       <c r="P179" s="11"/>
       <c r="Q179" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R179" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S179" s="22"/>
@@ -10714,11 +10965,11 @@
       <c r="O180" s="11"/>
       <c r="P180" s="11"/>
       <c r="Q180" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R180" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S180" s="22"/>
@@ -10744,11 +10995,11 @@
       <c r="O181" s="11"/>
       <c r="P181" s="11"/>
       <c r="Q181" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R181" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S181" s="22"/>
@@ -10774,11 +11025,11 @@
       <c r="O182" s="11"/>
       <c r="P182" s="11"/>
       <c r="Q182" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R182" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S182" s="22"/>
@@ -10804,11 +11055,11 @@
       <c r="O183" s="11"/>
       <c r="P183" s="11"/>
       <c r="Q183" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R183" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S183" s="22"/>
@@ -10834,11 +11085,11 @@
       <c r="O184" s="11"/>
       <c r="P184" s="11"/>
       <c r="Q184" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R184" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S184" s="22"/>
@@ -10864,11 +11115,11 @@
       <c r="O185" s="11"/>
       <c r="P185" s="11"/>
       <c r="Q185" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R185" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S185" s="22"/>
@@ -10894,11 +11145,11 @@
       <c r="O186" s="11"/>
       <c r="P186" s="11"/>
       <c r="Q186" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R186" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S186" s="22"/>
@@ -10924,11 +11175,11 @@
       <c r="O187" s="11"/>
       <c r="P187" s="11"/>
       <c r="Q187" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R187" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S187" s="22"/>
@@ -10954,11 +11205,11 @@
       <c r="O188" s="11"/>
       <c r="P188" s="11"/>
       <c r="Q188" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R188" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S188" s="22"/>
@@ -10984,11 +11235,11 @@
       <c r="O189" s="11"/>
       <c r="P189" s="11"/>
       <c r="Q189" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R189" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S189" s="22"/>
@@ -11014,11 +11265,11 @@
       <c r="O190" s="11"/>
       <c r="P190" s="11"/>
       <c r="Q190" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R190" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S190" s="22"/>
@@ -11044,11 +11295,11 @@
       <c r="O191" s="11"/>
       <c r="P191" s="11"/>
       <c r="Q191" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R191" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S191" s="22"/>
@@ -11074,11 +11325,11 @@
       <c r="O192" s="11"/>
       <c r="P192" s="11"/>
       <c r="Q192" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R192" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S192" s="22"/>
@@ -11104,11 +11355,11 @@
       <c r="O193" s="11"/>
       <c r="P193" s="11"/>
       <c r="Q193" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R193" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S193" s="22"/>
@@ -11134,11 +11385,11 @@
       <c r="O194" s="11"/>
       <c r="P194" s="11"/>
       <c r="Q194" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R194" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S194" s="22"/>
@@ -11164,11 +11415,11 @@
       <c r="O195" s="11"/>
       <c r="P195" s="11"/>
       <c r="Q195" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R195" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S195" s="22"/>
@@ -11194,11 +11445,11 @@
       <c r="O196" s="11"/>
       <c r="P196" s="11"/>
       <c r="Q196" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R196" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S196" s="22"/>
@@ -11224,11 +11475,11 @@
       <c r="O197" s="11"/>
       <c r="P197" s="11"/>
       <c r="Q197" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R197" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S197" s="22"/>
@@ -11254,11 +11505,11 @@
       <c r="O198" s="11"/>
       <c r="P198" s="11"/>
       <c r="Q198" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R198" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S198" s="22"/>
@@ -11284,11 +11535,11 @@
       <c r="O199" s="11"/>
       <c r="P199" s="11"/>
       <c r="Q199" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R199" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S199" s="22"/>
@@ -11314,11 +11565,11 @@
       <c r="O200" s="11"/>
       <c r="P200" s="11"/>
       <c r="Q200" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R200" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S200" s="22"/>
@@ -11344,11 +11595,11 @@
       <c r="O201" s="11"/>
       <c r="P201" s="11"/>
       <c r="Q201" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R201" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S201" s="22"/>
@@ -11374,11 +11625,11 @@
       <c r="O202" s="11"/>
       <c r="P202" s="11"/>
       <c r="Q202" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R202" s="19" t="str">
-        <f t="shared" ca="1" si="10"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S202" s="22"/>
@@ -11404,11 +11655,11 @@
       <c r="O203" s="11"/>
       <c r="P203" s="11"/>
       <c r="Q203" s="18" t="str">
-        <f t="shared" ref="Q203:Q210" si="11">IF(E203="","",E203+1)</f>
+        <f t="shared" ref="Q203:Q210" si="12">IF(E203="","",E203+1)</f>
         <v/>
       </c>
       <c r="R203" s="19" t="str">
-        <f t="shared" ref="R203:R210" ca="1" si="12">IF(E203="","",TODAY()-E203)</f>
+        <f t="shared" ref="R203:R210" ca="1" si="13">IF(E203="","",TODAY()-E203)</f>
         <v/>
       </c>
       <c r="S203" s="22"/>
@@ -11434,11 +11685,11 @@
       <c r="O204" s="11"/>
       <c r="P204" s="11"/>
       <c r="Q204" s="18" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="R204" s="19" t="str">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="13"/>
         <v/>
       </c>
       <c r="S204" s="22"/>
@@ -11464,11 +11715,11 @@
       <c r="O205" s="11"/>
       <c r="P205" s="11"/>
       <c r="Q205" s="18" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="R205" s="19" t="str">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="13"/>
         <v/>
       </c>
       <c r="S205" s="22"/>
@@ -11494,11 +11745,11 @@
       <c r="O206" s="11"/>
       <c r="P206" s="11"/>
       <c r="Q206" s="18" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="R206" s="19" t="str">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="13"/>
         <v/>
       </c>
       <c r="S206" s="22"/>
@@ -11524,11 +11775,11 @@
       <c r="O207" s="11"/>
       <c r="P207" s="11"/>
       <c r="Q207" s="18" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="R207" s="19" t="str">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="13"/>
         <v/>
       </c>
       <c r="S207" s="22"/>
@@ -11554,11 +11805,11 @@
       <c r="O208" s="11"/>
       <c r="P208" s="11"/>
       <c r="Q208" s="18" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="R208" s="19" t="str">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="13"/>
         <v/>
       </c>
       <c r="S208" s="22"/>
@@ -11584,11 +11835,11 @@
       <c r="O209" s="11"/>
       <c r="P209" s="11"/>
       <c r="Q209" s="18" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="R209" s="19" t="str">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="13"/>
         <v/>
       </c>
       <c r="S209" s="22"/>
@@ -11614,11 +11865,11 @@
       <c r="O210" s="14"/>
       <c r="P210" s="14"/>
       <c r="Q210" s="20" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="R210" s="21" t="str">
-        <f t="shared" ca="1" si="12"/>
+        <f t="shared" ca="1" si="13"/>
         <v/>
       </c>
       <c r="S210" s="23"/>

</xml_diff>

<commit_message>
[O6 22/09] Registro: 20 linhas O6 marcadas executadas pelo LEO; 5 linhas do Prime Day nao elegiveis a corrigir; decisao: esperar lista de 28/09
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -2270,6 +2270,9 @@
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="14" fontId="15" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2291,228 +2294,12 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
-  <dxfs count="35">
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9A3412"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFED7AA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF991B1B"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEE2E2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF374151"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF3F4F6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF166534"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDCFCE7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF3730A3"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE0E7FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF92400E"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEF3C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1E40AF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDBEAFE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9A3412"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFED7AA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF991B1B"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEE2E2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF374151"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF3F4F6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF166534"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDCFCE7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF3730A3"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE0E7FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF92400E"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEF3C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1E40AF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDBEAFE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9A3412"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFED7AA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF991B1B"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEE2E2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF374151"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF3F4F6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF166534"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDCFCE7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF3730A3"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE0E7FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF92400E"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEF3C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1E40AF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDBEAFE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="14">
     <dxf>
       <font>
         <b/>
@@ -2916,82 +2703,82 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
-      <c r="J1" s="48"/>
-      <c r="K1" s="48"/>
-      <c r="L1" s="48"/>
-      <c r="M1" s="48"/>
-      <c r="N1" s="48"/>
-      <c r="O1" s="48"/>
-      <c r="P1" s="48"/>
-      <c r="Q1" s="48"/>
-      <c r="R1" s="48"/>
-      <c r="S1" s="48"/>
-      <c r="T1" s="48"/>
-      <c r="U1" s="48"/>
-      <c r="V1" s="48"/>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
+      <c r="H1" s="51"/>
+      <c r="I1" s="51"/>
+      <c r="J1" s="51"/>
+      <c r="K1" s="51"/>
+      <c r="L1" s="51"/>
+      <c r="M1" s="51"/>
+      <c r="N1" s="51"/>
+      <c r="O1" s="51"/>
+      <c r="P1" s="51"/>
+      <c r="Q1" s="51"/>
+      <c r="R1" s="51"/>
+      <c r="S1" s="51"/>
+      <c r="T1" s="51"/>
+      <c r="U1" s="51"/>
+      <c r="V1" s="51"/>
     </row>
     <row r="2" spans="1:22" ht="30" customHeight="1">
-      <c r="A2" s="49" t="s">
+      <c r="A2" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
-      <c r="H2" s="49"/>
-      <c r="I2" s="49"/>
-      <c r="J2" s="49"/>
-      <c r="K2" s="49"/>
-      <c r="L2" s="49"/>
-      <c r="M2" s="49"/>
-      <c r="N2" s="49"/>
-      <c r="O2" s="49"/>
-      <c r="P2" s="49"/>
-      <c r="Q2" s="49"/>
-      <c r="R2" s="49"/>
-      <c r="S2" s="49"/>
-      <c r="T2" s="49"/>
-      <c r="U2" s="49"/>
-      <c r="V2" s="49"/>
+      <c r="B2" s="52"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="52"/>
+      <c r="J2" s="52"/>
+      <c r="K2" s="52"/>
+      <c r="L2" s="52"/>
+      <c r="M2" s="52"/>
+      <c r="N2" s="52"/>
+      <c r="O2" s="52"/>
+      <c r="P2" s="52"/>
+      <c r="Q2" s="52"/>
+      <c r="R2" s="52"/>
+      <c r="S2" s="52"/>
+      <c r="T2" s="52"/>
+      <c r="U2" s="52"/>
+      <c r="V2" s="52"/>
     </row>
     <row r="3" spans="1:22" ht="27.95" customHeight="1">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="50"/>
-      <c r="C3" s="50"/>
-      <c r="D3" s="50"/>
-      <c r="E3" s="50"/>
-      <c r="F3" s="50"/>
-      <c r="G3" s="50"/>
-      <c r="H3" s="50"/>
-      <c r="I3" s="50"/>
-      <c r="J3" s="50"/>
-      <c r="K3" s="50"/>
-      <c r="L3" s="50"/>
-      <c r="M3" s="50"/>
-      <c r="N3" s="50"/>
-      <c r="O3" s="50"/>
-      <c r="P3" s="50"/>
-      <c r="Q3" s="50"/>
-      <c r="R3" s="50"/>
-      <c r="S3" s="50"/>
-      <c r="T3" s="50"/>
-      <c r="U3" s="50"/>
-      <c r="V3" s="50"/>
+      <c r="B3" s="53"/>
+      <c r="C3" s="53"/>
+      <c r="D3" s="53"/>
+      <c r="E3" s="53"/>
+      <c r="F3" s="53"/>
+      <c r="G3" s="53"/>
+      <c r="H3" s="53"/>
+      <c r="I3" s="53"/>
+      <c r="J3" s="53"/>
+      <c r="K3" s="53"/>
+      <c r="L3" s="53"/>
+      <c r="M3" s="53"/>
+      <c r="N3" s="53"/>
+      <c r="O3" s="53"/>
+      <c r="P3" s="53"/>
+      <c r="Q3" s="53"/>
+      <c r="R3" s="53"/>
+      <c r="S3" s="53"/>
+      <c r="T3" s="53"/>
+      <c r="U3" s="53"/>
+      <c r="V3" s="53"/>
     </row>
     <row r="5" spans="1:22">
       <c r="A5" s="1" t="s">
@@ -3012,23 +2799,23 @@
       <c r="F5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H5" s="51" t="s">
+      <c r="H5" s="54" t="s">
         <v>9</v>
       </c>
-      <c r="I5" s="51"/>
-      <c r="J5" s="51"/>
-      <c r="K5" s="51"/>
-      <c r="L5" s="51"/>
-      <c r="M5" s="51"/>
-      <c r="N5" s="51"/>
-      <c r="O5" s="51"/>
-      <c r="P5" s="51"/>
-      <c r="Q5" s="51"/>
-      <c r="R5" s="51"/>
-      <c r="S5" s="51"/>
-      <c r="T5" s="51"/>
-      <c r="U5" s="51"/>
-      <c r="V5" s="51"/>
+      <c r="I5" s="54"/>
+      <c r="J5" s="54"/>
+      <c r="K5" s="54"/>
+      <c r="L5" s="54"/>
+      <c r="M5" s="54"/>
+      <c r="N5" s="54"/>
+      <c r="O5" s="54"/>
+      <c r="P5" s="54"/>
+      <c r="Q5" s="54"/>
+      <c r="R5" s="54"/>
+      <c r="S5" s="54"/>
+      <c r="T5" s="54"/>
+      <c r="U5" s="54"/>
+      <c r="V5" s="54"/>
     </row>
     <row r="6" spans="1:22" ht="26.1" customHeight="1">
       <c r="A6" s="2">
@@ -3041,7 +2828,7 @@
       </c>
       <c r="C6" s="3">
         <f>COUNTIF(O11:O210,"SIM")</f>
-        <v>51</v>
+        <v>71</v>
       </c>
       <c r="D6" s="3">
         <f>COUNTIF(P11:P210,"BLOQUEADA*")</f>
@@ -3049,53 +2836,53 @@
       </c>
       <c r="E6" s="3">
         <f>COUNTIF(P11:P210,"EXECUTADA - EM MATURAÇÃO")</f>
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="F6" s="4">
         <f>COUNTIF(P11:P210,"EXECUTADA - AVALIADA")</f>
         <v>38</v>
       </c>
-      <c r="H6" s="51"/>
-      <c r="I6" s="51"/>
-      <c r="J6" s="51"/>
-      <c r="K6" s="51"/>
-      <c r="L6" s="51"/>
-      <c r="M6" s="51"/>
-      <c r="N6" s="51"/>
-      <c r="O6" s="51"/>
-      <c r="P6" s="51"/>
-      <c r="Q6" s="51"/>
-      <c r="R6" s="51"/>
-      <c r="S6" s="51"/>
-      <c r="T6" s="51"/>
-      <c r="U6" s="51"/>
-      <c r="V6" s="51"/>
+      <c r="H6" s="54"/>
+      <c r="I6" s="54"/>
+      <c r="J6" s="54"/>
+      <c r="K6" s="54"/>
+      <c r="L6" s="54"/>
+      <c r="M6" s="54"/>
+      <c r="N6" s="54"/>
+      <c r="O6" s="54"/>
+      <c r="P6" s="54"/>
+      <c r="Q6" s="54"/>
+      <c r="R6" s="54"/>
+      <c r="S6" s="54"/>
+      <c r="T6" s="54"/>
+      <c r="U6" s="54"/>
+      <c r="V6" s="54"/>
     </row>
     <row r="8" spans="1:22" ht="21.95" customHeight="1">
-      <c r="A8" s="52" t="s">
+      <c r="A8" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="52"/>
-      <c r="C8" s="52"/>
-      <c r="D8" s="52"/>
-      <c r="E8" s="52"/>
-      <c r="F8" s="52"/>
-      <c r="G8" s="52"/>
-      <c r="H8" s="52"/>
-      <c r="I8" s="52"/>
-      <c r="J8" s="52"/>
-      <c r="K8" s="52"/>
-      <c r="L8" s="52"/>
-      <c r="M8" s="52"/>
-      <c r="N8" s="52"/>
-      <c r="O8" s="52"/>
-      <c r="P8" s="52"/>
-      <c r="Q8" s="52"/>
-      <c r="R8" s="52"/>
-      <c r="S8" s="52"/>
-      <c r="T8" s="52"/>
-      <c r="U8" s="52"/>
-      <c r="V8" s="52"/>
+      <c r="B8" s="55"/>
+      <c r="C8" s="55"/>
+      <c r="D8" s="55"/>
+      <c r="E8" s="55"/>
+      <c r="F8" s="55"/>
+      <c r="G8" s="55"/>
+      <c r="H8" s="55"/>
+      <c r="I8" s="55"/>
+      <c r="J8" s="55"/>
+      <c r="K8" s="55"/>
+      <c r="L8" s="55"/>
+      <c r="M8" s="55"/>
+      <c r="N8" s="55"/>
+      <c r="O8" s="55"/>
+      <c r="P8" s="55"/>
+      <c r="Q8" s="55"/>
+      <c r="R8" s="55"/>
+      <c r="S8" s="55"/>
+      <c r="T8" s="55"/>
+      <c r="U8" s="55"/>
+      <c r="V8" s="55"/>
     </row>
     <row r="10" spans="1:22" ht="38.1" customHeight="1">
       <c r="A10" s="5" t="s">
@@ -6770,13 +6557,13 @@
       <c r="B63" t="s">
         <v>464</v>
       </c>
-      <c r="C63" s="55">
+      <c r="C63" s="48">
         <v>46287</v>
       </c>
-      <c r="D63" s="55">
+      <c r="D63" s="48">
         <v>46287</v>
       </c>
-      <c r="E63" s="55">
+      <c r="E63" s="48">
         <v>46287</v>
       </c>
       <c r="F63" t="s">
@@ -6806,11 +6593,11 @@
       <c r="N63" t="s">
         <v>40</v>
       </c>
-      <c r="O63" t="s">
-        <v>44</v>
-      </c>
-      <c r="P63" t="s">
-        <v>43</v>
+      <c r="O63" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="P63" s="46" t="s">
+        <v>47</v>
       </c>
       <c r="Q63" s="18">
         <f t="shared" si="0"/>
@@ -6834,13 +6621,13 @@
       <c r="B64" t="s">
         <v>464</v>
       </c>
-      <c r="C64" s="55">
+      <c r="C64" s="48">
         <v>46287</v>
       </c>
-      <c r="D64" s="55">
+      <c r="D64" s="48">
         <v>46287</v>
       </c>
-      <c r="E64" s="55">
+      <c r="E64" s="48">
         <v>46287</v>
       </c>
       <c r="F64" t="s">
@@ -6870,11 +6657,11 @@
       <c r="N64" t="s">
         <v>40</v>
       </c>
-      <c r="O64" t="s">
-        <v>44</v>
-      </c>
-      <c r="P64" t="s">
-        <v>43</v>
+      <c r="O64" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="P64" s="46" t="s">
+        <v>47</v>
       </c>
       <c r="Q64" s="18">
         <f t="shared" si="0"/>
@@ -6898,13 +6685,13 @@
       <c r="B65" t="s">
         <v>464</v>
       </c>
-      <c r="C65" s="55">
+      <c r="C65" s="48">
         <v>46287</v>
       </c>
-      <c r="D65" s="55">
+      <c r="D65" s="48">
         <v>46287</v>
       </c>
-      <c r="E65" s="55">
+      <c r="E65" s="48">
         <v>46287</v>
       </c>
       <c r="F65" t="s">
@@ -6934,11 +6721,11 @@
       <c r="N65" t="s">
         <v>40</v>
       </c>
-      <c r="O65" t="s">
-        <v>44</v>
-      </c>
-      <c r="P65" t="s">
-        <v>43</v>
+      <c r="O65" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="P65" s="46" t="s">
+        <v>47</v>
       </c>
       <c r="Q65" s="18">
         <f t="shared" si="0"/>
@@ -6962,13 +6749,13 @@
       <c r="B66" t="s">
         <v>464</v>
       </c>
-      <c r="C66" s="55">
+      <c r="C66" s="48">
         <v>46287</v>
       </c>
-      <c r="D66" s="55">
+      <c r="D66" s="48">
         <v>46287</v>
       </c>
-      <c r="E66" s="55">
+      <c r="E66" s="48">
         <v>46287</v>
       </c>
       <c r="F66" t="s">
@@ -6998,11 +6785,11 @@
       <c r="N66" t="s">
         <v>40</v>
       </c>
-      <c r="O66" t="s">
-        <v>44</v>
-      </c>
-      <c r="P66" t="s">
-        <v>43</v>
+      <c r="O66" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="P66" s="46" t="s">
+        <v>47</v>
       </c>
       <c r="Q66" s="18">
         <f t="shared" si="0"/>
@@ -7026,13 +6813,13 @@
       <c r="B67" t="s">
         <v>464</v>
       </c>
-      <c r="C67" s="55">
+      <c r="C67" s="48">
         <v>46287</v>
       </c>
-      <c r="D67" s="55">
+      <c r="D67" s="48">
         <v>46287</v>
       </c>
-      <c r="E67" s="55">
+      <c r="E67" s="48">
         <v>46287</v>
       </c>
       <c r="F67" t="s">
@@ -7044,7 +6831,7 @@
       <c r="H67" t="s">
         <v>42</v>
       </c>
-      <c r="I67" s="56">
+      <c r="I67" s="49">
         <v>0.54</v>
       </c>
       <c r="J67" t="s">
@@ -7062,11 +6849,11 @@
       <c r="N67" t="s">
         <v>40</v>
       </c>
-      <c r="O67" t="s">
-        <v>44</v>
-      </c>
-      <c r="P67" t="s">
-        <v>43</v>
+      <c r="O67" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="P67" s="46" t="s">
+        <v>47</v>
       </c>
       <c r="Q67" s="18">
         <f t="shared" si="0"/>
@@ -7090,13 +6877,13 @@
       <c r="B68" t="s">
         <v>464</v>
       </c>
-      <c r="C68" s="55">
+      <c r="C68" s="48">
         <v>46287</v>
       </c>
-      <c r="D68" s="55">
+      <c r="D68" s="48">
         <v>46287</v>
       </c>
-      <c r="E68" s="55">
+      <c r="E68" s="48">
         <v>46287</v>
       </c>
       <c r="F68" t="s">
@@ -7126,11 +6913,11 @@
       <c r="N68" t="s">
         <v>40</v>
       </c>
-      <c r="O68" t="s">
-        <v>44</v>
-      </c>
-      <c r="P68" t="s">
-        <v>43</v>
+      <c r="O68" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="P68" s="46" t="s">
+        <v>47</v>
       </c>
       <c r="Q68" s="18">
         <f t="shared" si="0"/>
@@ -7140,7 +6927,7 @@
         <f t="shared" ca="1" si="2"/>
         <v>0</v>
       </c>
-      <c r="U68" s="57">
+      <c r="U68" s="50">
         <v>46293</v>
       </c>
       <c r="V68" t="s">
@@ -7154,13 +6941,13 @@
       <c r="B69" t="s">
         <v>464</v>
       </c>
-      <c r="C69" s="55">
+      <c r="C69" s="48">
         <v>46287</v>
       </c>
-      <c r="D69" s="55">
+      <c r="D69" s="48">
         <v>46287</v>
       </c>
-      <c r="E69" s="55">
+      <c r="E69" s="48">
         <v>46287</v>
       </c>
       <c r="F69" t="s">
@@ -7190,11 +6977,11 @@
       <c r="N69" t="s">
         <v>40</v>
       </c>
-      <c r="O69" t="s">
-        <v>44</v>
-      </c>
-      <c r="P69" t="s">
-        <v>43</v>
+      <c r="O69" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="P69" s="46" t="s">
+        <v>47</v>
       </c>
       <c r="Q69" s="18">
         <f t="shared" si="0"/>
@@ -7218,13 +7005,13 @@
       <c r="B70" t="s">
         <v>464</v>
       </c>
-      <c r="C70" s="55">
+      <c r="C70" s="48">
         <v>46287</v>
       </c>
-      <c r="D70" s="55">
+      <c r="D70" s="48">
         <v>46287</v>
       </c>
-      <c r="E70" s="55">
+      <c r="E70" s="48">
         <v>46287</v>
       </c>
       <c r="F70" t="s">
@@ -7254,11 +7041,11 @@
       <c r="N70" t="s">
         <v>40</v>
       </c>
-      <c r="O70" t="s">
-        <v>44</v>
-      </c>
-      <c r="P70" t="s">
-        <v>43</v>
+      <c r="O70" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="P70" s="46" t="s">
+        <v>47</v>
       </c>
       <c r="Q70" s="18">
         <f t="shared" si="0"/>
@@ -7282,13 +7069,13 @@
       <c r="B71" t="s">
         <v>464</v>
       </c>
-      <c r="C71" s="55">
+      <c r="C71" s="48">
         <v>46287</v>
       </c>
-      <c r="D71" s="55">
+      <c r="D71" s="48">
         <v>46287</v>
       </c>
-      <c r="E71" s="55">
+      <c r="E71" s="48">
         <v>46287</v>
       </c>
       <c r="F71" t="s">
@@ -7318,11 +7105,11 @@
       <c r="N71" t="s">
         <v>40</v>
       </c>
-      <c r="O71" t="s">
-        <v>44</v>
-      </c>
-      <c r="P71" t="s">
-        <v>43</v>
+      <c r="O71" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="P71" s="46" t="s">
+        <v>47</v>
       </c>
       <c r="Q71" s="18">
         <f t="shared" si="0"/>
@@ -7346,13 +7133,13 @@
       <c r="B72" t="s">
         <v>464</v>
       </c>
-      <c r="C72" s="55">
+      <c r="C72" s="48">
         <v>46287</v>
       </c>
-      <c r="D72" s="55">
+      <c r="D72" s="48">
         <v>46287</v>
       </c>
-      <c r="E72" s="55">
+      <c r="E72" s="48">
         <v>46287</v>
       </c>
       <c r="F72" t="s">
@@ -7382,11 +7169,11 @@
       <c r="N72" t="s">
         <v>40</v>
       </c>
-      <c r="O72" t="s">
-        <v>44</v>
-      </c>
-      <c r="P72" t="s">
-        <v>43</v>
+      <c r="O72" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="P72" s="46" t="s">
+        <v>47</v>
       </c>
       <c r="Q72" s="18">
         <f t="shared" si="0"/>
@@ -7410,13 +7197,13 @@
       <c r="B73" t="s">
         <v>464</v>
       </c>
-      <c r="C73" s="55">
+      <c r="C73" s="48">
         <v>46287</v>
       </c>
-      <c r="D73" s="55">
+      <c r="D73" s="48">
         <v>46287</v>
       </c>
-      <c r="E73" s="55">
+      <c r="E73" s="48">
         <v>46287</v>
       </c>
       <c r="F73" t="s">
@@ -7446,11 +7233,11 @@
       <c r="N73" t="s">
         <v>40</v>
       </c>
-      <c r="O73" t="s">
-        <v>44</v>
-      </c>
-      <c r="P73" t="s">
-        <v>43</v>
+      <c r="O73" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="P73" s="46" t="s">
+        <v>47</v>
       </c>
       <c r="Q73" s="18">
         <f t="shared" si="0"/>
@@ -7460,7 +7247,7 @@
         <f t="shared" ca="1" si="2"/>
         <v>0</v>
       </c>
-      <c r="U73" s="57">
+      <c r="U73" s="50">
         <v>46308</v>
       </c>
       <c r="V73" t="s">
@@ -7474,13 +7261,13 @@
       <c r="B74" t="s">
         <v>464</v>
       </c>
-      <c r="C74" s="55">
+      <c r="C74" s="48">
         <v>46287</v>
       </c>
-      <c r="D74" s="55">
+      <c r="D74" s="48">
         <v>46287</v>
       </c>
-      <c r="E74" s="55">
+      <c r="E74" s="48">
         <v>46287</v>
       </c>
       <c r="F74" t="s">
@@ -7510,11 +7297,11 @@
       <c r="N74" t="s">
         <v>40</v>
       </c>
-      <c r="O74" t="s">
-        <v>44</v>
-      </c>
-      <c r="P74" t="s">
-        <v>43</v>
+      <c r="O74" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="P74" s="46" t="s">
+        <v>47</v>
       </c>
       <c r="Q74" s="18">
         <f t="shared" si="0"/>
@@ -7524,7 +7311,7 @@
         <f t="shared" ca="1" si="2"/>
         <v>0</v>
       </c>
-      <c r="U74" s="57">
+      <c r="U74" s="50">
         <v>46308</v>
       </c>
     </row>
@@ -7535,13 +7322,13 @@
       <c r="B75" t="s">
         <v>464</v>
       </c>
-      <c r="C75" s="55">
+      <c r="C75" s="48">
         <v>46287</v>
       </c>
-      <c r="D75" s="55">
+      <c r="D75" s="48">
         <v>46287</v>
       </c>
-      <c r="E75" s="55">
+      <c r="E75" s="48">
         <v>46287</v>
       </c>
       <c r="F75" t="s">
@@ -7571,11 +7358,11 @@
       <c r="N75" t="s">
         <v>40</v>
       </c>
-      <c r="O75" t="s">
-        <v>44</v>
-      </c>
-      <c r="P75" t="s">
-        <v>43</v>
+      <c r="O75" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="P75" s="46" t="s">
+        <v>47</v>
       </c>
       <c r="Q75" s="18">
         <f t="shared" ref="Q75:Q82" si="3">IF(E75="","",E75+1)</f>
@@ -7585,7 +7372,7 @@
         <f t="shared" ca="1" si="2"/>
         <v>0</v>
       </c>
-      <c r="U75" s="57">
+      <c r="U75" s="50">
         <v>46308</v>
       </c>
       <c r="V75" t="s">
@@ -7599,13 +7386,13 @@
       <c r="B76" t="s">
         <v>464</v>
       </c>
-      <c r="C76" s="55">
+      <c r="C76" s="48">
         <v>46287</v>
       </c>
-      <c r="D76" s="55">
+      <c r="D76" s="48">
         <v>46287</v>
       </c>
-      <c r="E76" s="55">
+      <c r="E76" s="48">
         <v>46287</v>
       </c>
       <c r="F76" t="s">
@@ -7635,11 +7422,11 @@
       <c r="N76" t="s">
         <v>40</v>
       </c>
-      <c r="O76" t="s">
-        <v>44</v>
-      </c>
-      <c r="P76" t="s">
-        <v>43</v>
+      <c r="O76" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="P76" s="46" t="s">
+        <v>47</v>
       </c>
       <c r="Q76" s="18">
         <f t="shared" si="3"/>
@@ -7649,7 +7436,7 @@
         <f t="shared" ca="1" si="2"/>
         <v>0</v>
       </c>
-      <c r="U76" s="57">
+      <c r="U76" s="50">
         <v>46308</v>
       </c>
     </row>
@@ -7660,13 +7447,13 @@
       <c r="B77" t="s">
         <v>464</v>
       </c>
-      <c r="C77" s="55">
+      <c r="C77" s="48">
         <v>46287</v>
       </c>
-      <c r="D77" s="55">
+      <c r="D77" s="48">
         <v>46287</v>
       </c>
-      <c r="E77" s="55">
+      <c r="E77" s="48">
         <v>46287</v>
       </c>
       <c r="F77" t="s">
@@ -7696,11 +7483,11 @@
       <c r="N77" t="s">
         <v>40</v>
       </c>
-      <c r="O77" t="s">
-        <v>44</v>
-      </c>
-      <c r="P77" t="s">
-        <v>43</v>
+      <c r="O77" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="P77" s="46" t="s">
+        <v>47</v>
       </c>
       <c r="Q77" s="18">
         <f t="shared" si="3"/>
@@ -7710,7 +7497,7 @@
         <f t="shared" ca="1" si="2"/>
         <v>0</v>
       </c>
-      <c r="U77" s="57">
+      <c r="U77" s="50">
         <v>46308</v>
       </c>
       <c r="V77" t="s">
@@ -7724,13 +7511,13 @@
       <c r="B78" t="s">
         <v>464</v>
       </c>
-      <c r="C78" s="55">
+      <c r="C78" s="48">
         <v>46287</v>
       </c>
-      <c r="D78" s="55">
+      <c r="D78" s="48">
         <v>46287</v>
       </c>
-      <c r="E78" s="55">
+      <c r="E78" s="48">
         <v>46287</v>
       </c>
       <c r="F78" t="s">
@@ -7760,11 +7547,11 @@
       <c r="N78" t="s">
         <v>40</v>
       </c>
-      <c r="O78" t="s">
-        <v>44</v>
-      </c>
-      <c r="P78" t="s">
-        <v>43</v>
+      <c r="O78" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="P78" s="46" t="s">
+        <v>47</v>
       </c>
       <c r="Q78" s="18">
         <f t="shared" si="3"/>
@@ -7774,7 +7561,7 @@
         <f t="shared" ca="1" si="2"/>
         <v>0</v>
       </c>
-      <c r="U78" s="57">
+      <c r="U78" s="50">
         <v>46308</v>
       </c>
       <c r="V78" t="s">
@@ -7788,13 +7575,13 @@
       <c r="B79" t="s">
         <v>464</v>
       </c>
-      <c r="C79" s="55">
+      <c r="C79" s="48">
         <v>46287</v>
       </c>
-      <c r="D79" s="55">
+      <c r="D79" s="48">
         <v>46287</v>
       </c>
-      <c r="E79" s="55">
+      <c r="E79" s="48">
         <v>46287</v>
       </c>
       <c r="F79" t="s">
@@ -7824,11 +7611,11 @@
       <c r="N79" t="s">
         <v>40</v>
       </c>
-      <c r="O79" t="s">
-        <v>44</v>
-      </c>
-      <c r="P79" t="s">
-        <v>43</v>
+      <c r="O79" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="P79" s="46" t="s">
+        <v>47</v>
       </c>
       <c r="Q79" s="18">
         <f t="shared" si="3"/>
@@ -7838,7 +7625,7 @@
         <f t="shared" ca="1" si="2"/>
         <v>0</v>
       </c>
-      <c r="U79" s="57">
+      <c r="U79" s="50">
         <v>46308</v>
       </c>
       <c r="V79" t="s">
@@ -7852,13 +7639,13 @@
       <c r="B80" t="s">
         <v>464</v>
       </c>
-      <c r="C80" s="55">
+      <c r="C80" s="48">
         <v>46287</v>
       </c>
-      <c r="D80" s="55">
+      <c r="D80" s="48">
         <v>46287</v>
       </c>
-      <c r="E80" s="55">
+      <c r="E80" s="48">
         <v>46287</v>
       </c>
       <c r="F80" t="s">
@@ -7888,11 +7675,11 @@
       <c r="N80" t="s">
         <v>40</v>
       </c>
-      <c r="O80" t="s">
-        <v>44</v>
-      </c>
-      <c r="P80" t="s">
-        <v>43</v>
+      <c r="O80" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="P80" s="46" t="s">
+        <v>47</v>
       </c>
       <c r="Q80" s="18">
         <f t="shared" si="3"/>
@@ -7916,13 +7703,13 @@
       <c r="B81" t="s">
         <v>464</v>
       </c>
-      <c r="C81" s="55">
+      <c r="C81" s="48">
         <v>46287</v>
       </c>
-      <c r="D81" s="55">
+      <c r="D81" s="48">
         <v>46287</v>
       </c>
-      <c r="E81" s="55">
+      <c r="E81" s="48">
         <v>46287</v>
       </c>
       <c r="F81" t="s">
@@ -7952,11 +7739,11 @@
       <c r="N81" t="s">
         <v>40</v>
       </c>
-      <c r="O81" t="s">
-        <v>44</v>
-      </c>
-      <c r="P81" t="s">
-        <v>43</v>
+      <c r="O81" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="P81" s="46" t="s">
+        <v>47</v>
       </c>
       <c r="Q81" s="18">
         <f t="shared" si="3"/>
@@ -7980,13 +7767,13 @@
       <c r="B82" t="s">
         <v>464</v>
       </c>
-      <c r="C82" s="55">
+      <c r="C82" s="48">
         <v>46287</v>
       </c>
-      <c r="D82" s="55">
+      <c r="D82" s="48">
         <v>46287</v>
       </c>
-      <c r="E82" s="55">
+      <c r="E82" s="48">
         <v>46287</v>
       </c>
       <c r="F82" t="s">
@@ -8016,11 +7803,11 @@
       <c r="N82" t="s">
         <v>40</v>
       </c>
-      <c r="O82" t="s">
-        <v>44</v>
-      </c>
-      <c r="P82" t="s">
-        <v>43</v>
+      <c r="O82" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="P82" s="46" t="s">
+        <v>47</v>
       </c>
       <c r="Q82" s="18">
         <f t="shared" si="3"/>
@@ -8055,11 +7842,11 @@
       <c r="O83" s="11"/>
       <c r="P83" s="11"/>
       <c r="Q83" s="18" t="str">
-        <f t="shared" ref="Q75:Q106" si="4">IF(E83="","",E83+1)</f>
+        <f t="shared" ref="Q83:Q106" si="4">IF(E83="","",E83+1)</f>
         <v/>
       </c>
       <c r="R83" s="19" t="str">
-        <f t="shared" ref="R75:R106" ca="1" si="5">IF(E83="","",TODAY()-E83)</f>
+        <f t="shared" ref="R83:R106" ca="1" si="5">IF(E83="","",TODAY()-E83)</f>
         <v/>
       </c>
       <c r="S83" s="43"/>
@@ -11886,25 +11673,25 @@
     <mergeCell ref="A8:V8"/>
   </mergeCells>
   <conditionalFormatting sqref="P11:P210">
-    <cfRule type="expression" dxfId="34" priority="1">
+    <cfRule type="expression" dxfId="13" priority="1">
       <formula>P11="RECOMENDADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="33" priority="2">
+    <cfRule type="expression" dxfId="12" priority="2">
       <formula>P11="APROVADA - AGUARDANDO EXECUÇÃO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="32" priority="3">
+    <cfRule type="expression" dxfId="11" priority="3">
       <formula>P11="EXECUTADA - EM MATURAÇÃO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="31" priority="4">
+    <cfRule type="expression" dxfId="10" priority="4">
       <formula>P11="EXECUTADA - AVALIADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="30" priority="5">
+    <cfRule type="expression" dxfId="9" priority="5">
       <formula>P11="APROVADA - NÃO EXECUTADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="29" priority="6">
+    <cfRule type="expression" dxfId="8" priority="6">
       <formula>P11="REJEITADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="28" priority="7">
+    <cfRule type="expression" dxfId="7" priority="7">
       <formula>LEFT(P11,9)="BLOQUEADA"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11959,16 +11746,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.95" customHeight="1">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="56" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="53"/>
-      <c r="C1" s="53"/>
-      <c r="D1" s="53"/>
-      <c r="E1" s="53"/>
-      <c r="F1" s="53"/>
-      <c r="G1" s="53"/>
-      <c r="H1" s="53"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
     </row>
     <row r="3" spans="1:8" ht="15">
       <c r="A3" s="30" t="s">
@@ -12087,16 +11874,16 @@
       </c>
     </row>
     <row r="18" spans="1:8" ht="15">
-      <c r="A18" s="54" t="s">
+      <c r="A18" s="57" t="s">
         <v>64</v>
       </c>
-      <c r="B18" s="54"/>
-      <c r="C18" s="54"/>
-      <c r="D18" s="54"/>
-      <c r="E18" s="54"/>
-      <c r="F18" s="54"/>
-      <c r="G18" s="54"/>
-      <c r="H18" s="54"/>
+      <c r="B18" s="57"/>
+      <c r="C18" s="57"/>
+      <c r="D18" s="57"/>
+      <c r="E18" s="57"/>
+      <c r="F18" s="57"/>
+      <c r="G18" s="57"/>
+      <c r="H18" s="57"/>
     </row>
     <row r="19" spans="1:8" ht="29.25">
       <c r="A19" s="31" t="s">

</xml_diff>

<commit_message>
[O6 22/09] Prime Day: print confirma P3070 e PXP em Prime Big Deal Days 5-11/10; Registro 4a versao (O6-013 alterada por engano, a corrigir)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1190" uniqueCount="622">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1192" uniqueCount="624">
   <si>
     <t>REGISTRO DE ALTERAÇÕES — AMAZON ADS | WINNET METAIS</t>
   </si>
@@ -1631,9 +1631,6 @@
     <t>Converteu no 9.9 (3 un a −15%). Margem no preço da oferta 15,0% (Simulador SP Interior; piso 15%). Mínimo do evento 10% (LEO). Desconto no preço (EC-010) encerra 27/09 — sem empilhamento</t>
   </si>
   <si>
-    <t>Relâmpago vetada (EC-004). Conferir o preço de referência calculado pela Amazon na tela</t>
-  </si>
-  <si>
     <t>O6-012</t>
   </si>
   <si>
@@ -1664,9 +1661,6 @@
     <t>66 sessões em 10–20/09 (2º maior tráfego), margem 16,9% no preço da oferta (desconto máximo no piso 17,6%). Não está no desconto no preço</t>
   </si>
   <si>
-    <t>⚠️ Contamina a leitura de Ads da PI P3070 em 05–11/10 — descontar no gatilho O6-004</t>
-  </si>
-  <si>
     <t>O6-014</t>
   </si>
   <si>
@@ -1697,9 +1691,6 @@
     <t>26 sessões, maior ticket; margem 15,9% (máx. no piso 16,3%). EC-012 (10%) encerra 27/09</t>
   </si>
   <si>
-    <t>Classe Grandes: frete real = cobrado (sem subsídio de tabela)</t>
-  </si>
-  <si>
     <t>O6-016</t>
   </si>
   <si>
@@ -1715,9 +1706,6 @@
     <t>Opcional (aprovado em bloco no G11): 13 sessões, margem 17,8% (máx. no piso 14,0%). EC-015 encerra 27/09</t>
   </si>
   <si>
-    <t>LEO confirma na submissão se mantém</t>
-  </si>
-  <si>
     <t>O6-017</t>
   </si>
   <si>
@@ -1896,6 +1884,24 @@
   </si>
   <si>
     <t>NÃO AVALIÁVEL hoje. Primeira leitura 28/09 (sessões × conversão; primeira venda conferida pedido a pedido para fixar a regra de atribuição). Corte de série 23–27/09 a marcar na O7</t>
+  </si>
+  <si>
+    <t>não elegível na lista de 22/09; reconferir 28/09</t>
+  </si>
+  <si>
+    <t>não elegível na lista de 22/09; reconferir 28/10</t>
+  </si>
+  <si>
+    <t>não elegível na lista de 22/09; reconferir 28/11</t>
+  </si>
+  <si>
+    <t>não elegível na lista de 22/09; reconferir 28/12</t>
+  </si>
+  <si>
+    <t>não elegível na lista de 22/09; reconferir 28/13</t>
+  </si>
+  <si>
+    <t>não elegível na lista de 22/09; reconferir 28/14</t>
   </si>
 </sst>
 </file>
@@ -2299,7 +2305,78 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
-  <dxfs count="14">
+  <dxfs count="21">
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9A3412"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFED7AA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF991B1B"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF374151"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF3F4F6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF166534"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFDCFCE7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF3730A3"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFE0E7FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF92400E"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEF3C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1E40AF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFDBEAFE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -2828,7 +2905,7 @@
       </c>
       <c r="C6" s="3">
         <f>COUNTIF(O11:O210,"SIM")</f>
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="D6" s="3">
         <f>COUNTIF(P11:P210,"BLOQUEADA*")</f>
@@ -2836,7 +2913,7 @@
       </c>
       <c r="E6" s="3">
         <f>COUNTIF(P11:P210,"EXECUTADA - EM MATURAÇÃO")</f>
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="F6" s="4">
         <f>COUNTIF(P11:P210,"EXECUTADA - AVALIADA")</f>
@@ -4720,10 +4797,10 @@
         <v>13</v>
       </c>
       <c r="S36" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="T36" t="s">
-        <v>588</v>
+        <v>584</v>
       </c>
       <c r="U36" s="42">
         <v>46287</v>
@@ -4790,10 +4867,10 @@
         <v>13</v>
       </c>
       <c r="S37" t="s">
-        <v>589</v>
+        <v>585</v>
       </c>
       <c r="T37" t="s">
-        <v>590</v>
+        <v>586</v>
       </c>
       <c r="U37" s="42">
         <v>46287</v>
@@ -4860,10 +4937,10 @@
         <v>13</v>
       </c>
       <c r="S38" t="s">
-        <v>591</v>
+        <v>587</v>
       </c>
       <c r="T38" t="s">
-        <v>592</v>
+        <v>588</v>
       </c>
       <c r="U38" s="42">
         <v>46287</v>
@@ -4930,10 +5007,10 @@
         <v>13</v>
       </c>
       <c r="S39" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="T39" t="s">
-        <v>594</v>
+        <v>590</v>
       </c>
       <c r="U39" s="42">
         <v>46287</v>
@@ -5000,7 +5077,7 @@
         <v>13</v>
       </c>
       <c r="S40" t="s">
-        <v>595</v>
+        <v>591</v>
       </c>
       <c r="T40" t="s">
         <v>387</v>
@@ -5070,10 +5147,10 @@
         <v>13</v>
       </c>
       <c r="S41" t="s">
-        <v>596</v>
+        <v>592</v>
       </c>
       <c r="T41" t="s">
-        <v>597</v>
+        <v>593</v>
       </c>
       <c r="U41" s="42">
         <v>46287</v>
@@ -5140,10 +5217,10 @@
         <v>13</v>
       </c>
       <c r="S42" t="s">
-        <v>598</v>
+        <v>594</v>
       </c>
       <c r="T42" t="s">
-        <v>599</v>
+        <v>595</v>
       </c>
       <c r="U42" s="42">
         <v>46287</v>
@@ -5210,10 +5287,10 @@
         <v>13</v>
       </c>
       <c r="S43" t="s">
-        <v>600</v>
+        <v>596</v>
       </c>
       <c r="T43" t="s">
-        <v>601</v>
+        <v>597</v>
       </c>
       <c r="U43" s="42">
         <v>46308</v>
@@ -5280,10 +5357,10 @@
         <v>13</v>
       </c>
       <c r="S44" t="s">
-        <v>602</v>
+        <v>598</v>
       </c>
       <c r="T44" t="s">
-        <v>603</v>
+        <v>599</v>
       </c>
       <c r="U44" s="42">
         <v>46308</v>
@@ -5350,10 +5427,10 @@
         <v>13</v>
       </c>
       <c r="S45" t="s">
-        <v>604</v>
+        <v>600</v>
       </c>
       <c r="T45" t="s">
-        <v>605</v>
+        <v>601</v>
       </c>
       <c r="U45" s="42">
         <v>46287</v>
@@ -5420,10 +5497,10 @@
         <v>13</v>
       </c>
       <c r="S46" t="s">
-        <v>606</v>
+        <v>602</v>
       </c>
       <c r="T46" t="s">
-        <v>607</v>
+        <v>603</v>
       </c>
       <c r="U46" s="42">
         <v>46279</v>
@@ -5490,10 +5567,10 @@
         <v>13</v>
       </c>
       <c r="S47" t="s">
-        <v>608</v>
+        <v>604</v>
       </c>
       <c r="T47" t="s">
-        <v>609</v>
+        <v>605</v>
       </c>
       <c r="U47" s="39" t="s">
         <v>342</v>
@@ -5558,10 +5635,10 @@
         <v/>
       </c>
       <c r="S48" t="s">
-        <v>610</v>
+        <v>606</v>
       </c>
       <c r="T48" t="s">
-        <v>611</v>
+        <v>607</v>
       </c>
       <c r="U48" s="42">
         <v>46287</v>
@@ -5628,10 +5705,10 @@
         <v>13</v>
       </c>
       <c r="S49" t="s">
-        <v>612</v>
+        <v>608</v>
       </c>
       <c r="T49" t="s">
-        <v>613</v>
+        <v>609</v>
       </c>
       <c r="U49" s="42">
         <v>46279</v>
@@ -5698,10 +5775,10 @@
         <v>13</v>
       </c>
       <c r="S50" t="s">
-        <v>614</v>
+        <v>610</v>
       </c>
       <c r="T50" t="s">
-        <v>615</v>
+        <v>611</v>
       </c>
       <c r="U50" s="42">
         <v>46287</v>
@@ -5768,10 +5845,10 @@
         <v>13</v>
       </c>
       <c r="S51" t="s">
-        <v>616</v>
+        <v>612</v>
       </c>
       <c r="T51" t="s">
-        <v>617</v>
+        <v>613</v>
       </c>
       <c r="U51" s="42">
         <v>46287</v>
@@ -5838,10 +5915,10 @@
         <v>13</v>
       </c>
       <c r="S52" t="s">
-        <v>618</v>
+        <v>614</v>
       </c>
       <c r="T52" t="s">
-        <v>619</v>
+        <v>615</v>
       </c>
       <c r="U52" s="42">
         <v>46287</v>
@@ -5908,10 +5985,10 @@
         <v>4</v>
       </c>
       <c r="S53" t="s">
-        <v>620</v>
+        <v>616</v>
       </c>
       <c r="T53" t="s">
-        <v>621</v>
+        <v>617</v>
       </c>
       <c r="U53" s="47">
         <v>46293</v>
@@ -5978,10 +6055,10 @@
         <v>4</v>
       </c>
       <c r="S54" t="s">
-        <v>620</v>
+        <v>616</v>
       </c>
       <c r="T54" t="s">
-        <v>621</v>
+        <v>617</v>
       </c>
       <c r="U54" s="47">
         <v>46293</v>
@@ -6048,10 +6125,10 @@
         <v>4</v>
       </c>
       <c r="S55" t="s">
-        <v>620</v>
+        <v>616</v>
       </c>
       <c r="T55" t="s">
-        <v>621</v>
+        <v>617</v>
       </c>
       <c r="U55" s="47">
         <v>46293</v>
@@ -6118,10 +6195,10 @@
         <v>4</v>
       </c>
       <c r="S56" t="s">
-        <v>620</v>
+        <v>616</v>
       </c>
       <c r="T56" t="s">
-        <v>621</v>
+        <v>617</v>
       </c>
       <c r="U56" s="47">
         <v>46293</v>
@@ -6188,10 +6265,10 @@
         <v>4</v>
       </c>
       <c r="S57" t="s">
-        <v>620</v>
+        <v>616</v>
       </c>
       <c r="T57" t="s">
-        <v>621</v>
+        <v>617</v>
       </c>
       <c r="U57" s="47">
         <v>46293</v>
@@ -6258,10 +6335,10 @@
         <v>4</v>
       </c>
       <c r="S58" t="s">
-        <v>620</v>
+        <v>616</v>
       </c>
       <c r="T58" t="s">
-        <v>621</v>
+        <v>617</v>
       </c>
       <c r="U58" s="47">
         <v>46293</v>
@@ -6328,10 +6405,10 @@
         <v>4</v>
       </c>
       <c r="S59" t="s">
-        <v>620</v>
+        <v>616</v>
       </c>
       <c r="T59" t="s">
-        <v>621</v>
+        <v>617</v>
       </c>
       <c r="U59" s="47">
         <v>46293</v>
@@ -6398,10 +6475,10 @@
         <v>4</v>
       </c>
       <c r="S60" t="s">
-        <v>620</v>
+        <v>616</v>
       </c>
       <c r="T60" t="s">
-        <v>621</v>
+        <v>617</v>
       </c>
       <c r="U60" s="47">
         <v>46293</v>
@@ -6468,10 +6545,10 @@
         <v>4</v>
       </c>
       <c r="S61" t="s">
-        <v>620</v>
+        <v>616</v>
       </c>
       <c r="T61" t="s">
-        <v>621</v>
+        <v>617</v>
       </c>
       <c r="U61" s="47">
         <v>46293</v>
@@ -6538,10 +6615,10 @@
         <v>4</v>
       </c>
       <c r="S62" t="s">
-        <v>620</v>
+        <v>616</v>
       </c>
       <c r="T62" t="s">
-        <v>621</v>
+        <v>617</v>
       </c>
       <c r="U62" s="47">
         <v>46293</v>
@@ -7234,10 +7311,10 @@
         <v>40</v>
       </c>
       <c r="O73" s="46" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="P73" s="46" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="Q73" s="18">
         <f t="shared" si="0"/>
@@ -7248,15 +7325,15 @@
         <v>0</v>
       </c>
       <c r="U73" s="50">
-        <v>46308</v>
+        <v>46293</v>
       </c>
       <c r="V73" t="s">
-        <v>533</v>
+        <v>618</v>
       </c>
     </row>
     <row r="74" spans="1:22">
       <c r="A74" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B74" t="s">
         <v>464</v>
@@ -7274,19 +7351,19 @@
         <v>527</v>
       </c>
       <c r="G74" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="H74" t="s">
         <v>529</v>
       </c>
       <c r="I74" t="s">
+        <v>535</v>
+      </c>
+      <c r="J74" t="s">
         <v>536</v>
       </c>
-      <c r="J74" t="s">
+      <c r="K74" t="s">
         <v>537</v>
-      </c>
-      <c r="K74" t="s">
-        <v>538</v>
       </c>
       <c r="L74" t="s">
         <v>468</v>
@@ -7298,10 +7375,10 @@
         <v>40</v>
       </c>
       <c r="O74" s="46" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="P74" s="46" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="Q74" s="18">
         <f t="shared" si="0"/>
@@ -7312,12 +7389,15 @@
         <v>0</v>
       </c>
       <c r="U74" s="50">
-        <v>46308</v>
+        <v>46293</v>
+      </c>
+      <c r="V74" t="s">
+        <v>619</v>
       </c>
     </row>
     <row r="75" spans="1:22">
       <c r="A75" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="B75" t="s">
         <v>464</v>
@@ -7335,19 +7415,19 @@
         <v>527</v>
       </c>
       <c r="G75" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="H75" t="s">
         <v>529</v>
       </c>
       <c r="I75" t="s">
+        <v>540</v>
+      </c>
+      <c r="J75" t="s">
         <v>541</v>
       </c>
-      <c r="J75" t="s">
+      <c r="K75" t="s">
         <v>542</v>
-      </c>
-      <c r="K75" t="s">
-        <v>543</v>
       </c>
       <c r="L75" t="s">
         <v>468</v>
@@ -7359,10 +7439,10 @@
         <v>40</v>
       </c>
       <c r="O75" s="46" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="P75" s="46" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="Q75" s="18">
         <f t="shared" ref="Q75:Q82" si="3">IF(E75="","",E75+1)</f>
@@ -7373,15 +7453,15 @@
         <v>0</v>
       </c>
       <c r="U75" s="50">
-        <v>46308</v>
+        <v>46293</v>
       </c>
       <c r="V75" t="s">
-        <v>544</v>
+        <v>620</v>
       </c>
     </row>
     <row r="76" spans="1:22">
       <c r="A76" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="B76" t="s">
         <v>464</v>
@@ -7399,19 +7479,19 @@
         <v>527</v>
       </c>
       <c r="G76" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="H76" t="s">
         <v>529</v>
       </c>
       <c r="I76" t="s">
+        <v>545</v>
+      </c>
+      <c r="J76" t="s">
+        <v>546</v>
+      </c>
+      <c r="K76" t="s">
         <v>547</v>
-      </c>
-      <c r="J76" t="s">
-        <v>548</v>
-      </c>
-      <c r="K76" t="s">
-        <v>549</v>
       </c>
       <c r="L76" t="s">
         <v>468</v>
@@ -7423,10 +7503,10 @@
         <v>40</v>
       </c>
       <c r="O76" s="46" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="P76" s="46" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="Q76" s="18">
         <f t="shared" si="3"/>
@@ -7437,12 +7517,15 @@
         <v>0</v>
       </c>
       <c r="U76" s="50">
-        <v>46308</v>
+        <v>46293</v>
+      </c>
+      <c r="V76" t="s">
+        <v>621</v>
       </c>
     </row>
     <row r="77" spans="1:22">
       <c r="A77" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="B77" t="s">
         <v>464</v>
@@ -7460,19 +7543,19 @@
         <v>527</v>
       </c>
       <c r="G77" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="H77" t="s">
         <v>529</v>
       </c>
       <c r="I77" t="s">
+        <v>550</v>
+      </c>
+      <c r="J77" t="s">
+        <v>551</v>
+      </c>
+      <c r="K77" t="s">
         <v>552</v>
-      </c>
-      <c r="J77" t="s">
-        <v>553</v>
-      </c>
-      <c r="K77" t="s">
-        <v>554</v>
       </c>
       <c r="L77" t="s">
         <v>468</v>
@@ -7484,10 +7567,10 @@
         <v>40</v>
       </c>
       <c r="O77" s="46" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="P77" s="46" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="Q77" s="18">
         <f t="shared" si="3"/>
@@ -7498,15 +7581,15 @@
         <v>0</v>
       </c>
       <c r="U77" s="50">
-        <v>46308</v>
+        <v>46293</v>
       </c>
       <c r="V77" t="s">
-        <v>555</v>
+        <v>622</v>
       </c>
     </row>
     <row r="78" spans="1:22">
       <c r="A78" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
       <c r="B78" t="s">
         <v>464</v>
@@ -7524,19 +7607,19 @@
         <v>527</v>
       </c>
       <c r="G78" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="H78" t="s">
         <v>529</v>
       </c>
       <c r="I78" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
       <c r="J78" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="K78" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
       <c r="L78" t="s">
         <v>468</v>
@@ -7548,10 +7631,10 @@
         <v>40</v>
       </c>
       <c r="O78" s="46" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="P78" s="46" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="Q78" s="18">
         <f t="shared" si="3"/>
@@ -7562,15 +7645,15 @@
         <v>0</v>
       </c>
       <c r="U78" s="50">
-        <v>46308</v>
+        <v>46293</v>
       </c>
       <c r="V78" t="s">
-        <v>561</v>
+        <v>623</v>
       </c>
     </row>
     <row r="79" spans="1:22">
       <c r="A79" t="s">
-        <v>562</v>
+        <v>558</v>
       </c>
       <c r="B79" t="s">
         <v>464</v>
@@ -7588,19 +7671,19 @@
         <v>527</v>
       </c>
       <c r="G79" t="s">
-        <v>563</v>
+        <v>559</v>
       </c>
       <c r="H79" t="s">
         <v>529</v>
       </c>
       <c r="I79" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
       <c r="J79" t="s">
-        <v>565</v>
+        <v>561</v>
       </c>
       <c r="K79" t="s">
-        <v>566</v>
+        <v>562</v>
       </c>
       <c r="L79" t="s">
         <v>468</v>
@@ -7629,12 +7712,12 @@
         <v>46308</v>
       </c>
       <c r="V79" t="s">
-        <v>567</v>
+        <v>563</v>
       </c>
     </row>
     <row r="80" spans="1:22">
       <c r="A80" t="s">
-        <v>568</v>
+        <v>564</v>
       </c>
       <c r="B80" t="s">
         <v>464</v>
@@ -7649,22 +7732,22 @@
         <v>46287</v>
       </c>
       <c r="F80" t="s">
+        <v>565</v>
+      </c>
+      <c r="G80" t="s">
+        <v>566</v>
+      </c>
+      <c r="H80" t="s">
+        <v>567</v>
+      </c>
+      <c r="I80" t="s">
+        <v>568</v>
+      </c>
+      <c r="J80" t="s">
         <v>569</v>
       </c>
-      <c r="G80" t="s">
+      <c r="K80" t="s">
         <v>570</v>
-      </c>
-      <c r="H80" t="s">
-        <v>571</v>
-      </c>
-      <c r="I80" t="s">
-        <v>572</v>
-      </c>
-      <c r="J80" t="s">
-        <v>573</v>
-      </c>
-      <c r="K80" t="s">
-        <v>574</v>
       </c>
       <c r="L80" t="s">
         <v>468</v>
@@ -7693,12 +7776,12 @@
         <v>469</v>
       </c>
       <c r="V80" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
     </row>
     <row r="81" spans="1:22">
       <c r="A81" t="s">
-        <v>576</v>
+        <v>572</v>
       </c>
       <c r="B81" t="s">
         <v>464</v>
@@ -7716,19 +7799,19 @@
         <v>264</v>
       </c>
       <c r="G81" t="s">
-        <v>577</v>
+        <v>573</v>
       </c>
       <c r="H81" t="s">
         <v>506</v>
       </c>
       <c r="I81" t="s">
-        <v>578</v>
+        <v>574</v>
       </c>
       <c r="J81" t="s">
-        <v>579</v>
+        <v>575</v>
       </c>
       <c r="K81" t="s">
-        <v>580</v>
+        <v>576</v>
       </c>
       <c r="L81" t="s">
         <v>468</v>
@@ -7757,12 +7840,12 @@
         <v>469</v>
       </c>
       <c r="V81" t="s">
-        <v>581</v>
+        <v>577</v>
       </c>
     </row>
     <row r="82" spans="1:22">
       <c r="A82" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="B82" t="s">
         <v>464</v>
@@ -7777,7 +7860,7 @@
         <v>46287</v>
       </c>
       <c r="F82" t="s">
-        <v>583</v>
+        <v>579</v>
       </c>
       <c r="G82" t="s">
         <v>146</v>
@@ -7786,13 +7869,13 @@
         <v>138</v>
       </c>
       <c r="I82" t="s">
-        <v>584</v>
+        <v>580</v>
       </c>
       <c r="J82" t="s">
         <v>515</v>
       </c>
       <c r="K82" t="s">
-        <v>585</v>
+        <v>581</v>
       </c>
       <c r="L82" t="s">
         <v>468</v>
@@ -7821,7 +7904,7 @@
         <v>469</v>
       </c>
       <c r="V82" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
     </row>
     <row r="83" spans="1:22">
@@ -11673,25 +11756,25 @@
     <mergeCell ref="A8:V8"/>
   </mergeCells>
   <conditionalFormatting sqref="P11:P210">
-    <cfRule type="expression" dxfId="13" priority="1">
+    <cfRule type="expression" dxfId="20" priority="1">
       <formula>P11="RECOMENDADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="2">
+    <cfRule type="expression" dxfId="19" priority="2">
       <formula>P11="APROVADA - AGUARDANDO EXECUÇÃO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="3">
+    <cfRule type="expression" dxfId="18" priority="3">
       <formula>P11="EXECUTADA - EM MATURAÇÃO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="4">
+    <cfRule type="expression" dxfId="17" priority="4">
       <formula>P11="EXECUTADA - AVALIADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="5">
+    <cfRule type="expression" dxfId="16" priority="5">
       <formula>P11="APROVADA - NÃO EXECUTADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="6">
+    <cfRule type="expression" dxfId="15" priority="6">
       <formula>P11="REJEITADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="7">
+    <cfRule type="expression" dxfId="14" priority="7">
       <formula>LEFT(P11,9)="BLOQUEADA"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
[O6 22/09] Registro corrigido: 5 linhas do Prime Day aguardando lista de 28/09, O6-013 restaurada; 72 entradas
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1192" uniqueCount="624">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1192" uniqueCount="620">
   <si>
     <t>REGISTRO DE ALTERAÇÕES — AMAZON ADS | WINNET METAIS</t>
   </si>
@@ -1661,6 +1661,9 @@
     <t>66 sessões em 10–20/09 (2º maior tráfego), margem 16,9% no preço da oferta (desconto máximo no piso 17,6%). Não está no desconto no preço</t>
   </si>
   <si>
+    <t>⚠️ Contamina a leitura de Ads da PI P3070 em 05–11/10 — descontar no gatilho O6-004</t>
+  </si>
+  <si>
     <t>O6-014</t>
   </si>
   <si>
@@ -1887,21 +1890,6 @@
   </si>
   <si>
     <t>não elegível na lista de 22/09; reconferir 28/09</t>
-  </si>
-  <si>
-    <t>não elegível na lista de 22/09; reconferir 28/10</t>
-  </si>
-  <si>
-    <t>não elegível na lista de 22/09; reconferir 28/11</t>
-  </si>
-  <si>
-    <t>não elegível na lista de 22/09; reconferir 28/12</t>
-  </si>
-  <si>
-    <t>não elegível na lista de 22/09; reconferir 28/13</t>
-  </si>
-  <si>
-    <t>não elegível na lista de 22/09; reconferir 28/14</t>
   </si>
 </sst>
 </file>
@@ -2905,7 +2893,7 @@
       </c>
       <c r="C6" s="3">
         <f>COUNTIF(O11:O210,"SIM")</f>
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D6" s="3">
         <f>COUNTIF(P11:P210,"BLOQUEADA*")</f>
@@ -2913,7 +2901,7 @@
       </c>
       <c r="E6" s="3">
         <f>COUNTIF(P11:P210,"EXECUTADA - EM MATURAÇÃO")</f>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F6" s="4">
         <f>COUNTIF(P11:P210,"EXECUTADA - AVALIADA")</f>
@@ -4797,10 +4785,10 @@
         <v>13</v>
       </c>
       <c r="S36" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="T36" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="U36" s="42">
         <v>46287</v>
@@ -4867,10 +4855,10 @@
         <v>13</v>
       </c>
       <c r="S37" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="T37" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="U37" s="42">
         <v>46287</v>
@@ -4937,10 +4925,10 @@
         <v>13</v>
       </c>
       <c r="S38" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="T38" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="U38" s="42">
         <v>46287</v>
@@ -5007,10 +4995,10 @@
         <v>13</v>
       </c>
       <c r="S39" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="T39" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="U39" s="42">
         <v>46287</v>
@@ -5077,7 +5065,7 @@
         <v>13</v>
       </c>
       <c r="S40" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="T40" t="s">
         <v>387</v>
@@ -5147,10 +5135,10 @@
         <v>13</v>
       </c>
       <c r="S41" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="T41" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="U41" s="42">
         <v>46287</v>
@@ -5217,10 +5205,10 @@
         <v>13</v>
       </c>
       <c r="S42" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="T42" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="U42" s="42">
         <v>46287</v>
@@ -5287,10 +5275,10 @@
         <v>13</v>
       </c>
       <c r="S43" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="T43" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="U43" s="42">
         <v>46308</v>
@@ -5357,10 +5345,10 @@
         <v>13</v>
       </c>
       <c r="S44" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="T44" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="U44" s="42">
         <v>46308</v>
@@ -5427,10 +5415,10 @@
         <v>13</v>
       </c>
       <c r="S45" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="T45" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="U45" s="42">
         <v>46287</v>
@@ -5497,10 +5485,10 @@
         <v>13</v>
       </c>
       <c r="S46" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="T46" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="U46" s="42">
         <v>46279</v>
@@ -5567,10 +5555,10 @@
         <v>13</v>
       </c>
       <c r="S47" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="T47" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="U47" s="39" t="s">
         <v>342</v>
@@ -5635,10 +5623,10 @@
         <v/>
       </c>
       <c r="S48" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="T48" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="U48" s="42">
         <v>46287</v>
@@ -5705,10 +5693,10 @@
         <v>13</v>
       </c>
       <c r="S49" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="T49" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="U49" s="42">
         <v>46279</v>
@@ -5775,10 +5763,10 @@
         <v>13</v>
       </c>
       <c r="S50" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="T50" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="U50" s="42">
         <v>46287</v>
@@ -5845,10 +5833,10 @@
         <v>13</v>
       </c>
       <c r="S51" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="T51" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="U51" s="42">
         <v>46287</v>
@@ -5915,10 +5903,10 @@
         <v>13</v>
       </c>
       <c r="S52" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="T52" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="U52" s="42">
         <v>46287</v>
@@ -5985,10 +5973,10 @@
         <v>4</v>
       </c>
       <c r="S53" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="T53" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="U53" s="47">
         <v>46293</v>
@@ -6055,10 +6043,10 @@
         <v>4</v>
       </c>
       <c r="S54" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="T54" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="U54" s="47">
         <v>46293</v>
@@ -6125,10 +6113,10 @@
         <v>4</v>
       </c>
       <c r="S55" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="T55" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="U55" s="47">
         <v>46293</v>
@@ -6195,10 +6183,10 @@
         <v>4</v>
       </c>
       <c r="S56" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="T56" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="U56" s="47">
         <v>46293</v>
@@ -6265,10 +6253,10 @@
         <v>4</v>
       </c>
       <c r="S57" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="T57" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="U57" s="47">
         <v>46293</v>
@@ -6335,10 +6323,10 @@
         <v>4</v>
       </c>
       <c r="S58" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="T58" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="U58" s="47">
         <v>46293</v>
@@ -6405,10 +6393,10 @@
         <v>4</v>
       </c>
       <c r="S59" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="T59" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="U59" s="47">
         <v>46293</v>
@@ -6475,10 +6463,10 @@
         <v>4</v>
       </c>
       <c r="S60" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="T60" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="U60" s="47">
         <v>46293</v>
@@ -6545,10 +6533,10 @@
         <v>4</v>
       </c>
       <c r="S61" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="T61" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="U61" s="47">
         <v>46293</v>
@@ -6615,10 +6603,10 @@
         <v>4</v>
       </c>
       <c r="S62" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="T62" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="U62" s="47">
         <v>46293</v>
@@ -7280,9 +7268,7 @@
       <c r="D73" s="48">
         <v>46287</v>
       </c>
-      <c r="E73" s="48">
-        <v>46287</v>
-      </c>
+      <c r="E73" s="48"/>
       <c r="F73" t="s">
         <v>527</v>
       </c>
@@ -7316,19 +7302,19 @@
       <c r="P73" s="46" t="s">
         <v>43</v>
       </c>
-      <c r="Q73" s="18">
+      <c r="Q73" s="18" t="str">
         <f t="shared" si="0"/>
-        <v>46288</v>
-      </c>
-      <c r="R73" s="19">
+        <v/>
+      </c>
+      <c r="R73" s="19" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v/>
       </c>
       <c r="U73" s="50">
         <v>46293</v>
       </c>
       <c r="V73" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
     </row>
     <row r="74" spans="1:22">
@@ -7344,9 +7330,7 @@
       <c r="D74" s="48">
         <v>46287</v>
       </c>
-      <c r="E74" s="48">
-        <v>46287</v>
-      </c>
+      <c r="E74" s="48"/>
       <c r="F74" t="s">
         <v>527</v>
       </c>
@@ -7380,13 +7364,13 @@
       <c r="P74" s="46" t="s">
         <v>43</v>
       </c>
-      <c r="Q74" s="18">
+      <c r="Q74" s="18" t="str">
         <f t="shared" si="0"/>
-        <v>46288</v>
-      </c>
-      <c r="R74" s="19">
+        <v/>
+      </c>
+      <c r="R74" s="19" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v/>
       </c>
       <c r="U74" s="50">
         <v>46293</v>
@@ -7408,9 +7392,7 @@
       <c r="D75" s="48">
         <v>46287</v>
       </c>
-      <c r="E75" s="48">
-        <v>46287</v>
-      </c>
+      <c r="E75" s="48"/>
       <c r="F75" t="s">
         <v>527</v>
       </c>
@@ -7439,29 +7421,29 @@
         <v>40</v>
       </c>
       <c r="O75" s="46" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="P75" s="46" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q75" s="18">
+        <v>47</v>
+      </c>
+      <c r="Q75" s="18" t="str">
         <f t="shared" ref="Q75:Q82" si="3">IF(E75="","",E75+1)</f>
-        <v>46288</v>
-      </c>
-      <c r="R75" s="19">
+        <v/>
+      </c>
+      <c r="R75" s="19" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v/>
       </c>
       <c r="U75" s="50">
-        <v>46293</v>
+        <v>46308</v>
       </c>
       <c r="V75" t="s">
-        <v>620</v>
+        <v>543</v>
       </c>
     </row>
     <row r="76" spans="1:22">
       <c r="A76" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B76" t="s">
         <v>464</v>
@@ -7472,26 +7454,24 @@
       <c r="D76" s="48">
         <v>46287</v>
       </c>
-      <c r="E76" s="48">
-        <v>46287</v>
-      </c>
+      <c r="E76" s="48"/>
       <c r="F76" t="s">
         <v>527</v>
       </c>
       <c r="G76" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="H76" t="s">
         <v>529</v>
       </c>
       <c r="I76" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="J76" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="K76" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="L76" t="s">
         <v>468</v>
@@ -7508,24 +7488,24 @@
       <c r="P76" s="46" t="s">
         <v>43</v>
       </c>
-      <c r="Q76" s="18">
+      <c r="Q76" s="18" t="str">
         <f t="shared" si="3"/>
-        <v>46288</v>
-      </c>
-      <c r="R76" s="19">
+        <v/>
+      </c>
+      <c r="R76" s="19" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v/>
       </c>
       <c r="U76" s="50">
         <v>46293</v>
       </c>
       <c r="V76" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
     </row>
     <row r="77" spans="1:22">
       <c r="A77" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="B77" t="s">
         <v>464</v>
@@ -7536,26 +7516,24 @@
       <c r="D77" s="48">
         <v>46287</v>
       </c>
-      <c r="E77" s="48">
-        <v>46287</v>
-      </c>
+      <c r="E77" s="48"/>
       <c r="F77" t="s">
         <v>527</v>
       </c>
       <c r="G77" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="H77" t="s">
         <v>529</v>
       </c>
       <c r="I77" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="J77" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="K77" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="L77" t="s">
         <v>468</v>
@@ -7572,24 +7550,24 @@
       <c r="P77" s="46" t="s">
         <v>43</v>
       </c>
-      <c r="Q77" s="18">
+      <c r="Q77" s="18" t="str">
         <f t="shared" si="3"/>
-        <v>46288</v>
-      </c>
-      <c r="R77" s="19">
+        <v/>
+      </c>
+      <c r="R77" s="19" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v/>
       </c>
       <c r="U77" s="50">
         <v>46293</v>
       </c>
       <c r="V77" t="s">
-        <v>622</v>
+        <v>619</v>
       </c>
     </row>
     <row r="78" spans="1:22">
       <c r="A78" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="B78" t="s">
         <v>464</v>
@@ -7600,26 +7578,24 @@
       <c r="D78" s="48">
         <v>46287</v>
       </c>
-      <c r="E78" s="48">
-        <v>46287</v>
-      </c>
+      <c r="E78" s="48"/>
       <c r="F78" t="s">
         <v>527</v>
       </c>
       <c r="G78" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="H78" t="s">
         <v>529</v>
       </c>
       <c r="I78" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="J78" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="K78" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="L78" t="s">
         <v>468</v>
@@ -7636,24 +7612,24 @@
       <c r="P78" s="46" t="s">
         <v>43</v>
       </c>
-      <c r="Q78" s="18">
+      <c r="Q78" s="18" t="str">
         <f t="shared" si="3"/>
-        <v>46288</v>
-      </c>
-      <c r="R78" s="19">
+        <v/>
+      </c>
+      <c r="R78" s="19" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v/>
       </c>
       <c r="U78" s="50">
         <v>46293</v>
       </c>
       <c r="V78" t="s">
-        <v>623</v>
+        <v>619</v>
       </c>
     </row>
     <row r="79" spans="1:22">
       <c r="A79" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="B79" t="s">
         <v>464</v>
@@ -7671,19 +7647,19 @@
         <v>527</v>
       </c>
       <c r="G79" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="H79" t="s">
         <v>529</v>
       </c>
       <c r="I79" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="J79" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="K79" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="L79" t="s">
         <v>468</v>
@@ -7712,12 +7688,12 @@
         <v>46308</v>
       </c>
       <c r="V79" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
     </row>
     <row r="80" spans="1:22">
       <c r="A80" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="B80" t="s">
         <v>464</v>
@@ -7732,22 +7708,22 @@
         <v>46287</v>
       </c>
       <c r="F80" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="G80" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="H80" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="I80" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="J80" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="K80" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="L80" t="s">
         <v>468</v>
@@ -7776,12 +7752,12 @@
         <v>469</v>
       </c>
       <c r="V80" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
     <row r="81" spans="1:22">
       <c r="A81" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="B81" t="s">
         <v>464</v>
@@ -7799,19 +7775,19 @@
         <v>264</v>
       </c>
       <c r="G81" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="H81" t="s">
         <v>506</v>
       </c>
       <c r="I81" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="J81" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="K81" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="L81" t="s">
         <v>468</v>
@@ -7840,12 +7816,12 @@
         <v>469</v>
       </c>
       <c r="V81" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
     </row>
     <row r="82" spans="1:22">
       <c r="A82" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="B82" t="s">
         <v>464</v>
@@ -7860,7 +7836,7 @@
         <v>46287</v>
       </c>
       <c r="F82" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="G82" t="s">
         <v>146</v>
@@ -7869,13 +7845,13 @@
         <v>138</v>
       </c>
       <c r="I82" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="J82" t="s">
         <v>515</v>
       </c>
       <c r="K82" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="L82" t="s">
         <v>468</v>
@@ -7904,7 +7880,7 @@
         <v>469</v>
       </c>
       <c r="V82" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
     </row>
     <row r="83" spans="1:22">

</xml_diff>

<commit_message>
[O6 22/09] Registro fechado: data da O6-013 restaurada; 72 entradas conferidas
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -7392,7 +7392,9 @@
       <c r="D75" s="48">
         <v>46287</v>
       </c>
-      <c r="E75" s="48"/>
+      <c r="E75" s="48">
+        <v>46287</v>
+      </c>
       <c r="F75" t="s">
         <v>527</v>
       </c>
@@ -7426,13 +7428,13 @@
       <c r="P75" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="Q75" s="18" t="str">
+      <c r="Q75" s="18">
         <f t="shared" ref="Q75:Q82" si="3">IF(E75="","",E75+1)</f>
-        <v/>
-      </c>
-      <c r="R75" s="19" t="str">
+        <v>46288</v>
+      </c>
+      <c r="R75" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="U75" s="50">
         <v>46308</v>

</xml_diff>

<commit_message>
[Monitoramento 28/09] decisoes do LEO: nao recriar desconto; L1618-T e L2025-T no Prime Day a 5% (EC-017/018 propostas); Q2460-B a pausar na Geral; Registro com vereditos EC-007..016 conferido
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1192" uniqueCount="620">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2340" uniqueCount="638">
   <si>
     <t>REGISTRO DE ALTERAÇÕES — AMAZON ADS | WINNET METAIS</t>
   </si>
@@ -1890,6 +1890,60 @@
   </si>
   <si>
     <t>não elegível na lista de 22/09; reconferir 28/09</t>
+  </si>
+  <si>
+    <t>Semana 21–27/09 (painel TESTEDESCONTONOPRECO, Terminado): 2 un vendidas · R$ 220,40 · 41 visualizações no painel · conversão 4,9%. Total dos 10 SKUs: 7 un · R$ 1.187,20 · 166 visualizações · 4,2%. Desconto não gera tráfego (esperado); converteu em 2 de 10 SKUs.</t>
+  </si>
+  <si>
+    <t>POSITIVO — 2 un a R$ 110,20 em 27 sessões (BR 22–27/09); única lixeira que converteu. Regra de atribuição fixada com este SKU (Ads a preço com desconto).</t>
+  </si>
+  <si>
+    <t>Semana 21–27/09 (painel TESTEDESCONTONOPRECO, Terminado): 0 un · 38 visualizações. Total dos 10 SKUs: 7 un · R$ 1.187,20 · 166 visualizações · 4,2%. Desconto não gera tráfego (esperado); converteu em 2 de 10 SKUs.</t>
+  </si>
+  <si>
+    <t>SEM EFEITO — 0 venda em 26 sessões / 38 visualizações a −5%; maior tráfego do catálogo não converteu nem com oferta (9.9) nem com desconto no preço.</t>
+  </si>
+  <si>
+    <t>Semana 21–27/09 (painel TESTEDESCONTONOPRECO, Terminado): 0 un · 13 visualizações. Total dos 10 SKUs: 7 un · R$ 1.187,20 · 166 visualizações · 4,2%. Desconto não gera tráfego (esperado); converteu em 2 de 10 SKUs.</t>
+  </si>
+  <si>
+    <t>SEM EFEITO — 0 venda em 7 sessões / 13 visualizações; tráfego caiu (23 → 7 sessões/sem). Segue inscrito no Prime Day a −10%.</t>
+  </si>
+  <si>
+    <t>Semana 21–27/09 (painel TESTEDESCONTONOPRECO, Terminado): 5 un · R$ 966,80 · 10 visualizações · conversão 50%. Total dos 10 SKUs: 7 un · R$ 1.187,20 · 166 visualizações · 4,2%. Desconto não gera tráfego (esperado); converteu em 2 de 10 SKUs.</t>
+  </si>
+  <si>
+    <t>POSITIVO — 5 un em 2 pedidos (2 + 3) a R$ 193,36; converte com qualquer desconto (9.9: 3 un a −15%; agora 5 a −5%). No pedido de 3 a promoção de quantidade empilhou (−R$ 29,00) → margem 15,6% realizada.</t>
+  </si>
+  <si>
+    <t>Semana 21–27/09 (painel TESTEDESCONTONOPRECO, Terminado): 0 un · 12 visualizações · 0%. Total dos 10 SKUs: 7 un · R$ 1.187,20 · 166 visualizações · 4,2%. Desconto não gera tráfego (esperado); converteu em 2 de 10 SKUs.</t>
+  </si>
+  <si>
+    <t>NEGATIVO — 0 venda em 9 sessões / 12 visualizações; rodou sem preço riscado (sem preço de referência). Gatilho O6-006 disparou → pausar o anúncio do SKU na Geral (decisão do LEO).</t>
+  </si>
+  <si>
+    <t>Semana 21–27/09 (painel TESTEDESCONTONOPRECO, Terminado): 0 un · 18 visualizações. Total dos 10 SKUs: 7 un · R$ 1.187,20 · 166 visualizações · 4,2%. Desconto não gera tráfego (esperado); converteu em 2 de 10 SKUs.</t>
+  </si>
+  <si>
+    <t>SEM EFEITO — 0 venda em 13 sessões / 18 visualizações.</t>
+  </si>
+  <si>
+    <t>Semana 21–27/09 (painel TESTEDESCONTONOPRECO, Terminado): 0 un · 13 visualizações. Total dos 10 SKUs: 7 un · R$ 1.187,20 · 166 visualizações · 4,2%. Desconto não gera tráfego (esperado); converteu em 2 de 10 SKUs.o</t>
+  </si>
+  <si>
+    <t>SEM EFEITO — 0 venda em 12 sessões / 13 visualizações.</t>
+  </si>
+  <si>
+    <t>Semana 21–27/09 (painel TESTEDESCONTONOPRECO, Terminado): 0 un · 8 visualizações. Total dos 10 SKUs: 7 un · R$ 1.187,20 · 166 visualizações · 4,2%. Desconto não gera tráfego (esperado); converteu em 2 de 10 SKUs.</t>
+  </si>
+  <si>
+    <t>SEM EFEITO — 0 venda em 5 sessões / 8 visualizações.</t>
+  </si>
+  <si>
+    <t>Semana 21–27/09 (painel TESTEDESCONTONOPRECO, Terminado): 0 un · 5 visualizações. Total dos 10 SKUs: 7 un · R$ 1.187,20 · 166 visualizações · 4,2%. Desconto não gera tráfego (esperado); converteu em 2 de 10 SKUs.</t>
+  </si>
+  <si>
+    <t>SEM EFEITO — 0 venda em 3 sessões / 5 visualizações (opcional, tráfego marginal).</t>
   </si>
 </sst>
 </file>
@@ -2293,7 +2347,149 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
-  <dxfs count="21">
+  <dxfs count="35">
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9A3412"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFED7AA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF991B1B"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF374151"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF3F4F6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF166534"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFDCFCE7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF3730A3"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFE0E7FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF92400E"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEF3C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1E40AF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFDBEAFE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9A3412"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFED7AA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF991B1B"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF374151"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF3F4F6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF166534"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFDCFCE7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF3730A3"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFE0E7FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF92400E"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEF3C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1E40AF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFDBEAFE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -2901,11 +3097,11 @@
       </c>
       <c r="E6" s="3">
         <f>COUNTIF(P11:P210,"EXECUTADA - EM MATURAÇÃO")</f>
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="F6" s="4">
         <f>COUNTIF(P11:P210,"EXECUTADA - AVALIADA")</f>
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="H6" s="54"/>
       <c r="I6" s="54"/>
@@ -3070,7 +3266,7 @@
       </c>
       <c r="R11" s="17">
         <f t="shared" ref="R11:R42" ca="1" si="1">IF(E11="","",TODAY()-E11)</f>
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="S11" s="39" t="s">
         <v>362</v>
@@ -3136,7 +3332,7 @@
       </c>
       <c r="R12" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="S12" s="39" t="s">
         <v>363</v>
@@ -3200,7 +3396,7 @@
       </c>
       <c r="R13" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="S13" s="39" t="s">
         <v>364</v>
@@ -3268,7 +3464,7 @@
       </c>
       <c r="R14" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="S14" s="39" t="s">
         <v>365</v>
@@ -3338,7 +3534,7 @@
       </c>
       <c r="R15" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="S15" s="39" t="s">
         <v>366</v>
@@ -3408,7 +3604,7 @@
       </c>
       <c r="R16" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="S16" s="39" t="s">
         <v>367</v>
@@ -3478,7 +3674,7 @@
       </c>
       <c r="R17" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="S17" s="39" t="s">
         <v>368</v>
@@ -3546,7 +3742,7 @@
       </c>
       <c r="R18" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="S18" s="39" t="s">
         <v>369</v>
@@ -3616,7 +3812,7 @@
       </c>
       <c r="R19" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="S19" s="39" t="s">
         <v>370</v>
@@ -3686,7 +3882,7 @@
       </c>
       <c r="R20" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="S20" s="39" t="s">
         <v>371</v>
@@ -3754,7 +3950,7 @@
       </c>
       <c r="R21" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="S21" s="39" t="s">
         <v>372</v>
@@ -3820,7 +4016,7 @@
       </c>
       <c r="R22" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="S22" s="39" t="s">
         <v>373</v>
@@ -3886,7 +4082,7 @@
       </c>
       <c r="R23" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="S23" s="39" t="s">
         <v>372</v>
@@ -3952,7 +4148,7 @@
       </c>
       <c r="R24" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="S24" s="39" t="s">
         <v>374</v>
@@ -4022,7 +4218,7 @@
       </c>
       <c r="R25" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="S25" s="39" t="s">
         <v>375</v>
@@ -4088,7 +4284,7 @@
       </c>
       <c r="R26" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="S26" s="39" t="s">
         <v>376</v>
@@ -4156,7 +4352,7 @@
       </c>
       <c r="R27" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="S27" s="39" t="s">
         <v>377</v>
@@ -4226,7 +4422,7 @@
       </c>
       <c r="R28" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="S28" s="39" t="s">
         <v>378</v>
@@ -4296,7 +4492,7 @@
       </c>
       <c r="R29" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="S29" s="39" t="s">
         <v>379</v>
@@ -4366,7 +4562,7 @@
       </c>
       <c r="R30" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="S30" s="39" t="s">
         <v>380</v>
@@ -4436,7 +4632,7 @@
       </c>
       <c r="R31" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="S31" s="39" t="s">
         <v>381</v>
@@ -4506,7 +4702,7 @@
       </c>
       <c r="R32" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="S32" s="39" t="s">
         <v>401</v>
@@ -4574,7 +4770,7 @@
       </c>
       <c r="R33" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="S33" s="39" t="s">
         <v>402</v>
@@ -4642,7 +4838,7 @@
       </c>
       <c r="R34" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="S34" s="43" t="s">
         <v>459</v>
@@ -4712,7 +4908,7 @@
       </c>
       <c r="R35" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="S35" s="43" t="s">
         <v>460</v>
@@ -4782,7 +4978,7 @@
       </c>
       <c r="R36" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="S36" t="s">
         <v>584</v>
@@ -4852,7 +5048,7 @@
       </c>
       <c r="R37" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="S37" t="s">
         <v>586</v>
@@ -4922,7 +5118,7 @@
       </c>
       <c r="R38" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="S38" t="s">
         <v>588</v>
@@ -4992,7 +5188,7 @@
       </c>
       <c r="R39" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="S39" t="s">
         <v>590</v>
@@ -5062,7 +5258,7 @@
       </c>
       <c r="R40" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="S40" t="s">
         <v>592</v>
@@ -5132,7 +5328,7 @@
       </c>
       <c r="R41" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="S41" t="s">
         <v>593</v>
@@ -5202,7 +5398,7 @@
       </c>
       <c r="R42" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="S42" t="s">
         <v>595</v>
@@ -5272,7 +5468,7 @@
       </c>
       <c r="R43" s="19">
         <f t="shared" ref="R43:R82" ca="1" si="2">IF(E43="","",TODAY()-E43)</f>
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="S43" t="s">
         <v>597</v>
@@ -5342,7 +5538,7 @@
       </c>
       <c r="R44" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="S44" t="s">
         <v>599</v>
@@ -5412,7 +5608,7 @@
       </c>
       <c r="R45" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="S45" t="s">
         <v>601</v>
@@ -5482,7 +5678,7 @@
       </c>
       <c r="R46" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="S46" t="s">
         <v>603</v>
@@ -5552,7 +5748,7 @@
       </c>
       <c r="R47" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="S47" t="s">
         <v>605</v>
@@ -5690,7 +5886,7 @@
       </c>
       <c r="R49" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="S49" t="s">
         <v>609</v>
@@ -5760,7 +5956,7 @@
       </c>
       <c r="R50" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="S50" t="s">
         <v>611</v>
@@ -5830,7 +6026,7 @@
       </c>
       <c r="R51" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="S51" t="s">
         <v>613</v>
@@ -5900,7 +6096,7 @@
       </c>
       <c r="R52" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="S52" t="s">
         <v>615</v>
@@ -5961,8 +6157,8 @@
       <c r="O53" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="P53" s="46" t="s">
-        <v>47</v>
+      <c r="P53" s="39" t="s">
+        <v>51</v>
       </c>
       <c r="Q53" s="18">
         <f t="shared" si="0"/>
@@ -5970,13 +6166,13 @@
       </c>
       <c r="R53" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="S53" t="s">
-        <v>617</v>
+        <v>620</v>
       </c>
       <c r="T53" t="s">
-        <v>618</v>
+        <v>621</v>
       </c>
       <c r="U53" s="47">
         <v>46293</v>
@@ -6031,8 +6227,8 @@
       <c r="O54" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="P54" s="46" t="s">
-        <v>47</v>
+      <c r="P54" s="39" t="s">
+        <v>51</v>
       </c>
       <c r="Q54" s="18">
         <f t="shared" si="0"/>
@@ -6040,13 +6236,13 @@
       </c>
       <c r="R54" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="S54" t="s">
-        <v>617</v>
+        <v>622</v>
       </c>
       <c r="T54" t="s">
-        <v>618</v>
+        <v>623</v>
       </c>
       <c r="U54" s="47">
         <v>46293</v>
@@ -6101,8 +6297,8 @@
       <c r="O55" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="P55" s="46" t="s">
-        <v>47</v>
+      <c r="P55" s="39" t="s">
+        <v>51</v>
       </c>
       <c r="Q55" s="18">
         <f t="shared" si="0"/>
@@ -6110,13 +6306,13 @@
       </c>
       <c r="R55" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="S55" t="s">
-        <v>617</v>
+        <v>624</v>
       </c>
       <c r="T55" t="s">
-        <v>618</v>
+        <v>625</v>
       </c>
       <c r="U55" s="47">
         <v>46293</v>
@@ -6171,8 +6367,8 @@
       <c r="O56" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="P56" s="46" t="s">
-        <v>47</v>
+      <c r="P56" s="39" t="s">
+        <v>51</v>
       </c>
       <c r="Q56" s="18">
         <f t="shared" si="0"/>
@@ -6180,13 +6376,13 @@
       </c>
       <c r="R56" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="S56" t="s">
-        <v>617</v>
+        <v>626</v>
       </c>
       <c r="T56" t="s">
-        <v>618</v>
+        <v>627</v>
       </c>
       <c r="U56" s="47">
         <v>46293</v>
@@ -6241,8 +6437,8 @@
       <c r="O57" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="P57" s="46" t="s">
-        <v>47</v>
+      <c r="P57" s="39" t="s">
+        <v>51</v>
       </c>
       <c r="Q57" s="18">
         <f t="shared" si="0"/>
@@ -6250,13 +6446,13 @@
       </c>
       <c r="R57" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="S57" t="s">
-        <v>617</v>
+        <v>628</v>
       </c>
       <c r="T57" t="s">
-        <v>618</v>
+        <v>629</v>
       </c>
       <c r="U57" s="47">
         <v>46293</v>
@@ -6311,8 +6507,8 @@
       <c r="O58" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="P58" s="46" t="s">
-        <v>47</v>
+      <c r="P58" s="39" t="s">
+        <v>51</v>
       </c>
       <c r="Q58" s="18">
         <f t="shared" si="0"/>
@@ -6320,13 +6516,13 @@
       </c>
       <c r="R58" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="S58" t="s">
-        <v>617</v>
+        <v>630</v>
       </c>
       <c r="T58" t="s">
-        <v>618</v>
+        <v>631</v>
       </c>
       <c r="U58" s="47">
         <v>46293</v>
@@ -6381,8 +6577,8 @@
       <c r="O59" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="P59" s="46" t="s">
-        <v>47</v>
+      <c r="P59" s="39" t="s">
+        <v>51</v>
       </c>
       <c r="Q59" s="18">
         <f t="shared" si="0"/>
@@ -6390,13 +6586,13 @@
       </c>
       <c r="R59" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="S59" t="s">
-        <v>617</v>
+        <v>632</v>
       </c>
       <c r="T59" t="s">
-        <v>618</v>
+        <v>633</v>
       </c>
       <c r="U59" s="47">
         <v>46293</v>
@@ -6451,8 +6647,8 @@
       <c r="O60" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="P60" s="46" t="s">
-        <v>47</v>
+      <c r="P60" s="39" t="s">
+        <v>51</v>
       </c>
       <c r="Q60" s="18">
         <f t="shared" si="0"/>
@@ -6460,13 +6656,13 @@
       </c>
       <c r="R60" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="S60" t="s">
-        <v>617</v>
+        <v>634</v>
       </c>
       <c r="T60" t="s">
-        <v>618</v>
+        <v>635</v>
       </c>
       <c r="U60" s="47">
         <v>46293</v>
@@ -6521,8 +6717,8 @@
       <c r="O61" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="P61" s="46" t="s">
-        <v>47</v>
+      <c r="P61" s="39" t="s">
+        <v>51</v>
       </c>
       <c r="Q61" s="18">
         <f t="shared" si="0"/>
@@ -6530,13 +6726,13 @@
       </c>
       <c r="R61" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="S61" t="s">
-        <v>617</v>
+        <v>634</v>
       </c>
       <c r="T61" t="s">
-        <v>618</v>
+        <v>635</v>
       </c>
       <c r="U61" s="47">
         <v>46293</v>
@@ -6591,8 +6787,8 @@
       <c r="O62" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="P62" s="46" t="s">
-        <v>47</v>
+      <c r="P62" s="39" t="s">
+        <v>51</v>
       </c>
       <c r="Q62" s="18">
         <f t="shared" si="0"/>
@@ -6600,13 +6796,13 @@
       </c>
       <c r="R62" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="S62" t="s">
-        <v>617</v>
+        <v>636</v>
       </c>
       <c r="T62" t="s">
-        <v>618</v>
+        <v>637</v>
       </c>
       <c r="U62" s="47">
         <v>46293</v>
@@ -6670,7 +6866,7 @@
       </c>
       <c r="R63" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U63" t="s">
         <v>469</v>
@@ -6734,7 +6930,7 @@
       </c>
       <c r="R64" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U64" t="s">
         <v>474</v>
@@ -6798,7 +6994,7 @@
       </c>
       <c r="R65" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U65" t="s">
         <v>146</v>
@@ -6862,7 +7058,7 @@
       </c>
       <c r="R66" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U66" t="s">
         <v>469</v>
@@ -6926,7 +7122,7 @@
       </c>
       <c r="R67" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U67" t="s">
         <v>469</v>
@@ -6990,7 +7186,7 @@
       </c>
       <c r="R68" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U68" s="50">
         <v>46293</v>
@@ -7054,7 +7250,7 @@
       </c>
       <c r="R69" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U69" t="s">
         <v>146</v>
@@ -7118,7 +7314,7 @@
       </c>
       <c r="R70" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U70" t="s">
         <v>469</v>
@@ -7182,7 +7378,7 @@
       </c>
       <c r="R71" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U71" t="s">
         <v>146</v>
@@ -7246,7 +7442,7 @@
       </c>
       <c r="R72" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U72" t="s">
         <v>469</v>
@@ -7434,7 +7630,7 @@
       </c>
       <c r="R75" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U75" s="50">
         <v>46308</v>
@@ -7684,7 +7880,7 @@
       </c>
       <c r="R79" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U79" s="50">
         <v>46308</v>
@@ -7748,7 +7944,7 @@
       </c>
       <c r="R80" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U80" t="s">
         <v>469</v>
@@ -7812,7 +8008,7 @@
       </c>
       <c r="R81" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U81" t="s">
         <v>469</v>
@@ -7876,7 +8072,7 @@
       </c>
       <c r="R82" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U82" t="s">
         <v>469</v>
@@ -11734,25 +11930,25 @@
     <mergeCell ref="A8:V8"/>
   </mergeCells>
   <conditionalFormatting sqref="P11:P210">
-    <cfRule type="expression" dxfId="20" priority="1">
+    <cfRule type="expression" dxfId="34" priority="1">
       <formula>P11="RECOMENDADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="19" priority="2">
+    <cfRule type="expression" dxfId="33" priority="2">
       <formula>P11="APROVADA - AGUARDANDO EXECUÇÃO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="3">
+    <cfRule type="expression" dxfId="32" priority="3">
       <formula>P11="EXECUTADA - EM MATURAÇÃO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="17" priority="4">
+    <cfRule type="expression" dxfId="31" priority="4">
       <formula>P11="EXECUTADA - AVALIADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="5">
+    <cfRule type="expression" dxfId="30" priority="5">
       <formula>P11="APROVADA - NÃO EXECUTADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="6">
+    <cfRule type="expression" dxfId="29" priority="6">
       <formula>P11="REJEITADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="7">
+    <cfRule type="expression" dxfId="28" priority="7">
       <formula>LEFT(P11,9)="BLOQUEADA"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
[Monitoramento 28/09] minimo do Prime Day e 10% (correcao de 22/09 estava errada): L1618-T e L2025-T caem abaixo do piso, decisao a reconfirmar; Q2460-B pausado na Geral (print); Registro com EC-017/018 em 83-84
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2340" uniqueCount="638">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2370" uniqueCount="651">
   <si>
     <t>REGISTRO DE ALTERAÇÕES — AMAZON ADS | WINNET METAIS</t>
   </si>
@@ -1944,6 +1944,45 @@
   </si>
   <si>
     <t>SEM EFEITO — 0 venda em 3 sessões / 5 visualizações (opcional, tráfego marginal).</t>
+  </si>
+  <si>
+    <t>EC-017</t>
+  </si>
+  <si>
+    <t>L1618-T (B0H3QQLFFY) — desconto 5% (mínimo do evento)</t>
+  </si>
+  <si>
+    <t>Sem oferta inscrita; preço de tabela R$ 116,00</t>
+  </si>
+  <si>
+    <t>Melhor Oferta −5% → R$ 110,20 · Prime Big Deal Days 05–11/10</t>
+  </si>
+  <si>
+    <t>Entrou na lista de recomendações de 28/09 (não estava em 22/09). Converteu 2 un a −5% com desconto no preço em 21–27/09 (27 sessões) — única lixeira que converteu com desconto; no 9.9 com oferta: 0. Margem SP Interior 15,3% — no piso. Se a promo de quantidade empilhasse (3+): 12,1%; no 9.9 a Melhor …</t>
+  </si>
+  <si>
+    <t>ciclos/Monitoramento-28-09.md + relatorios/amazon/monitoramento-28-09/ (lista do Prime Day de 28/09) + Simulador Mestra v4.3.4</t>
+  </si>
+  <si>
+    <t>Não empilha com desconto no preço (nenhum ativo). Conferir preço de referência na tela. Leitura na O7 (13/10) junto com P3070 e PXP; o evento contamina a leitura de Ads do SKU na Geral em 05–11/10.</t>
+  </si>
+  <si>
+    <t>Motor de tráfego da Geral: em 05–11/10 a atribuição do SKU sai a preço da oferta (R$ 126,26). Marcar na O7.</t>
+  </si>
+  <si>
+    <t>Entrou na lista de recomendações de 28/09. Maior tráfego do catálogo; 0 conversão a −5% com desconto no preço (26 sessões, 21–27/09) e 0 com oferta no 9.9 — vende orgânico e por promo de quantidade. Teste do selo do evento. Margem SP Interior 16,5%; a 10% cairia a 13,1% (por isso 5%).</t>
+  </si>
+  <si>
+    <t>Melhor Oferta −5% → R$ 126,26 · Prime Big Deal Days 05–11/10</t>
+  </si>
+  <si>
+    <t>Sem oferta inscrita; preço de tabela R$ 132,90</t>
+  </si>
+  <si>
+    <t>L2025-T (B0H6C5CTSC) — desconto 5% (mínimo do evento)</t>
+  </si>
+  <si>
+    <t>EC-018</t>
   </si>
 </sst>
 </file>
@@ -2347,7 +2386,78 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
-  <dxfs count="35">
+  <dxfs count="42">
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9A3412"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFED7AA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF991B1B"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF374151"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF3F4F6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF166534"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFDCFCE7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF3730A3"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFE0E7FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF92400E"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEF3C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1E40AF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFDBEAFE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -3081,15 +3191,15 @@
     <row r="6" spans="1:22" ht="26.1" customHeight="1">
       <c r="A6" s="2">
         <f>COUNTIF(A11:A210,"&lt;&gt;")</f>
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B6" s="3">
         <f>COUNTIF(N11:N210,"SIM")</f>
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C6" s="3">
         <f>COUNTIF(O11:O210,"SIM")</f>
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D6" s="3">
         <f>COUNTIF(P11:P210,"BLOQUEADA*")</f>
@@ -3097,7 +3207,7 @@
       </c>
       <c r="E6" s="3">
         <f>COUNTIF(P11:P210,"EXECUTADA - EM MATURAÇÃO")</f>
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F6" s="4">
         <f>COUNTIF(P11:P210,"EXECUTADA - AVALIADA")</f>
@@ -8082,64 +8192,136 @@
       </c>
     </row>
     <row r="83" spans="1:22">
-      <c r="A83" s="10"/>
-      <c r="B83" s="11"/>
-      <c r="C83" s="12"/>
-      <c r="D83" s="12"/>
-      <c r="E83" s="12"/>
-      <c r="F83" s="43"/>
-      <c r="G83" s="43"/>
-      <c r="H83" s="11"/>
-      <c r="I83" s="11"/>
-      <c r="J83" s="11"/>
-      <c r="K83" s="11"/>
-      <c r="L83" s="11"/>
-      <c r="M83" s="11"/>
-      <c r="N83" s="11"/>
-      <c r="O83" s="11"/>
-      <c r="P83" s="11"/>
-      <c r="Q83" s="18" t="str">
+      <c r="A83" s="10" t="s">
+        <v>638</v>
+      </c>
+      <c r="B83" s="11" t="s">
+        <v>215</v>
+      </c>
+      <c r="C83" s="12">
+        <v>46293</v>
+      </c>
+      <c r="D83" s="12">
+        <v>46293</v>
+      </c>
+      <c r="E83" s="12">
+        <v>46293</v>
+      </c>
+      <c r="F83" s="43" t="s">
+        <v>527</v>
+      </c>
+      <c r="G83" s="43" t="s">
+        <v>639</v>
+      </c>
+      <c r="H83" s="11" t="s">
+        <v>529</v>
+      </c>
+      <c r="I83" s="11" t="s">
+        <v>640</v>
+      </c>
+      <c r="J83" s="11" t="s">
+        <v>641</v>
+      </c>
+      <c r="K83" s="11" t="s">
+        <v>642</v>
+      </c>
+      <c r="L83" s="11" t="s">
+        <v>643</v>
+      </c>
+      <c r="M83" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="N83" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O83" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="P83" s="46" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q83" s="18">
         <f t="shared" ref="Q83:Q106" si="4">IF(E83="","",E83+1)</f>
-        <v/>
-      </c>
-      <c r="R83" s="19" t="str">
+        <v>46294</v>
+      </c>
+      <c r="R83" s="19">
         <f t="shared" ref="R83:R106" ca="1" si="5">IF(E83="","",TODAY()-E83)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S83" s="43"/>
       <c r="T83" s="43"/>
-      <c r="U83" s="7"/>
-      <c r="V83" s="41"/>
+      <c r="U83" t="s">
+        <v>469</v>
+      </c>
+      <c r="V83" s="41" t="s">
+        <v>644</v>
+      </c>
     </row>
     <row r="84" spans="1:22">
-      <c r="A84" s="10"/>
-      <c r="B84" s="11"/>
-      <c r="C84" s="12"/>
-      <c r="D84" s="12"/>
-      <c r="E84" s="12"/>
-      <c r="F84" s="43"/>
-      <c r="G84" s="43"/>
-      <c r="H84" s="11"/>
-      <c r="I84" s="11"/>
-      <c r="J84" s="11"/>
-      <c r="K84" s="11"/>
-      <c r="L84" s="11"/>
-      <c r="M84" s="11"/>
-      <c r="N84" s="11"/>
-      <c r="O84" s="11"/>
-      <c r="P84" s="11"/>
-      <c r="Q84" s="18" t="str">
+      <c r="A84" s="10" t="s">
+        <v>650</v>
+      </c>
+      <c r="B84" s="11" t="s">
+        <v>215</v>
+      </c>
+      <c r="C84" s="12">
+        <v>46293</v>
+      </c>
+      <c r="D84" s="12">
+        <v>46293</v>
+      </c>
+      <c r="E84" s="12">
+        <v>46293</v>
+      </c>
+      <c r="F84" s="43" t="s">
+        <v>527</v>
+      </c>
+      <c r="G84" s="43" t="s">
+        <v>649</v>
+      </c>
+      <c r="H84" s="11" t="s">
+        <v>529</v>
+      </c>
+      <c r="I84" s="11" t="s">
+        <v>648</v>
+      </c>
+      <c r="J84" s="11" t="s">
+        <v>647</v>
+      </c>
+      <c r="K84" s="11" t="s">
+        <v>646</v>
+      </c>
+      <c r="L84" s="11" t="s">
+        <v>643</v>
+      </c>
+      <c r="M84" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N84" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O84" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="P84" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q84" s="18">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R84" s="19" t="str">
+        <v>46294</v>
+      </c>
+      <c r="R84" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S84" s="43"/>
       <c r="T84" s="43"/>
-      <c r="U84" s="7"/>
-      <c r="V84" s="41"/>
+      <c r="U84" t="s">
+        <v>469</v>
+      </c>
+      <c r="V84" s="41" t="s">
+        <v>645</v>
+      </c>
     </row>
     <row r="85" spans="1:22">
       <c r="A85" s="10"/>
@@ -11930,25 +12112,25 @@
     <mergeCell ref="A8:V8"/>
   </mergeCells>
   <conditionalFormatting sqref="P11:P210">
-    <cfRule type="expression" dxfId="34" priority="1">
+    <cfRule type="expression" dxfId="41" priority="1">
       <formula>P11="RECOMENDADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="33" priority="2">
+    <cfRule type="expression" dxfId="40" priority="2">
       <formula>P11="APROVADA - AGUARDANDO EXECUÇÃO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="32" priority="3">
+    <cfRule type="expression" dxfId="39" priority="3">
       <formula>P11="EXECUTADA - EM MATURAÇÃO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="31" priority="4">
+    <cfRule type="expression" dxfId="38" priority="4">
       <formula>P11="EXECUTADA - AVALIADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="30" priority="5">
+    <cfRule type="expression" dxfId="37" priority="5">
       <formula>P11="APROVADA - NÃO EXECUTADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="29" priority="6">
+    <cfRule type="expression" dxfId="36" priority="6">
       <formula>P11="REJEITADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="28" priority="7">
+    <cfRule type="expression" dxfId="35" priority="7">
       <formula>LEFT(P11,9)="BLOQUEADA"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
[Monitoramento 28/09] encerrado: L1618-T e L2025-T ficam fora do Prime Day (minimo 10% fura o piso); evento fecha com P3070 e PXP; O6-006 fechada no Registro
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2370" uniqueCount="651">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1193" uniqueCount="637">
   <si>
     <t>REGISTRO DE ALTERAÇÕES — AMAZON ADS | WINNET METAIS</t>
   </si>
@@ -1883,12 +1883,6 @@
     <t>CONFIRMADA; dúvida RESOLVIDA POR FONTE</t>
   </si>
   <si>
-    <t>Começou em 21/09 — 1 dia dentro da Era; sem dado</t>
-  </si>
-  <si>
-    <t>NÃO AVALIÁVEL hoje. Primeira leitura 28/09 (sessões × conversão; primeira venda conferida pedido a pedido para fixar a regra de atribuição). Corte de série 23–27/09 a marcar na O7</t>
-  </si>
-  <si>
     <t>não elegível na lista de 22/09; reconferir 28/09</t>
   </si>
   <si>
@@ -1946,43 +1940,7 @@
     <t>SEM EFEITO — 0 venda em 3 sessões / 5 visualizações (opcional, tráfego marginal).</t>
   </si>
   <si>
-    <t>EC-017</t>
-  </si>
-  <si>
-    <t>L1618-T (B0H3QQLFFY) — desconto 5% (mínimo do evento)</t>
-  </si>
-  <si>
-    <t>Sem oferta inscrita; preço de tabela R$ 116,00</t>
-  </si>
-  <si>
-    <t>Melhor Oferta −5% → R$ 110,20 · Prime Big Deal Days 05–11/10</t>
-  </si>
-  <si>
-    <t>Entrou na lista de recomendações de 28/09 (não estava em 22/09). Converteu 2 un a −5% com desconto no preço em 21–27/09 (27 sessões) — única lixeira que converteu com desconto; no 9.9 com oferta: 0. Margem SP Interior 15,3% — no piso. Se a promo de quantidade empilhasse (3+): 12,1%; no 9.9 a Melhor …</t>
-  </si>
-  <si>
-    <t>ciclos/Monitoramento-28-09.md + relatorios/amazon/monitoramento-28-09/ (lista do Prime Day de 28/09) + Simulador Mestra v4.3.4</t>
-  </si>
-  <si>
-    <t>Não empilha com desconto no preço (nenhum ativo). Conferir preço de referência na tela. Leitura na O7 (13/10) junto com P3070 e PXP; o evento contamina a leitura de Ads do SKU na Geral em 05–11/10.</t>
-  </si>
-  <si>
-    <t>Motor de tráfego da Geral: em 05–11/10 a atribuição do SKU sai a preço da oferta (R$ 126,26). Marcar na O7.</t>
-  </si>
-  <si>
-    <t>Entrou na lista de recomendações de 28/09. Maior tráfego do catálogo; 0 conversão a −5% com desconto no preço (26 sessões, 21–27/09) e 0 com oferta no 9.9 — vende orgânico e por promo de quantidade. Teste do selo do evento. Margem SP Interior 16,5%; a 10% cairia a 13,1% (por isso 5%).</t>
-  </si>
-  <si>
-    <t>Melhor Oferta −5% → R$ 126,26 · Prime Big Deal Days 05–11/10</t>
-  </si>
-  <si>
-    <t>Sem oferta inscrita; preço de tabela R$ 132,90</t>
-  </si>
-  <si>
-    <t>L2025-T (B0H6C5CTSC) — desconto 5% (mínimo do evento)</t>
-  </si>
-  <si>
-    <t>EC-018</t>
+    <t>gatilho disparou em 28/09, anúncio pausado</t>
   </si>
 </sst>
 </file>
@@ -2386,362 +2344,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
-  <dxfs count="42">
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9A3412"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFED7AA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF991B1B"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEE2E2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF374151"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF3F4F6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF166534"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDCFCE7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF3730A3"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE0E7FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF92400E"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEF3C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1E40AF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDBEAFE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9A3412"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFED7AA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF991B1B"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEE2E2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF374151"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF3F4F6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF166534"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDCFCE7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF3730A3"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE0E7FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF92400E"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEF3C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1E40AF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDBEAFE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9A3412"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFED7AA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF991B1B"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEE2E2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF374151"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF3F4F6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF166534"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDCFCE7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF3730A3"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE0E7FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF92400E"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEF3C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1E40AF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDBEAFE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9A3412"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFED7AA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF991B1B"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEE2E2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF374151"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF3F4F6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF166534"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDCFCE7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF3730A3"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE0E7FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF92400E"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEF3C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1E40AF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDBEAFE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9A3412"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFED7AA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF991B1B"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEE2E2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF374151"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF3F4F6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF166534"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDCFCE7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF3730A3"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE0E7FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF92400E"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEF3C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1E40AF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDBEAFE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="7">
     <dxf>
       <font>
         <b/>
@@ -2827,7 +2430,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RegistroAlteracoesAds" displayName="RegistroAlteracoesAds" ref="A10:V210" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RegistroAlteracoesAds" displayName="RegistroAlteracoesAds" ref="A10:V208" totalsRowShown="0">
   <tableColumns count="22">
     <tableColumn id="1" name="ID da alteração"/>
     <tableColumn id="2" name="Ciclo"/>
@@ -3051,7 +2654,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:V210"/>
+  <dimension ref="A1:V208"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -3190,27 +2793,27 @@
     </row>
     <row r="6" spans="1:22" ht="26.1" customHeight="1">
       <c r="A6" s="2">
-        <f>COUNTIF(A11:A210,"&lt;&gt;")</f>
-        <v>74</v>
+        <f>COUNTIF(A11:A208,"&lt;&gt;")</f>
+        <v>72</v>
       </c>
       <c r="B6" s="3">
-        <f>COUNTIF(N11:N210,"SIM")</f>
-        <v>74</v>
+        <f>COUNTIF(N11:N208,"SIM")</f>
+        <v>72</v>
       </c>
       <c r="C6" s="3">
-        <f>COUNTIF(O11:O210,"SIM")</f>
-        <v>68</v>
+        <f>COUNTIF(O11:O208,"SIM")</f>
+        <v>66</v>
       </c>
       <c r="D6" s="3">
-        <f>COUNTIF(P11:P210,"BLOQUEADA*")</f>
+        <f>COUNTIF(P11:P208,"BLOQUEADA*")</f>
         <v>0</v>
       </c>
       <c r="E6" s="3">
-        <f>COUNTIF(P11:P210,"EXECUTADA - EM MATURAÇÃO")</f>
-        <v>20</v>
+        <f>COUNTIF(P11:P208,"EXECUTADA - EM MATURAÇÃO")</f>
+        <v>18</v>
       </c>
       <c r="F6" s="4">
-        <f>COUNTIF(P11:P210,"EXECUTADA - AVALIADA")</f>
+        <f>COUNTIF(P11:P208,"EXECUTADA - AVALIADA")</f>
         <v>48</v>
       </c>
       <c r="H6" s="54"/>
@@ -6279,10 +5882,10 @@
         <v>10</v>
       </c>
       <c r="S53" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="T53" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="U53" s="47">
         <v>46293</v>
@@ -6349,10 +5952,10 @@
         <v>10</v>
       </c>
       <c r="S54" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="T54" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="U54" s="47">
         <v>46293</v>
@@ -6419,10 +6022,10 @@
         <v>10</v>
       </c>
       <c r="S55" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="T55" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="U55" s="47">
         <v>46293</v>
@@ -6489,10 +6092,10 @@
         <v>10</v>
       </c>
       <c r="S56" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="T56" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="U56" s="47">
         <v>46293</v>
@@ -6559,10 +6162,10 @@
         <v>10</v>
       </c>
       <c r="S57" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="T57" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="U57" s="47">
         <v>46293</v>
@@ -6629,10 +6232,10 @@
         <v>10</v>
       </c>
       <c r="S58" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="T58" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="U58" s="47">
         <v>46293</v>
@@ -6699,10 +6302,10 @@
         <v>10</v>
       </c>
       <c r="S59" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="T59" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="U59" s="47">
         <v>46293</v>
@@ -6769,10 +6372,10 @@
         <v>10</v>
       </c>
       <c r="S60" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="T60" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="U60" s="47">
         <v>46293</v>
@@ -6839,10 +6442,10 @@
         <v>10</v>
       </c>
       <c r="S61" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="T61" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="U61" s="47">
         <v>46293</v>
@@ -6909,10 +6512,10 @@
         <v>10</v>
       </c>
       <c r="S62" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="T62" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="U62" s="47">
         <v>46293</v>
@@ -7298,8 +6901,11 @@
         <f t="shared" ca="1" si="2"/>
         <v>6</v>
       </c>
+      <c r="T68" t="s">
+        <v>636</v>
+      </c>
       <c r="U68" s="50">
-        <v>46293</v>
+        <v>46308</v>
       </c>
       <c r="V68" t="s">
         <v>497</v>
@@ -7620,7 +7226,7 @@
         <v>46293</v>
       </c>
       <c r="V73" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
     </row>
     <row r="74" spans="1:22">
@@ -7682,7 +7288,7 @@
         <v>46293</v>
       </c>
       <c r="V74" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
     </row>
     <row r="75" spans="1:22">
@@ -7808,7 +7414,7 @@
         <v>46293</v>
       </c>
       <c r="V76" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
     </row>
     <row r="77" spans="1:22">
@@ -7870,7 +7476,7 @@
         <v>46293</v>
       </c>
       <c r="V77" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
     </row>
     <row r="78" spans="1:22">
@@ -7932,7 +7538,7 @@
         <v>46293</v>
       </c>
       <c r="V78" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
     </row>
     <row r="79" spans="1:22">
@@ -8192,136 +7798,64 @@
       </c>
     </row>
     <row r="83" spans="1:22">
-      <c r="A83" s="10" t="s">
-        <v>638</v>
-      </c>
-      <c r="B83" s="11" t="s">
-        <v>215</v>
-      </c>
-      <c r="C83" s="12">
-        <v>46293</v>
-      </c>
-      <c r="D83" s="12">
-        <v>46293</v>
-      </c>
-      <c r="E83" s="12">
-        <v>46293</v>
-      </c>
-      <c r="F83" s="43" t="s">
-        <v>527</v>
-      </c>
-      <c r="G83" s="43" t="s">
-        <v>639</v>
-      </c>
-      <c r="H83" s="11" t="s">
-        <v>529</v>
-      </c>
-      <c r="I83" s="11" t="s">
-        <v>640</v>
-      </c>
-      <c r="J83" s="11" t="s">
-        <v>641</v>
-      </c>
-      <c r="K83" s="11" t="s">
-        <v>642</v>
-      </c>
-      <c r="L83" s="11" t="s">
-        <v>643</v>
-      </c>
-      <c r="M83" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="N83" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="O83" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="P83" s="46" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q83" s="18">
-        <f t="shared" ref="Q83:Q106" si="4">IF(E83="","",E83+1)</f>
-        <v>46294</v>
-      </c>
-      <c r="R83" s="19">
-        <f t="shared" ref="R83:R106" ca="1" si="5">IF(E83="","",TODAY()-E83)</f>
-        <v>0</v>
+      <c r="A83" s="10"/>
+      <c r="B83" s="11"/>
+      <c r="C83" s="12"/>
+      <c r="D83" s="12"/>
+      <c r="E83" s="12"/>
+      <c r="F83" s="43"/>
+      <c r="G83" s="43"/>
+      <c r="H83" s="11"/>
+      <c r="I83" s="11"/>
+      <c r="J83" s="11"/>
+      <c r="K83" s="11"/>
+      <c r="L83" s="11"/>
+      <c r="M83" s="11"/>
+      <c r="N83" s="11"/>
+      <c r="O83" s="11"/>
+      <c r="P83" s="11"/>
+      <c r="Q83" s="18" t="str">
+        <f t="shared" ref="Q83:Q104" si="4">IF(E83="","",E83+1)</f>
+        <v/>
+      </c>
+      <c r="R83" s="19" t="str">
+        <f t="shared" ref="R83:R104" ca="1" si="5">IF(E83="","",TODAY()-E83)</f>
+        <v/>
       </c>
       <c r="S83" s="43"/>
       <c r="T83" s="43"/>
-      <c r="U83" t="s">
-        <v>469</v>
-      </c>
-      <c r="V83" s="41" t="s">
-        <v>644</v>
-      </c>
+      <c r="U83" s="7"/>
+      <c r="V83" s="41"/>
     </row>
     <row r="84" spans="1:22">
-      <c r="A84" s="10" t="s">
-        <v>650</v>
-      </c>
-      <c r="B84" s="11" t="s">
-        <v>215</v>
-      </c>
-      <c r="C84" s="12">
-        <v>46293</v>
-      </c>
-      <c r="D84" s="12">
-        <v>46293</v>
-      </c>
-      <c r="E84" s="12">
-        <v>46293</v>
-      </c>
-      <c r="F84" s="43" t="s">
-        <v>527</v>
-      </c>
-      <c r="G84" s="43" t="s">
-        <v>649</v>
-      </c>
-      <c r="H84" s="11" t="s">
-        <v>529</v>
-      </c>
-      <c r="I84" s="11" t="s">
-        <v>648</v>
-      </c>
-      <c r="J84" s="11" t="s">
-        <v>647</v>
-      </c>
-      <c r="K84" s="11" t="s">
-        <v>646</v>
-      </c>
-      <c r="L84" s="11" t="s">
-        <v>643</v>
-      </c>
-      <c r="M84" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="N84" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="O84" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="P84" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q84" s="18">
+      <c r="A84" s="10"/>
+      <c r="B84" s="11"/>
+      <c r="C84" s="12"/>
+      <c r="D84" s="12"/>
+      <c r="E84" s="12"/>
+      <c r="F84" s="43"/>
+      <c r="G84" s="43"/>
+      <c r="H84" s="11"/>
+      <c r="I84" s="11"/>
+      <c r="J84" s="11"/>
+      <c r="K84" s="11"/>
+      <c r="L84" s="11"/>
+      <c r="M84" s="11"/>
+      <c r="N84" s="11"/>
+      <c r="O84" s="11"/>
+      <c r="P84" s="11"/>
+      <c r="Q84" s="18" t="str">
         <f t="shared" si="4"/>
-        <v>46294</v>
-      </c>
-      <c r="R84" s="19">
+        <v/>
+      </c>
+      <c r="R84" s="19" t="str">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v/>
       </c>
       <c r="S84" s="43"/>
       <c r="T84" s="43"/>
-      <c r="U84" t="s">
-        <v>469</v>
-      </c>
-      <c r="V84" s="41" t="s">
-        <v>645</v>
-      </c>
+      <c r="U84" s="7"/>
+      <c r="V84" s="41"/>
     </row>
     <row r="85" spans="1:22">
       <c r="A85" s="10"/>
@@ -8941,11 +8475,11 @@
       <c r="O105" s="11"/>
       <c r="P105" s="11"/>
       <c r="Q105" s="18" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="Q105:Q136" si="6">IF(E105="","",E105+1)</f>
         <v/>
       </c>
       <c r="R105" s="19" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ref="R105:R136" ca="1" si="7">IF(E105="","",TODAY()-E105)</f>
         <v/>
       </c>
       <c r="S105" s="43"/>
@@ -8971,11 +8505,11 @@
       <c r="O106" s="11"/>
       <c r="P106" s="11"/>
       <c r="Q106" s="18" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R106" s="19" t="str">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S106" s="43"/>
@@ -9001,11 +8535,11 @@
       <c r="O107" s="11"/>
       <c r="P107" s="11"/>
       <c r="Q107" s="18" t="str">
-        <f t="shared" ref="Q107:Q138" si="6">IF(E107="","",E107+1)</f>
+        <f t="shared" si="6"/>
         <v/>
       </c>
       <c r="R107" s="19" t="str">
-        <f t="shared" ref="R107:R138" ca="1" si="7">IF(E107="","",TODAY()-E107)</f>
+        <f t="shared" ca="1" si="7"/>
         <v/>
       </c>
       <c r="S107" s="43"/>
@@ -9901,11 +9435,11 @@
       <c r="O137" s="11"/>
       <c r="P137" s="11"/>
       <c r="Q137" s="18" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="Q137:Q168" si="8">IF(E137="","",E137+1)</f>
         <v/>
       </c>
       <c r="R137" s="19" t="str">
-        <f t="shared" ca="1" si="7"/>
+        <f t="shared" ref="R137:R168" ca="1" si="9">IF(E137="","",TODAY()-E137)</f>
         <v/>
       </c>
       <c r="S137" s="43"/>
@@ -9931,11 +9465,11 @@
       <c r="O138" s="11"/>
       <c r="P138" s="11"/>
       <c r="Q138" s="18" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R138" s="19" t="str">
-        <f t="shared" ca="1" si="7"/>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S138" s="43"/>
@@ -9961,11 +9495,11 @@
       <c r="O139" s="11"/>
       <c r="P139" s="11"/>
       <c r="Q139" s="18" t="str">
-        <f t="shared" ref="Q139:Q170" si="8">IF(E139="","",E139+1)</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
       <c r="R139" s="19" t="str">
-        <f t="shared" ref="R139:R170" ca="1" si="9">IF(E139="","",TODAY()-E139)</f>
+        <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
       <c r="S139" s="43"/>
@@ -10519,13 +10053,13 @@
       <c r="C158" s="12"/>
       <c r="D158" s="12"/>
       <c r="E158" s="12"/>
-      <c r="F158" s="43"/>
-      <c r="G158" s="43"/>
+      <c r="F158" s="22"/>
+      <c r="G158" s="22"/>
       <c r="H158" s="11"/>
-      <c r="I158" s="11"/>
-      <c r="J158" s="11"/>
-      <c r="K158" s="11"/>
-      <c r="L158" s="11"/>
+      <c r="I158" s="24"/>
+      <c r="J158" s="24"/>
+      <c r="K158" s="24"/>
+      <c r="L158" s="24"/>
       <c r="M158" s="11"/>
       <c r="N158" s="11"/>
       <c r="O158" s="11"/>
@@ -10538,10 +10072,10 @@
         <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
-      <c r="S158" s="43"/>
-      <c r="T158" s="43"/>
+      <c r="S158" s="22"/>
+      <c r="T158" s="22"/>
       <c r="U158" s="7"/>
-      <c r="V158" s="41"/>
+      <c r="V158" s="26"/>
     </row>
     <row r="159" spans="1:22">
       <c r="A159" s="10"/>
@@ -10549,13 +10083,13 @@
       <c r="C159" s="12"/>
       <c r="D159" s="12"/>
       <c r="E159" s="12"/>
-      <c r="F159" s="43"/>
-      <c r="G159" s="43"/>
+      <c r="F159" s="22"/>
+      <c r="G159" s="22"/>
       <c r="H159" s="11"/>
-      <c r="I159" s="11"/>
-      <c r="J159" s="11"/>
-      <c r="K159" s="11"/>
-      <c r="L159" s="11"/>
+      <c r="I159" s="24"/>
+      <c r="J159" s="24"/>
+      <c r="K159" s="24"/>
+      <c r="L159" s="24"/>
       <c r="M159" s="11"/>
       <c r="N159" s="11"/>
       <c r="O159" s="11"/>
@@ -10568,10 +10102,10 @@
         <f t="shared" ca="1" si="9"/>
         <v/>
       </c>
-      <c r="S159" s="43"/>
-      <c r="T159" s="43"/>
+      <c r="S159" s="22"/>
+      <c r="T159" s="22"/>
       <c r="U159" s="7"/>
-      <c r="V159" s="41"/>
+      <c r="V159" s="26"/>
     </row>
     <row r="160" spans="1:22">
       <c r="A160" s="10"/>
@@ -10861,11 +10395,11 @@
       <c r="O169" s="11"/>
       <c r="P169" s="11"/>
       <c r="Q169" s="18" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="Q169:Q200" si="10">IF(E169="","",E169+1)</f>
         <v/>
       </c>
       <c r="R169" s="19" t="str">
-        <f t="shared" ca="1" si="9"/>
+        <f t="shared" ref="R169:R200" ca="1" si="11">IF(E169="","",TODAY()-E169)</f>
         <v/>
       </c>
       <c r="S169" s="22"/>
@@ -10891,11 +10425,11 @@
       <c r="O170" s="11"/>
       <c r="P170" s="11"/>
       <c r="Q170" s="18" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R170" s="19" t="str">
-        <f t="shared" ca="1" si="9"/>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S170" s="22"/>
@@ -10921,11 +10455,11 @@
       <c r="O171" s="11"/>
       <c r="P171" s="11"/>
       <c r="Q171" s="18" t="str">
-        <f t="shared" ref="Q171:Q202" si="10">IF(E171="","",E171+1)</f>
+        <f t="shared" si="10"/>
         <v/>
       </c>
       <c r="R171" s="19" t="str">
-        <f t="shared" ref="R171:R202" ca="1" si="11">IF(E171="","",TODAY()-E171)</f>
+        <f t="shared" ca="1" si="11"/>
         <v/>
       </c>
       <c r="S171" s="22"/>
@@ -11821,11 +11355,11 @@
       <c r="O201" s="11"/>
       <c r="P201" s="11"/>
       <c r="Q201" s="18" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" ref="Q201:Q208" si="12">IF(E201="","",E201+1)</f>
         <v/>
       </c>
       <c r="R201" s="19" t="str">
-        <f t="shared" ca="1" si="11"/>
+        <f t="shared" ref="R201:R208" ca="1" si="13">IF(E201="","",TODAY()-E201)</f>
         <v/>
       </c>
       <c r="S201" s="22"/>
@@ -11851,11 +11385,11 @@
       <c r="O202" s="11"/>
       <c r="P202" s="11"/>
       <c r="Q202" s="18" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="R202" s="19" t="str">
-        <f t="shared" ca="1" si="11"/>
+        <f t="shared" ca="1" si="13"/>
         <v/>
       </c>
       <c r="S202" s="22"/>
@@ -11881,11 +11415,11 @@
       <c r="O203" s="11"/>
       <c r="P203" s="11"/>
       <c r="Q203" s="18" t="str">
-        <f t="shared" ref="Q203:Q210" si="12">IF(E203="","",E203+1)</f>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="R203" s="19" t="str">
-        <f t="shared" ref="R203:R210" ca="1" si="13">IF(E203="","",TODAY()-E203)</f>
+        <f t="shared" ca="1" si="13"/>
         <v/>
       </c>
       <c r="S203" s="22"/>
@@ -12014,94 +11548,34 @@
       <c r="V207" s="26"/>
     </row>
     <row r="208" spans="1:22">
-      <c r="A208" s="10"/>
-      <c r="B208" s="11"/>
-      <c r="C208" s="12"/>
-      <c r="D208" s="12"/>
-      <c r="E208" s="12"/>
-      <c r="F208" s="22"/>
-      <c r="G208" s="22"/>
-      <c r="H208" s="11"/>
-      <c r="I208" s="24"/>
-      <c r="J208" s="24"/>
-      <c r="K208" s="24"/>
-      <c r="L208" s="24"/>
-      <c r="M208" s="11"/>
-      <c r="N208" s="11"/>
-      <c r="O208" s="11"/>
-      <c r="P208" s="11"/>
-      <c r="Q208" s="18" t="str">
+      <c r="A208" s="13"/>
+      <c r="B208" s="14"/>
+      <c r="C208" s="15"/>
+      <c r="D208" s="15"/>
+      <c r="E208" s="15"/>
+      <c r="F208" s="23"/>
+      <c r="G208" s="23"/>
+      <c r="H208" s="14"/>
+      <c r="I208" s="25"/>
+      <c r="J208" s="25"/>
+      <c r="K208" s="25"/>
+      <c r="L208" s="25"/>
+      <c r="M208" s="14"/>
+      <c r="N208" s="14"/>
+      <c r="O208" s="14"/>
+      <c r="P208" s="14"/>
+      <c r="Q208" s="20" t="str">
         <f t="shared" si="12"/>
         <v/>
       </c>
-      <c r="R208" s="19" t="str">
+      <c r="R208" s="21" t="str">
         <f t="shared" ca="1" si="13"/>
         <v/>
       </c>
-      <c r="S208" s="22"/>
-      <c r="T208" s="22"/>
-      <c r="U208" s="7"/>
-      <c r="V208" s="26"/>
-    </row>
-    <row r="209" spans="1:22">
-      <c r="A209" s="10"/>
-      <c r="B209" s="11"/>
-      <c r="C209" s="12"/>
-      <c r="D209" s="12"/>
-      <c r="E209" s="12"/>
-      <c r="F209" s="22"/>
-      <c r="G209" s="22"/>
-      <c r="H209" s="11"/>
-      <c r="I209" s="24"/>
-      <c r="J209" s="24"/>
-      <c r="K209" s="24"/>
-      <c r="L209" s="24"/>
-      <c r="M209" s="11"/>
-      <c r="N209" s="11"/>
-      <c r="O209" s="11"/>
-      <c r="P209" s="11"/>
-      <c r="Q209" s="18" t="str">
-        <f t="shared" si="12"/>
-        <v/>
-      </c>
-      <c r="R209" s="19" t="str">
-        <f t="shared" ca="1" si="13"/>
-        <v/>
-      </c>
-      <c r="S209" s="22"/>
-      <c r="T209" s="22"/>
-      <c r="U209" s="7"/>
-      <c r="V209" s="26"/>
-    </row>
-    <row r="210" spans="1:22">
-      <c r="A210" s="13"/>
-      <c r="B210" s="14"/>
-      <c r="C210" s="15"/>
-      <c r="D210" s="15"/>
-      <c r="E210" s="15"/>
-      <c r="F210" s="23"/>
-      <c r="G210" s="23"/>
-      <c r="H210" s="14"/>
-      <c r="I210" s="25"/>
-      <c r="J210" s="25"/>
-      <c r="K210" s="25"/>
-      <c r="L210" s="25"/>
-      <c r="M210" s="14"/>
-      <c r="N210" s="14"/>
-      <c r="O210" s="14"/>
-      <c r="P210" s="14"/>
-      <c r="Q210" s="20" t="str">
-        <f t="shared" si="12"/>
-        <v/>
-      </c>
-      <c r="R210" s="21" t="str">
-        <f t="shared" ca="1" si="13"/>
-        <v/>
-      </c>
-      <c r="S210" s="23"/>
-      <c r="T210" s="23"/>
-      <c r="U210" s="8"/>
-      <c r="V210" s="27"/>
+      <c r="S208" s="23"/>
+      <c r="T208" s="23"/>
+      <c r="U208" s="8"/>
+      <c r="V208" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -12111,26 +11585,26 @@
     <mergeCell ref="H5:V6"/>
     <mergeCell ref="A8:V8"/>
   </mergeCells>
-  <conditionalFormatting sqref="P11:P210">
-    <cfRule type="expression" dxfId="41" priority="1">
+  <conditionalFormatting sqref="P11:P208">
+    <cfRule type="expression" dxfId="6" priority="1">
       <formula>P11="RECOMENDADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="40" priority="2">
+    <cfRule type="expression" dxfId="5" priority="2">
       <formula>P11="APROVADA - AGUARDANDO EXECUÇÃO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="39" priority="3">
+    <cfRule type="expression" dxfId="4" priority="3">
       <formula>P11="EXECUTADA - EM MATURAÇÃO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="38" priority="4">
+    <cfRule type="expression" dxfId="3" priority="4">
       <formula>P11="EXECUTADA - AVALIADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="37" priority="5">
+    <cfRule type="expression" dxfId="2" priority="5">
       <formula>P11="APROVADA - NÃO EXECUTADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="36" priority="6">
+    <cfRule type="expression" dxfId="1" priority="6">
       <formula>P11="REJEITADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="35" priority="7">
+    <cfRule type="expression" dxfId="0" priority="7">
       <formula>LEFT(P11,9)="BLOQUEADA"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12146,25 +11620,25 @@
           <x14:formula1>
             <xm:f>Listas!$A$4:$A$15</xm:f>
           </x14:formula1>
-          <xm:sqref>H11:H29 H31:H210</xm:sqref>
+          <xm:sqref>H11:H29 H31:H208</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list">
           <x14:formula1>
             <xm:f>Listas!$G$4:$G$6</xm:f>
           </x14:formula1>
-          <xm:sqref>M11:M210</xm:sqref>
+          <xm:sqref>M11:M208</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list">
           <x14:formula1>
             <xm:f>Listas!$E$4:$E$6</xm:f>
           </x14:formula1>
-          <xm:sqref>N11:O210</xm:sqref>
+          <xm:sqref>N11:O208</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list">
           <x14:formula1>
             <xm:f>Listas!$C$4:$C$11</xm:f>
           </x14:formula1>
-          <xm:sqref>P11:P210</xm:sqref>
+          <xm:sqref>P11:P208</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
[30/09] Registro com EC-017..019 (75 entradas); tela do desconto no preco permite vincular ao evento Prime Big Deal Days (publico Prime, preco fixo)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1193" uniqueCount="637">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1235" uniqueCount="650">
   <si>
     <t>REGISTRO DE ALTERAÇÕES — AMAZON ADS | WINNET METAIS</t>
   </si>
@@ -1941,6 +1941,45 @@
   </si>
   <si>
     <t>gatilho disparou em 28/09, anúncio pausado</t>
+  </si>
+  <si>
+    <t>EC-017</t>
+  </si>
+  <si>
+    <t>Desconto no preço (promoção) — semana do Prime Day</t>
+  </si>
+  <si>
+    <t>PXM (B0H4S3FHG6) — desconto no preço 10%</t>
+  </si>
+  <si>
+    <t>Desconto 10% → R$ 183,19 · piso R$ 183,09 · 05/10 00:00 a 11/10 23:59</t>
+  </si>
+  <si>
+    <t>Converte com qualquer desconto (9.9: 3 un a −15%; 21–27/09: 5 un a −5%). Margem SP Interior 15,0% — no piso; com promo de quantidade empilhada: 11,7% (3+) / 9,5% (5+), risco aceito (o pedido de 3 PXM de 24/09 saiu a 15,6% realizados).</t>
+  </si>
+  <si>
+    <t>ciclos/Monitoramento-28-09.md (adendo 30/09) + Simulador Mestra v4.3.4 + relatorios/amazon/monitoramento-28-09/</t>
+  </si>
+  <si>
+    <t>Plano B do Prime Day: SKU de margem e tráfego adequados que a Amazon não abriu para Melhor Oferta (listas de 22 e 28/09). Sem selo do evento; preço riscado na busca. Não conflita com P3070/PXP (Melhor Oferta). Atribuição do Ads: preço com desconto (regra de 28/09). ⚠️ A promoção de quantidade empilh…</t>
+  </si>
+  <si>
+    <t>EC-018</t>
+  </si>
+  <si>
+    <t>Desconto 10% → R$ 223,88 · piso R$ 217,76 · 05/10 00:00 a 11/10 23:59</t>
+  </si>
+  <si>
+    <t>Converteu com Melhor Oferta a −10% no 9.9 (1 un); 0 a −10% em 21–27/09 (5 sessões). Margem SP Interior 16,7%; com promo de quantidade: 13,5% (3+) / 11,5% (5+).</t>
+  </si>
+  <si>
+    <t>EC-019</t>
+  </si>
+  <si>
+    <t>Desconto 10% → R$ 460,28 · piso R$ 404,24 · 05/10 00:00 a 11/10 23:59</t>
+  </si>
+  <si>
+    <t>Não respondeu a −10% em 21–27/09 (12 sessões, 0 un), mas tem a maior folga entre os com tráfego: 22,6%; com promo de quantidade 19,7% (3+) / 17,8% (5+) — absorve o empilhamento. Teste na semana de maior tráfego.</t>
   </si>
 </sst>
 </file>
@@ -2794,15 +2833,15 @@
     <row r="6" spans="1:22" ht="26.1" customHeight="1">
       <c r="A6" s="2">
         <f>COUNTIF(A11:A208,"&lt;&gt;")</f>
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B6" s="3">
         <f>COUNTIF(N11:N208,"SIM")</f>
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C6" s="3">
         <f>COUNTIF(O11:O208,"SIM")</f>
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D6" s="3">
         <f>COUNTIF(P11:P208,"BLOQUEADA*")</f>
@@ -2810,7 +2849,7 @@
       </c>
       <c r="E6" s="3">
         <f>COUNTIF(P11:P208,"EXECUTADA - EM MATURAÇÃO")</f>
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F6" s="4">
         <f>COUNTIF(P11:P208,"EXECUTADA - AVALIADA")</f>
@@ -2979,7 +3018,7 @@
       </c>
       <c r="R11" s="17">
         <f t="shared" ref="R11:R42" ca="1" si="1">IF(E11="","",TODAY()-E11)</f>
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="S11" s="39" t="s">
         <v>362</v>
@@ -3045,7 +3084,7 @@
       </c>
       <c r="R12" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="S12" s="39" t="s">
         <v>363</v>
@@ -3109,7 +3148,7 @@
       </c>
       <c r="R13" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="S13" s="39" t="s">
         <v>364</v>
@@ -3177,7 +3216,7 @@
       </c>
       <c r="R14" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="S14" s="39" t="s">
         <v>365</v>
@@ -3247,7 +3286,7 @@
       </c>
       <c r="R15" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="S15" s="39" t="s">
         <v>366</v>
@@ -3317,7 +3356,7 @@
       </c>
       <c r="R16" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="S16" s="39" t="s">
         <v>367</v>
@@ -3387,7 +3426,7 @@
       </c>
       <c r="R17" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="S17" s="39" t="s">
         <v>368</v>
@@ -3455,7 +3494,7 @@
       </c>
       <c r="R18" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="S18" s="39" t="s">
         <v>369</v>
@@ -3525,7 +3564,7 @@
       </c>
       <c r="R19" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="S19" s="39" t="s">
         <v>370</v>
@@ -3595,7 +3634,7 @@
       </c>
       <c r="R20" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="S20" s="39" t="s">
         <v>371</v>
@@ -3663,7 +3702,7 @@
       </c>
       <c r="R21" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="S21" s="39" t="s">
         <v>372</v>
@@ -3729,7 +3768,7 @@
       </c>
       <c r="R22" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="S22" s="39" t="s">
         <v>373</v>
@@ -3795,7 +3834,7 @@
       </c>
       <c r="R23" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="S23" s="39" t="s">
         <v>372</v>
@@ -3861,7 +3900,7 @@
       </c>
       <c r="R24" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="S24" s="39" t="s">
         <v>374</v>
@@ -3931,7 +3970,7 @@
       </c>
       <c r="R25" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="S25" s="39" t="s">
         <v>375</v>
@@ -3997,7 +4036,7 @@
       </c>
       <c r="R26" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="S26" s="39" t="s">
         <v>376</v>
@@ -4065,7 +4104,7 @@
       </c>
       <c r="R27" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="S27" s="39" t="s">
         <v>377</v>
@@ -4135,7 +4174,7 @@
       </c>
       <c r="R28" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="S28" s="39" t="s">
         <v>378</v>
@@ -4205,7 +4244,7 @@
       </c>
       <c r="R29" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="S29" s="39" t="s">
         <v>379</v>
@@ -4275,7 +4314,7 @@
       </c>
       <c r="R30" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="S30" s="39" t="s">
         <v>380</v>
@@ -4345,7 +4384,7 @@
       </c>
       <c r="R31" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="S31" s="39" t="s">
         <v>381</v>
@@ -4415,7 +4454,7 @@
       </c>
       <c r="R32" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="S32" s="39" t="s">
         <v>401</v>
@@ -4483,7 +4522,7 @@
       </c>
       <c r="R33" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="S33" s="39" t="s">
         <v>402</v>
@@ -4551,7 +4590,7 @@
       </c>
       <c r="R34" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="S34" s="43" t="s">
         <v>459</v>
@@ -4621,7 +4660,7 @@
       </c>
       <c r="R35" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="S35" s="43" t="s">
         <v>460</v>
@@ -4691,7 +4730,7 @@
       </c>
       <c r="R36" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="S36" t="s">
         <v>584</v>
@@ -4761,7 +4800,7 @@
       </c>
       <c r="R37" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="S37" t="s">
         <v>586</v>
@@ -4831,7 +4870,7 @@
       </c>
       <c r="R38" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="S38" t="s">
         <v>588</v>
@@ -4901,7 +4940,7 @@
       </c>
       <c r="R39" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="S39" t="s">
         <v>590</v>
@@ -4971,7 +5010,7 @@
       </c>
       <c r="R40" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="S40" t="s">
         <v>592</v>
@@ -5041,7 +5080,7 @@
       </c>
       <c r="R41" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="S41" t="s">
         <v>593</v>
@@ -5111,7 +5150,7 @@
       </c>
       <c r="R42" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="S42" t="s">
         <v>595</v>
@@ -5181,7 +5220,7 @@
       </c>
       <c r="R43" s="19">
         <f t="shared" ref="R43:R82" ca="1" si="2">IF(E43="","",TODAY()-E43)</f>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="S43" t="s">
         <v>597</v>
@@ -5251,7 +5290,7 @@
       </c>
       <c r="R44" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="S44" t="s">
         <v>599</v>
@@ -5321,7 +5360,7 @@
       </c>
       <c r="R45" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="S45" t="s">
         <v>601</v>
@@ -5391,7 +5430,7 @@
       </c>
       <c r="R46" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="S46" t="s">
         <v>603</v>
@@ -5461,7 +5500,7 @@
       </c>
       <c r="R47" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="S47" t="s">
         <v>605</v>
@@ -5599,7 +5638,7 @@
       </c>
       <c r="R49" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="S49" t="s">
         <v>609</v>
@@ -5669,7 +5708,7 @@
       </c>
       <c r="R50" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="S50" t="s">
         <v>611</v>
@@ -5739,7 +5778,7 @@
       </c>
       <c r="R51" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="S51" t="s">
         <v>613</v>
@@ -5809,7 +5848,7 @@
       </c>
       <c r="R52" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="S52" t="s">
         <v>615</v>
@@ -5879,7 +5918,7 @@
       </c>
       <c r="R53" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="S53" t="s">
         <v>618</v>
@@ -5949,7 +5988,7 @@
       </c>
       <c r="R54" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="S54" t="s">
         <v>620</v>
@@ -6019,7 +6058,7 @@
       </c>
       <c r="R55" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="S55" t="s">
         <v>622</v>
@@ -6089,7 +6128,7 @@
       </c>
       <c r="R56" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="S56" t="s">
         <v>624</v>
@@ -6159,7 +6198,7 @@
       </c>
       <c r="R57" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="S57" t="s">
         <v>626</v>
@@ -6229,7 +6268,7 @@
       </c>
       <c r="R58" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="S58" t="s">
         <v>628</v>
@@ -6299,7 +6338,7 @@
       </c>
       <c r="R59" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="S59" t="s">
         <v>630</v>
@@ -6369,7 +6408,7 @@
       </c>
       <c r="R60" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="S60" t="s">
         <v>632</v>
@@ -6439,7 +6478,7 @@
       </c>
       <c r="R61" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="S61" t="s">
         <v>632</v>
@@ -6509,7 +6548,7 @@
       </c>
       <c r="R62" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="S62" t="s">
         <v>634</v>
@@ -6579,7 +6618,7 @@
       </c>
       <c r="R63" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U63" t="s">
         <v>469</v>
@@ -6643,7 +6682,7 @@
       </c>
       <c r="R64" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U64" t="s">
         <v>474</v>
@@ -6707,7 +6746,7 @@
       </c>
       <c r="R65" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U65" t="s">
         <v>146</v>
@@ -6771,7 +6810,7 @@
       </c>
       <c r="R66" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U66" t="s">
         <v>469</v>
@@ -6835,7 +6874,7 @@
       </c>
       <c r="R67" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U67" t="s">
         <v>469</v>
@@ -6899,7 +6938,7 @@
       </c>
       <c r="R68" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="T68" t="s">
         <v>636</v>
@@ -6966,7 +7005,7 @@
       </c>
       <c r="R69" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U69" t="s">
         <v>146</v>
@@ -7030,7 +7069,7 @@
       </c>
       <c r="R70" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U70" t="s">
         <v>469</v>
@@ -7094,7 +7133,7 @@
       </c>
       <c r="R71" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U71" t="s">
         <v>146</v>
@@ -7158,7 +7197,7 @@
       </c>
       <c r="R72" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U72" t="s">
         <v>469</v>
@@ -7346,7 +7385,7 @@
       </c>
       <c r="R75" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U75" s="50">
         <v>46308</v>
@@ -7596,7 +7635,7 @@
       </c>
       <c r="R79" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U79" s="50">
         <v>46308</v>
@@ -7660,7 +7699,7 @@
       </c>
       <c r="R80" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U80" t="s">
         <v>469</v>
@@ -7724,7 +7763,7 @@
       </c>
       <c r="R81" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U81" t="s">
         <v>469</v>
@@ -7788,7 +7827,7 @@
       </c>
       <c r="R82" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U82" t="s">
         <v>469</v>
@@ -7798,94 +7837,202 @@
       </c>
     </row>
     <row r="83" spans="1:22">
-      <c r="A83" s="10"/>
-      <c r="B83" s="11"/>
-      <c r="C83" s="12"/>
-      <c r="D83" s="12"/>
-      <c r="E83" s="12"/>
-      <c r="F83" s="43"/>
-      <c r="G83" s="43"/>
-      <c r="H83" s="11"/>
-      <c r="I83" s="11"/>
-      <c r="J83" s="11"/>
-      <c r="K83" s="11"/>
-      <c r="L83" s="11"/>
-      <c r="M83" s="11"/>
-      <c r="N83" s="11"/>
-      <c r="O83" s="11"/>
-      <c r="P83" s="11"/>
-      <c r="Q83" s="18" t="str">
+      <c r="A83" s="10" t="s">
+        <v>637</v>
+      </c>
+      <c r="B83" s="11" t="s">
+        <v>215</v>
+      </c>
+      <c r="C83" s="12">
+        <v>46295</v>
+      </c>
+      <c r="D83" s="12">
+        <v>46295</v>
+      </c>
+      <c r="E83" s="12">
+        <v>46295</v>
+      </c>
+      <c r="F83" s="43" t="s">
+        <v>638</v>
+      </c>
+      <c r="G83" s="43" t="s">
+        <v>639</v>
+      </c>
+      <c r="H83" s="11" t="s">
+        <v>408</v>
+      </c>
+      <c r="I83" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="J83" s="11" t="s">
+        <v>640</v>
+      </c>
+      <c r="K83" s="11" t="s">
+        <v>641</v>
+      </c>
+      <c r="L83" s="11" t="s">
+        <v>642</v>
+      </c>
+      <c r="M83" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="N83" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O83" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="P83" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q83" s="18">
         <f t="shared" ref="Q83:Q104" si="4">IF(E83="","",E83+1)</f>
-        <v/>
-      </c>
-      <c r="R83" s="19" t="str">
+        <v>46296</v>
+      </c>
+      <c r="R83" s="19">
         <f t="shared" ref="R83:R104" ca="1" si="5">IF(E83="","",TODAY()-E83)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S83" s="43"/>
       <c r="T83" s="43"/>
-      <c r="U83" s="7"/>
-      <c r="V83" s="41"/>
+      <c r="U83" s="7">
+        <v>46308</v>
+      </c>
+      <c r="V83" s="41" t="s">
+        <v>643</v>
+      </c>
     </row>
     <row r="84" spans="1:22">
-      <c r="A84" s="10"/>
-      <c r="B84" s="11"/>
-      <c r="C84" s="12"/>
-      <c r="D84" s="12"/>
-      <c r="E84" s="12"/>
-      <c r="F84" s="43"/>
-      <c r="G84" s="43"/>
-      <c r="H84" s="11"/>
-      <c r="I84" s="11"/>
-      <c r="J84" s="11"/>
-      <c r="K84" s="11"/>
-      <c r="L84" s="11"/>
-      <c r="M84" s="11"/>
-      <c r="N84" s="11"/>
-      <c r="O84" s="11"/>
-      <c r="P84" s="11"/>
-      <c r="Q84" s="18" t="str">
+      <c r="A84" s="10" t="s">
+        <v>644</v>
+      </c>
+      <c r="B84" s="11" t="s">
+        <v>215</v>
+      </c>
+      <c r="C84" s="12">
+        <v>46295</v>
+      </c>
+      <c r="D84" s="12">
+        <v>46295</v>
+      </c>
+      <c r="E84" s="12">
+        <v>46295</v>
+      </c>
+      <c r="F84" s="43" t="s">
+        <v>638</v>
+      </c>
+      <c r="G84" s="43" t="s">
+        <v>445</v>
+      </c>
+      <c r="H84" s="11" t="s">
+        <v>408</v>
+      </c>
+      <c r="I84" s="11" t="s">
+        <v>446</v>
+      </c>
+      <c r="J84" s="11" t="s">
+        <v>645</v>
+      </c>
+      <c r="K84" s="11" t="s">
+        <v>646</v>
+      </c>
+      <c r="L84" s="11" t="s">
+        <v>642</v>
+      </c>
+      <c r="M84" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="N84" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O84" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="P84" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q84" s="18">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R84" s="19" t="str">
+        <v>46296</v>
+      </c>
+      <c r="R84" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S84" s="43"/>
       <c r="T84" s="43"/>
-      <c r="U84" s="7"/>
-      <c r="V84" s="41"/>
+      <c r="U84" s="7">
+        <v>46308</v>
+      </c>
+      <c r="V84" s="41" t="s">
+        <v>643</v>
+      </c>
     </row>
     <row r="85" spans="1:22">
-      <c r="A85" s="10"/>
-      <c r="B85" s="11"/>
-      <c r="C85" s="12"/>
-      <c r="D85" s="12"/>
-      <c r="E85" s="12"/>
-      <c r="F85" s="43"/>
-      <c r="G85" s="43"/>
-      <c r="H85" s="11"/>
-      <c r="I85" s="11"/>
-      <c r="J85" s="11"/>
-      <c r="K85" s="11"/>
-      <c r="L85" s="11"/>
-      <c r="M85" s="11"/>
-      <c r="N85" s="11"/>
-      <c r="O85" s="11"/>
-      <c r="P85" s="11"/>
-      <c r="Q85" s="18" t="str">
+      <c r="A85" s="10" t="s">
+        <v>647</v>
+      </c>
+      <c r="B85" s="11" t="s">
+        <v>215</v>
+      </c>
+      <c r="C85" s="12">
+        <v>46295</v>
+      </c>
+      <c r="D85" s="12">
+        <v>46295</v>
+      </c>
+      <c r="E85" s="12">
+        <v>46295</v>
+      </c>
+      <c r="F85" s="43" t="s">
+        <v>638</v>
+      </c>
+      <c r="G85" s="43" t="s">
+        <v>440</v>
+      </c>
+      <c r="H85" s="11" t="s">
+        <v>408</v>
+      </c>
+      <c r="I85" s="11" t="s">
+        <v>441</v>
+      </c>
+      <c r="J85" s="11" t="s">
+        <v>648</v>
+      </c>
+      <c r="K85" s="11" t="s">
+        <v>649</v>
+      </c>
+      <c r="L85" s="11" t="s">
+        <v>642</v>
+      </c>
+      <c r="M85" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="N85" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O85" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="P85" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q85" s="18">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R85" s="19" t="str">
+        <v>46296</v>
+      </c>
+      <c r="R85" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S85" s="43"/>
       <c r="T85" s="43"/>
-      <c r="U85" s="7"/>
-      <c r="V85" s="41"/>
+      <c r="U85" s="7">
+        <v>46308</v>
+      </c>
+      <c r="V85" s="41" t="s">
+        <v>643</v>
+      </c>
     </row>
     <row r="86" spans="1:22">
       <c r="A86" s="10"/>

</xml_diff>

<commit_message>
[30/09] Registro com EC-020 e vereditos EC-017/018/019 (76 entradas); lista dos 48 SKUs sem preco de referencia = 48 sem venda registrada — regra na Memoria
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1235" uniqueCount="650">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1255" uniqueCount="664">
   <si>
     <t>REGISTRO DE ALTERAÇÕES — AMAZON ADS | WINNET METAIS</t>
   </si>
@@ -1980,6 +1980,48 @@
   </si>
   <si>
     <t>Não respondeu a −10% em 21–27/09 (12 sessões, 0 un), mas tem a maior folga entre os com tráfego: 22,6%; com promo de quantidade 19,7% (3+) / 17,8% (5+) — absorve o empilhamento. Teste na semana de maior tráfego.</t>
+  </si>
+  <si>
+    <t>EC-020</t>
+  </si>
+  <si>
+    <t>Desconto no preço comum PRECOPRIMEALTERNATIVO — 05–11/10 (semana do Prime Day, sem vínculo com o evento)</t>
+  </si>
+  <si>
+    <t>Lote de 12 SKUs: L2460-CP, EGC, Q4070-A, L2470-B, L3070-B, P4080, P3050, P3060, PXM, L2460-AML, Q3060-A, L3085-B</t>
+  </si>
+  <si>
+    <t>Preço de tabela nos 12, sem promoção (referência da Amazon = preço de tabela da Mestra, conferido no modelo de upload)</t>
+  </si>
+  <si>
+    <t>Preço fixo a 10% em cada SKU: L2460-CP 302,11 · EGC 607,15 · Q4070-A 947,85 · L2470-B 358,51 · L3070-B 489,46 · P4080 963,15 · P3050 420,90 · P3060 460,27 · PXM 183,18 · L2460-AML 261,15 · Q3060-A 522,46 · L3085-B 578,01 · público Todos os clientes · 05/10 00:00 a 11/10 23:59 · unidades = estoque (2…</t>
+  </si>
+  <si>
+    <t>Prime Day largo aprovado pelo LEO (A+B+C, 59 SKUs + PXM/P3060). O desconto vinculado ao evento (EC-017/019) exigiu frete grátis para envio pelo vendedor e foi descartado; frete grátis + 10% deixaria todo o catálogo abaixo do piso (Mestra SP Interior). O desconto comum não exige frete grátis (provado…</t>
+  </si>
+  <si>
+    <t>ciclos/Monitoramento-28-09.md (adendos 30/09) + dados/PROPOSTA_PrimeDay_desconto_evento_catalogo.csv + Simulador Mestra v4.3.4 + relatorios/amazon/monitoramento-28-09/ (upload_desconto-comum_13-skus_10pct_final_30-09.xlsx, prints etapa 3 e painel 'Em breve')</t>
+  </si>
+  <si>
+    <t>Sem selo do evento e sem 'Preço exclusivo do Prime': preço riscado '10% off' na busca e na página, para todos os clientes. Não conflita com P3070/PXP (Melhor Oferta, sem exigência de frete — conferido no painel em 30/09). 48 SKUs ficaram fora por 'Sem preço de referência' (regra de plataforma: sem v…</t>
+  </si>
+  <si>
+    <t>Criado em 30/09 no desconto vinculado ao evento (PRIMEDAY-DESCONTO-10) e marcado 'Inválido — O SKU não oferece frete grátis' na Etapa 3 (aba de erros marcou todos os participantes).</t>
+  </si>
+  <si>
+    <t>DESCARTADA 30/09 — o desconto vinculado ao evento exige frete grátis para envio pelo vendedor; substituída pela EC-020 (desconto comum, mesmo preço R$ 183,18).</t>
+  </si>
+  <si>
+    <t>DESCARTADA 30/09 — sem preço de referência (desconto invisível); fora do Prime Day; recuperar referência para a Black Friday.</t>
+  </si>
+  <si>
+    <t>Criado em 30/09 a 5% (R$ 236,31) e 'Sem preço de referência'; excluído pelo LEO no mesmo dia, antes do descarte do desconto do evento.</t>
+  </si>
+  <si>
+    <t>Criado em 30/09 no desconto vinculado ao evento e marcado 'Inválido — O SKU não oferece frete grátis' na Etapa 3.</t>
+  </si>
+  <si>
+    <t>DESCARTADA 30/09 — mesma regra da EC-017; substituída pela EC-020 (desconto comum, mesmo preço R$ 460,27).</t>
   </si>
 </sst>
 </file>
@@ -2383,7 +2425,149 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="21">
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9A3412"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFED7AA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF991B1B"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF374151"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF3F4F6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF166534"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFDCFCE7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF3730A3"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFE0E7FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF92400E"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEF3C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1E40AF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFDBEAFE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9A3412"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFED7AA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF991B1B"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF374151"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF3F4F6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF166534"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFDCFCE7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF3730A3"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFE0E7FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF92400E"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEF3C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1E40AF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFDBEAFE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -2833,15 +3017,15 @@
     <row r="6" spans="1:22" ht="26.1" customHeight="1">
       <c r="A6" s="2">
         <f>COUNTIF(A11:A208,"&lt;&gt;")</f>
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B6" s="3">
         <f>COUNTIF(N11:N208,"SIM")</f>
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C6" s="3">
         <f>COUNTIF(O11:O208,"SIM")</f>
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D6" s="3">
         <f>COUNTIF(P11:P208,"BLOQUEADA*")</f>
@@ -2849,11 +3033,11 @@
       </c>
       <c r="E6" s="3">
         <f>COUNTIF(P11:P208,"EXECUTADA - EM MATURAÇÃO")</f>
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F6" s="4">
         <f>COUNTIF(P11:P208,"EXECUTADA - AVALIADA")</f>
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="H6" s="54"/>
       <c r="I6" s="54"/>
@@ -7883,7 +8067,7 @@
         <v>40</v>
       </c>
       <c r="P83" s="11" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="Q83" s="18">
         <f t="shared" ref="Q83:Q104" si="4">IF(E83="","",E83+1)</f>
@@ -7893,11 +8077,13 @@
         <f t="shared" ref="R83:R104" ca="1" si="5">IF(E83="","",TODAY()-E83)</f>
         <v>0</v>
       </c>
-      <c r="S83" s="43"/>
-      <c r="T83" s="43"/>
-      <c r="U83" s="7">
-        <v>46308</v>
-      </c>
+      <c r="S83" s="43" t="s">
+        <v>658</v>
+      </c>
+      <c r="T83" s="43" t="s">
+        <v>659</v>
+      </c>
+      <c r="U83" s="7"/>
       <c r="V83" s="41" t="s">
         <v>643</v>
       </c>
@@ -7949,7 +8135,7 @@
         <v>40</v>
       </c>
       <c r="P84" s="11" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="Q84" s="18">
         <f t="shared" si="4"/>
@@ -7959,11 +8145,13 @@
         <f t="shared" ca="1" si="5"/>
         <v>0</v>
       </c>
-      <c r="S84" s="43"/>
-      <c r="T84" s="43"/>
-      <c r="U84" s="7">
-        <v>46308</v>
-      </c>
+      <c r="S84" s="43" t="s">
+        <v>661</v>
+      </c>
+      <c r="T84" s="43" t="s">
+        <v>660</v>
+      </c>
+      <c r="U84" s="7"/>
       <c r="V84" s="41" t="s">
         <v>643</v>
       </c>
@@ -8015,7 +8203,7 @@
         <v>40</v>
       </c>
       <c r="P85" s="11" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="Q85" s="18">
         <f t="shared" si="4"/>
@@ -8025,8 +8213,12 @@
         <f t="shared" ca="1" si="5"/>
         <v>0</v>
       </c>
-      <c r="S85" s="43"/>
-      <c r="T85" s="43"/>
+      <c r="S85" s="43" t="s">
+        <v>662</v>
+      </c>
+      <c r="T85" s="43" t="s">
+        <v>663</v>
+      </c>
       <c r="U85" s="7">
         <v>46308</v>
       </c>
@@ -8035,34 +8227,70 @@
       </c>
     </row>
     <row r="86" spans="1:22">
-      <c r="A86" s="10"/>
-      <c r="B86" s="11"/>
-      <c r="C86" s="12"/>
-      <c r="D86" s="12"/>
-      <c r="E86" s="12"/>
-      <c r="F86" s="43"/>
-      <c r="G86" s="43"/>
-      <c r="H86" s="11"/>
-      <c r="I86" s="11"/>
-      <c r="J86" s="11"/>
-      <c r="K86" s="11"/>
-      <c r="L86" s="11"/>
-      <c r="M86" s="11"/>
-      <c r="N86" s="11"/>
-      <c r="O86" s="11"/>
-      <c r="P86" s="11"/>
-      <c r="Q86" s="18" t="str">
+      <c r="A86" s="10" t="s">
+        <v>650</v>
+      </c>
+      <c r="B86" s="11" t="s">
+        <v>215</v>
+      </c>
+      <c r="C86" s="12">
+        <v>46295</v>
+      </c>
+      <c r="D86" s="12">
+        <v>46295</v>
+      </c>
+      <c r="E86" s="12">
+        <v>46295</v>
+      </c>
+      <c r="F86" s="43" t="s">
+        <v>651</v>
+      </c>
+      <c r="G86" s="43" t="s">
+        <v>652</v>
+      </c>
+      <c r="H86" s="11" t="s">
+        <v>408</v>
+      </c>
+      <c r="I86" s="11" t="s">
+        <v>653</v>
+      </c>
+      <c r="J86" s="11" t="s">
+        <v>654</v>
+      </c>
+      <c r="K86" s="11" t="s">
+        <v>655</v>
+      </c>
+      <c r="L86" s="11" t="s">
+        <v>656</v>
+      </c>
+      <c r="M86" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="N86" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O86" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="P86" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q86" s="18">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R86" s="19" t="str">
+        <v>46296</v>
+      </c>
+      <c r="R86" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S86" s="43"/>
       <c r="T86" s="43"/>
-      <c r="U86" s="7"/>
-      <c r="V86" s="41"/>
+      <c r="U86" s="7">
+        <v>46308</v>
+      </c>
+      <c r="V86" s="41" t="s">
+        <v>657</v>
+      </c>
     </row>
     <row r="87" spans="1:22">
       <c r="A87" s="10"/>
@@ -11733,25 +11961,25 @@
     <mergeCell ref="A8:V8"/>
   </mergeCells>
   <conditionalFormatting sqref="P11:P208">
-    <cfRule type="expression" dxfId="6" priority="1">
+    <cfRule type="expression" dxfId="20" priority="1">
       <formula>P11="RECOMENDADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="2">
+    <cfRule type="expression" dxfId="19" priority="2">
       <formula>P11="APROVADA - AGUARDANDO EXECUÇÃO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="3">
+    <cfRule type="expression" dxfId="18" priority="3">
       <formula>P11="EXECUTADA - EM MATURAÇÃO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="17" priority="4">
       <formula>P11="EXECUTADA - AVALIADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="5">
+    <cfRule type="expression" dxfId="16" priority="5">
       <formula>P11="APROVADA - NÃO EXECUTADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="6">
+    <cfRule type="expression" dxfId="15" priority="6">
       <formula>P11="REJEITADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="7">
+    <cfRule type="expression" dxfId="14" priority="7">
       <formula>LEFT(P11,9)="BLOQUEADA"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
[01/10] Registro: celulas J/K/V da EC-020 recoladas sem corte (versao curta); 76 entradas, validacoes intactas
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -1994,18 +1994,9 @@
     <t>Preço de tabela nos 12, sem promoção (referência da Amazon = preço de tabela da Mestra, conferido no modelo de upload)</t>
   </si>
   <si>
-    <t>Preço fixo a 10% em cada SKU: L2460-CP 302,11 · EGC 607,15 · Q4070-A 947,85 · L2470-B 358,51 · L3070-B 489,46 · P4080 963,15 · P3050 420,90 · P3060 460,27 · PXM 183,18 · L2460-AML 261,15 · Q3060-A 522,46 · L3085-B 578,01 · público Todos os clientes · 05/10 00:00 a 11/10 23:59 · unidades = estoque (2…</t>
-  </si>
-  <si>
-    <t>Prime Day largo aprovado pelo LEO (A+B+C, 59 SKUs + PXM/P3060). O desconto vinculado ao evento (EC-017/019) exigiu frete grátis para envio pelo vendedor e foi descartado; frete grátis + 10% deixaria todo o catálogo abaixo do piso (Mestra SP Interior). O desconto comum não exige frete grátis (provado…</t>
-  </si>
-  <si>
     <t>ciclos/Monitoramento-28-09.md (adendos 30/09) + dados/PROPOSTA_PrimeDay_desconto_evento_catalogo.csv + Simulador Mestra v4.3.4 + relatorios/amazon/monitoramento-28-09/ (upload_desconto-comum_13-skus_10pct_final_30-09.xlsx, prints etapa 3 e painel 'Em breve')</t>
   </si>
   <si>
-    <t>Sem selo do evento e sem 'Preço exclusivo do Prime': preço riscado '10% off' na busca e na página, para todos os clientes. Não conflita com P3070/PXP (Melhor Oferta, sem exigência de frete — conferido no painel em 30/09). 48 SKUs ficaram fora por 'Sem preço de referência' (regra de plataforma: sem v…</t>
-  </si>
-  <si>
     <t>Criado em 30/09 no desconto vinculado ao evento (PRIMEDAY-DESCONTO-10) e marcado 'Inválido — O SKU não oferece frete grátis' na Etapa 3 (aba de erros marcou todos os participantes).</t>
   </si>
   <si>
@@ -2022,6 +2013,18 @@
   </si>
   <si>
     <t>DESCARTADA 30/09 — mesma regra da EC-017; substituída pela EC-020 (desconto comum, mesmo preço R$ 460,27).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preço fixo a 10%: L2460-CP 302,11 · EGC 607,15 · Q4070-A 947,85 · L2470-B 358,51 · L3070-B 489,46 · P4080 963,15 · P3050 420,90 · P3060 460,27 · PXM 183,18 · L2460-AML 261,15 · Q3060-A 522,46 · L3085-B 578,01 · Todos os clientes · 05/10 00:00–11/10 23:59 · unidades = estoque
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prime Day largo (A+B+C) aprovado pelo LEO. Desconto do evento exigiu frete grátis → descartado (frete grátis + 10% deixa tudo abaixo do piso). Dos 61, só 13 tinham preço de referência; L2450--CZ caiu por ASIN restrito → 12. Margem a 10%: 15,0% (PXM) a 22,6% (P3060); 4 no piso; promo de qtd empilha.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sem selo do evento; riscado '10% off' para todos. Não conflita com P3070/PXP (Melhor Oferta). 48 SKUs fora por 'Sem preço de referência' = nunca venderam (Registro_Vendas); SP-01 inelegível. Ads atribui a preço com desconto. Ler na O7 em 2 blocos. Painel PRECOPRIMEALTERNATIVO Em breve, 12 ASINs.
+</t>
   </si>
 </sst>
 </file>
@@ -2425,149 +2428,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
-  <dxfs count="21">
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9A3412"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFED7AA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF991B1B"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEE2E2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF374151"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF3F4F6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF166534"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDCFCE7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF3730A3"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE0E7FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF92400E"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEF3C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1E40AF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDBEAFE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9A3412"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFED7AA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF991B1B"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEE2E2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF374151"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF3F4F6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF166534"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDCFCE7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF3730A3"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE0E7FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF92400E"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEF3C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1E40AF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDBEAFE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="7">
     <dxf>
       <font>
         <b/>
@@ -3202,7 +3063,7 @@
       </c>
       <c r="R11" s="17">
         <f t="shared" ref="R11:R42" ca="1" si="1">IF(E11="","",TODAY()-E11)</f>
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="S11" s="39" t="s">
         <v>362</v>
@@ -3268,7 +3129,7 @@
       </c>
       <c r="R12" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="S12" s="39" t="s">
         <v>363</v>
@@ -3332,7 +3193,7 @@
       </c>
       <c r="R13" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S13" s="39" t="s">
         <v>364</v>
@@ -3400,7 +3261,7 @@
       </c>
       <c r="R14" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S14" s="39" t="s">
         <v>365</v>
@@ -3470,7 +3331,7 @@
       </c>
       <c r="R15" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S15" s="39" t="s">
         <v>366</v>
@@ -3540,7 +3401,7 @@
       </c>
       <c r="R16" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S16" s="39" t="s">
         <v>367</v>
@@ -3610,7 +3471,7 @@
       </c>
       <c r="R17" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S17" s="39" t="s">
         <v>368</v>
@@ -3678,7 +3539,7 @@
       </c>
       <c r="R18" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S18" s="39" t="s">
         <v>369</v>
@@ -3748,7 +3609,7 @@
       </c>
       <c r="R19" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S19" s="39" t="s">
         <v>370</v>
@@ -3818,7 +3679,7 @@
       </c>
       <c r="R20" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S20" s="39" t="s">
         <v>371</v>
@@ -3886,7 +3747,7 @@
       </c>
       <c r="R21" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S21" s="39" t="s">
         <v>372</v>
@@ -3952,7 +3813,7 @@
       </c>
       <c r="R22" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S22" s="39" t="s">
         <v>373</v>
@@ -4018,7 +3879,7 @@
       </c>
       <c r="R23" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S23" s="39" t="s">
         <v>372</v>
@@ -4084,7 +3945,7 @@
       </c>
       <c r="R24" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S24" s="39" t="s">
         <v>374</v>
@@ -4154,7 +4015,7 @@
       </c>
       <c r="R25" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S25" s="39" t="s">
         <v>375</v>
@@ -4220,7 +4081,7 @@
       </c>
       <c r="R26" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S26" s="39" t="s">
         <v>376</v>
@@ -4288,7 +4149,7 @@
       </c>
       <c r="R27" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S27" s="39" t="s">
         <v>377</v>
@@ -4358,7 +4219,7 @@
       </c>
       <c r="R28" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S28" s="39" t="s">
         <v>378</v>
@@ -4428,7 +4289,7 @@
       </c>
       <c r="R29" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S29" s="39" t="s">
         <v>379</v>
@@ -4498,7 +4359,7 @@
       </c>
       <c r="R30" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="S30" s="39" t="s">
         <v>380</v>
@@ -4568,7 +4429,7 @@
       </c>
       <c r="R31" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S31" s="39" t="s">
         <v>381</v>
@@ -4638,7 +4499,7 @@
       </c>
       <c r="R32" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="S32" s="39" t="s">
         <v>401</v>
@@ -4706,7 +4567,7 @@
       </c>
       <c r="R33" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="S33" s="39" t="s">
         <v>402</v>
@@ -4774,7 +4635,7 @@
       </c>
       <c r="R34" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="S34" s="43" t="s">
         <v>459</v>
@@ -4844,7 +4705,7 @@
       </c>
       <c r="R35" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="S35" s="43" t="s">
         <v>460</v>
@@ -4914,7 +4775,7 @@
       </c>
       <c r="R36" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S36" t="s">
         <v>584</v>
@@ -4984,7 +4845,7 @@
       </c>
       <c r="R37" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S37" t="s">
         <v>586</v>
@@ -5054,7 +4915,7 @@
       </c>
       <c r="R38" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S38" t="s">
         <v>588</v>
@@ -5124,7 +4985,7 @@
       </c>
       <c r="R39" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S39" t="s">
         <v>590</v>
@@ -5194,7 +5055,7 @@
       </c>
       <c r="R40" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S40" t="s">
         <v>592</v>
@@ -5264,7 +5125,7 @@
       </c>
       <c r="R41" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S41" t="s">
         <v>593</v>
@@ -5334,7 +5195,7 @@
       </c>
       <c r="R42" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S42" t="s">
         <v>595</v>
@@ -5404,7 +5265,7 @@
       </c>
       <c r="R43" s="19">
         <f t="shared" ref="R43:R82" ca="1" si="2">IF(E43="","",TODAY()-E43)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S43" t="s">
         <v>597</v>
@@ -5474,7 +5335,7 @@
       </c>
       <c r="R44" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S44" t="s">
         <v>599</v>
@@ -5544,7 +5405,7 @@
       </c>
       <c r="R45" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S45" t="s">
         <v>601</v>
@@ -5614,7 +5475,7 @@
       </c>
       <c r="R46" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S46" t="s">
         <v>603</v>
@@ -5684,7 +5545,7 @@
       </c>
       <c r="R47" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S47" t="s">
         <v>605</v>
@@ -5822,7 +5683,7 @@
       </c>
       <c r="R49" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S49" t="s">
         <v>609</v>
@@ -5892,7 +5753,7 @@
       </c>
       <c r="R50" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S50" t="s">
         <v>611</v>
@@ -5962,7 +5823,7 @@
       </c>
       <c r="R51" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S51" t="s">
         <v>613</v>
@@ -6032,7 +5893,7 @@
       </c>
       <c r="R52" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S52" t="s">
         <v>615</v>
@@ -6102,7 +5963,7 @@
       </c>
       <c r="R53" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S53" t="s">
         <v>618</v>
@@ -6172,7 +6033,7 @@
       </c>
       <c r="R54" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S54" t="s">
         <v>620</v>
@@ -6242,7 +6103,7 @@
       </c>
       <c r="R55" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S55" t="s">
         <v>622</v>
@@ -6312,7 +6173,7 @@
       </c>
       <c r="R56" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S56" t="s">
         <v>624</v>
@@ -6382,7 +6243,7 @@
       </c>
       <c r="R57" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S57" t="s">
         <v>626</v>
@@ -6452,7 +6313,7 @@
       </c>
       <c r="R58" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S58" t="s">
         <v>628</v>
@@ -6522,7 +6383,7 @@
       </c>
       <c r="R59" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S59" t="s">
         <v>630</v>
@@ -6592,7 +6453,7 @@
       </c>
       <c r="R60" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S60" t="s">
         <v>632</v>
@@ -6662,7 +6523,7 @@
       </c>
       <c r="R61" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S61" t="s">
         <v>632</v>
@@ -6732,7 +6593,7 @@
       </c>
       <c r="R62" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S62" t="s">
         <v>634</v>
@@ -6802,7 +6663,7 @@
       </c>
       <c r="R63" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U63" t="s">
         <v>469</v>
@@ -6866,7 +6727,7 @@
       </c>
       <c r="R64" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U64" t="s">
         <v>474</v>
@@ -6930,7 +6791,7 @@
       </c>
       <c r="R65" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U65" t="s">
         <v>146</v>
@@ -6994,7 +6855,7 @@
       </c>
       <c r="R66" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U66" t="s">
         <v>469</v>
@@ -7058,7 +6919,7 @@
       </c>
       <c r="R67" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U67" t="s">
         <v>469</v>
@@ -7122,7 +6983,7 @@
       </c>
       <c r="R68" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T68" t="s">
         <v>636</v>
@@ -7189,7 +7050,7 @@
       </c>
       <c r="R69" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U69" t="s">
         <v>146</v>
@@ -7253,7 +7114,7 @@
       </c>
       <c r="R70" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U70" t="s">
         <v>469</v>
@@ -7317,7 +7178,7 @@
       </c>
       <c r="R71" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U71" t="s">
         <v>146</v>
@@ -7381,7 +7242,7 @@
       </c>
       <c r="R72" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U72" t="s">
         <v>469</v>
@@ -7569,7 +7430,7 @@
       </c>
       <c r="R75" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U75" s="50">
         <v>46308</v>
@@ -7819,7 +7680,7 @@
       </c>
       <c r="R79" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U79" s="50">
         <v>46308</v>
@@ -7883,7 +7744,7 @@
       </c>
       <c r="R80" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U80" t="s">
         <v>469</v>
@@ -7947,7 +7808,7 @@
       </c>
       <c r="R81" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U81" t="s">
         <v>469</v>
@@ -8011,7 +7872,7 @@
       </c>
       <c r="R82" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U82" t="s">
         <v>469</v>
@@ -8075,13 +7936,13 @@
       </c>
       <c r="R83" s="19">
         <f t="shared" ref="R83:R104" ca="1" si="5">IF(E83="","",TODAY()-E83)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S83" s="43" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
       <c r="T83" s="43" t="s">
-        <v>659</v>
+        <v>656</v>
       </c>
       <c r="U83" s="7"/>
       <c r="V83" s="41" t="s">
@@ -8143,13 +8004,13 @@
       </c>
       <c r="R84" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S84" s="43" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
       <c r="T84" s="43" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
       <c r="U84" s="7"/>
       <c r="V84" s="41" t="s">
@@ -8211,13 +8072,13 @@
       </c>
       <c r="R85" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S85" s="43" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="T85" s="43" t="s">
-        <v>663</v>
+        <v>660</v>
       </c>
       <c r="U85" s="7">
         <v>46308</v>
@@ -8255,13 +8116,13 @@
         <v>653</v>
       </c>
       <c r="J86" s="11" t="s">
+        <v>661</v>
+      </c>
+      <c r="K86" s="11" t="s">
+        <v>662</v>
+      </c>
+      <c r="L86" s="11" t="s">
         <v>654</v>
-      </c>
-      <c r="K86" s="11" t="s">
-        <v>655</v>
-      </c>
-      <c r="L86" s="11" t="s">
-        <v>656</v>
       </c>
       <c r="M86" s="11" t="s">
         <v>45</v>
@@ -8281,7 +8142,7 @@
       </c>
       <c r="R86" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S86" s="43"/>
       <c r="T86" s="43"/>
@@ -8289,7 +8150,7 @@
         <v>46308</v>
       </c>
       <c r="V86" s="41" t="s">
-        <v>657</v>
+        <v>663</v>
       </c>
     </row>
     <row r="87" spans="1:22">
@@ -11961,25 +11822,25 @@
     <mergeCell ref="A8:V8"/>
   </mergeCells>
   <conditionalFormatting sqref="P11:P208">
-    <cfRule type="expression" dxfId="20" priority="1">
+    <cfRule type="expression" dxfId="6" priority="1">
       <formula>P11="RECOMENDADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="19" priority="2">
+    <cfRule type="expression" dxfId="5" priority="2">
       <formula>P11="APROVADA - AGUARDANDO EXECUÇÃO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="3">
+    <cfRule type="expression" dxfId="4" priority="3">
       <formula>P11="EXECUTADA - EM MATURAÇÃO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="17" priority="4">
+    <cfRule type="expression" dxfId="3" priority="4">
       <formula>P11="EXECUTADA - AVALIADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="5">
+    <cfRule type="expression" dxfId="2" priority="5">
       <formula>P11="APROVADA - NÃO EXECUTADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="6">
+    <cfRule type="expression" dxfId="1" priority="6">
       <formula>P11="REJEITADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="7">
+    <cfRule type="expression" dxfId="0" priority="7">
       <formula>LEFT(P11,9)="BLOQUEADA"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
[O7 13/10] Registro: 18 linhas O7-001..018 coladas pelo LEO (98 entradas); vereditos da O6 em blocos para colar (P63/S63/U63 + EC-020)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1255" uniqueCount="664">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1512" uniqueCount="766">
   <si>
     <t>REGISTRO DE ALTERAÇÕES — AMAZON ADS | WINNET METAIS</t>
   </si>
@@ -2026,12 +2026,319 @@
     <t xml:space="preserve">Sem selo do evento; riscado '10% off' para todos. Não conflita com P3070/PXP (Melhor Oferta). 48 SKUs fora por 'Sem preço de referência' = nunca venderam (Registro_Vendas); SP-01 inelegível. Ads atribui a preço com desconto. Ler na O7 em 2 blocos. Painel PRECOPRIMEALTERNATIVO Em breve, 12 ASINs.
 </t>
   </si>
+  <si>
+    <t>O7-001</t>
+  </si>
+  <si>
+    <t>O7</t>
+  </si>
+  <si>
+    <t>segmentação close-match (Correspondência aproximada)</t>
+  </si>
+  <si>
+    <t>R$ 0,65 (+20%)</t>
+  </si>
+  <si>
+    <t>ACOS 4,4% em 179 cli / 8 compras (30d); Era da campanha 4,5%; orçamento folgado (12%). Objetivo 9% dá margem para comprar entrega.</t>
+  </si>
+  <si>
+    <t>ciclos/O7-13-10.md + relatorios/amazon/o7-13-10/</t>
+  </si>
+  <si>
+    <t>27/10/2026</t>
+  </si>
+  <si>
+    <t>Reler na O8: se ACOS da segmentação passar de 9%, voltar a 0,54.</t>
+  </si>
+  <si>
+    <t>O7-002</t>
+  </si>
+  <si>
+    <t>segmentação substitutes (Substitutos)</t>
+  </si>
+  <si>
+    <t>ACOS 4,2% em 131 cli / 5 compras (30d). Devolve o lance pré-O5 com evidência de conversão.</t>
+  </si>
+  <si>
+    <t>Mesma régua de saída da O7-001.</t>
+  </si>
+  <si>
+    <t>O7-003</t>
+  </si>
+  <si>
+    <t>alvo asin="B0CYWMQ93Y" (exato, lance 0,90)</t>
+  </si>
+  <si>
+    <t>Ativo</t>
+  </si>
+  <si>
+    <t>18 cliques vitalícios / R$ 17,10 / 0 venda — régua de alvo (15+). Campanha segue ativa (3 vendas vitalícias, ACOS 15,1%).</t>
+  </si>
+  <si>
+    <t>Não converter em pausa de campanha.</t>
+  </si>
+  <si>
+    <t>O7-004</t>
+  </si>
+  <si>
+    <t>ASIN B076VYNP9W (substitutes)</t>
+  </si>
+  <si>
+    <t>Servindo</t>
+  </si>
+  <si>
+    <t>Negativado</t>
+  </si>
+  <si>
+    <t>20 cliques / R$ 9,37 / 0 em 30d — maior dreno da Geral sem venda. Não é irrelevância semântica (é concorrente), por isso MÉDIA.</t>
+  </si>
+  <si>
+    <t>Reavaliar se o SKU anunciado (L2025-T) perder entrega.</t>
+  </si>
+  <si>
+    <t>O7-005</t>
+  </si>
+  <si>
+    <t>frase "dourada"</t>
+  </si>
+  <si>
+    <t>Negativado (frase)</t>
+  </si>
+  <si>
+    <t>"lixeira dourada" 3 cli / R$ 2,07 / 0 — a Winnet não vende acabamento dourado.</t>
+  </si>
+  <si>
+    <t>O7-006</t>
+  </si>
+  <si>
+    <t>6B Lixeiras banheiro + Manual L3070-B</t>
+  </si>
+  <si>
+    <t>estratégia de lance (piloto O4-014 / O5-009 / O6-010)</t>
+  </si>
+  <si>
+    <t>ALTERAR ESTRATÉGIA DE LANCE</t>
+  </si>
+  <si>
+    <t>Lances dinâmicos (aumento e redução)</t>
+  </si>
+  <si>
+    <t>Lances fixos</t>
+  </si>
+  <si>
+    <t>Contrato de saída da O6-010: zero diferença contra o controle em 2 Eras (6B 12 cli/0; L3070-B 2 cli/0; controle 0–1 cli). Piloto encerrado como SEM EFEITO.</t>
+  </si>
+  <si>
+    <t>Conferir no console a estratégia real antes de alterar.</t>
+  </si>
+  <si>
+    <t>O7-007</t>
+  </si>
+  <si>
+    <t>6B Lixeiras banheiro</t>
+  </si>
+  <si>
+    <t>palavra-chave exata "lixo banheiro" (L1618-T + L2025-T)</t>
+  </si>
+  <si>
+    <t>Não existe</t>
+  </si>
+  <si>
+    <t>Exata, lance R$ 0,80</t>
+  </si>
+  <si>
+    <t>Termo provou valor na Geral: 10 cli / R$ 7,31 / 2 compras / R$ 395,70 (ACOS 1,8%). Exata &gt; Frase. CPC médio 0,73.</t>
+  </si>
+  <si>
+    <t>Entra com a 6B já em lances fixos (O7-006).</t>
+  </si>
+  <si>
+    <t>O7-008</t>
+  </si>
+  <si>
+    <t>alvos asin-expanded (lance 1,10)</t>
+  </si>
+  <si>
+    <t>R$ 1,32 (+20%)</t>
+  </si>
+  <si>
+    <t>Radar: 1.015 impressões/30d, 4 cli, 1 compra; vitalício 12 cli / 3 compras. Objetivo é amostra, não gasto (R$ 2,52 em 30d).</t>
+  </si>
+  <si>
+    <t>Contrato de saída: O8 sem aumento de entrega → voltar a 1,10.</t>
+  </si>
+  <si>
+    <t>O7-009</t>
+  </si>
+  <si>
+    <t>alvos asin exatos (lance 0,90)</t>
+  </si>
+  <si>
+    <t>R$ 1,08 (+20%)</t>
+  </si>
+  <si>
+    <t>Régua da assessoria: campanha gastou &lt; R$ 5 em 30d (R$ 2,52) com ACOS abaixo do Máximo → +20% em TODAS as segmentações. Complementa a O7-008.</t>
+  </si>
+  <si>
+    <t>ciclos/O7-13-10_lista-refeita-regua-henrique.md + docs/referencia/Otimizacao_de_ADS_assessoria_Henrique.pdf + relatorios/amazon/o7-13-10/</t>
+  </si>
+  <si>
+    <t>Os dois métodos convergem (Radar + regra "&lt; R$ 5").</t>
+  </si>
+  <si>
+    <t>O7-010</t>
+  </si>
+  <si>
+    <t>Extintor Palavra-Chave Exato Manual</t>
+  </si>
+  <si>
+    <t>exata "suporte para extintor de incêndio"</t>
+  </si>
+  <si>
+    <t>R$ 3,12 (+20%)</t>
+  </si>
+  <si>
+    <t>Regra "&lt; R$ 5 → +20%" reativada pelo LEO em 13/10: 143 impr · 1 cli · R$ 0,72 em 30d. ACOS indefinido (sem venda) lido como "não acima do Máximo".</t>
+  </si>
+  <si>
+    <t>Ressalva: TOS IS 76% — pouca busca, não pouco lance. Ler na O8; se impressões não subirem, a alavanca não é lance.</t>
+  </si>
+  <si>
+    <t>O7-011</t>
+  </si>
+  <si>
+    <t>Cinzeiros 6C</t>
+  </si>
+  <si>
+    <t>exata "lixeira com cinzeiro"</t>
+  </si>
+  <si>
+    <t>R$ 1,92 (+20%)</t>
+  </si>
+  <si>
+    <t>Regra "&lt; R$ 5 → +20%" reativada: 258 impr · 1 cli · R$ 1,56 em 30d.</t>
+  </si>
+  <si>
+    <t>L2460-CZ vendeu pela Geral ("cinzeiro externo"), não por esta manual.</t>
+  </si>
+  <si>
+    <t>O7-012</t>
+  </si>
+  <si>
+    <t>Manual Bituqueiras Space</t>
+  </si>
+  <si>
+    <t>exata "bituqueira de parede"</t>
+  </si>
+  <si>
+    <t>R$ 1,44 (+20%)</t>
+  </si>
+  <si>
+    <t>Regra "&lt; R$ 5 → +20%" reativada: 17 impr · 1 cli · R$ 1,09 em 30d. Anúncios 13/10: SP-PP, SP-FF, SP-T em inserção; SP-01 suspensa (caso 21652133321).</t>
+  </si>
+  <si>
+    <t>Conferir no console se a campanha segue ativa (relatório de 30d termina em 06/10).</t>
+  </si>
+  <si>
+    <t>O7-013</t>
+  </si>
+  <si>
+    <t>Manual Palavra-Chave L3070-B</t>
+  </si>
+  <si>
+    <t>exata "lixeira basculante 50 litros"</t>
+  </si>
+  <si>
+    <t>Regra "&lt; R$ 5 → +20%" reativada: 460 impr · 2 cli · R$ 2,44 em 30d.</t>
+  </si>
+  <si>
+    <t>Executar DEPOIS da O7-006 (estratégia volta a fixo) para o lance novo valer como fixo.</t>
+  </si>
+  <si>
+    <t>O7-014</t>
+  </si>
+  <si>
+    <t>exata "lixeira banheiro 7 litros"</t>
+  </si>
+  <si>
+    <t>R$ 1,80 (+20%)</t>
+  </si>
+  <si>
+    <t>Regra "&lt; R$ 5 → +20%" reativada: 1.196 impr · 1 cli · R$ 2,30 em 30d.</t>
+  </si>
+  <si>
+    <t>Ressalva: CTR 0,08% — lance maior compra impressão, não clique. Se na O8 seguir sem clique, é CORRIGIR CTR, não lance. Não mexer na exata "pia de cozinha" (14/15, vigia).</t>
+  </si>
+  <si>
+    <t>O7-015</t>
+  </si>
+  <si>
+    <t>auto PXP-o311/08</t>
+  </si>
+  <si>
+    <t>R$ 1,58 (+20%)</t>
+  </si>
+  <si>
+    <t>Regra "&lt; R$ 5 → +20%" reativada: 2.879 impr · 3 cli · R$ 3,03 em 30d.</t>
+  </si>
+  <si>
+    <t>Conflita com a vigia da campanha (10/15 cli sem venda em 30d). Checkpoint de 15 cliques continua valendo: se disparar, abre diagnóstico de conversão do PXP antes de qualquer novo aumento.</t>
+  </si>
+  <si>
+    <t>O7-016</t>
+  </si>
+  <si>
+    <t>R$ 80 (+100%)</t>
+  </si>
+  <si>
+    <t>Regra 8 da assessoria: ACOS 0,4% abaixo do Objetivo → +100%. Aprovado pelo LEO. Sem efeito prático: campanha consome 0,2% do orçamento.</t>
+  </si>
+  <si>
+    <t>Executado por fidelidade à régua original; não é alavanca (decisão O4 segue válida para leitura).</t>
+  </si>
+  <si>
+    <t>O7-017</t>
+  </si>
+  <si>
+    <t>R$ 24 (+20%)</t>
+  </si>
+  <si>
+    <t>Regra 8 da assessoria: ACOS 13,0% entre Objetivo e Máximo → +20%. Aprovado pelo LEO. Consome 27% do orçamento.</t>
+  </si>
+  <si>
+    <t>Idem O7-016. Campanha segue sem mexida de lance (gatilho O6-004 não disparou).</t>
+  </si>
+  <si>
+    <t>O7-018</t>
+  </si>
+  <si>
+    <t>Conta (método)</t>
+  </si>
+  <si>
+    <t>réguas de ACOS — Parâmetros §1</t>
+  </si>
+  <si>
+    <t>ALTERAR RÉGUA DE ACOS</t>
+  </si>
+  <si>
+    <t>Objetivo 9% · Máximo 18% · Emergência 36% (fixos)</t>
+  </si>
+  <si>
+    <t>Máximo = margem média 30d (Mestra) · Objetivo = metade · Emergência = dobro → 25% · 12,5% · 50% (margem 13/09–12/10: 25,1%)</t>
+  </si>
+  <si>
+    <t>Definição da assessoria (PDF): ACOS Máximo = margem média bruta dos últimos 30 dias; Objetivo = metade. Aplicado com a margem líquida da Mestra (fonte oficial de margem). Recalcular a cada Ox.</t>
+  </si>
+  <si>
+    <t>Não é ação no console. Print do Gestor Seller (margem bruta) pode refinar o número; até lá vale a Mestra. Diagnóstico da O7 relido: ACOS 5,4% da Era = 43% do Objetivo novo.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <numFmts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="6" formatCode="&quot;R$&quot;\ #,##0;[Red]\-&quot;R$&quot;\ #,##0"/>
     <numFmt numFmtId="8" formatCode="&quot;R$&quot;\ #,##0.00;[Red]\-&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
   <fonts count="16">
@@ -2272,7 +2579,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="14"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2422,6 +2729,12 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2878,11 +3191,11 @@
     <row r="6" spans="1:22" ht="26.1" customHeight="1">
       <c r="A6" s="2">
         <f>COUNTIF(A11:A208,"&lt;&gt;")</f>
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="B6" s="3">
         <f>COUNTIF(N11:N208,"SIM")</f>
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="C6" s="3">
         <f>COUNTIF(O11:O208,"SIM")</f>
@@ -3063,7 +3376,7 @@
       </c>
       <c r="R11" s="17">
         <f t="shared" ref="R11:R42" ca="1" si="1">IF(E11="","",TODAY()-E11)</f>
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="S11" s="39" t="s">
         <v>362</v>
@@ -3129,7 +3442,7 @@
       </c>
       <c r="R12" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="S12" s="39" t="s">
         <v>363</v>
@@ -3193,7 +3506,7 @@
       </c>
       <c r="R13" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="S13" s="39" t="s">
         <v>364</v>
@@ -3261,7 +3574,7 @@
       </c>
       <c r="R14" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="S14" s="39" t="s">
         <v>365</v>
@@ -3331,7 +3644,7 @@
       </c>
       <c r="R15" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="S15" s="39" t="s">
         <v>366</v>
@@ -3401,7 +3714,7 @@
       </c>
       <c r="R16" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="S16" s="39" t="s">
         <v>367</v>
@@ -3471,7 +3784,7 @@
       </c>
       <c r="R17" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="S17" s="39" t="s">
         <v>368</v>
@@ -3539,7 +3852,7 @@
       </c>
       <c r="R18" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="S18" s="39" t="s">
         <v>369</v>
@@ -3609,7 +3922,7 @@
       </c>
       <c r="R19" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="S19" s="39" t="s">
         <v>370</v>
@@ -3679,7 +3992,7 @@
       </c>
       <c r="R20" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="S20" s="39" t="s">
         <v>371</v>
@@ -3747,7 +4060,7 @@
       </c>
       <c r="R21" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="S21" s="39" t="s">
         <v>372</v>
@@ -3813,7 +4126,7 @@
       </c>
       <c r="R22" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="S22" s="39" t="s">
         <v>373</v>
@@ -3879,7 +4192,7 @@
       </c>
       <c r="R23" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="S23" s="39" t="s">
         <v>372</v>
@@ -3945,7 +4258,7 @@
       </c>
       <c r="R24" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="S24" s="39" t="s">
         <v>374</v>
@@ -4015,7 +4328,7 @@
       </c>
       <c r="R25" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="S25" s="39" t="s">
         <v>375</v>
@@ -4081,7 +4394,7 @@
       </c>
       <c r="R26" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="S26" s="39" t="s">
         <v>376</v>
@@ -4149,7 +4462,7 @@
       </c>
       <c r="R27" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="S27" s="39" t="s">
         <v>377</v>
@@ -4219,7 +4532,7 @@
       </c>
       <c r="R28" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="S28" s="39" t="s">
         <v>378</v>
@@ -4289,7 +4602,7 @@
       </c>
       <c r="R29" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="S29" s="39" t="s">
         <v>379</v>
@@ -4359,7 +4672,7 @@
       </c>
       <c r="R30" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="S30" s="39" t="s">
         <v>380</v>
@@ -4429,7 +4742,7 @@
       </c>
       <c r="R31" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="S31" s="39" t="s">
         <v>381</v>
@@ -4499,7 +4812,7 @@
       </c>
       <c r="R32" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="S32" s="39" t="s">
         <v>401</v>
@@ -4567,7 +4880,7 @@
       </c>
       <c r="R33" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="S33" s="39" t="s">
         <v>402</v>
@@ -4635,7 +4948,7 @@
       </c>
       <c r="R34" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="S34" s="43" t="s">
         <v>459</v>
@@ -4705,7 +5018,7 @@
       </c>
       <c r="R35" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="S35" s="43" t="s">
         <v>460</v>
@@ -4775,7 +5088,7 @@
       </c>
       <c r="R36" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="S36" t="s">
         <v>584</v>
@@ -4845,7 +5158,7 @@
       </c>
       <c r="R37" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="S37" t="s">
         <v>586</v>
@@ -4915,7 +5228,7 @@
       </c>
       <c r="R38" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="S38" t="s">
         <v>588</v>
@@ -4985,7 +5298,7 @@
       </c>
       <c r="R39" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="S39" t="s">
         <v>590</v>
@@ -5055,7 +5368,7 @@
       </c>
       <c r="R40" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="S40" t="s">
         <v>592</v>
@@ -5125,7 +5438,7 @@
       </c>
       <c r="R41" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="S41" t="s">
         <v>593</v>
@@ -5195,7 +5508,7 @@
       </c>
       <c r="R42" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="S42" t="s">
         <v>595</v>
@@ -5265,7 +5578,7 @@
       </c>
       <c r="R43" s="19">
         <f t="shared" ref="R43:R82" ca="1" si="2">IF(E43="","",TODAY()-E43)</f>
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="S43" t="s">
         <v>597</v>
@@ -5335,7 +5648,7 @@
       </c>
       <c r="R44" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="S44" t="s">
         <v>599</v>
@@ -5405,7 +5718,7 @@
       </c>
       <c r="R45" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="S45" t="s">
         <v>601</v>
@@ -5475,7 +5788,7 @@
       </c>
       <c r="R46" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="S46" t="s">
         <v>603</v>
@@ -5545,7 +5858,7 @@
       </c>
       <c r="R47" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="S47" t="s">
         <v>605</v>
@@ -5683,7 +5996,7 @@
       </c>
       <c r="R49" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="S49" t="s">
         <v>609</v>
@@ -5753,7 +6066,7 @@
       </c>
       <c r="R50" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="S50" t="s">
         <v>611</v>
@@ -5823,7 +6136,7 @@
       </c>
       <c r="R51" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="S51" t="s">
         <v>613</v>
@@ -5893,7 +6206,7 @@
       </c>
       <c r="R52" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="S52" t="s">
         <v>615</v>
@@ -5963,7 +6276,7 @@
       </c>
       <c r="R53" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="S53" t="s">
         <v>618</v>
@@ -6033,7 +6346,7 @@
       </c>
       <c r="R54" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="S54" t="s">
         <v>620</v>
@@ -6103,7 +6416,7 @@
       </c>
       <c r="R55" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="S55" t="s">
         <v>622</v>
@@ -6173,7 +6486,7 @@
       </c>
       <c r="R56" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="S56" t="s">
         <v>624</v>
@@ -6243,7 +6556,7 @@
       </c>
       <c r="R57" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="S57" t="s">
         <v>626</v>
@@ -6313,7 +6626,7 @@
       </c>
       <c r="R58" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="S58" t="s">
         <v>628</v>
@@ -6383,7 +6696,7 @@
       </c>
       <c r="R59" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="S59" t="s">
         <v>630</v>
@@ -6453,7 +6766,7 @@
       </c>
       <c r="R60" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="S60" t="s">
         <v>632</v>
@@ -6523,7 +6836,7 @@
       </c>
       <c r="R61" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="S61" t="s">
         <v>632</v>
@@ -6593,7 +6906,7 @@
       </c>
       <c r="R62" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="S62" t="s">
         <v>634</v>
@@ -6663,7 +6976,7 @@
       </c>
       <c r="R63" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="U63" t="s">
         <v>469</v>
@@ -6727,7 +7040,7 @@
       </c>
       <c r="R64" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="U64" t="s">
         <v>474</v>
@@ -6791,7 +7104,7 @@
       </c>
       <c r="R65" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="U65" t="s">
         <v>146</v>
@@ -6855,7 +7168,7 @@
       </c>
       <c r="R66" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="U66" t="s">
         <v>469</v>
@@ -6919,7 +7232,7 @@
       </c>
       <c r="R67" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="U67" t="s">
         <v>469</v>
@@ -6983,7 +7296,7 @@
       </c>
       <c r="R68" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="T68" t="s">
         <v>636</v>
@@ -7050,7 +7363,7 @@
       </c>
       <c r="R69" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="U69" t="s">
         <v>146</v>
@@ -7114,7 +7427,7 @@
       </c>
       <c r="R70" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="U70" t="s">
         <v>469</v>
@@ -7178,7 +7491,7 @@
       </c>
       <c r="R71" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="U71" t="s">
         <v>146</v>
@@ -7242,7 +7555,7 @@
       </c>
       <c r="R72" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="U72" t="s">
         <v>469</v>
@@ -7430,7 +7743,7 @@
       </c>
       <c r="R75" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="U75" s="50">
         <v>46308</v>
@@ -7680,7 +7993,7 @@
       </c>
       <c r="R79" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="U79" s="50">
         <v>46308</v>
@@ -7744,7 +8057,7 @@
       </c>
       <c r="R80" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="U80" t="s">
         <v>469</v>
@@ -7808,7 +8121,7 @@
       </c>
       <c r="R81" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="U81" t="s">
         <v>469</v>
@@ -7872,7 +8185,7 @@
       </c>
       <c r="R82" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="U82" t="s">
         <v>469</v>
@@ -7936,7 +8249,7 @@
       </c>
       <c r="R83" s="19">
         <f t="shared" ref="R83:R104" ca="1" si="5">IF(E83="","",TODAY()-E83)</f>
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="S83" s="43" t="s">
         <v>655</v>
@@ -8004,7 +8317,7 @@
       </c>
       <c r="R84" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="S84" s="43" t="s">
         <v>658</v>
@@ -8072,7 +8385,7 @@
       </c>
       <c r="R85" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="S85" s="43" t="s">
         <v>659</v>
@@ -8142,7 +8455,7 @@
       </c>
       <c r="R86" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="S86" s="43"/>
       <c r="T86" s="43"/>
@@ -8154,544 +8467,1190 @@
       </c>
     </row>
     <row r="87" spans="1:22">
-      <c r="A87" s="10"/>
-      <c r="B87" s="11"/>
-      <c r="C87" s="12"/>
-      <c r="D87" s="12"/>
-      <c r="E87" s="12"/>
-      <c r="F87" s="43"/>
-      <c r="G87" s="43"/>
-      <c r="H87" s="11"/>
-      <c r="I87" s="11"/>
-      <c r="J87" s="11"/>
-      <c r="K87" s="11"/>
-      <c r="L87" s="11"/>
-      <c r="M87" s="11"/>
-      <c r="N87" s="11"/>
-      <c r="O87" s="11"/>
-      <c r="P87" s="11"/>
-      <c r="Q87" s="18" t="str">
+      <c r="A87" s="10" t="s">
+        <v>664</v>
+      </c>
+      <c r="B87" s="11" t="s">
+        <v>665</v>
+      </c>
+      <c r="C87" s="12">
+        <v>46308</v>
+      </c>
+      <c r="D87" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E87" s="12">
+        <v>46308</v>
+      </c>
+      <c r="F87" s="43" t="s">
+        <v>264</v>
+      </c>
+      <c r="G87" s="43" t="s">
+        <v>666</v>
+      </c>
+      <c r="H87" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="I87" s="58">
+        <v>0.54</v>
+      </c>
+      <c r="J87" s="11" t="s">
+        <v>667</v>
+      </c>
+      <c r="K87" s="11" t="s">
+        <v>668</v>
+      </c>
+      <c r="L87" s="11" t="s">
+        <v>669</v>
+      </c>
+      <c r="M87" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="N87" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O87" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="P87" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q87" s="18">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R87" s="19" t="str">
+        <v>46309</v>
+      </c>
+      <c r="R87" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S87" s="43"/>
       <c r="T87" s="43"/>
-      <c r="U87" s="7"/>
-      <c r="V87" s="41"/>
+      <c r="U87" s="7" t="s">
+        <v>670</v>
+      </c>
+      <c r="V87" s="41" t="s">
+        <v>671</v>
+      </c>
     </row>
     <row r="88" spans="1:22">
-      <c r="A88" s="10"/>
-      <c r="B88" s="11"/>
-      <c r="C88" s="12"/>
-      <c r="D88" s="12"/>
-      <c r="E88" s="12"/>
-      <c r="F88" s="43"/>
-      <c r="G88" s="43"/>
-      <c r="H88" s="11"/>
-      <c r="I88" s="11"/>
-      <c r="J88" s="11"/>
-      <c r="K88" s="11"/>
-      <c r="L88" s="11"/>
-      <c r="M88" s="11"/>
-      <c r="N88" s="11"/>
-      <c r="O88" s="11"/>
-      <c r="P88" s="11"/>
-      <c r="Q88" s="18" t="str">
+      <c r="A88" s="10" t="s">
+        <v>672</v>
+      </c>
+      <c r="B88" s="11" t="s">
+        <v>665</v>
+      </c>
+      <c r="C88" s="12">
+        <v>46308</v>
+      </c>
+      <c r="D88" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E88" s="12">
+        <v>46308</v>
+      </c>
+      <c r="F88" s="43" t="s">
+        <v>264</v>
+      </c>
+      <c r="G88" s="43" t="s">
+        <v>673</v>
+      </c>
+      <c r="H88" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="I88" s="58">
+        <v>0.45</v>
+      </c>
+      <c r="J88" s="11" t="s">
+        <v>304</v>
+      </c>
+      <c r="K88" s="11" t="s">
+        <v>674</v>
+      </c>
+      <c r="L88" s="11" t="s">
+        <v>669</v>
+      </c>
+      <c r="M88" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="N88" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O88" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="P88" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q88" s="18">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R88" s="19" t="str">
+        <v>46309</v>
+      </c>
+      <c r="R88" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S88" s="43"/>
       <c r="T88" s="43"/>
-      <c r="U88" s="7"/>
-      <c r="V88" s="41"/>
+      <c r="U88" s="7" t="s">
+        <v>670</v>
+      </c>
+      <c r="V88" s="41" t="s">
+        <v>675</v>
+      </c>
     </row>
     <row r="89" spans="1:22">
-      <c r="A89" s="10"/>
-      <c r="B89" s="11"/>
-      <c r="C89" s="12"/>
-      <c r="D89" s="12"/>
-      <c r="E89" s="12"/>
-      <c r="F89" s="43"/>
-      <c r="G89" s="43"/>
-      <c r="H89" s="11"/>
-      <c r="I89" s="11"/>
-      <c r="J89" s="11"/>
-      <c r="K89" s="11"/>
-      <c r="L89" s="11"/>
-      <c r="M89" s="11"/>
-      <c r="N89" s="11"/>
-      <c r="O89" s="11"/>
-      <c r="P89" s="11"/>
-      <c r="Q89" s="18" t="str">
+      <c r="A89" s="10" t="s">
+        <v>676</v>
+      </c>
+      <c r="B89" s="11" t="s">
+        <v>665</v>
+      </c>
+      <c r="C89" s="12">
+        <v>46308</v>
+      </c>
+      <c r="D89" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E89" s="12">
+        <v>46308</v>
+      </c>
+      <c r="F89" s="43" t="s">
+        <v>270</v>
+      </c>
+      <c r="G89" s="43" t="s">
+        <v>677</v>
+      </c>
+      <c r="H89" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="I89" s="11" t="s">
+        <v>678</v>
+      </c>
+      <c r="J89" s="11" t="s">
+        <v>479</v>
+      </c>
+      <c r="K89" s="11" t="s">
+        <v>679</v>
+      </c>
+      <c r="L89" s="11" t="s">
+        <v>669</v>
+      </c>
+      <c r="M89" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="N89" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O89" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="P89" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q89" s="18">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R89" s="19" t="str">
+        <v>46309</v>
+      </c>
+      <c r="R89" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S89" s="43"/>
       <c r="T89" s="43"/>
-      <c r="U89" s="7"/>
-      <c r="V89" s="41"/>
+      <c r="U89" s="7" t="s">
+        <v>670</v>
+      </c>
+      <c r="V89" s="41" t="s">
+        <v>680</v>
+      </c>
     </row>
     <row r="90" spans="1:22">
-      <c r="A90" s="10"/>
-      <c r="B90" s="11"/>
-      <c r="C90" s="12"/>
-      <c r="D90" s="12"/>
-      <c r="E90" s="12"/>
-      <c r="F90" s="43"/>
-      <c r="G90" s="43"/>
-      <c r="H90" s="11"/>
-      <c r="I90" s="11"/>
-      <c r="J90" s="11"/>
-      <c r="K90" s="11"/>
-      <c r="L90" s="11"/>
-      <c r="M90" s="11"/>
-      <c r="N90" s="11"/>
-      <c r="O90" s="11"/>
-      <c r="P90" s="11"/>
-      <c r="Q90" s="18" t="str">
+      <c r="A90" s="10" t="s">
+        <v>681</v>
+      </c>
+      <c r="B90" s="11" t="s">
+        <v>665</v>
+      </c>
+      <c r="C90" s="12">
+        <v>46308</v>
+      </c>
+      <c r="D90" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E90" s="12">
+        <v>46308</v>
+      </c>
+      <c r="F90" s="43" t="s">
+        <v>264</v>
+      </c>
+      <c r="G90" s="43" t="s">
+        <v>682</v>
+      </c>
+      <c r="H90" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="I90" s="11" t="s">
+        <v>683</v>
+      </c>
+      <c r="J90" s="11" t="s">
+        <v>684</v>
+      </c>
+      <c r="K90" s="11" t="s">
+        <v>685</v>
+      </c>
+      <c r="L90" s="11" t="s">
+        <v>669</v>
+      </c>
+      <c r="M90" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="N90" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O90" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="P90" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q90" s="18">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R90" s="19" t="str">
+        <v>46309</v>
+      </c>
+      <c r="R90" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S90" s="43"/>
       <c r="T90" s="43"/>
-      <c r="U90" s="7"/>
-      <c r="V90" s="41"/>
+      <c r="U90" s="7" t="s">
+        <v>670</v>
+      </c>
+      <c r="V90" s="41" t="s">
+        <v>686</v>
+      </c>
     </row>
     <row r="91" spans="1:22">
-      <c r="A91" s="10"/>
-      <c r="B91" s="11"/>
-      <c r="C91" s="12"/>
-      <c r="D91" s="12"/>
-      <c r="E91" s="12"/>
-      <c r="F91" s="43"/>
-      <c r="G91" s="43"/>
-      <c r="H91" s="11"/>
-      <c r="I91" s="11"/>
-      <c r="J91" s="11"/>
-      <c r="K91" s="11"/>
-      <c r="L91" s="11"/>
-      <c r="M91" s="11"/>
-      <c r="N91" s="11"/>
-      <c r="O91" s="11"/>
-      <c r="P91" s="11"/>
-      <c r="Q91" s="18" t="str">
+      <c r="A91" s="10" t="s">
+        <v>687</v>
+      </c>
+      <c r="B91" s="11" t="s">
+        <v>665</v>
+      </c>
+      <c r="C91" s="12">
+        <v>46308</v>
+      </c>
+      <c r="D91" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E91" s="12">
+        <v>46308</v>
+      </c>
+      <c r="F91" s="43" t="s">
+        <v>264</v>
+      </c>
+      <c r="G91" s="43" t="s">
+        <v>688</v>
+      </c>
+      <c r="H91" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="I91" s="11" t="s">
+        <v>683</v>
+      </c>
+      <c r="J91" s="11" t="s">
+        <v>689</v>
+      </c>
+      <c r="K91" s="11" t="s">
+        <v>690</v>
+      </c>
+      <c r="L91" s="11" t="s">
+        <v>669</v>
+      </c>
+      <c r="M91" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="N91" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O91" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="P91" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q91" s="18">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R91" s="19" t="str">
+        <v>46309</v>
+      </c>
+      <c r="R91" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S91" s="43"/>
       <c r="T91" s="43"/>
-      <c r="U91" s="7"/>
+      <c r="U91" s="7" t="s">
+        <v>670</v>
+      </c>
       <c r="V91" s="41"/>
     </row>
     <row r="92" spans="1:22">
-      <c r="A92" s="10"/>
-      <c r="B92" s="11"/>
-      <c r="C92" s="12"/>
-      <c r="D92" s="12"/>
-      <c r="E92" s="12"/>
-      <c r="F92" s="43"/>
-      <c r="G92" s="43"/>
-      <c r="H92" s="11"/>
-      <c r="I92" s="11"/>
-      <c r="J92" s="11"/>
-      <c r="K92" s="11"/>
-      <c r="L92" s="11"/>
-      <c r="M92" s="11"/>
-      <c r="N92" s="11"/>
-      <c r="O92" s="11"/>
-      <c r="P92" s="11"/>
-      <c r="Q92" s="18" t="str">
+      <c r="A92" s="10" t="s">
+        <v>691</v>
+      </c>
+      <c r="B92" s="11" t="s">
+        <v>665</v>
+      </c>
+      <c r="C92" s="12">
+        <v>46308</v>
+      </c>
+      <c r="D92" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E92" s="12">
+        <v>46308</v>
+      </c>
+      <c r="F92" s="43" t="s">
+        <v>692</v>
+      </c>
+      <c r="G92" s="43" t="s">
+        <v>693</v>
+      </c>
+      <c r="H92" s="11" t="s">
+        <v>694</v>
+      </c>
+      <c r="I92" s="11" t="s">
+        <v>695</v>
+      </c>
+      <c r="J92" s="11" t="s">
+        <v>696</v>
+      </c>
+      <c r="K92" s="11" t="s">
+        <v>697</v>
+      </c>
+      <c r="L92" s="11" t="s">
+        <v>669</v>
+      </c>
+      <c r="M92" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="N92" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O92" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="P92" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q92" s="18">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R92" s="19" t="str">
+        <v>46309</v>
+      </c>
+      <c r="R92" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S92" s="43"/>
       <c r="T92" s="43"/>
-      <c r="U92" s="7"/>
-      <c r="V92" s="41"/>
+      <c r="U92" s="7" t="s">
+        <v>670</v>
+      </c>
+      <c r="V92" s="41" t="s">
+        <v>698</v>
+      </c>
     </row>
     <row r="93" spans="1:22">
-      <c r="A93" s="10"/>
-      <c r="B93" s="11"/>
-      <c r="C93" s="12"/>
-      <c r="D93" s="12"/>
-      <c r="E93" s="12"/>
-      <c r="F93" s="43"/>
-      <c r="G93" s="43"/>
-      <c r="H93" s="11"/>
-      <c r="I93" s="11"/>
-      <c r="J93" s="11"/>
-      <c r="K93" s="11"/>
-      <c r="L93" s="11"/>
-      <c r="M93" s="11"/>
-      <c r="N93" s="11"/>
-      <c r="O93" s="11"/>
-      <c r="P93" s="11"/>
-      <c r="Q93" s="18" t="str">
+      <c r="A93" s="10" t="s">
+        <v>699</v>
+      </c>
+      <c r="B93" s="11" t="s">
+        <v>665</v>
+      </c>
+      <c r="C93" s="12">
+        <v>46308</v>
+      </c>
+      <c r="D93" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E93" s="12">
+        <v>46308</v>
+      </c>
+      <c r="F93" s="43" t="s">
+        <v>700</v>
+      </c>
+      <c r="G93" s="43" t="s">
+        <v>701</v>
+      </c>
+      <c r="H93" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="I93" s="11" t="s">
+        <v>702</v>
+      </c>
+      <c r="J93" s="11" t="s">
+        <v>703</v>
+      </c>
+      <c r="K93" s="11" t="s">
+        <v>704</v>
+      </c>
+      <c r="L93" s="11" t="s">
+        <v>669</v>
+      </c>
+      <c r="M93" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="N93" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O93" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="P93" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q93" s="18">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R93" s="19" t="str">
+        <v>46309</v>
+      </c>
+      <c r="R93" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S93" s="43"/>
       <c r="T93" s="43"/>
-      <c r="U93" s="7"/>
-      <c r="V93" s="41"/>
+      <c r="U93" s="7" t="s">
+        <v>670</v>
+      </c>
+      <c r="V93" s="41" t="s">
+        <v>705</v>
+      </c>
     </row>
     <row r="94" spans="1:22">
-      <c r="A94" s="10"/>
-      <c r="B94" s="11"/>
-      <c r="C94" s="12"/>
-      <c r="D94" s="12"/>
-      <c r="E94" s="12"/>
-      <c r="F94" s="43"/>
-      <c r="G94" s="43"/>
-      <c r="H94" s="11"/>
-      <c r="I94" s="11"/>
-      <c r="J94" s="11"/>
-      <c r="K94" s="11"/>
-      <c r="L94" s="11"/>
-      <c r="M94" s="11"/>
-      <c r="N94" s="11"/>
-      <c r="O94" s="11"/>
-      <c r="P94" s="11"/>
-      <c r="Q94" s="18" t="str">
+      <c r="A94" s="10" t="s">
+        <v>706</v>
+      </c>
+      <c r="B94" s="11" t="s">
+        <v>665</v>
+      </c>
+      <c r="C94" s="12">
+        <v>46308</v>
+      </c>
+      <c r="D94" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E94" s="12">
+        <v>46308</v>
+      </c>
+      <c r="F94" s="43" t="s">
+        <v>272</v>
+      </c>
+      <c r="G94" s="43" t="s">
+        <v>707</v>
+      </c>
+      <c r="H94" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="I94" s="58">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="J94" s="11" t="s">
+        <v>708</v>
+      </c>
+      <c r="K94" s="11" t="s">
+        <v>709</v>
+      </c>
+      <c r="L94" s="11" t="s">
+        <v>669</v>
+      </c>
+      <c r="M94" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="N94" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O94" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="P94" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q94" s="18">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R94" s="19" t="str">
+        <v>46309</v>
+      </c>
+      <c r="R94" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S94" s="43"/>
       <c r="T94" s="43"/>
-      <c r="U94" s="7"/>
-      <c r="V94" s="41"/>
+      <c r="U94" s="7" t="s">
+        <v>670</v>
+      </c>
+      <c r="V94" s="41" t="s">
+        <v>710</v>
+      </c>
     </row>
     <row r="95" spans="1:22">
-      <c r="A95" s="10"/>
-      <c r="B95" s="11"/>
-      <c r="C95" s="12"/>
-      <c r="D95" s="12"/>
-      <c r="E95" s="12"/>
-      <c r="F95" s="43"/>
-      <c r="G95" s="43"/>
-      <c r="H95" s="11"/>
-      <c r="I95" s="11"/>
-      <c r="J95" s="11"/>
-      <c r="K95" s="11"/>
-      <c r="L95" s="11"/>
-      <c r="M95" s="11"/>
-      <c r="N95" s="11"/>
-      <c r="O95" s="11"/>
-      <c r="P95" s="11"/>
-      <c r="Q95" s="18" t="str">
+      <c r="A95" s="10" t="s">
+        <v>711</v>
+      </c>
+      <c r="B95" s="11" t="s">
+        <v>665</v>
+      </c>
+      <c r="C95" s="12">
+        <v>46308</v>
+      </c>
+      <c r="D95" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E95" s="12">
+        <v>46308</v>
+      </c>
+      <c r="F95" s="43" t="s">
+        <v>272</v>
+      </c>
+      <c r="G95" s="43" t="s">
+        <v>712</v>
+      </c>
+      <c r="H95" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="I95" s="58">
+        <v>0.9</v>
+      </c>
+      <c r="J95" s="11" t="s">
+        <v>713</v>
+      </c>
+      <c r="K95" s="11" t="s">
+        <v>714</v>
+      </c>
+      <c r="L95" s="11" t="s">
+        <v>715</v>
+      </c>
+      <c r="M95" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="N95" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O95" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="P95" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q95" s="18">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R95" s="19" t="str">
+        <v>46309</v>
+      </c>
+      <c r="R95" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S95" s="43"/>
       <c r="T95" s="43"/>
-      <c r="U95" s="7"/>
-      <c r="V95" s="41"/>
+      <c r="U95" s="7" t="s">
+        <v>670</v>
+      </c>
+      <c r="V95" s="41" t="s">
+        <v>716</v>
+      </c>
     </row>
     <row r="96" spans="1:22">
-      <c r="A96" s="10"/>
-      <c r="B96" s="11"/>
-      <c r="C96" s="12"/>
-      <c r="D96" s="12"/>
-      <c r="E96" s="12"/>
-      <c r="F96" s="43"/>
-      <c r="G96" s="43"/>
-      <c r="H96" s="11"/>
-      <c r="I96" s="11"/>
-      <c r="J96" s="11"/>
-      <c r="K96" s="11"/>
-      <c r="L96" s="11"/>
-      <c r="M96" s="11"/>
-      <c r="N96" s="11"/>
-      <c r="O96" s="11"/>
-      <c r="P96" s="11"/>
-      <c r="Q96" s="18" t="str">
+      <c r="A96" s="10" t="s">
+        <v>717</v>
+      </c>
+      <c r="B96" s="11" t="s">
+        <v>665</v>
+      </c>
+      <c r="C96" s="12">
+        <v>46308</v>
+      </c>
+      <c r="D96" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E96" s="12">
+        <v>46308</v>
+      </c>
+      <c r="F96" s="43" t="s">
+        <v>718</v>
+      </c>
+      <c r="G96" s="43" t="s">
+        <v>719</v>
+      </c>
+      <c r="H96" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="I96" s="58">
+        <v>2.6</v>
+      </c>
+      <c r="J96" s="11" t="s">
+        <v>720</v>
+      </c>
+      <c r="K96" s="11" t="s">
+        <v>721</v>
+      </c>
+      <c r="L96" s="11" t="s">
+        <v>715</v>
+      </c>
+      <c r="M96" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N96" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O96" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="P96" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q96" s="18">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R96" s="19" t="str">
+        <v>46309</v>
+      </c>
+      <c r="R96" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S96" s="43"/>
       <c r="T96" s="43"/>
-      <c r="U96" s="7"/>
-      <c r="V96" s="41"/>
+      <c r="U96" s="7" t="s">
+        <v>670</v>
+      </c>
+      <c r="V96" s="41" t="s">
+        <v>722</v>
+      </c>
     </row>
     <row r="97" spans="1:22">
-      <c r="A97" s="10"/>
-      <c r="B97" s="11"/>
-      <c r="C97" s="12"/>
-      <c r="D97" s="12"/>
-      <c r="E97" s="12"/>
-      <c r="F97" s="43"/>
-      <c r="G97" s="43"/>
-      <c r="H97" s="11"/>
-      <c r="I97" s="11"/>
-      <c r="J97" s="11"/>
-      <c r="K97" s="11"/>
-      <c r="L97" s="11"/>
-      <c r="M97" s="11"/>
-      <c r="N97" s="11"/>
-      <c r="O97" s="11"/>
-      <c r="P97" s="11"/>
-      <c r="Q97" s="18" t="str">
+      <c r="A97" s="10" t="s">
+        <v>723</v>
+      </c>
+      <c r="B97" s="11" t="s">
+        <v>665</v>
+      </c>
+      <c r="C97" s="12">
+        <v>46308</v>
+      </c>
+      <c r="D97" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E97" s="12">
+        <v>46308</v>
+      </c>
+      <c r="F97" s="43" t="s">
+        <v>724</v>
+      </c>
+      <c r="G97" s="43" t="s">
+        <v>725</v>
+      </c>
+      <c r="H97" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="I97" s="58">
+        <v>1.6</v>
+      </c>
+      <c r="J97" s="11" t="s">
+        <v>726</v>
+      </c>
+      <c r="K97" s="11" t="s">
+        <v>727</v>
+      </c>
+      <c r="L97" s="11" t="s">
+        <v>715</v>
+      </c>
+      <c r="M97" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N97" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O97" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="P97" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q97" s="18">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R97" s="19" t="str">
+        <v>46309</v>
+      </c>
+      <c r="R97" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S97" s="43"/>
       <c r="T97" s="43"/>
-      <c r="U97" s="7"/>
-      <c r="V97" s="41"/>
+      <c r="U97" s="7" t="s">
+        <v>670</v>
+      </c>
+      <c r="V97" s="41" t="s">
+        <v>728</v>
+      </c>
     </row>
     <row r="98" spans="1:22">
-      <c r="A98" s="10"/>
-      <c r="B98" s="11"/>
-      <c r="C98" s="12"/>
-      <c r="D98" s="12"/>
-      <c r="E98" s="12"/>
-      <c r="F98" s="43"/>
-      <c r="G98" s="43"/>
-      <c r="H98" s="11"/>
-      <c r="I98" s="11"/>
-      <c r="J98" s="11"/>
-      <c r="K98" s="11"/>
-      <c r="L98" s="11"/>
-      <c r="M98" s="11"/>
-      <c r="N98" s="11"/>
-      <c r="O98" s="11"/>
-      <c r="P98" s="11"/>
-      <c r="Q98" s="18" t="str">
+      <c r="A98" s="10" t="s">
+        <v>729</v>
+      </c>
+      <c r="B98" s="11" t="s">
+        <v>665</v>
+      </c>
+      <c r="C98" s="12">
+        <v>46308</v>
+      </c>
+      <c r="D98" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E98" s="12">
+        <v>46308</v>
+      </c>
+      <c r="F98" s="43" t="s">
+        <v>730</v>
+      </c>
+      <c r="G98" s="43" t="s">
+        <v>731</v>
+      </c>
+      <c r="H98" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="I98" s="58">
+        <v>1.2</v>
+      </c>
+      <c r="J98" s="11" t="s">
+        <v>732</v>
+      </c>
+      <c r="K98" s="11" t="s">
+        <v>733</v>
+      </c>
+      <c r="L98" s="11" t="s">
+        <v>715</v>
+      </c>
+      <c r="M98" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N98" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O98" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="P98" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q98" s="18">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R98" s="19" t="str">
+        <v>46309</v>
+      </c>
+      <c r="R98" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S98" s="43"/>
       <c r="T98" s="43"/>
-      <c r="U98" s="7"/>
-      <c r="V98" s="41"/>
+      <c r="U98" s="7" t="s">
+        <v>670</v>
+      </c>
+      <c r="V98" s="41" t="s">
+        <v>734</v>
+      </c>
     </row>
     <row r="99" spans="1:22">
-      <c r="A99" s="10"/>
-      <c r="B99" s="11"/>
-      <c r="C99" s="12"/>
-      <c r="D99" s="12"/>
-      <c r="E99" s="12"/>
-      <c r="F99" s="43"/>
-      <c r="G99" s="43"/>
-      <c r="H99" s="11"/>
-      <c r="I99" s="11"/>
-      <c r="J99" s="11"/>
-      <c r="K99" s="11"/>
-      <c r="L99" s="11"/>
-      <c r="M99" s="11"/>
-      <c r="N99" s="11"/>
-      <c r="O99" s="11"/>
-      <c r="P99" s="11"/>
-      <c r="Q99" s="18" t="str">
+      <c r="A99" s="10" t="s">
+        <v>735</v>
+      </c>
+      <c r="B99" s="11" t="s">
+        <v>665</v>
+      </c>
+      <c r="C99" s="12">
+        <v>46308</v>
+      </c>
+      <c r="D99" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E99" s="12">
+        <v>46308</v>
+      </c>
+      <c r="F99" s="43" t="s">
+        <v>736</v>
+      </c>
+      <c r="G99" s="43" t="s">
+        <v>737</v>
+      </c>
+      <c r="H99" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="I99" s="58">
+        <v>1.2</v>
+      </c>
+      <c r="J99" s="11" t="s">
+        <v>732</v>
+      </c>
+      <c r="K99" s="11" t="s">
+        <v>738</v>
+      </c>
+      <c r="L99" s="11" t="s">
+        <v>715</v>
+      </c>
+      <c r="M99" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N99" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O99" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="P99" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q99" s="18">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R99" s="19" t="str">
+        <v>46309</v>
+      </c>
+      <c r="R99" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S99" s="43"/>
       <c r="T99" s="43"/>
-      <c r="U99" s="7"/>
-      <c r="V99" s="41"/>
+      <c r="U99" s="7" t="s">
+        <v>670</v>
+      </c>
+      <c r="V99" s="41" t="s">
+        <v>739</v>
+      </c>
     </row>
     <row r="100" spans="1:22">
-      <c r="A100" s="10"/>
-      <c r="B100" s="11"/>
-      <c r="C100" s="12"/>
-      <c r="D100" s="12"/>
-      <c r="E100" s="12"/>
-      <c r="F100" s="43"/>
-      <c r="G100" s="43"/>
-      <c r="H100" s="11"/>
-      <c r="I100" s="11"/>
-      <c r="J100" s="11"/>
-      <c r="K100" s="11"/>
-      <c r="L100" s="11"/>
-      <c r="M100" s="11"/>
-      <c r="N100" s="11"/>
-      <c r="O100" s="11"/>
-      <c r="P100" s="11"/>
-      <c r="Q100" s="18" t="str">
+      <c r="A100" s="10" t="s">
+        <v>740</v>
+      </c>
+      <c r="B100" s="11" t="s">
+        <v>665</v>
+      </c>
+      <c r="C100" s="12">
+        <v>46308</v>
+      </c>
+      <c r="D100" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E100" s="12">
+        <v>46308</v>
+      </c>
+      <c r="F100" s="43" t="s">
+        <v>700</v>
+      </c>
+      <c r="G100" s="43" t="s">
+        <v>741</v>
+      </c>
+      <c r="H100" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="I100" s="58">
+        <v>1.5</v>
+      </c>
+      <c r="J100" s="11" t="s">
+        <v>742</v>
+      </c>
+      <c r="K100" s="11" t="s">
+        <v>743</v>
+      </c>
+      <c r="L100" s="11" t="s">
+        <v>715</v>
+      </c>
+      <c r="M100" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N100" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O100" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="P100" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q100" s="18">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R100" s="19" t="str">
+        <v>46309</v>
+      </c>
+      <c r="R100" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S100" s="43"/>
       <c r="T100" s="43"/>
-      <c r="U100" s="7"/>
-      <c r="V100" s="41"/>
+      <c r="U100" s="7" t="s">
+        <v>670</v>
+      </c>
+      <c r="V100" s="41" t="s">
+        <v>744</v>
+      </c>
     </row>
     <row r="101" spans="1:22">
-      <c r="A101" s="10"/>
-      <c r="B101" s="11"/>
-      <c r="C101" s="12"/>
-      <c r="D101" s="12"/>
-      <c r="E101" s="12"/>
-      <c r="F101" s="43"/>
-      <c r="G101" s="43"/>
-      <c r="H101" s="11"/>
-      <c r="I101" s="11"/>
-      <c r="J101" s="11"/>
-      <c r="K101" s="11"/>
-      <c r="L101" s="11"/>
-      <c r="M101" s="11"/>
-      <c r="N101" s="11"/>
-      <c r="O101" s="11"/>
-      <c r="P101" s="11"/>
-      <c r="Q101" s="18" t="str">
+      <c r="A101" s="10" t="s">
+        <v>745</v>
+      </c>
+      <c r="B101" s="11" t="s">
+        <v>665</v>
+      </c>
+      <c r="C101" s="12">
+        <v>46308</v>
+      </c>
+      <c r="D101" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E101" s="12">
+        <v>46308</v>
+      </c>
+      <c r="F101" s="43" t="s">
+        <v>746</v>
+      </c>
+      <c r="G101" s="43" t="s">
+        <v>116</v>
+      </c>
+      <c r="H101" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="I101" s="58">
+        <v>1.32</v>
+      </c>
+      <c r="J101" s="11" t="s">
+        <v>747</v>
+      </c>
+      <c r="K101" s="11" t="s">
+        <v>748</v>
+      </c>
+      <c r="L101" s="11" t="s">
+        <v>715</v>
+      </c>
+      <c r="M101" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N101" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O101" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="P101" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q101" s="18">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R101" s="19" t="str">
+        <v>46309</v>
+      </c>
+      <c r="R101" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S101" s="43"/>
       <c r="T101" s="43"/>
-      <c r="U101" s="7"/>
-      <c r="V101" s="41"/>
+      <c r="U101" s="7" t="s">
+        <v>670</v>
+      </c>
+      <c r="V101" s="41" t="s">
+        <v>749</v>
+      </c>
     </row>
     <row r="102" spans="1:22">
-      <c r="A102" s="10"/>
-      <c r="B102" s="11"/>
-      <c r="C102" s="12"/>
-      <c r="D102" s="12"/>
-      <c r="E102" s="12"/>
-      <c r="F102" s="43"/>
-      <c r="G102" s="43"/>
-      <c r="H102" s="11"/>
-      <c r="I102" s="11"/>
-      <c r="J102" s="11"/>
-      <c r="K102" s="11"/>
-      <c r="L102" s="11"/>
-      <c r="M102" s="11"/>
-      <c r="N102" s="11"/>
-      <c r="O102" s="11"/>
-      <c r="P102" s="11"/>
-      <c r="Q102" s="18" t="str">
+      <c r="A102" s="10" t="s">
+        <v>750</v>
+      </c>
+      <c r="B102" s="11" t="s">
+        <v>665</v>
+      </c>
+      <c r="C102" s="12">
+        <v>46308</v>
+      </c>
+      <c r="D102" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E102" s="12">
+        <v>46308</v>
+      </c>
+      <c r="F102" s="43" t="s">
+        <v>272</v>
+      </c>
+      <c r="G102" s="43" t="s">
+        <v>276</v>
+      </c>
+      <c r="H102" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="I102" s="59">
+        <v>40</v>
+      </c>
+      <c r="J102" s="11" t="s">
+        <v>751</v>
+      </c>
+      <c r="K102" s="11" t="s">
+        <v>752</v>
+      </c>
+      <c r="L102" s="11" t="s">
+        <v>715</v>
+      </c>
+      <c r="M102" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N102" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O102" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="P102" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q102" s="18">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R102" s="19" t="str">
+        <v>46309</v>
+      </c>
+      <c r="R102" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S102" s="43"/>
       <c r="T102" s="43"/>
-      <c r="U102" s="7"/>
-      <c r="V102" s="41"/>
+      <c r="U102" s="7" t="s">
+        <v>670</v>
+      </c>
+      <c r="V102" s="41" t="s">
+        <v>753</v>
+      </c>
     </row>
     <row r="103" spans="1:22">
-      <c r="A103" s="10"/>
-      <c r="B103" s="11"/>
-      <c r="C103" s="12"/>
-      <c r="D103" s="12"/>
-      <c r="E103" s="12"/>
-      <c r="F103" s="43"/>
-      <c r="G103" s="43"/>
-      <c r="H103" s="11"/>
-      <c r="I103" s="11"/>
-      <c r="J103" s="11"/>
-      <c r="K103" s="11"/>
-      <c r="L103" s="11"/>
-      <c r="M103" s="11"/>
-      <c r="N103" s="11"/>
-      <c r="O103" s="11"/>
-      <c r="P103" s="11"/>
-      <c r="Q103" s="18" t="str">
+      <c r="A103" s="10" t="s">
+        <v>754</v>
+      </c>
+      <c r="B103" s="11" t="s">
+        <v>665</v>
+      </c>
+      <c r="C103" s="12">
+        <v>46308</v>
+      </c>
+      <c r="D103" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E103" s="12">
+        <v>46308</v>
+      </c>
+      <c r="F103" s="43" t="s">
+        <v>270</v>
+      </c>
+      <c r="G103" s="43" t="s">
+        <v>276</v>
+      </c>
+      <c r="H103" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="I103" s="59">
+        <v>20</v>
+      </c>
+      <c r="J103" s="11" t="s">
+        <v>755</v>
+      </c>
+      <c r="K103" s="11" t="s">
+        <v>756</v>
+      </c>
+      <c r="L103" s="11" t="s">
+        <v>715</v>
+      </c>
+      <c r="M103" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="N103" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O103" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="P103" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q103" s="18">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R103" s="19" t="str">
+        <v>46309</v>
+      </c>
+      <c r="R103" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S103" s="43"/>
       <c r="T103" s="43"/>
-      <c r="U103" s="7"/>
-      <c r="V103" s="41"/>
+      <c r="U103" s="7" t="s">
+        <v>670</v>
+      </c>
+      <c r="V103" s="41" t="s">
+        <v>757</v>
+      </c>
     </row>
     <row r="104" spans="1:22">
-      <c r="A104" s="10"/>
-      <c r="B104" s="11"/>
-      <c r="C104" s="12"/>
-      <c r="D104" s="12"/>
-      <c r="E104" s="12"/>
-      <c r="F104" s="43"/>
-      <c r="G104" s="43"/>
-      <c r="H104" s="11"/>
-      <c r="I104" s="11"/>
-      <c r="J104" s="11"/>
-      <c r="K104" s="11"/>
-      <c r="L104" s="11"/>
-      <c r="M104" s="11"/>
-      <c r="N104" s="11"/>
-      <c r="O104" s="11"/>
-      <c r="P104" s="11"/>
-      <c r="Q104" s="18" t="str">
+      <c r="A104" s="10" t="s">
+        <v>758</v>
+      </c>
+      <c r="B104" s="11" t="s">
+        <v>665</v>
+      </c>
+      <c r="C104" s="12">
+        <v>46308</v>
+      </c>
+      <c r="D104" s="12">
+        <v>46308</v>
+      </c>
+      <c r="E104" s="12">
+        <v>46308</v>
+      </c>
+      <c r="F104" s="43" t="s">
+        <v>759</v>
+      </c>
+      <c r="G104" s="43" t="s">
+        <v>760</v>
+      </c>
+      <c r="H104" s="11" t="s">
+        <v>761</v>
+      </c>
+      <c r="I104" s="11" t="s">
+        <v>762</v>
+      </c>
+      <c r="J104" s="11" t="s">
+        <v>763</v>
+      </c>
+      <c r="K104" s="11" t="s">
+        <v>764</v>
+      </c>
+      <c r="L104" s="11" t="s">
+        <v>715</v>
+      </c>
+      <c r="M104" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="N104" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O104" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="P104" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q104" s="18">
         <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R104" s="19" t="str">
+        <v>46309</v>
+      </c>
+      <c r="R104" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S104" s="43"/>
       <c r="T104" s="43"/>
-      <c r="U104" s="7"/>
-      <c r="V104" s="41"/>
+      <c r="U104" s="7" t="s">
+        <v>670</v>
+      </c>
+      <c r="V104" s="41" t="s">
+        <v>765</v>
+      </c>
     </row>
     <row r="105" spans="1:22">
       <c r="A105" s="10"/>

</xml_diff>

<commit_message>
[O7 13/10] Registro arrumado pelo LEO: O7-001..018 executadas em 13/10 (em maturacao), vereditos da O6 lancados; conferencia contra export/prints pendente
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1512" uniqueCount="766">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1554" uniqueCount="797">
   <si>
     <t>REGISTRO DE ALTERAÇÕES — AMAZON ADS | WINNET METAIS</t>
   </si>
@@ -1439,9 +1439,6 @@
     <t>ciclos/O6-22-09.md + relatorios/amazon/o6-22-09/ (export 10-21_09, recorrentes 30d 22/08–20/09, exports vitalícios de alvos, segmentação da Geral na Era, BR 10–20/09)</t>
   </si>
   <si>
-    <t>O7 13/10</t>
-  </si>
-  <si>
     <t>Cobertura do SP-PP mantida pela Geral (30d: 2.370 impr, 4 cli, R$ 2,76) e pela Manual Bituqueiras. Executar antes das mudanças de lance (reversível)</t>
   </si>
   <si>
@@ -1454,9 +1451,6 @@
     <t>Gatilho O5-007 disparado nas duas condições: 0 vendas E CTR 0,17% (&lt; 0,3%) na Era (10 cli, R$ 7,58). 30d: 8.534 impr, 11 cli, CTR 0,129%, 0 venda; 4.695 impr no termo "guarda chuva" com 2 cli. Melhor Oferta −10% no 9.9 zerou. BR: 24 sessões / 0 un</t>
   </si>
   <si>
-    <t>quando a página do EGC for revisada</t>
-  </si>
-  <si>
     <t>EGC segue anunciado na Geral (72 impr / 1 cli em 30d). Lance 0,84 registrado para eventual retorno. Sai do grupo de controle do piloto de lance</t>
   </si>
   <si>
@@ -1938,9 +1932,6 @@
   </si>
   <si>
     <t>SEM EFEITO — 0 venda em 3 sessões / 5 visualizações (opcional, tráfego marginal).</t>
-  </si>
-  <si>
-    <t>gatilho disparou em 28/09, anúncio pausado</t>
   </si>
   <si>
     <t>EC-017</t>
@@ -2331,6 +2322,108 @@
   </si>
   <si>
     <t>Não é ação no console. Print do Gestor Seller (margem bruta) pode refinar o número; até lá vale a Mestra. Diagnóstico da O7 relido: ACOS 5,4% da Era = 43% do Objetivo novo.</t>
+  </si>
+  <si>
+    <t>SP-PP pausada; 0 atividade na Era</t>
+  </si>
+  <si>
+    <t>MANTIDA — venda orgânica não reabilita a auto</t>
+  </si>
+  <si>
+    <t>EGC pausada; SKU vendeu 1 un orgânica (23/09) e teve 24 sessões na Era sem Ads</t>
+  </si>
+  <si>
+    <t>alvo B09YDLC69D pausado; 16 cli vit / 0 congelados</t>
+  </si>
+  <si>
+    <t>PRECOPRIMEALTERNATIVO (12 SKUs a 10%, 05–11/10): 108 visualizações · 0 un · R$ 0</t>
+  </si>
+  <si>
+    <t>SEM EFEITO — 3ª leitura de desconto a 10% sem conversão; não repetir fora de evento com selo</t>
+  </si>
+  <si>
+    <t>MANTIDAS</t>
+  </si>
+  <si>
+    <t>Geral R$ 90/dia, consumo 12%; auto PXP 10 cli/0 em 30d; PI L2030-B 7 cli/0 (vit 3 compras em 1 alvo)</t>
+  </si>
+  <si>
+    <t>VIGIA MANTIDA — dupla (Geral 5/15; PI 14/15)</t>
+  </si>
+  <si>
+    <t>B0BHMZBZW9: Geral 5 cli / 0 em 30d (régua 15); como alvo da PI P3070 14 cli vit / 1</t>
+  </si>
+  <si>
+    <t>Migração: GS1 reenviado 05/10; gate físico sem data</t>
+  </si>
+  <si>
+    <t>NÃO DECIDIR AINDA (mantido)</t>
+  </si>
+  <si>
+    <t>O8</t>
+  </si>
+  <si>
+    <t>Melhor Oferta PXP 10% (exceção ao piso): 23 visualizações · 0 un</t>
+  </si>
+  <si>
+    <t>SEM EFEITO — exceção ao piso não se repete</t>
+  </si>
+  <si>
+    <t>P3050 não elegível; no desconto comum: 11 sessões / 0</t>
+  </si>
+  <si>
+    <t>NÃO ELEGÍVEL</t>
+  </si>
+  <si>
+    <t>P3060 não elegível; no desconto comum: 12 sessões / 0</t>
+  </si>
+  <si>
+    <t>P4080 não elegível; no desconto comum: 21 sessões / 0</t>
+  </si>
+  <si>
+    <t>Melhor Oferta P3070 15%: 124 visualizações · 1 un · R$ 523,75 · 0,8%; BR 108 sessões na semana</t>
+  </si>
+  <si>
+    <t>POSITIVO FRACO — tráfego sim, 1 conversão; repetir só com selo de evento</t>
+  </si>
+  <si>
+    <t>PG2460 não elegível; sem preço de referência</t>
+  </si>
+  <si>
+    <t>PXM nunca entrou na lista de Melhor Oferta</t>
+  </si>
+  <si>
+    <t>NÃO ELEGÍVEL — substituída pelo desconto comum (EC-020), 0 venda</t>
+  </si>
+  <si>
+    <t>Piloto +1 Era: 6B 12 cli/0, L3070-B 2 cli/0; controle 0–1 cli</t>
+  </si>
+  <si>
+    <t>SEM EFEITO — encerrar (O7-006)</t>
+  </si>
+  <si>
+    <t>exata "lixeira inox para pia de cozinha": 14 cli / R$ 16,18 / 0 em 30d</t>
+  </si>
+  <si>
+    <t>VIGIA MANTIDA — dispara com 1 clique (→ 1,20 ou pausar)</t>
+  </si>
+  <si>
+    <t>Q2460-B pausado na Geral em 28/09; BR 19 → 1 sessão por bloco</t>
+  </si>
+  <si>
+    <t>CONFIRMADA — SKU vai à fila de página</t>
+  </si>
+  <si>
+    <t>loose-match a 0,45: 153 cli · R$ 96,49 · 4 compras · ACOS 9,4% (30d); era o dreno de 60% do custo</t>
+  </si>
+  <si>
+    <t>POSITIVO — mantido em 0,45</t>
+  </si>
+  <si>
+    <t>PI P3070 na Era: 70 cli · R$ 89,35 · 1 venda (30/09, alvo B0CTMZHJFJ) · ACOS 14,5%</t>
+  </si>
+  <si>
+    <t>GATILHO NÃO DISPAROU — lances mantidos; alvo B0CYWMQ93Y → O7-003</t>
   </si>
 </sst>
 </file>
@@ -2579,7 +2672,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="14"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2708,7 +2801,6 @@
     <xf numFmtId="14" fontId="15" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2741,7 +2833,362 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="42">
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9A3412"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFED7AA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF991B1B"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF374151"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF3F4F6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF166534"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFDCFCE7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF3730A3"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFE0E7FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF92400E"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEF3C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1E40AF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFDBEAFE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9A3412"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFED7AA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF991B1B"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF374151"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF3F4F6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF166534"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFDCFCE7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF3730A3"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFE0E7FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF92400E"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEF3C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1E40AF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFDBEAFE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9A3412"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFED7AA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF991B1B"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF374151"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF3F4F6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF166534"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFDCFCE7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF3730A3"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFE0E7FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF92400E"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEF3C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1E40AF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFDBEAFE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9A3412"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFED7AA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF991B1B"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF374151"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF3F4F6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF166534"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFDCFCE7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF3730A3"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFE0E7FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF92400E"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEF3C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1E40AF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFDBEAFE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9A3412"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFED7AA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF991B1B"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF374151"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF3F4F6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF166534"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFDCFCE7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF3730A3"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFE0E7FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF92400E"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFEF3C7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1E40AF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFDBEAFE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -3074,82 +3521,82 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="50" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51"/>
-      <c r="E1" s="51"/>
-      <c r="F1" s="51"/>
-      <c r="G1" s="51"/>
-      <c r="H1" s="51"/>
-      <c r="I1" s="51"/>
-      <c r="J1" s="51"/>
-      <c r="K1" s="51"/>
-      <c r="L1" s="51"/>
-      <c r="M1" s="51"/>
-      <c r="N1" s="51"/>
-      <c r="O1" s="51"/>
-      <c r="P1" s="51"/>
-      <c r="Q1" s="51"/>
-      <c r="R1" s="51"/>
-      <c r="S1" s="51"/>
-      <c r="T1" s="51"/>
-      <c r="U1" s="51"/>
-      <c r="V1" s="51"/>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="E1" s="50"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="H1" s="50"/>
+      <c r="I1" s="50"/>
+      <c r="J1" s="50"/>
+      <c r="K1" s="50"/>
+      <c r="L1" s="50"/>
+      <c r="M1" s="50"/>
+      <c r="N1" s="50"/>
+      <c r="O1" s="50"/>
+      <c r="P1" s="50"/>
+      <c r="Q1" s="50"/>
+      <c r="R1" s="50"/>
+      <c r="S1" s="50"/>
+      <c r="T1" s="50"/>
+      <c r="U1" s="50"/>
+      <c r="V1" s="50"/>
     </row>
     <row r="2" spans="1:22" ht="30" customHeight="1">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="51" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="52"/>
-      <c r="F2" s="52"/>
-      <c r="G2" s="52"/>
-      <c r="H2" s="52"/>
-      <c r="I2" s="52"/>
-      <c r="J2" s="52"/>
-      <c r="K2" s="52"/>
-      <c r="L2" s="52"/>
-      <c r="M2" s="52"/>
-      <c r="N2" s="52"/>
-      <c r="O2" s="52"/>
-      <c r="P2" s="52"/>
-      <c r="Q2" s="52"/>
-      <c r="R2" s="52"/>
-      <c r="S2" s="52"/>
-      <c r="T2" s="52"/>
-      <c r="U2" s="52"/>
-      <c r="V2" s="52"/>
+      <c r="B2" s="51"/>
+      <c r="C2" s="51"/>
+      <c r="D2" s="51"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
+      <c r="H2" s="51"/>
+      <c r="I2" s="51"/>
+      <c r="J2" s="51"/>
+      <c r="K2" s="51"/>
+      <c r="L2" s="51"/>
+      <c r="M2" s="51"/>
+      <c r="N2" s="51"/>
+      <c r="O2" s="51"/>
+      <c r="P2" s="51"/>
+      <c r="Q2" s="51"/>
+      <c r="R2" s="51"/>
+      <c r="S2" s="51"/>
+      <c r="T2" s="51"/>
+      <c r="U2" s="51"/>
+      <c r="V2" s="51"/>
     </row>
     <row r="3" spans="1:22" ht="27.95" customHeight="1">
-      <c r="A3" s="53" t="s">
+      <c r="A3" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="53"/>
-      <c r="D3" s="53"/>
-      <c r="E3" s="53"/>
-      <c r="F3" s="53"/>
-      <c r="G3" s="53"/>
-      <c r="H3" s="53"/>
-      <c r="I3" s="53"/>
-      <c r="J3" s="53"/>
-      <c r="K3" s="53"/>
-      <c r="L3" s="53"/>
-      <c r="M3" s="53"/>
-      <c r="N3" s="53"/>
-      <c r="O3" s="53"/>
-      <c r="P3" s="53"/>
-      <c r="Q3" s="53"/>
-      <c r="R3" s="53"/>
-      <c r="S3" s="53"/>
-      <c r="T3" s="53"/>
-      <c r="U3" s="53"/>
-      <c r="V3" s="53"/>
+      <c r="B3" s="52"/>
+      <c r="C3" s="52"/>
+      <c r="D3" s="52"/>
+      <c r="E3" s="52"/>
+      <c r="F3" s="52"/>
+      <c r="G3" s="52"/>
+      <c r="H3" s="52"/>
+      <c r="I3" s="52"/>
+      <c r="J3" s="52"/>
+      <c r="K3" s="52"/>
+      <c r="L3" s="52"/>
+      <c r="M3" s="52"/>
+      <c r="N3" s="52"/>
+      <c r="O3" s="52"/>
+      <c r="P3" s="52"/>
+      <c r="Q3" s="52"/>
+      <c r="R3" s="52"/>
+      <c r="S3" s="52"/>
+      <c r="T3" s="52"/>
+      <c r="U3" s="52"/>
+      <c r="V3" s="52"/>
     </row>
     <row r="5" spans="1:22">
       <c r="A5" s="1" t="s">
@@ -3170,23 +3617,23 @@
       <c r="F5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H5" s="54" t="s">
+      <c r="H5" s="53" t="s">
         <v>9</v>
       </c>
-      <c r="I5" s="54"/>
-      <c r="J5" s="54"/>
-      <c r="K5" s="54"/>
-      <c r="L5" s="54"/>
-      <c r="M5" s="54"/>
-      <c r="N5" s="54"/>
-      <c r="O5" s="54"/>
-      <c r="P5" s="54"/>
-      <c r="Q5" s="54"/>
-      <c r="R5" s="54"/>
-      <c r="S5" s="54"/>
-      <c r="T5" s="54"/>
-      <c r="U5" s="54"/>
-      <c r="V5" s="54"/>
+      <c r="I5" s="53"/>
+      <c r="J5" s="53"/>
+      <c r="K5" s="53"/>
+      <c r="L5" s="53"/>
+      <c r="M5" s="53"/>
+      <c r="N5" s="53"/>
+      <c r="O5" s="53"/>
+      <c r="P5" s="53"/>
+      <c r="Q5" s="53"/>
+      <c r="R5" s="53"/>
+      <c r="S5" s="53"/>
+      <c r="T5" s="53"/>
+      <c r="U5" s="53"/>
+      <c r="V5" s="53"/>
     </row>
     <row r="6" spans="1:22" ht="26.1" customHeight="1">
       <c r="A6" s="2">
@@ -3199,7 +3646,7 @@
       </c>
       <c r="C6" s="3">
         <f>COUNTIF(O11:O208,"SIM")</f>
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="D6" s="3">
         <f>COUNTIF(P11:P208,"BLOQUEADA*")</f>
@@ -3207,53 +3654,53 @@
       </c>
       <c r="E6" s="3">
         <f>COUNTIF(P11:P208,"EXECUTADA - EM MATURAÇÃO")</f>
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="F6" s="4">
         <f>COUNTIF(P11:P208,"EXECUTADA - AVALIADA")</f>
-        <v>51</v>
-      </c>
-      <c r="H6" s="54"/>
-      <c r="I6" s="54"/>
-      <c r="J6" s="54"/>
-      <c r="K6" s="54"/>
-      <c r="L6" s="54"/>
-      <c r="M6" s="54"/>
-      <c r="N6" s="54"/>
-      <c r="O6" s="54"/>
-      <c r="P6" s="54"/>
-      <c r="Q6" s="54"/>
-      <c r="R6" s="54"/>
-      <c r="S6" s="54"/>
-      <c r="T6" s="54"/>
-      <c r="U6" s="54"/>
-      <c r="V6" s="54"/>
+        <v>65</v>
+      </c>
+      <c r="H6" s="53"/>
+      <c r="I6" s="53"/>
+      <c r="J6" s="53"/>
+      <c r="K6" s="53"/>
+      <c r="L6" s="53"/>
+      <c r="M6" s="53"/>
+      <c r="N6" s="53"/>
+      <c r="O6" s="53"/>
+      <c r="P6" s="53"/>
+      <c r="Q6" s="53"/>
+      <c r="R6" s="53"/>
+      <c r="S6" s="53"/>
+      <c r="T6" s="53"/>
+      <c r="U6" s="53"/>
+      <c r="V6" s="53"/>
     </row>
     <row r="8" spans="1:22" ht="21.95" customHeight="1">
-      <c r="A8" s="55" t="s">
+      <c r="A8" s="54" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="55"/>
-      <c r="C8" s="55"/>
-      <c r="D8" s="55"/>
-      <c r="E8" s="55"/>
-      <c r="F8" s="55"/>
-      <c r="G8" s="55"/>
-      <c r="H8" s="55"/>
-      <c r="I8" s="55"/>
-      <c r="J8" s="55"/>
-      <c r="K8" s="55"/>
-      <c r="L8" s="55"/>
-      <c r="M8" s="55"/>
-      <c r="N8" s="55"/>
-      <c r="O8" s="55"/>
-      <c r="P8" s="55"/>
-      <c r="Q8" s="55"/>
-      <c r="R8" s="55"/>
-      <c r="S8" s="55"/>
-      <c r="T8" s="55"/>
-      <c r="U8" s="55"/>
-      <c r="V8" s="55"/>
+      <c r="B8" s="54"/>
+      <c r="C8" s="54"/>
+      <c r="D8" s="54"/>
+      <c r="E8" s="54"/>
+      <c r="F8" s="54"/>
+      <c r="G8" s="54"/>
+      <c r="H8" s="54"/>
+      <c r="I8" s="54"/>
+      <c r="J8" s="54"/>
+      <c r="K8" s="54"/>
+      <c r="L8" s="54"/>
+      <c r="M8" s="54"/>
+      <c r="N8" s="54"/>
+      <c r="O8" s="54"/>
+      <c r="P8" s="54"/>
+      <c r="Q8" s="54"/>
+      <c r="R8" s="54"/>
+      <c r="S8" s="54"/>
+      <c r="T8" s="54"/>
+      <c r="U8" s="54"/>
+      <c r="V8" s="54"/>
     </row>
     <row r="10" spans="1:22" ht="38.1" customHeight="1">
       <c r="A10" s="5" t="s">
@@ -5091,10 +5538,10 @@
         <v>34</v>
       </c>
       <c r="S36" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="T36" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="U36" s="42">
         <v>46287</v>
@@ -5161,10 +5608,10 @@
         <v>34</v>
       </c>
       <c r="S37" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="T37" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="U37" s="42">
         <v>46287</v>
@@ -5231,10 +5678,10 @@
         <v>34</v>
       </c>
       <c r="S38" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="T38" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="U38" s="42">
         <v>46287</v>
@@ -5301,10 +5748,10 @@
         <v>34</v>
       </c>
       <c r="S39" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="T39" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="U39" s="42">
         <v>46287</v>
@@ -5371,7 +5818,7 @@
         <v>34</v>
       </c>
       <c r="S40" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="T40" t="s">
         <v>387</v>
@@ -5441,10 +5888,10 @@
         <v>34</v>
       </c>
       <c r="S41" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="T41" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="U41" s="42">
         <v>46287</v>
@@ -5511,10 +5958,10 @@
         <v>34</v>
       </c>
       <c r="S42" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="T42" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="U42" s="42">
         <v>46287</v>
@@ -5581,10 +6028,10 @@
         <v>34</v>
       </c>
       <c r="S43" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="T43" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="U43" s="42">
         <v>46308</v>
@@ -5651,10 +6098,10 @@
         <v>34</v>
       </c>
       <c r="S44" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="T44" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="U44" s="42">
         <v>46308</v>
@@ -5721,10 +6168,10 @@
         <v>34</v>
       </c>
       <c r="S45" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="T45" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="U45" s="42">
         <v>46287</v>
@@ -5791,10 +6238,10 @@
         <v>34</v>
       </c>
       <c r="S46" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="T46" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="U46" s="42">
         <v>46279</v>
@@ -5861,10 +6308,10 @@
         <v>34</v>
       </c>
       <c r="S47" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="T47" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="U47" s="39" t="s">
         <v>342</v>
@@ -5929,10 +6376,10 @@
         <v/>
       </c>
       <c r="S48" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="T48" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="U48" s="42">
         <v>46287</v>
@@ -5999,10 +6446,10 @@
         <v>34</v>
       </c>
       <c r="S49" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="T49" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="U49" s="42">
         <v>46279</v>
@@ -6069,10 +6516,10 @@
         <v>34</v>
       </c>
       <c r="S50" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="T50" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="U50" s="42">
         <v>46287</v>
@@ -6139,10 +6586,10 @@
         <v>34</v>
       </c>
       <c r="S51" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="T51" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="U51" s="42">
         <v>46287</v>
@@ -6209,10 +6656,10 @@
         <v>34</v>
       </c>
       <c r="S52" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="T52" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="U52" s="42">
         <v>46287</v>
@@ -6279,10 +6726,10 @@
         <v>25</v>
       </c>
       <c r="S53" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="T53" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="U53" s="47">
         <v>46293</v>
@@ -6349,10 +6796,10 @@
         <v>25</v>
       </c>
       <c r="S54" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="T54" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="U54" s="47">
         <v>46293</v>
@@ -6419,10 +6866,10 @@
         <v>25</v>
       </c>
       <c r="S55" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="T55" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="U55" s="47">
         <v>46293</v>
@@ -6489,10 +6936,10 @@
         <v>25</v>
       </c>
       <c r="S56" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="T56" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="U56" s="47">
         <v>46293</v>
@@ -6559,10 +7006,10 @@
         <v>25</v>
       </c>
       <c r="S57" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="T57" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="U57" s="47">
         <v>46293</v>
@@ -6629,10 +7076,10 @@
         <v>25</v>
       </c>
       <c r="S58" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="T58" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="U58" s="47">
         <v>46293</v>
@@ -6699,10 +7146,10 @@
         <v>25</v>
       </c>
       <c r="S59" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="T59" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="U59" s="47">
         <v>46293</v>
@@ -6769,10 +7216,10 @@
         <v>25</v>
       </c>
       <c r="S60" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="T60" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="U60" s="47">
         <v>46293</v>
@@ -6839,10 +7286,10 @@
         <v>25</v>
       </c>
       <c r="S61" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="T61" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="U61" s="47">
         <v>46293</v>
@@ -6909,10 +7356,10 @@
         <v>25</v>
       </c>
       <c r="S62" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="T62" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="U62" s="47">
         <v>46293</v>
@@ -6968,7 +7415,7 @@
         <v>40</v>
       </c>
       <c r="P63" s="46" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="Q63" s="18">
         <f t="shared" si="0"/>
@@ -6978,16 +7425,22 @@
         <f t="shared" ca="1" si="2"/>
         <v>21</v>
       </c>
+      <c r="S63" t="s">
+        <v>763</v>
+      </c>
+      <c r="T63" t="s">
+        <v>392</v>
+      </c>
       <c r="U63" t="s">
+        <v>146</v>
+      </c>
+      <c r="V63" t="s">
         <v>469</v>
-      </c>
-      <c r="V63" t="s">
-        <v>470</v>
       </c>
     </row>
     <row r="64" spans="1:22">
       <c r="A64" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="B64" t="s">
         <v>464</v>
@@ -7011,13 +7464,13 @@
         <v>54</v>
       </c>
       <c r="I64" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="J64" t="s">
         <v>143</v>
       </c>
       <c r="K64" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="L64" t="s">
         <v>468</v>
@@ -7032,7 +7485,7 @@
         <v>40</v>
       </c>
       <c r="P64" s="46" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="Q64" s="18">
         <f t="shared" si="0"/>
@@ -7042,16 +7495,22 @@
         <f t="shared" ca="1" si="2"/>
         <v>21</v>
       </c>
+      <c r="S64" t="s">
+        <v>765</v>
+      </c>
+      <c r="T64" t="s">
+        <v>764</v>
+      </c>
       <c r="U64" t="s">
-        <v>474</v>
+        <v>146</v>
       </c>
       <c r="V64" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
     </row>
     <row r="65" spans="1:22">
       <c r="A65" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="B65" t="s">
         <v>464</v>
@@ -7069,19 +7528,19 @@
         <v>270</v>
       </c>
       <c r="G65" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="H65" t="s">
         <v>52</v>
       </c>
       <c r="I65" t="s">
+        <v>476</v>
+      </c>
+      <c r="J65" t="s">
+        <v>477</v>
+      </c>
+      <c r="K65" t="s">
         <v>478</v>
-      </c>
-      <c r="J65" t="s">
-        <v>479</v>
-      </c>
-      <c r="K65" t="s">
-        <v>480</v>
       </c>
       <c r="L65" t="s">
         <v>468</v>
@@ -7096,7 +7555,7 @@
         <v>40</v>
       </c>
       <c r="P65" s="46" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="Q65" s="18">
         <f t="shared" si="0"/>
@@ -7106,16 +7565,22 @@
         <f t="shared" ca="1" si="2"/>
         <v>21</v>
       </c>
+      <c r="S65" t="s">
+        <v>766</v>
+      </c>
+      <c r="T65" t="s">
+        <v>392</v>
+      </c>
       <c r="U65" t="s">
         <v>146</v>
       </c>
       <c r="V65" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
     </row>
     <row r="66" spans="1:22">
       <c r="A66" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="B66" t="s">
         <v>464</v>
@@ -7136,16 +7601,16 @@
         <v>114</v>
       </c>
       <c r="H66" t="s">
+        <v>481</v>
+      </c>
+      <c r="I66" t="s">
+        <v>482</v>
+      </c>
+      <c r="J66" t="s">
         <v>483</v>
       </c>
-      <c r="I66" t="s">
+      <c r="K66" t="s">
         <v>484</v>
-      </c>
-      <c r="J66" t="s">
-        <v>485</v>
-      </c>
-      <c r="K66" t="s">
-        <v>486</v>
       </c>
       <c r="L66" t="s">
         <v>468</v>
@@ -7160,7 +7625,7 @@
         <v>40</v>
       </c>
       <c r="P66" s="46" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="Q66" s="18">
         <f t="shared" si="0"/>
@@ -7170,16 +7635,22 @@
         <f t="shared" ca="1" si="2"/>
         <v>21</v>
       </c>
-      <c r="U66" t="s">
-        <v>469</v>
+      <c r="S66" t="s">
+        <v>795</v>
+      </c>
+      <c r="T66" t="s">
+        <v>796</v>
+      </c>
+      <c r="U66" s="48">
+        <v>46322</v>
       </c>
       <c r="V66" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
     </row>
     <row r="67" spans="1:22">
       <c r="A67" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="B67" t="s">
         <v>464</v>
@@ -7209,7 +7680,7 @@
         <v>303</v>
       </c>
       <c r="K67" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="L67" t="s">
         <v>468</v>
@@ -7224,7 +7695,7 @@
         <v>40</v>
       </c>
       <c r="P67" s="46" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="Q67" s="18">
         <f t="shared" si="0"/>
@@ -7234,16 +7705,22 @@
         <f t="shared" ca="1" si="2"/>
         <v>21</v>
       </c>
-      <c r="U67" t="s">
-        <v>469</v>
+      <c r="S67" t="s">
+        <v>793</v>
+      </c>
+      <c r="T67" t="s">
+        <v>794</v>
+      </c>
+      <c r="U67" s="48">
+        <v>46322</v>
       </c>
       <c r="V67" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
     </row>
     <row r="68" spans="1:22">
       <c r="A68" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="B68" t="s">
         <v>464</v>
@@ -7261,19 +7738,19 @@
         <v>264</v>
       </c>
       <c r="G68" t="s">
+        <v>490</v>
+      </c>
+      <c r="H68" t="s">
+        <v>491</v>
+      </c>
+      <c r="I68" t="s">
         <v>492</v>
       </c>
-      <c r="H68" t="s">
+      <c r="J68" t="s">
         <v>493</v>
       </c>
-      <c r="I68" t="s">
+      <c r="K68" t="s">
         <v>494</v>
-      </c>
-      <c r="J68" t="s">
-        <v>495</v>
-      </c>
-      <c r="K68" t="s">
-        <v>496</v>
       </c>
       <c r="L68" t="s">
         <v>468</v>
@@ -7288,7 +7765,7 @@
         <v>40</v>
       </c>
       <c r="P68" s="46" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="Q68" s="18">
         <f t="shared" si="0"/>
@@ -7298,19 +7775,22 @@
         <f t="shared" ca="1" si="2"/>
         <v>21</v>
       </c>
+      <c r="S68" t="s">
+        <v>791</v>
+      </c>
       <c r="T68" t="s">
-        <v>636</v>
-      </c>
-      <c r="U68" s="50">
-        <v>46308</v>
+        <v>792</v>
+      </c>
+      <c r="U68" t="s">
+        <v>146</v>
       </c>
       <c r="V68" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
     </row>
     <row r="69" spans="1:22">
       <c r="A69" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="B69" t="s">
         <v>464</v>
@@ -7328,19 +7808,19 @@
         <v>112</v>
       </c>
       <c r="G69" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="H69" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="I69" t="s">
         <v>57</v>
       </c>
       <c r="J69" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="K69" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="L69" t="s">
         <v>468</v>
@@ -7369,12 +7849,12 @@
         <v>146</v>
       </c>
       <c r="V69" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
     </row>
     <row r="70" spans="1:22">
       <c r="A70" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="B70" t="s">
         <v>464</v>
@@ -7392,19 +7872,19 @@
         <v>112</v>
       </c>
       <c r="G70" t="s">
+        <v>503</v>
+      </c>
+      <c r="H70" t="s">
+        <v>504</v>
+      </c>
+      <c r="I70" t="s">
         <v>505</v>
       </c>
-      <c r="H70" t="s">
+      <c r="J70" t="s">
         <v>506</v>
       </c>
-      <c r="I70" t="s">
+      <c r="K70" t="s">
         <v>507</v>
-      </c>
-      <c r="J70" t="s">
-        <v>508</v>
-      </c>
-      <c r="K70" t="s">
-        <v>509</v>
       </c>
       <c r="L70" t="s">
         <v>468</v>
@@ -7419,7 +7899,7 @@
         <v>40</v>
       </c>
       <c r="P70" s="46" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="Q70" s="18">
         <f t="shared" si="0"/>
@@ -7429,16 +7909,22 @@
         <f t="shared" ca="1" si="2"/>
         <v>21</v>
       </c>
-      <c r="U70" t="s">
-        <v>469</v>
+      <c r="S70" t="s">
+        <v>789</v>
+      </c>
+      <c r="T70" t="s">
+        <v>790</v>
+      </c>
+      <c r="U70" s="48">
+        <v>46315</v>
       </c>
       <c r="V70" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
     </row>
     <row r="71" spans="1:22">
       <c r="A71" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="B71" t="s">
         <v>464</v>
@@ -7456,19 +7942,19 @@
         <v>112</v>
       </c>
       <c r="G71" t="s">
+        <v>510</v>
+      </c>
+      <c r="H71" t="s">
+        <v>511</v>
+      </c>
+      <c r="I71" t="s">
         <v>512</v>
       </c>
-      <c r="H71" t="s">
+      <c r="J71" t="s">
         <v>513</v>
       </c>
-      <c r="I71" t="s">
+      <c r="K71" t="s">
         <v>514</v>
-      </c>
-      <c r="J71" t="s">
-        <v>515</v>
-      </c>
-      <c r="K71" t="s">
-        <v>516</v>
       </c>
       <c r="L71" t="s">
         <v>468</v>
@@ -7497,12 +7983,12 @@
         <v>146</v>
       </c>
       <c r="V71" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
     </row>
     <row r="72" spans="1:22">
       <c r="A72" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="B72" t="s">
         <v>464</v>
@@ -7517,22 +8003,22 @@
         <v>46287</v>
       </c>
       <c r="F72" t="s">
+        <v>517</v>
+      </c>
+      <c r="G72" t="s">
+        <v>518</v>
+      </c>
+      <c r="H72" t="s">
         <v>519</v>
       </c>
-      <c r="G72" t="s">
+      <c r="I72" t="s">
         <v>520</v>
       </c>
-      <c r="H72" t="s">
+      <c r="J72" t="s">
         <v>521</v>
       </c>
-      <c r="I72" t="s">
+      <c r="K72" t="s">
         <v>522</v>
-      </c>
-      <c r="J72" t="s">
-        <v>523</v>
-      </c>
-      <c r="K72" t="s">
-        <v>524</v>
       </c>
       <c r="L72" t="s">
         <v>468</v>
@@ -7547,7 +8033,7 @@
         <v>40</v>
       </c>
       <c r="P72" s="46" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="Q72" s="18">
         <f t="shared" si="0"/>
@@ -7557,16 +8043,22 @@
         <f t="shared" ca="1" si="2"/>
         <v>21</v>
       </c>
+      <c r="S72" t="s">
+        <v>787</v>
+      </c>
+      <c r="T72" t="s">
+        <v>788</v>
+      </c>
       <c r="U72" t="s">
-        <v>469</v>
+        <v>146</v>
       </c>
       <c r="V72" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
     </row>
     <row r="73" spans="1:22">
       <c r="A73" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="B73" t="s">
         <v>464</v>
@@ -7579,22 +8071,22 @@
       </c>
       <c r="E73" s="48"/>
       <c r="F73" t="s">
+        <v>525</v>
+      </c>
+      <c r="G73" t="s">
+        <v>526</v>
+      </c>
+      <c r="H73" t="s">
         <v>527</v>
       </c>
-      <c r="G73" t="s">
+      <c r="I73" t="s">
         <v>528</v>
       </c>
-      <c r="H73" t="s">
+      <c r="J73" t="s">
         <v>529</v>
       </c>
-      <c r="I73" t="s">
+      <c r="K73" t="s">
         <v>530</v>
-      </c>
-      <c r="J73" t="s">
-        <v>531</v>
-      </c>
-      <c r="K73" t="s">
-        <v>532</v>
       </c>
       <c r="L73" t="s">
         <v>468</v>
@@ -7609,7 +8101,7 @@
         <v>44</v>
       </c>
       <c r="P73" s="46" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="Q73" s="18" t="str">
         <f t="shared" si="0"/>
@@ -7619,16 +8111,22 @@
         <f t="shared" ca="1" si="2"/>
         <v/>
       </c>
-      <c r="U73" s="50">
-        <v>46293</v>
+      <c r="S73" t="s">
+        <v>785</v>
+      </c>
+      <c r="T73" t="s">
+        <v>786</v>
+      </c>
+      <c r="U73" t="s">
+        <v>146</v>
       </c>
       <c r="V73" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
     </row>
     <row r="74" spans="1:22">
       <c r="A74" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="B74" t="s">
         <v>464</v>
@@ -7641,22 +8139,22 @@
       </c>
       <c r="E74" s="48"/>
       <c r="F74" t="s">
+        <v>525</v>
+      </c>
+      <c r="G74" t="s">
+        <v>532</v>
+      </c>
+      <c r="H74" t="s">
         <v>527</v>
       </c>
-      <c r="G74" t="s">
+      <c r="I74" t="s">
+        <v>533</v>
+      </c>
+      <c r="J74" t="s">
         <v>534</v>
       </c>
-      <c r="H74" t="s">
-        <v>529</v>
-      </c>
-      <c r="I74" t="s">
+      <c r="K74" t="s">
         <v>535</v>
-      </c>
-      <c r="J74" t="s">
-        <v>536</v>
-      </c>
-      <c r="K74" t="s">
-        <v>537</v>
       </c>
       <c r="L74" t="s">
         <v>468</v>
@@ -7671,7 +8169,7 @@
         <v>44</v>
       </c>
       <c r="P74" s="46" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="Q74" s="18" t="str">
         <f t="shared" si="0"/>
@@ -7681,16 +8179,22 @@
         <f t="shared" ca="1" si="2"/>
         <v/>
       </c>
-      <c r="U74" s="50">
-        <v>46293</v>
+      <c r="S74" t="s">
+        <v>784</v>
+      </c>
+      <c r="T74" t="s">
+        <v>779</v>
+      </c>
+      <c r="U74" t="s">
+        <v>146</v>
       </c>
       <c r="V74" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
     </row>
     <row r="75" spans="1:22">
       <c r="A75" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="B75" t="s">
         <v>464</v>
@@ -7705,22 +8209,22 @@
         <v>46287</v>
       </c>
       <c r="F75" t="s">
+        <v>525</v>
+      </c>
+      <c r="G75" t="s">
+        <v>537</v>
+      </c>
+      <c r="H75" t="s">
         <v>527</v>
       </c>
-      <c r="G75" t="s">
+      <c r="I75" t="s">
+        <v>538</v>
+      </c>
+      <c r="J75" t="s">
         <v>539</v>
       </c>
-      <c r="H75" t="s">
-        <v>529</v>
-      </c>
-      <c r="I75" t="s">
+      <c r="K75" t="s">
         <v>540</v>
-      </c>
-      <c r="J75" t="s">
-        <v>541</v>
-      </c>
-      <c r="K75" t="s">
-        <v>542</v>
       </c>
       <c r="L75" t="s">
         <v>468</v>
@@ -7735,7 +8239,7 @@
         <v>40</v>
       </c>
       <c r="P75" s="46" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="Q75" s="18">
         <f t="shared" ref="Q75:Q82" si="3">IF(E75="","",E75+1)</f>
@@ -7745,16 +8249,22 @@
         <f t="shared" ca="1" si="2"/>
         <v>21</v>
       </c>
-      <c r="U75" s="50">
-        <v>46308</v>
+      <c r="S75" t="s">
+        <v>782</v>
+      </c>
+      <c r="T75" t="s">
+        <v>783</v>
+      </c>
+      <c r="U75" t="s">
+        <v>146</v>
       </c>
       <c r="V75" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
     </row>
     <row r="76" spans="1:22">
       <c r="A76" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="B76" t="s">
         <v>464</v>
@@ -7767,22 +8277,22 @@
       </c>
       <c r="E76" s="48"/>
       <c r="F76" t="s">
+        <v>525</v>
+      </c>
+      <c r="G76" t="s">
+        <v>543</v>
+      </c>
+      <c r="H76" t="s">
         <v>527</v>
       </c>
-      <c r="G76" t="s">
+      <c r="I76" t="s">
+        <v>544</v>
+      </c>
+      <c r="J76" t="s">
         <v>545</v>
       </c>
-      <c r="H76" t="s">
-        <v>529</v>
-      </c>
-      <c r="I76" t="s">
+      <c r="K76" t="s">
         <v>546</v>
-      </c>
-      <c r="J76" t="s">
-        <v>547</v>
-      </c>
-      <c r="K76" t="s">
-        <v>548</v>
       </c>
       <c r="L76" t="s">
         <v>468</v>
@@ -7797,7 +8307,7 @@
         <v>44</v>
       </c>
       <c r="P76" s="46" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="Q76" s="18" t="str">
         <f t="shared" si="3"/>
@@ -7807,16 +8317,22 @@
         <f t="shared" ca="1" si="2"/>
         <v/>
       </c>
-      <c r="U76" s="50">
-        <v>46293</v>
+      <c r="S76" t="s">
+        <v>780</v>
+      </c>
+      <c r="T76" t="s">
+        <v>779</v>
+      </c>
+      <c r="U76" t="s">
+        <v>146</v>
       </c>
       <c r="V76" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
     </row>
     <row r="77" spans="1:22">
       <c r="A77" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="B77" t="s">
         <v>464</v>
@@ -7829,22 +8345,22 @@
       </c>
       <c r="E77" s="48"/>
       <c r="F77" t="s">
+        <v>525</v>
+      </c>
+      <c r="G77" t="s">
+        <v>548</v>
+      </c>
+      <c r="H77" t="s">
         <v>527</v>
       </c>
-      <c r="G77" t="s">
+      <c r="I77" t="s">
+        <v>549</v>
+      </c>
+      <c r="J77" t="s">
         <v>550</v>
       </c>
-      <c r="H77" t="s">
-        <v>529</v>
-      </c>
-      <c r="I77" t="s">
+      <c r="K77" t="s">
         <v>551</v>
-      </c>
-      <c r="J77" t="s">
-        <v>552</v>
-      </c>
-      <c r="K77" t="s">
-        <v>553</v>
       </c>
       <c r="L77" t="s">
         <v>468</v>
@@ -7859,7 +8375,7 @@
         <v>44</v>
       </c>
       <c r="P77" s="46" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="Q77" s="18" t="str">
         <f t="shared" si="3"/>
@@ -7869,16 +8385,22 @@
         <f t="shared" ca="1" si="2"/>
         <v/>
       </c>
-      <c r="U77" s="50">
-        <v>46293</v>
+      <c r="S77" t="s">
+        <v>781</v>
+      </c>
+      <c r="T77" t="s">
+        <v>779</v>
+      </c>
+      <c r="U77" t="s">
+        <v>146</v>
       </c>
       <c r="V77" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
     </row>
     <row r="78" spans="1:22">
       <c r="A78" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B78" t="s">
         <v>464</v>
@@ -7891,22 +8413,22 @@
       </c>
       <c r="E78" s="48"/>
       <c r="F78" t="s">
+        <v>525</v>
+      </c>
+      <c r="G78" t="s">
+        <v>553</v>
+      </c>
+      <c r="H78" t="s">
         <v>527</v>
       </c>
-      <c r="G78" t="s">
+      <c r="I78" t="s">
+        <v>554</v>
+      </c>
+      <c r="J78" t="s">
         <v>555</v>
       </c>
-      <c r="H78" t="s">
-        <v>529</v>
-      </c>
-      <c r="I78" t="s">
+      <c r="K78" t="s">
         <v>556</v>
-      </c>
-      <c r="J78" t="s">
-        <v>557</v>
-      </c>
-      <c r="K78" t="s">
-        <v>558</v>
       </c>
       <c r="L78" t="s">
         <v>468</v>
@@ -7921,7 +8443,7 @@
         <v>44</v>
       </c>
       <c r="P78" s="46" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="Q78" s="18" t="str">
         <f t="shared" si="3"/>
@@ -7931,16 +8453,22 @@
         <f t="shared" ca="1" si="2"/>
         <v/>
       </c>
-      <c r="U78" s="50">
-        <v>46293</v>
+      <c r="S78" t="s">
+        <v>778</v>
+      </c>
+      <c r="T78" t="s">
+        <v>779</v>
+      </c>
+      <c r="U78" t="s">
+        <v>146</v>
       </c>
       <c r="V78" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
     </row>
     <row r="79" spans="1:22">
       <c r="A79" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="B79" t="s">
         <v>464</v>
@@ -7955,22 +8483,22 @@
         <v>46287</v>
       </c>
       <c r="F79" t="s">
+        <v>525</v>
+      </c>
+      <c r="G79" t="s">
+        <v>558</v>
+      </c>
+      <c r="H79" t="s">
         <v>527</v>
       </c>
-      <c r="G79" t="s">
+      <c r="I79" t="s">
+        <v>559</v>
+      </c>
+      <c r="J79" t="s">
         <v>560</v>
       </c>
-      <c r="H79" t="s">
-        <v>529</v>
-      </c>
-      <c r="I79" t="s">
+      <c r="K79" t="s">
         <v>561</v>
-      </c>
-      <c r="J79" t="s">
-        <v>562</v>
-      </c>
-      <c r="K79" t="s">
-        <v>563</v>
       </c>
       <c r="L79" t="s">
         <v>468</v>
@@ -7985,7 +8513,7 @@
         <v>40</v>
       </c>
       <c r="P79" s="46" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="Q79" s="18">
         <f t="shared" si="3"/>
@@ -7995,16 +8523,22 @@
         <f t="shared" ca="1" si="2"/>
         <v>21</v>
       </c>
-      <c r="U79" s="50">
-        <v>46308</v>
+      <c r="S79" t="s">
+        <v>776</v>
+      </c>
+      <c r="T79" t="s">
+        <v>777</v>
+      </c>
+      <c r="U79" t="s">
+        <v>146</v>
       </c>
       <c r="V79" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
     </row>
     <row r="80" spans="1:22">
       <c r="A80" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="B80" t="s">
         <v>464</v>
@@ -8019,22 +8553,22 @@
         <v>46287</v>
       </c>
       <c r="F80" t="s">
+        <v>564</v>
+      </c>
+      <c r="G80" t="s">
+        <v>565</v>
+      </c>
+      <c r="H80" t="s">
         <v>566</v>
       </c>
-      <c r="G80" t="s">
+      <c r="I80" t="s">
         <v>567</v>
       </c>
-      <c r="H80" t="s">
+      <c r="J80" t="s">
         <v>568</v>
       </c>
-      <c r="I80" t="s">
+      <c r="K80" t="s">
         <v>569</v>
-      </c>
-      <c r="J80" t="s">
-        <v>570</v>
-      </c>
-      <c r="K80" t="s">
-        <v>571</v>
       </c>
       <c r="L80" t="s">
         <v>468</v>
@@ -8049,7 +8583,7 @@
         <v>40</v>
       </c>
       <c r="P80" s="46" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="Q80" s="18">
         <f t="shared" si="3"/>
@@ -8059,16 +8593,22 @@
         <f t="shared" ca="1" si="2"/>
         <v>21</v>
       </c>
-      <c r="U80" t="s">
-        <v>469</v>
+      <c r="S80" t="s">
+        <v>773</v>
+      </c>
+      <c r="T80" t="s">
+        <v>774</v>
+      </c>
+      <c r="U80" s="48" t="s">
+        <v>775</v>
       </c>
       <c r="V80" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
     </row>
     <row r="81" spans="1:22">
       <c r="A81" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="B81" t="s">
         <v>464</v>
@@ -8086,19 +8626,19 @@
         <v>264</v>
       </c>
       <c r="G81" t="s">
+        <v>572</v>
+      </c>
+      <c r="H81" t="s">
+        <v>504</v>
+      </c>
+      <c r="I81" t="s">
+        <v>573</v>
+      </c>
+      <c r="J81" t="s">
         <v>574</v>
       </c>
-      <c r="H81" t="s">
-        <v>506</v>
-      </c>
-      <c r="I81" t="s">
+      <c r="K81" t="s">
         <v>575</v>
-      </c>
-      <c r="J81" t="s">
-        <v>576</v>
-      </c>
-      <c r="K81" t="s">
-        <v>577</v>
       </c>
       <c r="L81" t="s">
         <v>468</v>
@@ -8113,7 +8653,7 @@
         <v>40</v>
       </c>
       <c r="P81" s="46" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="Q81" s="18">
         <f t="shared" si="3"/>
@@ -8123,16 +8663,22 @@
         <f t="shared" ca="1" si="2"/>
         <v>21</v>
       </c>
-      <c r="U81" t="s">
-        <v>469</v>
+      <c r="S81" t="s">
+        <v>772</v>
+      </c>
+      <c r="T81" t="s">
+        <v>771</v>
+      </c>
+      <c r="U81" s="48">
+        <v>46322</v>
       </c>
       <c r="V81" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
     </row>
     <row r="82" spans="1:22">
       <c r="A82" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="B82" t="s">
         <v>464</v>
@@ -8147,7 +8693,7 @@
         <v>46287</v>
       </c>
       <c r="F82" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="G82" t="s">
         <v>146</v>
@@ -8156,13 +8702,13 @@
         <v>138</v>
       </c>
       <c r="I82" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="J82" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="K82" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="L82" t="s">
         <v>468</v>
@@ -8177,7 +8723,7 @@
         <v>40</v>
       </c>
       <c r="P82" s="46" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="Q82" s="18">
         <f t="shared" si="3"/>
@@ -8187,16 +8733,22 @@
         <f t="shared" ca="1" si="2"/>
         <v>21</v>
       </c>
+      <c r="S82" t="s">
+        <v>770</v>
+      </c>
+      <c r="T82" t="s">
+        <v>769</v>
+      </c>
       <c r="U82" t="s">
-        <v>469</v>
+        <v>146</v>
       </c>
       <c r="V82" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
     </row>
     <row r="83" spans="1:22">
       <c r="A83" s="10" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
       <c r="B83" s="11" t="s">
         <v>215</v>
@@ -8211,10 +8763,10 @@
         <v>46295</v>
       </c>
       <c r="F83" s="43" t="s">
-        <v>638</v>
+        <v>635</v>
       </c>
       <c r="G83" s="43" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
       <c r="H83" s="11" t="s">
         <v>408</v>
@@ -8223,13 +8775,13 @@
         <v>426</v>
       </c>
       <c r="J83" s="11" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="K83" s="11" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
       <c r="L83" s="11" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
       <c r="M83" s="11" t="s">
         <v>45</v>
@@ -8252,19 +8804,19 @@
         <v>13</v>
       </c>
       <c r="S83" s="43" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="T83" s="43" t="s">
-        <v>656</v>
+        <v>653</v>
       </c>
       <c r="U83" s="7"/>
       <c r="V83" s="41" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
     </row>
     <row r="84" spans="1:22">
       <c r="A84" s="10" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="B84" s="11" t="s">
         <v>215</v>
@@ -8279,7 +8831,7 @@
         <v>46295</v>
       </c>
       <c r="F84" s="43" t="s">
-        <v>638</v>
+        <v>635</v>
       </c>
       <c r="G84" s="43" t="s">
         <v>445</v>
@@ -8291,13 +8843,13 @@
         <v>446</v>
       </c>
       <c r="J84" s="11" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="K84" s="11" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="L84" s="11" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
       <c r="M84" s="11" t="s">
         <v>45</v>
@@ -8320,19 +8872,19 @@
         <v>13</v>
       </c>
       <c r="S84" s="43" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
       <c r="T84" s="43" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
       <c r="U84" s="7"/>
       <c r="V84" s="41" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
     </row>
     <row r="85" spans="1:22">
       <c r="A85" s="10" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="B85" s="11" t="s">
         <v>215</v>
@@ -8347,7 +8899,7 @@
         <v>46295</v>
       </c>
       <c r="F85" s="43" t="s">
-        <v>638</v>
+        <v>635</v>
       </c>
       <c r="G85" s="43" t="s">
         <v>440</v>
@@ -8359,13 +8911,13 @@
         <v>441</v>
       </c>
       <c r="J85" s="11" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
       <c r="K85" s="11" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="L85" s="11" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
       <c r="M85" s="11" t="s">
         <v>45</v>
@@ -8388,21 +8940,21 @@
         <v>13</v>
       </c>
       <c r="S85" s="43" t="s">
-        <v>659</v>
+        <v>656</v>
       </c>
       <c r="T85" s="43" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
       <c r="U85" s="7">
         <v>46308</v>
       </c>
       <c r="V85" s="41" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
     </row>
     <row r="86" spans="1:22">
       <c r="A86" s="10" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
       <c r="B86" s="11" t="s">
         <v>215</v>
@@ -8417,25 +8969,25 @@
         <v>46295</v>
       </c>
       <c r="F86" s="43" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
       <c r="G86" s="43" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="H86" s="11" t="s">
         <v>408</v>
       </c>
       <c r="I86" s="11" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="J86" s="11" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
       <c r="K86" s="11" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="L86" s="11" t="s">
-        <v>654</v>
+        <v>651</v>
       </c>
       <c r="M86" s="11" t="s">
         <v>45</v>
@@ -8447,7 +8999,7 @@
         <v>40</v>
       </c>
       <c r="P86" s="11" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="Q86" s="18">
         <f t="shared" si="4"/>
@@ -8457,21 +9009,25 @@
         <f t="shared" ca="1" si="5"/>
         <v>13</v>
       </c>
-      <c r="S86" s="43"/>
-      <c r="T86" s="43"/>
-      <c r="U86" s="7">
-        <v>46308</v>
+      <c r="S86" s="43" t="s">
+        <v>767</v>
+      </c>
+      <c r="T86" s="43" t="s">
+        <v>768</v>
+      </c>
+      <c r="U86" s="7" t="s">
+        <v>146</v>
       </c>
       <c r="V86" s="41" t="s">
-        <v>663</v>
+        <v>660</v>
       </c>
     </row>
     <row r="87" spans="1:22">
       <c r="A87" s="10" t="s">
-        <v>664</v>
+        <v>661</v>
       </c>
       <c r="B87" s="11" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="C87" s="12">
         <v>46308</v>
@@ -8486,22 +9042,22 @@
         <v>264</v>
       </c>
       <c r="G87" s="43" t="s">
-        <v>666</v>
+        <v>663</v>
       </c>
       <c r="H87" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="I87" s="58">
+      <c r="I87" s="57">
         <v>0.54</v>
       </c>
       <c r="J87" s="11" t="s">
-        <v>667</v>
+        <v>664</v>
       </c>
       <c r="K87" s="11" t="s">
-        <v>668</v>
+        <v>665</v>
       </c>
       <c r="L87" s="11" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="M87" s="11" t="s">
         <v>45</v>
@@ -8510,10 +9066,10 @@
         <v>40</v>
       </c>
       <c r="O87" s="11" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="P87" s="11" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="Q87" s="18">
         <f t="shared" si="4"/>
@@ -8526,18 +9082,18 @@
       <c r="S87" s="43"/>
       <c r="T87" s="43"/>
       <c r="U87" s="7" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="V87" s="41" t="s">
-        <v>671</v>
+        <v>668</v>
       </c>
     </row>
     <row r="88" spans="1:22">
       <c r="A88" s="10" t="s">
-        <v>672</v>
+        <v>669</v>
       </c>
       <c r="B88" s="11" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="C88" s="12">
         <v>46308</v>
@@ -8552,22 +9108,22 @@
         <v>264</v>
       </c>
       <c r="G88" s="43" t="s">
-        <v>673</v>
+        <v>670</v>
       </c>
       <c r="H88" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="I88" s="58">
+      <c r="I88" s="57">
         <v>0.45</v>
       </c>
       <c r="J88" s="11" t="s">
         <v>304</v>
       </c>
       <c r="K88" s="11" t="s">
-        <v>674</v>
+        <v>671</v>
       </c>
       <c r="L88" s="11" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="M88" s="11" t="s">
         <v>45</v>
@@ -8576,10 +9132,10 @@
         <v>40</v>
       </c>
       <c r="O88" s="11" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="P88" s="11" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="Q88" s="18">
         <f t="shared" si="4"/>
@@ -8592,18 +9148,18 @@
       <c r="S88" s="43"/>
       <c r="T88" s="43"/>
       <c r="U88" s="7" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="V88" s="41" t="s">
-        <v>675</v>
+        <v>672</v>
       </c>
     </row>
     <row r="89" spans="1:22">
       <c r="A89" s="10" t="s">
-        <v>676</v>
+        <v>673</v>
       </c>
       <c r="B89" s="11" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="C89" s="12">
         <v>46308</v>
@@ -8618,22 +9174,22 @@
         <v>270</v>
       </c>
       <c r="G89" s="43" t="s">
-        <v>677</v>
+        <v>674</v>
       </c>
       <c r="H89" s="11" t="s">
         <v>52</v>
       </c>
       <c r="I89" s="11" t="s">
-        <v>678</v>
+        <v>675</v>
       </c>
       <c r="J89" s="11" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="K89" s="11" t="s">
-        <v>679</v>
+        <v>676</v>
       </c>
       <c r="L89" s="11" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="M89" s="11" t="s">
         <v>41</v>
@@ -8642,10 +9198,10 @@
         <v>40</v>
       </c>
       <c r="O89" s="11" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="P89" s="11" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="Q89" s="18">
         <f t="shared" si="4"/>
@@ -8658,18 +9214,18 @@
       <c r="S89" s="43"/>
       <c r="T89" s="43"/>
       <c r="U89" s="7" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="V89" s="41" t="s">
-        <v>680</v>
+        <v>677</v>
       </c>
     </row>
     <row r="90" spans="1:22">
       <c r="A90" s="10" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
       <c r="B90" s="11" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="C90" s="12">
         <v>46308</v>
@@ -8684,22 +9240,22 @@
         <v>264</v>
       </c>
       <c r="G90" s="43" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
       <c r="H90" s="11" t="s">
         <v>61</v>
       </c>
       <c r="I90" s="11" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
       <c r="J90" s="11" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
       <c r="K90" s="11" t="s">
-        <v>685</v>
+        <v>682</v>
       </c>
       <c r="L90" s="11" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="M90" s="11" t="s">
         <v>45</v>
@@ -8708,10 +9264,10 @@
         <v>40</v>
       </c>
       <c r="O90" s="11" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="P90" s="11" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="Q90" s="18">
         <f t="shared" si="4"/>
@@ -8724,18 +9280,18 @@
       <c r="S90" s="43"/>
       <c r="T90" s="43"/>
       <c r="U90" s="7" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="V90" s="41" t="s">
-        <v>686</v>
+        <v>683</v>
       </c>
     </row>
     <row r="91" spans="1:22">
       <c r="A91" s="10" t="s">
-        <v>687</v>
+        <v>684</v>
       </c>
       <c r="B91" s="11" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="C91" s="12">
         <v>46308</v>
@@ -8750,22 +9306,22 @@
         <v>264</v>
       </c>
       <c r="G91" s="43" t="s">
-        <v>688</v>
+        <v>685</v>
       </c>
       <c r="H91" s="11" t="s">
         <v>60</v>
       </c>
       <c r="I91" s="11" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
       <c r="J91" s="11" t="s">
-        <v>689</v>
+        <v>686</v>
       </c>
       <c r="K91" s="11" t="s">
-        <v>690</v>
+        <v>687</v>
       </c>
       <c r="L91" s="11" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="M91" s="11" t="s">
         <v>41</v>
@@ -8774,10 +9330,10 @@
         <v>40</v>
       </c>
       <c r="O91" s="11" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="P91" s="11" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="Q91" s="18">
         <f t="shared" si="4"/>
@@ -8790,16 +9346,16 @@
       <c r="S91" s="43"/>
       <c r="T91" s="43"/>
       <c r="U91" s="7" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="V91" s="41"/>
     </row>
     <row r="92" spans="1:22">
       <c r="A92" s="10" t="s">
-        <v>691</v>
+        <v>688</v>
       </c>
       <c r="B92" s="11" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="C92" s="12">
         <v>46308</v>
@@ -8811,25 +9367,25 @@
         <v>46308</v>
       </c>
       <c r="F92" s="43" t="s">
+        <v>689</v>
+      </c>
+      <c r="G92" s="43" t="s">
+        <v>690</v>
+      </c>
+      <c r="H92" s="11" t="s">
+        <v>691</v>
+      </c>
+      <c r="I92" s="11" t="s">
         <v>692</v>
       </c>
-      <c r="G92" s="43" t="s">
+      <c r="J92" s="11" t="s">
         <v>693</v>
       </c>
-      <c r="H92" s="11" t="s">
+      <c r="K92" s="11" t="s">
         <v>694</v>
       </c>
-      <c r="I92" s="11" t="s">
-        <v>695</v>
-      </c>
-      <c r="J92" s="11" t="s">
-        <v>696</v>
-      </c>
-      <c r="K92" s="11" t="s">
-        <v>697</v>
-      </c>
       <c r="L92" s="11" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="M92" s="11" t="s">
         <v>41</v>
@@ -8838,10 +9394,10 @@
         <v>40</v>
       </c>
       <c r="O92" s="11" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="P92" s="11" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="Q92" s="18">
         <f t="shared" si="4"/>
@@ -8854,18 +9410,18 @@
       <c r="S92" s="43"/>
       <c r="T92" s="43"/>
       <c r="U92" s="7" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="V92" s="41" t="s">
-        <v>698</v>
+        <v>695</v>
       </c>
     </row>
     <row r="93" spans="1:22">
       <c r="A93" s="10" t="s">
-        <v>699</v>
+        <v>696</v>
       </c>
       <c r="B93" s="11" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="C93" s="12">
         <v>46308</v>
@@ -8877,25 +9433,25 @@
         <v>46308</v>
       </c>
       <c r="F93" s="43" t="s">
-        <v>700</v>
+        <v>697</v>
       </c>
       <c r="G93" s="43" t="s">
-        <v>701</v>
+        <v>698</v>
       </c>
       <c r="H93" s="11" t="s">
         <v>62</v>
       </c>
       <c r="I93" s="11" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="J93" s="11" t="s">
-        <v>703</v>
+        <v>700</v>
       </c>
       <c r="K93" s="11" t="s">
-        <v>704</v>
+        <v>701</v>
       </c>
       <c r="L93" s="11" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="M93" s="11" t="s">
         <v>45</v>
@@ -8904,10 +9460,10 @@
         <v>40</v>
       </c>
       <c r="O93" s="11" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="P93" s="11" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="Q93" s="18">
         <f t="shared" si="4"/>
@@ -8920,18 +9476,18 @@
       <c r="S93" s="43"/>
       <c r="T93" s="43"/>
       <c r="U93" s="7" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="V93" s="41" t="s">
-        <v>705</v>
+        <v>702</v>
       </c>
     </row>
     <row r="94" spans="1:22">
       <c r="A94" s="10" t="s">
-        <v>706</v>
+        <v>703</v>
       </c>
       <c r="B94" s="11" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="C94" s="12">
         <v>46308</v>
@@ -8946,22 +9502,22 @@
         <v>272</v>
       </c>
       <c r="G94" s="43" t="s">
-        <v>707</v>
+        <v>704</v>
       </c>
       <c r="H94" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="I94" s="58">
+      <c r="I94" s="57">
         <v>1.1000000000000001</v>
       </c>
       <c r="J94" s="11" t="s">
-        <v>708</v>
+        <v>705</v>
       </c>
       <c r="K94" s="11" t="s">
-        <v>709</v>
+        <v>706</v>
       </c>
       <c r="L94" s="11" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="M94" s="11" t="s">
         <v>45</v>
@@ -8970,10 +9526,10 @@
         <v>40</v>
       </c>
       <c r="O94" s="11" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="P94" s="11" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="Q94" s="18">
         <f t="shared" si="4"/>
@@ -8986,18 +9542,18 @@
       <c r="S94" s="43"/>
       <c r="T94" s="43"/>
       <c r="U94" s="7" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="V94" s="41" t="s">
-        <v>710</v>
+        <v>707</v>
       </c>
     </row>
     <row r="95" spans="1:22">
       <c r="A95" s="10" t="s">
-        <v>711</v>
+        <v>708</v>
       </c>
       <c r="B95" s="11" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="C95" s="12">
         <v>46308</v>
@@ -9012,22 +9568,22 @@
         <v>272</v>
       </c>
       <c r="G95" s="43" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
       <c r="H95" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="I95" s="58">
+      <c r="I95" s="57">
         <v>0.9</v>
       </c>
       <c r="J95" s="11" t="s">
-        <v>713</v>
+        <v>710</v>
       </c>
       <c r="K95" s="11" t="s">
-        <v>714</v>
+        <v>711</v>
       </c>
       <c r="L95" s="11" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="M95" s="11" t="s">
         <v>41</v>
@@ -9036,10 +9592,10 @@
         <v>40</v>
       </c>
       <c r="O95" s="11" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="P95" s="11" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="Q95" s="18">
         <f t="shared" si="4"/>
@@ -9052,18 +9608,18 @@
       <c r="S95" s="43"/>
       <c r="T95" s="43"/>
       <c r="U95" s="7" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="V95" s="41" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
     </row>
     <row r="96" spans="1:22">
       <c r="A96" s="10" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="B96" s="11" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="C96" s="12">
         <v>46308</v>
@@ -9075,25 +9631,25 @@
         <v>46308</v>
       </c>
       <c r="F96" s="43" t="s">
-        <v>718</v>
+        <v>715</v>
       </c>
       <c r="G96" s="43" t="s">
-        <v>719</v>
+        <v>716</v>
       </c>
       <c r="H96" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="I96" s="58">
+      <c r="I96" s="57">
         <v>2.6</v>
       </c>
       <c r="J96" s="11" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="K96" s="11" t="s">
-        <v>721</v>
+        <v>718</v>
       </c>
       <c r="L96" s="11" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="M96" s="11" t="s">
         <v>49</v>
@@ -9102,10 +9658,10 @@
         <v>40</v>
       </c>
       <c r="O96" s="11" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="P96" s="11" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="Q96" s="18">
         <f t="shared" si="4"/>
@@ -9118,18 +9674,18 @@
       <c r="S96" s="43"/>
       <c r="T96" s="43"/>
       <c r="U96" s="7" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="V96" s="41" t="s">
-        <v>722</v>
+        <v>719</v>
       </c>
     </row>
     <row r="97" spans="1:22">
       <c r="A97" s="10" t="s">
-        <v>723</v>
+        <v>720</v>
       </c>
       <c r="B97" s="11" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="C97" s="12">
         <v>46308</v>
@@ -9141,25 +9697,25 @@
         <v>46308</v>
       </c>
       <c r="F97" s="43" t="s">
-        <v>724</v>
+        <v>721</v>
       </c>
       <c r="G97" s="43" t="s">
-        <v>725</v>
+        <v>722</v>
       </c>
       <c r="H97" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="I97" s="58">
+      <c r="I97" s="57">
         <v>1.6</v>
       </c>
       <c r="J97" s="11" t="s">
-        <v>726</v>
+        <v>723</v>
       </c>
       <c r="K97" s="11" t="s">
-        <v>727</v>
+        <v>724</v>
       </c>
       <c r="L97" s="11" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="M97" s="11" t="s">
         <v>49</v>
@@ -9168,10 +9724,10 @@
         <v>40</v>
       </c>
       <c r="O97" s="11" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="P97" s="11" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="Q97" s="18">
         <f t="shared" si="4"/>
@@ -9184,18 +9740,18 @@
       <c r="S97" s="43"/>
       <c r="T97" s="43"/>
       <c r="U97" s="7" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="V97" s="41" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
     </row>
     <row r="98" spans="1:22">
       <c r="A98" s="10" t="s">
-        <v>729</v>
+        <v>726</v>
       </c>
       <c r="B98" s="11" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="C98" s="12">
         <v>46308</v>
@@ -9207,25 +9763,25 @@
         <v>46308</v>
       </c>
       <c r="F98" s="43" t="s">
-        <v>730</v>
+        <v>727</v>
       </c>
       <c r="G98" s="43" t="s">
-        <v>731</v>
+        <v>728</v>
       </c>
       <c r="H98" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="I98" s="58">
+      <c r="I98" s="57">
         <v>1.2</v>
       </c>
       <c r="J98" s="11" t="s">
-        <v>732</v>
+        <v>729</v>
       </c>
       <c r="K98" s="11" t="s">
-        <v>733</v>
+        <v>730</v>
       </c>
       <c r="L98" s="11" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="M98" s="11" t="s">
         <v>49</v>
@@ -9234,10 +9790,10 @@
         <v>40</v>
       </c>
       <c r="O98" s="11" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="P98" s="11" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="Q98" s="18">
         <f t="shared" si="4"/>
@@ -9250,18 +9806,18 @@
       <c r="S98" s="43"/>
       <c r="T98" s="43"/>
       <c r="U98" s="7" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="V98" s="41" t="s">
-        <v>734</v>
+        <v>731</v>
       </c>
     </row>
     <row r="99" spans="1:22">
       <c r="A99" s="10" t="s">
-        <v>735</v>
+        <v>732</v>
       </c>
       <c r="B99" s="11" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="C99" s="12">
         <v>46308</v>
@@ -9273,25 +9829,25 @@
         <v>46308</v>
       </c>
       <c r="F99" s="43" t="s">
-        <v>736</v>
+        <v>733</v>
       </c>
       <c r="G99" s="43" t="s">
-        <v>737</v>
+        <v>734</v>
       </c>
       <c r="H99" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="I99" s="58">
+      <c r="I99" s="57">
         <v>1.2</v>
       </c>
       <c r="J99" s="11" t="s">
-        <v>732</v>
+        <v>729</v>
       </c>
       <c r="K99" s="11" t="s">
-        <v>738</v>
+        <v>735</v>
       </c>
       <c r="L99" s="11" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="M99" s="11" t="s">
         <v>49</v>
@@ -9300,10 +9856,10 @@
         <v>40</v>
       </c>
       <c r="O99" s="11" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="P99" s="11" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="Q99" s="18">
         <f t="shared" si="4"/>
@@ -9316,18 +9872,18 @@
       <c r="S99" s="43"/>
       <c r="T99" s="43"/>
       <c r="U99" s="7" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="V99" s="41" t="s">
-        <v>739</v>
+        <v>736</v>
       </c>
     </row>
     <row r="100" spans="1:22">
       <c r="A100" s="10" t="s">
-        <v>740</v>
+        <v>737</v>
       </c>
       <c r="B100" s="11" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="C100" s="12">
         <v>46308</v>
@@ -9339,25 +9895,25 @@
         <v>46308</v>
       </c>
       <c r="F100" s="43" t="s">
-        <v>700</v>
+        <v>697</v>
       </c>
       <c r="G100" s="43" t="s">
-        <v>741</v>
+        <v>738</v>
       </c>
       <c r="H100" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="I100" s="58">
+      <c r="I100" s="57">
         <v>1.5</v>
       </c>
       <c r="J100" s="11" t="s">
-        <v>742</v>
+        <v>739</v>
       </c>
       <c r="K100" s="11" t="s">
-        <v>743</v>
+        <v>740</v>
       </c>
       <c r="L100" s="11" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="M100" s="11" t="s">
         <v>49</v>
@@ -9366,10 +9922,10 @@
         <v>40</v>
       </c>
       <c r="O100" s="11" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="P100" s="11" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="Q100" s="18">
         <f t="shared" si="4"/>
@@ -9382,18 +9938,18 @@
       <c r="S100" s="43"/>
       <c r="T100" s="43"/>
       <c r="U100" s="7" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="V100" s="41" t="s">
-        <v>744</v>
+        <v>741</v>
       </c>
     </row>
     <row r="101" spans="1:22">
       <c r="A101" s="10" t="s">
-        <v>745</v>
+        <v>742</v>
       </c>
       <c r="B101" s="11" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="C101" s="12">
         <v>46308</v>
@@ -9405,7 +9961,7 @@
         <v>46308</v>
       </c>
       <c r="F101" s="43" t="s">
-        <v>746</v>
+        <v>743</v>
       </c>
       <c r="G101" s="43" t="s">
         <v>116</v>
@@ -9413,17 +9969,17 @@
       <c r="H101" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="I101" s="58">
+      <c r="I101" s="57">
         <v>1.32</v>
       </c>
       <c r="J101" s="11" t="s">
-        <v>747</v>
+        <v>744</v>
       </c>
       <c r="K101" s="11" t="s">
-        <v>748</v>
+        <v>745</v>
       </c>
       <c r="L101" s="11" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="M101" s="11" t="s">
         <v>49</v>
@@ -9432,10 +9988,10 @@
         <v>40</v>
       </c>
       <c r="O101" s="11" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="P101" s="11" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="Q101" s="18">
         <f t="shared" si="4"/>
@@ -9448,18 +10004,18 @@
       <c r="S101" s="43"/>
       <c r="T101" s="43"/>
       <c r="U101" s="7" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="V101" s="41" t="s">
-        <v>749</v>
+        <v>746</v>
       </c>
     </row>
     <row r="102" spans="1:22">
       <c r="A102" s="10" t="s">
-        <v>750</v>
+        <v>747</v>
       </c>
       <c r="B102" s="11" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="C102" s="12">
         <v>46308</v>
@@ -9479,17 +10035,17 @@
       <c r="H102" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="I102" s="59">
+      <c r="I102" s="58">
         <v>40</v>
       </c>
       <c r="J102" s="11" t="s">
-        <v>751</v>
+        <v>748</v>
       </c>
       <c r="K102" s="11" t="s">
-        <v>752</v>
+        <v>749</v>
       </c>
       <c r="L102" s="11" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="M102" s="11" t="s">
         <v>49</v>
@@ -9498,10 +10054,10 @@
         <v>40</v>
       </c>
       <c r="O102" s="11" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="P102" s="11" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="Q102" s="18">
         <f t="shared" si="4"/>
@@ -9514,18 +10070,18 @@
       <c r="S102" s="43"/>
       <c r="T102" s="43"/>
       <c r="U102" s="7" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="V102" s="41" t="s">
-        <v>753</v>
+        <v>750</v>
       </c>
     </row>
     <row r="103" spans="1:22">
       <c r="A103" s="10" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="B103" s="11" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="C103" s="12">
         <v>46308</v>
@@ -9545,17 +10101,17 @@
       <c r="H103" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="I103" s="59">
+      <c r="I103" s="58">
         <v>20</v>
       </c>
       <c r="J103" s="11" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="K103" s="11" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="L103" s="11" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="M103" s="11" t="s">
         <v>49</v>
@@ -9564,10 +10120,10 @@
         <v>40</v>
       </c>
       <c r="O103" s="11" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="P103" s="11" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="Q103" s="18">
         <f t="shared" si="4"/>
@@ -9580,18 +10136,18 @@
       <c r="S103" s="43"/>
       <c r="T103" s="43"/>
       <c r="U103" s="7" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="V103" s="41" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
     </row>
     <row r="104" spans="1:22">
       <c r="A104" s="10" t="s">
-        <v>758</v>
+        <v>755</v>
       </c>
       <c r="B104" s="11" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="C104" s="12">
         <v>46308</v>
@@ -9603,25 +10159,25 @@
         <v>46308</v>
       </c>
       <c r="F104" s="43" t="s">
+        <v>756</v>
+      </c>
+      <c r="G104" s="43" t="s">
+        <v>757</v>
+      </c>
+      <c r="H104" s="11" t="s">
+        <v>758</v>
+      </c>
+      <c r="I104" s="11" t="s">
         <v>759</v>
       </c>
-      <c r="G104" s="43" t="s">
+      <c r="J104" s="11" t="s">
         <v>760</v>
       </c>
-      <c r="H104" s="11" t="s">
+      <c r="K104" s="11" t="s">
         <v>761</v>
       </c>
-      <c r="I104" s="11" t="s">
-        <v>762</v>
-      </c>
-      <c r="J104" s="11" t="s">
-        <v>763</v>
-      </c>
-      <c r="K104" s="11" t="s">
-        <v>764</v>
-      </c>
       <c r="L104" s="11" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="M104" s="11" t="s">
         <v>41</v>
@@ -9630,10 +10186,10 @@
         <v>40</v>
       </c>
       <c r="O104" s="11" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="P104" s="11" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="Q104" s="18">
         <f t="shared" si="4"/>
@@ -9646,10 +10202,10 @@
       <c r="S104" s="43"/>
       <c r="T104" s="43"/>
       <c r="U104" s="7" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="V104" s="41" t="s">
-        <v>765</v>
+        <v>762</v>
       </c>
     </row>
     <row r="105" spans="1:22">
@@ -12781,25 +13337,25 @@
     <mergeCell ref="A8:V8"/>
   </mergeCells>
   <conditionalFormatting sqref="P11:P208">
-    <cfRule type="expression" dxfId="6" priority="1">
+    <cfRule type="expression" dxfId="41" priority="1">
       <formula>P11="RECOMENDADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="2">
+    <cfRule type="expression" dxfId="40" priority="2">
       <formula>P11="APROVADA - AGUARDANDO EXECUÇÃO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="3">
+    <cfRule type="expression" dxfId="39" priority="3">
       <formula>P11="EXECUTADA - EM MATURAÇÃO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="38" priority="4">
       <formula>P11="EXECUTADA - AVALIADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="5">
+    <cfRule type="expression" dxfId="37" priority="5">
       <formula>P11="APROVADA - NÃO EXECUTADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="6">
+    <cfRule type="expression" dxfId="36" priority="6">
       <formula>P11="REJEITADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="7">
+    <cfRule type="expression" dxfId="35" priority="7">
       <formula>LEFT(P11,9)="BLOQUEADA"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12854,16 +13410,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.95" customHeight="1">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="55" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
+      <c r="B1" s="55"/>
+      <c r="C1" s="55"/>
+      <c r="D1" s="55"/>
+      <c r="E1" s="55"/>
+      <c r="F1" s="55"/>
+      <c r="G1" s="55"/>
+      <c r="H1" s="55"/>
     </row>
     <row r="3" spans="1:8" ht="15">
       <c r="A3" s="30" t="s">
@@ -12982,16 +13538,16 @@
       </c>
     </row>
     <row r="18" spans="1:8" ht="15">
-      <c r="A18" s="57" t="s">
+      <c r="A18" s="56" t="s">
         <v>64</v>
       </c>
-      <c r="B18" s="57"/>
-      <c r="C18" s="57"/>
-      <c r="D18" s="57"/>
-      <c r="E18" s="57"/>
-      <c r="F18" s="57"/>
-      <c r="G18" s="57"/>
-      <c r="H18" s="57"/>
+      <c r="B18" s="56"/>
+      <c r="C18" s="56"/>
+      <c r="D18" s="56"/>
+      <c r="E18" s="56"/>
+      <c r="F18" s="56"/>
+      <c r="G18" s="56"/>
+      <c r="H18" s="56"/>
     </row>
     <row r="19" spans="1:8" ht="29.25">
       <c r="A19" s="31" t="s">

</xml_diff>

<commit_message>
[O7 13/10] Registro: vereditos O6-007 e O6-009 preenchidos pelo LEO (98 entradas completas)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1554" uniqueCount="797">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1558" uniqueCount="801">
   <si>
     <t>REGISTRO DE ALTERAÇÕES — AMAZON ADS | WINNET METAIS</t>
   </si>
@@ -1577,9 +1577,6 @@
     <t>30d: perna L2025-B do termo "lixeira banheiro 7 litros" com 3 cli, R$ 5,34, 0 venda — sem clique novo desde a O5. Amostra não mudou</t>
   </si>
   <si>
-    <t>Custo desprezível; reabrir só se a perna voltar a consumir</t>
-  </si>
-  <si>
     <t>O6-010</t>
   </si>
   <si>
@@ -2424,6 +2421,21 @@
   </si>
   <si>
     <t>GATILHO NÃO DISPAROU — lances mantidos; alvo B0CYWMQ93Y → O7-003</t>
+  </si>
+  <si>
+    <t>O5-013 cancelada em 22/09; nada a promover</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENCERRADA </t>
+  </si>
+  <si>
+    <t>L2025-B segue no grupo da 6B; exatas da 6B sem venda em 30d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MANTIDA </t>
+  </si>
+  <si>
+    <t>grupo recebe a exata "lixo banheiro" (O7-007)</t>
   </si>
 </sst>
 </file>
@@ -2801,6 +2813,12 @@
     <xf numFmtId="14" fontId="15" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2822,373 +2840,12 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
-  <dxfs count="42">
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9A3412"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFED7AA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF991B1B"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEE2E2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF374151"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF3F4F6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF166534"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDCFCE7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF3730A3"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE0E7FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF92400E"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEF3C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1E40AF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDBEAFE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9A3412"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFED7AA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF991B1B"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEE2E2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF374151"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF3F4F6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF166534"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDCFCE7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF3730A3"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE0E7FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF92400E"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEF3C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1E40AF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDBEAFE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9A3412"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFED7AA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF991B1B"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEE2E2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF374151"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF3F4F6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF166534"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDCFCE7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF3730A3"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE0E7FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF92400E"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEF3C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1E40AF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDBEAFE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9A3412"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFED7AA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF991B1B"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEE2E2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF374151"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF3F4F6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF166534"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDCFCE7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF3730A3"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE0E7FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF92400E"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEF3C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1E40AF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDBEAFE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9A3412"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFED7AA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF991B1B"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEE2E2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF374151"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF3F4F6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF166534"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDCFCE7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF3730A3"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE0E7FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF92400E"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFEF3C7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF1E40AF"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFDBEAFE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="7">
     <dxf>
       <font>
         <b/>
@@ -3521,82 +3178,82 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="30" customHeight="1">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="50"/>
-      <c r="D1" s="50"/>
-      <c r="E1" s="50"/>
-      <c r="F1" s="50"/>
-      <c r="G1" s="50"/>
-      <c r="H1" s="50"/>
-      <c r="I1" s="50"/>
-      <c r="J1" s="50"/>
-      <c r="K1" s="50"/>
-      <c r="L1" s="50"/>
-      <c r="M1" s="50"/>
-      <c r="N1" s="50"/>
-      <c r="O1" s="50"/>
-      <c r="P1" s="50"/>
-      <c r="Q1" s="50"/>
-      <c r="R1" s="50"/>
-      <c r="S1" s="50"/>
-      <c r="T1" s="50"/>
-      <c r="U1" s="50"/>
-      <c r="V1" s="50"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="52"/>
+      <c r="H1" s="52"/>
+      <c r="I1" s="52"/>
+      <c r="J1" s="52"/>
+      <c r="K1" s="52"/>
+      <c r="L1" s="52"/>
+      <c r="M1" s="52"/>
+      <c r="N1" s="52"/>
+      <c r="O1" s="52"/>
+      <c r="P1" s="52"/>
+      <c r="Q1" s="52"/>
+      <c r="R1" s="52"/>
+      <c r="S1" s="52"/>
+      <c r="T1" s="52"/>
+      <c r="U1" s="52"/>
+      <c r="V1" s="52"/>
     </row>
     <row r="2" spans="1:22" ht="30" customHeight="1">
-      <c r="A2" s="51" t="s">
+      <c r="A2" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="51"/>
-      <c r="C2" s="51"/>
-      <c r="D2" s="51"/>
-      <c r="E2" s="51"/>
-      <c r="F2" s="51"/>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
-      <c r="I2" s="51"/>
-      <c r="J2" s="51"/>
-      <c r="K2" s="51"/>
-      <c r="L2" s="51"/>
-      <c r="M2" s="51"/>
-      <c r="N2" s="51"/>
-      <c r="O2" s="51"/>
-      <c r="P2" s="51"/>
-      <c r="Q2" s="51"/>
-      <c r="R2" s="51"/>
-      <c r="S2" s="51"/>
-      <c r="T2" s="51"/>
-      <c r="U2" s="51"/>
-      <c r="V2" s="51"/>
+      <c r="B2" s="53"/>
+      <c r="C2" s="53"/>
+      <c r="D2" s="53"/>
+      <c r="E2" s="53"/>
+      <c r="F2" s="53"/>
+      <c r="G2" s="53"/>
+      <c r="H2" s="53"/>
+      <c r="I2" s="53"/>
+      <c r="J2" s="53"/>
+      <c r="K2" s="53"/>
+      <c r="L2" s="53"/>
+      <c r="M2" s="53"/>
+      <c r="N2" s="53"/>
+      <c r="O2" s="53"/>
+      <c r="P2" s="53"/>
+      <c r="Q2" s="53"/>
+      <c r="R2" s="53"/>
+      <c r="S2" s="53"/>
+      <c r="T2" s="53"/>
+      <c r="U2" s="53"/>
+      <c r="V2" s="53"/>
     </row>
     <row r="3" spans="1:22" ht="27.95" customHeight="1">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="54" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="52"/>
-      <c r="C3" s="52"/>
-      <c r="D3" s="52"/>
-      <c r="E3" s="52"/>
-      <c r="F3" s="52"/>
-      <c r="G3" s="52"/>
-      <c r="H3" s="52"/>
-      <c r="I3" s="52"/>
-      <c r="J3" s="52"/>
-      <c r="K3" s="52"/>
-      <c r="L3" s="52"/>
-      <c r="M3" s="52"/>
-      <c r="N3" s="52"/>
-      <c r="O3" s="52"/>
-      <c r="P3" s="52"/>
-      <c r="Q3" s="52"/>
-      <c r="R3" s="52"/>
-      <c r="S3" s="52"/>
-      <c r="T3" s="52"/>
-      <c r="U3" s="52"/>
-      <c r="V3" s="52"/>
+      <c r="B3" s="54"/>
+      <c r="C3" s="54"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
+      <c r="G3" s="54"/>
+      <c r="H3" s="54"/>
+      <c r="I3" s="54"/>
+      <c r="J3" s="54"/>
+      <c r="K3" s="54"/>
+      <c r="L3" s="54"/>
+      <c r="M3" s="54"/>
+      <c r="N3" s="54"/>
+      <c r="O3" s="54"/>
+      <c r="P3" s="54"/>
+      <c r="Q3" s="54"/>
+      <c r="R3" s="54"/>
+      <c r="S3" s="54"/>
+      <c r="T3" s="54"/>
+      <c r="U3" s="54"/>
+      <c r="V3" s="54"/>
     </row>
     <row r="5" spans="1:22">
       <c r="A5" s="1" t="s">
@@ -3617,23 +3274,23 @@
       <c r="F5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H5" s="53" t="s">
+      <c r="H5" s="55" t="s">
         <v>9</v>
       </c>
-      <c r="I5" s="53"/>
-      <c r="J5" s="53"/>
-      <c r="K5" s="53"/>
-      <c r="L5" s="53"/>
-      <c r="M5" s="53"/>
-      <c r="N5" s="53"/>
-      <c r="O5" s="53"/>
-      <c r="P5" s="53"/>
-      <c r="Q5" s="53"/>
-      <c r="R5" s="53"/>
-      <c r="S5" s="53"/>
-      <c r="T5" s="53"/>
-      <c r="U5" s="53"/>
-      <c r="V5" s="53"/>
+      <c r="I5" s="55"/>
+      <c r="J5" s="55"/>
+      <c r="K5" s="55"/>
+      <c r="L5" s="55"/>
+      <c r="M5" s="55"/>
+      <c r="N5" s="55"/>
+      <c r="O5" s="55"/>
+      <c r="P5" s="55"/>
+      <c r="Q5" s="55"/>
+      <c r="R5" s="55"/>
+      <c r="S5" s="55"/>
+      <c r="T5" s="55"/>
+      <c r="U5" s="55"/>
+      <c r="V5" s="55"/>
     </row>
     <row r="6" spans="1:22" ht="26.1" customHeight="1">
       <c r="A6" s="2">
@@ -3660,47 +3317,47 @@
         <f>COUNTIF(P11:P208,"EXECUTADA - AVALIADA")</f>
         <v>65</v>
       </c>
-      <c r="H6" s="53"/>
-      <c r="I6" s="53"/>
-      <c r="J6" s="53"/>
-      <c r="K6" s="53"/>
-      <c r="L6" s="53"/>
-      <c r="M6" s="53"/>
-      <c r="N6" s="53"/>
-      <c r="O6" s="53"/>
-      <c r="P6" s="53"/>
-      <c r="Q6" s="53"/>
-      <c r="R6" s="53"/>
-      <c r="S6" s="53"/>
-      <c r="T6" s="53"/>
-      <c r="U6" s="53"/>
-      <c r="V6" s="53"/>
+      <c r="H6" s="55"/>
+      <c r="I6" s="55"/>
+      <c r="J6" s="55"/>
+      <c r="K6" s="55"/>
+      <c r="L6" s="55"/>
+      <c r="M6" s="55"/>
+      <c r="N6" s="55"/>
+      <c r="O6" s="55"/>
+      <c r="P6" s="55"/>
+      <c r="Q6" s="55"/>
+      <c r="R6" s="55"/>
+      <c r="S6" s="55"/>
+      <c r="T6" s="55"/>
+      <c r="U6" s="55"/>
+      <c r="V6" s="55"/>
     </row>
     <row r="8" spans="1:22" ht="21.95" customHeight="1">
-      <c r="A8" s="54" t="s">
+      <c r="A8" s="56" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="54"/>
-      <c r="C8" s="54"/>
-      <c r="D8" s="54"/>
-      <c r="E8" s="54"/>
-      <c r="F8" s="54"/>
-      <c r="G8" s="54"/>
-      <c r="H8" s="54"/>
-      <c r="I8" s="54"/>
-      <c r="J8" s="54"/>
-      <c r="K8" s="54"/>
-      <c r="L8" s="54"/>
-      <c r="M8" s="54"/>
-      <c r="N8" s="54"/>
-      <c r="O8" s="54"/>
-      <c r="P8" s="54"/>
-      <c r="Q8" s="54"/>
-      <c r="R8" s="54"/>
-      <c r="S8" s="54"/>
-      <c r="T8" s="54"/>
-      <c r="U8" s="54"/>
-      <c r="V8" s="54"/>
+      <c r="B8" s="56"/>
+      <c r="C8" s="56"/>
+      <c r="D8" s="56"/>
+      <c r="E8" s="56"/>
+      <c r="F8" s="56"/>
+      <c r="G8" s="56"/>
+      <c r="H8" s="56"/>
+      <c r="I8" s="56"/>
+      <c r="J8" s="56"/>
+      <c r="K8" s="56"/>
+      <c r="L8" s="56"/>
+      <c r="M8" s="56"/>
+      <c r="N8" s="56"/>
+      <c r="O8" s="56"/>
+      <c r="P8" s="56"/>
+      <c r="Q8" s="56"/>
+      <c r="R8" s="56"/>
+      <c r="S8" s="56"/>
+      <c r="T8" s="56"/>
+      <c r="U8" s="56"/>
+      <c r="V8" s="56"/>
     </row>
     <row r="10" spans="1:22" ht="38.1" customHeight="1">
       <c r="A10" s="5" t="s">
@@ -5538,10 +5195,10 @@
         <v>34</v>
       </c>
       <c r="S36" t="s">
+        <v>581</v>
+      </c>
+      <c r="T36" t="s">
         <v>582</v>
-      </c>
-      <c r="T36" t="s">
-        <v>583</v>
       </c>
       <c r="U36" s="42">
         <v>46287</v>
@@ -5608,10 +5265,10 @@
         <v>34</v>
       </c>
       <c r="S37" t="s">
+        <v>583</v>
+      </c>
+      <c r="T37" t="s">
         <v>584</v>
-      </c>
-      <c r="T37" t="s">
-        <v>585</v>
       </c>
       <c r="U37" s="42">
         <v>46287</v>
@@ -5678,10 +5335,10 @@
         <v>34</v>
       </c>
       <c r="S38" t="s">
+        <v>585</v>
+      </c>
+      <c r="T38" t="s">
         <v>586</v>
-      </c>
-      <c r="T38" t="s">
-        <v>587</v>
       </c>
       <c r="U38" s="42">
         <v>46287</v>
@@ -5748,10 +5405,10 @@
         <v>34</v>
       </c>
       <c r="S39" t="s">
+        <v>587</v>
+      </c>
+      <c r="T39" t="s">
         <v>588</v>
-      </c>
-      <c r="T39" t="s">
-        <v>589</v>
       </c>
       <c r="U39" s="42">
         <v>46287</v>
@@ -5818,7 +5475,7 @@
         <v>34</v>
       </c>
       <c r="S40" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="T40" t="s">
         <v>387</v>
@@ -5888,10 +5545,10 @@
         <v>34</v>
       </c>
       <c r="S41" t="s">
+        <v>590</v>
+      </c>
+      <c r="T41" t="s">
         <v>591</v>
-      </c>
-      <c r="T41" t="s">
-        <v>592</v>
       </c>
       <c r="U41" s="42">
         <v>46287</v>
@@ -5958,10 +5615,10 @@
         <v>34</v>
       </c>
       <c r="S42" t="s">
+        <v>592</v>
+      </c>
+      <c r="T42" t="s">
         <v>593</v>
-      </c>
-      <c r="T42" t="s">
-        <v>594</v>
       </c>
       <c r="U42" s="42">
         <v>46287</v>
@@ -6028,10 +5685,10 @@
         <v>34</v>
       </c>
       <c r="S43" t="s">
+        <v>594</v>
+      </c>
+      <c r="T43" t="s">
         <v>595</v>
-      </c>
-      <c r="T43" t="s">
-        <v>596</v>
       </c>
       <c r="U43" s="42">
         <v>46308</v>
@@ -6098,10 +5755,10 @@
         <v>34</v>
       </c>
       <c r="S44" t="s">
+        <v>596</v>
+      </c>
+      <c r="T44" t="s">
         <v>597</v>
-      </c>
-      <c r="T44" t="s">
-        <v>598</v>
       </c>
       <c r="U44" s="42">
         <v>46308</v>
@@ -6168,10 +5825,10 @@
         <v>34</v>
       </c>
       <c r="S45" t="s">
+        <v>598</v>
+      </c>
+      <c r="T45" t="s">
         <v>599</v>
-      </c>
-      <c r="T45" t="s">
-        <v>600</v>
       </c>
       <c r="U45" s="42">
         <v>46287</v>
@@ -6238,10 +5895,10 @@
         <v>34</v>
       </c>
       <c r="S46" t="s">
+        <v>600</v>
+      </c>
+      <c r="T46" t="s">
         <v>601</v>
-      </c>
-      <c r="T46" t="s">
-        <v>602</v>
       </c>
       <c r="U46" s="42">
         <v>46279</v>
@@ -6308,10 +5965,10 @@
         <v>34</v>
       </c>
       <c r="S47" t="s">
+        <v>602</v>
+      </c>
+      <c r="T47" t="s">
         <v>603</v>
-      </c>
-      <c r="T47" t="s">
-        <v>604</v>
       </c>
       <c r="U47" s="39" t="s">
         <v>342</v>
@@ -6376,10 +6033,10 @@
         <v/>
       </c>
       <c r="S48" t="s">
+        <v>604</v>
+      </c>
+      <c r="T48" t="s">
         <v>605</v>
-      </c>
-      <c r="T48" t="s">
-        <v>606</v>
       </c>
       <c r="U48" s="42">
         <v>46287</v>
@@ -6446,10 +6103,10 @@
         <v>34</v>
       </c>
       <c r="S49" t="s">
+        <v>606</v>
+      </c>
+      <c r="T49" t="s">
         <v>607</v>
-      </c>
-      <c r="T49" t="s">
-        <v>608</v>
       </c>
       <c r="U49" s="42">
         <v>46279</v>
@@ -6516,10 +6173,10 @@
         <v>34</v>
       </c>
       <c r="S50" t="s">
+        <v>608</v>
+      </c>
+      <c r="T50" t="s">
         <v>609</v>
-      </c>
-      <c r="T50" t="s">
-        <v>610</v>
       </c>
       <c r="U50" s="42">
         <v>46287</v>
@@ -6586,10 +6243,10 @@
         <v>34</v>
       </c>
       <c r="S51" t="s">
+        <v>610</v>
+      </c>
+      <c r="T51" t="s">
         <v>611</v>
-      </c>
-      <c r="T51" t="s">
-        <v>612</v>
       </c>
       <c r="U51" s="42">
         <v>46287</v>
@@ -6656,10 +6313,10 @@
         <v>34</v>
       </c>
       <c r="S52" t="s">
+        <v>612</v>
+      </c>
+      <c r="T52" t="s">
         <v>613</v>
-      </c>
-      <c r="T52" t="s">
-        <v>614</v>
       </c>
       <c r="U52" s="42">
         <v>46287</v>
@@ -6726,10 +6383,10 @@
         <v>25</v>
       </c>
       <c r="S53" t="s">
+        <v>615</v>
+      </c>
+      <c r="T53" t="s">
         <v>616</v>
-      </c>
-      <c r="T53" t="s">
-        <v>617</v>
       </c>
       <c r="U53" s="47">
         <v>46293</v>
@@ -6796,10 +6453,10 @@
         <v>25</v>
       </c>
       <c r="S54" t="s">
+        <v>617</v>
+      </c>
+      <c r="T54" t="s">
         <v>618</v>
-      </c>
-      <c r="T54" t="s">
-        <v>619</v>
       </c>
       <c r="U54" s="47">
         <v>46293</v>
@@ -6866,10 +6523,10 @@
         <v>25</v>
       </c>
       <c r="S55" t="s">
+        <v>619</v>
+      </c>
+      <c r="T55" t="s">
         <v>620</v>
-      </c>
-      <c r="T55" t="s">
-        <v>621</v>
       </c>
       <c r="U55" s="47">
         <v>46293</v>
@@ -6936,10 +6593,10 @@
         <v>25</v>
       </c>
       <c r="S56" t="s">
+        <v>621</v>
+      </c>
+      <c r="T56" t="s">
         <v>622</v>
-      </c>
-      <c r="T56" t="s">
-        <v>623</v>
       </c>
       <c r="U56" s="47">
         <v>46293</v>
@@ -7006,10 +6663,10 @@
         <v>25</v>
       </c>
       <c r="S57" t="s">
+        <v>623</v>
+      </c>
+      <c r="T57" t="s">
         <v>624</v>
-      </c>
-      <c r="T57" t="s">
-        <v>625</v>
       </c>
       <c r="U57" s="47">
         <v>46293</v>
@@ -7076,10 +6733,10 @@
         <v>25</v>
       </c>
       <c r="S58" t="s">
+        <v>625</v>
+      </c>
+      <c r="T58" t="s">
         <v>626</v>
-      </c>
-      <c r="T58" t="s">
-        <v>627</v>
       </c>
       <c r="U58" s="47">
         <v>46293</v>
@@ -7146,10 +6803,10 @@
         <v>25</v>
       </c>
       <c r="S59" t="s">
+        <v>627</v>
+      </c>
+      <c r="T59" t="s">
         <v>628</v>
-      </c>
-      <c r="T59" t="s">
-        <v>629</v>
       </c>
       <c r="U59" s="47">
         <v>46293</v>
@@ -7216,10 +6873,10 @@
         <v>25</v>
       </c>
       <c r="S60" t="s">
+        <v>629</v>
+      </c>
+      <c r="T60" t="s">
         <v>630</v>
-      </c>
-      <c r="T60" t="s">
-        <v>631</v>
       </c>
       <c r="U60" s="47">
         <v>46293</v>
@@ -7286,10 +6943,10 @@
         <v>25</v>
       </c>
       <c r="S61" t="s">
+        <v>629</v>
+      </c>
+      <c r="T61" t="s">
         <v>630</v>
-      </c>
-      <c r="T61" t="s">
-        <v>631</v>
       </c>
       <c r="U61" s="47">
         <v>46293</v>
@@ -7356,10 +7013,10 @@
         <v>25</v>
       </c>
       <c r="S62" t="s">
+        <v>631</v>
+      </c>
+      <c r="T62" t="s">
         <v>632</v>
-      </c>
-      <c r="T62" t="s">
-        <v>633</v>
       </c>
       <c r="U62" s="47">
         <v>46293</v>
@@ -7426,7 +7083,7 @@
         <v>21</v>
       </c>
       <c r="S63" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="T63" t="s">
         <v>392</v>
@@ -7496,10 +7153,10 @@
         <v>21</v>
       </c>
       <c r="S64" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="T64" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="U64" t="s">
         <v>146</v>
@@ -7566,7 +7223,7 @@
         <v>21</v>
       </c>
       <c r="S65" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="T65" t="s">
         <v>392</v>
@@ -7636,10 +7293,10 @@
         <v>21</v>
       </c>
       <c r="S66" t="s">
+        <v>794</v>
+      </c>
+      <c r="T66" t="s">
         <v>795</v>
-      </c>
-      <c r="T66" t="s">
-        <v>796</v>
       </c>
       <c r="U66" s="48">
         <v>46322</v>
@@ -7706,10 +7363,10 @@
         <v>21</v>
       </c>
       <c r="S67" t="s">
+        <v>792</v>
+      </c>
+      <c r="T67" t="s">
         <v>793</v>
-      </c>
-      <c r="T67" t="s">
-        <v>794</v>
       </c>
       <c r="U67" s="48">
         <v>46322</v>
@@ -7776,10 +7433,10 @@
         <v>21</v>
       </c>
       <c r="S68" t="s">
+        <v>790</v>
+      </c>
+      <c r="T68" t="s">
         <v>791</v>
-      </c>
-      <c r="T68" t="s">
-        <v>792</v>
       </c>
       <c r="U68" t="s">
         <v>146</v>
@@ -7845,6 +7502,12 @@
         <f t="shared" ca="1" si="2"/>
         <v>21</v>
       </c>
+      <c r="S69" t="s">
+        <v>796</v>
+      </c>
+      <c r="T69" t="s">
+        <v>797</v>
+      </c>
       <c r="U69" t="s">
         <v>146</v>
       </c>
@@ -7910,10 +7573,10 @@
         <v>21</v>
       </c>
       <c r="S70" t="s">
+        <v>788</v>
+      </c>
+      <c r="T70" t="s">
         <v>789</v>
-      </c>
-      <c r="T70" t="s">
-        <v>790</v>
       </c>
       <c r="U70" s="48">
         <v>46315</v>
@@ -7979,16 +7642,22 @@
         <f t="shared" ca="1" si="2"/>
         <v>21</v>
       </c>
+      <c r="S71" t="s">
+        <v>798</v>
+      </c>
+      <c r="T71" t="s">
+        <v>799</v>
+      </c>
       <c r="U71" t="s">
         <v>146</v>
       </c>
       <c r="V71" t="s">
-        <v>515</v>
+        <v>800</v>
       </c>
     </row>
     <row r="72" spans="1:22">
       <c r="A72" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="B72" t="s">
         <v>464</v>
@@ -8003,22 +7672,22 @@
         <v>46287</v>
       </c>
       <c r="F72" t="s">
+        <v>516</v>
+      </c>
+      <c r="G72" t="s">
         <v>517</v>
       </c>
-      <c r="G72" t="s">
+      <c r="H72" t="s">
         <v>518</v>
       </c>
-      <c r="H72" t="s">
+      <c r="I72" t="s">
         <v>519</v>
       </c>
-      <c r="I72" t="s">
+      <c r="J72" t="s">
         <v>520</v>
       </c>
-      <c r="J72" t="s">
+      <c r="K72" t="s">
         <v>521</v>
-      </c>
-      <c r="K72" t="s">
-        <v>522</v>
       </c>
       <c r="L72" t="s">
         <v>468</v>
@@ -8044,21 +7713,21 @@
         <v>21</v>
       </c>
       <c r="S72" t="s">
+        <v>786</v>
+      </c>
+      <c r="T72" t="s">
         <v>787</v>
-      </c>
-      <c r="T72" t="s">
-        <v>788</v>
       </c>
       <c r="U72" t="s">
         <v>146</v>
       </c>
       <c r="V72" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="73" spans="1:22">
       <c r="A73" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B73" t="s">
         <v>464</v>
@@ -8071,22 +7740,22 @@
       </c>
       <c r="E73" s="48"/>
       <c r="F73" t="s">
+        <v>524</v>
+      </c>
+      <c r="G73" t="s">
         <v>525</v>
       </c>
-      <c r="G73" t="s">
+      <c r="H73" t="s">
         <v>526</v>
       </c>
-      <c r="H73" t="s">
+      <c r="I73" t="s">
         <v>527</v>
       </c>
-      <c r="I73" t="s">
+      <c r="J73" t="s">
         <v>528</v>
       </c>
-      <c r="J73" t="s">
+      <c r="K73" t="s">
         <v>529</v>
-      </c>
-      <c r="K73" t="s">
-        <v>530</v>
       </c>
       <c r="L73" t="s">
         <v>468</v>
@@ -8112,21 +7781,21 @@
         <v/>
       </c>
       <c r="S73" t="s">
+        <v>784</v>
+      </c>
+      <c r="T73" t="s">
         <v>785</v>
-      </c>
-      <c r="T73" t="s">
-        <v>786</v>
       </c>
       <c r="U73" t="s">
         <v>146</v>
       </c>
       <c r="V73" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
     </row>
     <row r="74" spans="1:22">
       <c r="A74" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B74" t="s">
         <v>464</v>
@@ -8139,22 +7808,22 @@
       </c>
       <c r="E74" s="48"/>
       <c r="F74" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="G74" t="s">
+        <v>531</v>
+      </c>
+      <c r="H74" t="s">
+        <v>526</v>
+      </c>
+      <c r="I74" t="s">
         <v>532</v>
       </c>
-      <c r="H74" t="s">
-        <v>527</v>
-      </c>
-      <c r="I74" t="s">
+      <c r="J74" t="s">
         <v>533</v>
       </c>
-      <c r="J74" t="s">
+      <c r="K74" t="s">
         <v>534</v>
-      </c>
-      <c r="K74" t="s">
-        <v>535</v>
       </c>
       <c r="L74" t="s">
         <v>468</v>
@@ -8180,21 +7849,21 @@
         <v/>
       </c>
       <c r="S74" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="T74" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="U74" t="s">
         <v>146</v>
       </c>
       <c r="V74" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
     </row>
     <row r="75" spans="1:22">
       <c r="A75" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="B75" t="s">
         <v>464</v>
@@ -8209,22 +7878,22 @@
         <v>46287</v>
       </c>
       <c r="F75" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="G75" t="s">
+        <v>536</v>
+      </c>
+      <c r="H75" t="s">
+        <v>526</v>
+      </c>
+      <c r="I75" t="s">
         <v>537</v>
       </c>
-      <c r="H75" t="s">
-        <v>527</v>
-      </c>
-      <c r="I75" t="s">
+      <c r="J75" t="s">
         <v>538</v>
       </c>
-      <c r="J75" t="s">
+      <c r="K75" t="s">
         <v>539</v>
-      </c>
-      <c r="K75" t="s">
-        <v>540</v>
       </c>
       <c r="L75" t="s">
         <v>468</v>
@@ -8250,21 +7919,21 @@
         <v>21</v>
       </c>
       <c r="S75" t="s">
+        <v>781</v>
+      </c>
+      <c r="T75" t="s">
         <v>782</v>
-      </c>
-      <c r="T75" t="s">
-        <v>783</v>
       </c>
       <c r="U75" t="s">
         <v>146</v>
       </c>
       <c r="V75" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
     </row>
     <row r="76" spans="1:22">
       <c r="A76" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="B76" t="s">
         <v>464</v>
@@ -8277,22 +7946,22 @@
       </c>
       <c r="E76" s="48"/>
       <c r="F76" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="G76" t="s">
+        <v>542</v>
+      </c>
+      <c r="H76" t="s">
+        <v>526</v>
+      </c>
+      <c r="I76" t="s">
         <v>543</v>
       </c>
-      <c r="H76" t="s">
-        <v>527</v>
-      </c>
-      <c r="I76" t="s">
+      <c r="J76" t="s">
         <v>544</v>
       </c>
-      <c r="J76" t="s">
+      <c r="K76" t="s">
         <v>545</v>
-      </c>
-      <c r="K76" t="s">
-        <v>546</v>
       </c>
       <c r="L76" t="s">
         <v>468</v>
@@ -8318,21 +7987,21 @@
         <v/>
       </c>
       <c r="S76" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="T76" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="U76" t="s">
         <v>146</v>
       </c>
       <c r="V76" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
     </row>
     <row r="77" spans="1:22">
       <c r="A77" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="B77" t="s">
         <v>464</v>
@@ -8345,22 +8014,22 @@
       </c>
       <c r="E77" s="48"/>
       <c r="F77" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="G77" t="s">
+        <v>547</v>
+      </c>
+      <c r="H77" t="s">
+        <v>526</v>
+      </c>
+      <c r="I77" t="s">
         <v>548</v>
       </c>
-      <c r="H77" t="s">
-        <v>527</v>
-      </c>
-      <c r="I77" t="s">
+      <c r="J77" t="s">
         <v>549</v>
       </c>
-      <c r="J77" t="s">
+      <c r="K77" t="s">
         <v>550</v>
-      </c>
-      <c r="K77" t="s">
-        <v>551</v>
       </c>
       <c r="L77" t="s">
         <v>468</v>
@@ -8386,21 +8055,21 @@
         <v/>
       </c>
       <c r="S77" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="T77" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="U77" t="s">
         <v>146</v>
       </c>
       <c r="V77" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
     </row>
     <row r="78" spans="1:22">
       <c r="A78" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="B78" t="s">
         <v>464</v>
@@ -8413,22 +8082,22 @@
       </c>
       <c r="E78" s="48"/>
       <c r="F78" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="G78" t="s">
+        <v>552</v>
+      </c>
+      <c r="H78" t="s">
+        <v>526</v>
+      </c>
+      <c r="I78" t="s">
         <v>553</v>
       </c>
-      <c r="H78" t="s">
-        <v>527</v>
-      </c>
-      <c r="I78" t="s">
+      <c r="J78" t="s">
         <v>554</v>
       </c>
-      <c r="J78" t="s">
+      <c r="K78" t="s">
         <v>555</v>
-      </c>
-      <c r="K78" t="s">
-        <v>556</v>
       </c>
       <c r="L78" t="s">
         <v>468</v>
@@ -8454,21 +8123,21 @@
         <v/>
       </c>
       <c r="S78" t="s">
+        <v>777</v>
+      </c>
+      <c r="T78" t="s">
         <v>778</v>
-      </c>
-      <c r="T78" t="s">
-        <v>779</v>
       </c>
       <c r="U78" t="s">
         <v>146</v>
       </c>
       <c r="V78" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
     </row>
     <row r="79" spans="1:22">
       <c r="A79" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="B79" t="s">
         <v>464</v>
@@ -8483,22 +8152,22 @@
         <v>46287</v>
       </c>
       <c r="F79" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="G79" t="s">
+        <v>557</v>
+      </c>
+      <c r="H79" t="s">
+        <v>526</v>
+      </c>
+      <c r="I79" t="s">
         <v>558</v>
       </c>
-      <c r="H79" t="s">
-        <v>527</v>
-      </c>
-      <c r="I79" t="s">
+      <c r="J79" t="s">
         <v>559</v>
       </c>
-      <c r="J79" t="s">
+      <c r="K79" t="s">
         <v>560</v>
-      </c>
-      <c r="K79" t="s">
-        <v>561</v>
       </c>
       <c r="L79" t="s">
         <v>468</v>
@@ -8524,21 +8193,21 @@
         <v>21</v>
       </c>
       <c r="S79" t="s">
+        <v>775</v>
+      </c>
+      <c r="T79" t="s">
         <v>776</v>
-      </c>
-      <c r="T79" t="s">
-        <v>777</v>
       </c>
       <c r="U79" t="s">
         <v>146</v>
       </c>
       <c r="V79" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="80" spans="1:22">
       <c r="A80" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="B80" t="s">
         <v>464</v>
@@ -8553,22 +8222,22 @@
         <v>46287</v>
       </c>
       <c r="F80" t="s">
+        <v>563</v>
+      </c>
+      <c r="G80" t="s">
         <v>564</v>
       </c>
-      <c r="G80" t="s">
+      <c r="H80" t="s">
         <v>565</v>
       </c>
-      <c r="H80" t="s">
+      <c r="I80" t="s">
         <v>566</v>
       </c>
-      <c r="I80" t="s">
+      <c r="J80" t="s">
         <v>567</v>
       </c>
-      <c r="J80" t="s">
+      <c r="K80" t="s">
         <v>568</v>
-      </c>
-      <c r="K80" t="s">
-        <v>569</v>
       </c>
       <c r="L80" t="s">
         <v>468</v>
@@ -8594,21 +8263,21 @@
         <v>21</v>
       </c>
       <c r="S80" t="s">
+        <v>772</v>
+      </c>
+      <c r="T80" t="s">
         <v>773</v>
       </c>
-      <c r="T80" t="s">
+      <c r="U80" s="48" t="s">
         <v>774</v>
       </c>
-      <c r="U80" s="48" t="s">
-        <v>775</v>
-      </c>
       <c r="V80" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
     </row>
     <row r="81" spans="1:22">
       <c r="A81" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="B81" t="s">
         <v>464</v>
@@ -8626,19 +8295,19 @@
         <v>264</v>
       </c>
       <c r="G81" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="H81" t="s">
         <v>504</v>
       </c>
       <c r="I81" t="s">
+        <v>572</v>
+      </c>
+      <c r="J81" t="s">
         <v>573</v>
       </c>
-      <c r="J81" t="s">
+      <c r="K81" t="s">
         <v>574</v>
-      </c>
-      <c r="K81" t="s">
-        <v>575</v>
       </c>
       <c r="L81" t="s">
         <v>468</v>
@@ -8664,21 +8333,21 @@
         <v>21</v>
       </c>
       <c r="S81" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="T81" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="U81" s="48">
         <v>46322</v>
       </c>
       <c r="V81" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
     </row>
     <row r="82" spans="1:22">
       <c r="A82" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="B82" t="s">
         <v>464</v>
@@ -8693,7 +8362,7 @@
         <v>46287</v>
       </c>
       <c r="F82" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="G82" t="s">
         <v>146</v>
@@ -8702,13 +8371,13 @@
         <v>138</v>
       </c>
       <c r="I82" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="J82" t="s">
         <v>513</v>
       </c>
       <c r="K82" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="L82" t="s">
         <v>468</v>
@@ -8734,21 +8403,21 @@
         <v>21</v>
       </c>
       <c r="S82" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="T82" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="U82" t="s">
         <v>146</v>
       </c>
       <c r="V82" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="83" spans="1:22">
       <c r="A83" s="10" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="B83" s="11" t="s">
         <v>215</v>
@@ -8763,10 +8432,10 @@
         <v>46295</v>
       </c>
       <c r="F83" s="43" t="s">
+        <v>634</v>
+      </c>
+      <c r="G83" s="43" t="s">
         <v>635</v>
-      </c>
-      <c r="G83" s="43" t="s">
-        <v>636</v>
       </c>
       <c r="H83" s="11" t="s">
         <v>408</v>
@@ -8775,13 +8444,13 @@
         <v>426</v>
       </c>
       <c r="J83" s="11" t="s">
+        <v>636</v>
+      </c>
+      <c r="K83" s="11" t="s">
         <v>637</v>
       </c>
-      <c r="K83" s="11" t="s">
+      <c r="L83" s="11" t="s">
         <v>638</v>
-      </c>
-      <c r="L83" s="11" t="s">
-        <v>639</v>
       </c>
       <c r="M83" s="11" t="s">
         <v>45</v>
@@ -8804,19 +8473,19 @@
         <v>13</v>
       </c>
       <c r="S83" s="43" t="s">
+        <v>651</v>
+      </c>
+      <c r="T83" s="43" t="s">
         <v>652</v>
-      </c>
-      <c r="T83" s="43" t="s">
-        <v>653</v>
       </c>
       <c r="U83" s="7"/>
       <c r="V83" s="41" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="84" spans="1:22">
       <c r="A84" s="10" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="B84" s="11" t="s">
         <v>215</v>
@@ -8831,7 +8500,7 @@
         <v>46295</v>
       </c>
       <c r="F84" s="43" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="G84" s="43" t="s">
         <v>445</v>
@@ -8843,13 +8512,13 @@
         <v>446</v>
       </c>
       <c r="J84" s="11" t="s">
+        <v>641</v>
+      </c>
+      <c r="K84" s="11" t="s">
         <v>642</v>
       </c>
-      <c r="K84" s="11" t="s">
-        <v>643</v>
-      </c>
       <c r="L84" s="11" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="M84" s="11" t="s">
         <v>45</v>
@@ -8872,19 +8541,19 @@
         <v>13</v>
       </c>
       <c r="S84" s="43" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="T84" s="43" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="U84" s="7"/>
       <c r="V84" s="41" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="85" spans="1:22">
       <c r="A85" s="10" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B85" s="11" t="s">
         <v>215</v>
@@ -8899,7 +8568,7 @@
         <v>46295</v>
       </c>
       <c r="F85" s="43" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="G85" s="43" t="s">
         <v>440</v>
@@ -8911,13 +8580,13 @@
         <v>441</v>
       </c>
       <c r="J85" s="11" t="s">
+        <v>644</v>
+      </c>
+      <c r="K85" s="11" t="s">
         <v>645</v>
       </c>
-      <c r="K85" s="11" t="s">
-        <v>646</v>
-      </c>
       <c r="L85" s="11" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="M85" s="11" t="s">
         <v>45</v>
@@ -8940,21 +8609,21 @@
         <v>13</v>
       </c>
       <c r="S85" s="43" t="s">
+        <v>655</v>
+      </c>
+      <c r="T85" s="43" t="s">
         <v>656</v>
-      </c>
-      <c r="T85" s="43" t="s">
-        <v>657</v>
       </c>
       <c r="U85" s="7">
         <v>46308</v>
       </c>
       <c r="V85" s="41" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="86" spans="1:22">
       <c r="A86" s="10" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="B86" s="11" t="s">
         <v>215</v>
@@ -8969,25 +8638,25 @@
         <v>46295</v>
       </c>
       <c r="F86" s="43" t="s">
+        <v>647</v>
+      </c>
+      <c r="G86" s="43" t="s">
         <v>648</v>
-      </c>
-      <c r="G86" s="43" t="s">
-        <v>649</v>
       </c>
       <c r="H86" s="11" t="s">
         <v>408</v>
       </c>
       <c r="I86" s="11" t="s">
+        <v>649</v>
+      </c>
+      <c r="J86" s="11" t="s">
+        <v>657</v>
+      </c>
+      <c r="K86" s="11" t="s">
+        <v>658</v>
+      </c>
+      <c r="L86" s="11" t="s">
         <v>650</v>
-      </c>
-      <c r="J86" s="11" t="s">
-        <v>658</v>
-      </c>
-      <c r="K86" s="11" t="s">
-        <v>659</v>
-      </c>
-      <c r="L86" s="11" t="s">
-        <v>651</v>
       </c>
       <c r="M86" s="11" t="s">
         <v>45</v>
@@ -9010,24 +8679,24 @@
         <v>13</v>
       </c>
       <c r="S86" s="43" t="s">
+        <v>766</v>
+      </c>
+      <c r="T86" s="43" t="s">
         <v>767</v>
-      </c>
-      <c r="T86" s="43" t="s">
-        <v>768</v>
       </c>
       <c r="U86" s="7" t="s">
         <v>146</v>
       </c>
       <c r="V86" s="41" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
     </row>
     <row r="87" spans="1:22">
       <c r="A87" s="10" t="s">
+        <v>660</v>
+      </c>
+      <c r="B87" s="11" t="s">
         <v>661</v>
-      </c>
-      <c r="B87" s="11" t="s">
-        <v>662</v>
       </c>
       <c r="C87" s="12">
         <v>46308</v>
@@ -9042,22 +8711,22 @@
         <v>264</v>
       </c>
       <c r="G87" s="43" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="H87" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="I87" s="57">
+      <c r="I87" s="50">
         <v>0.54</v>
       </c>
       <c r="J87" s="11" t="s">
+        <v>663</v>
+      </c>
+      <c r="K87" s="11" t="s">
         <v>664</v>
       </c>
-      <c r="K87" s="11" t="s">
+      <c r="L87" s="11" t="s">
         <v>665</v>
-      </c>
-      <c r="L87" s="11" t="s">
-        <v>666</v>
       </c>
       <c r="M87" s="11" t="s">
         <v>45</v>
@@ -9082,18 +8751,18 @@
       <c r="S87" s="43"/>
       <c r="T87" s="43"/>
       <c r="U87" s="7" t="s">
+        <v>666</v>
+      </c>
+      <c r="V87" s="41" t="s">
         <v>667</v>
-      </c>
-      <c r="V87" s="41" t="s">
-        <v>668</v>
       </c>
     </row>
     <row r="88" spans="1:22">
       <c r="A88" s="10" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="B88" s="11" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C88" s="12">
         <v>46308</v>
@@ -9108,22 +8777,22 @@
         <v>264</v>
       </c>
       <c r="G88" s="43" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="H88" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="I88" s="57">
+      <c r="I88" s="50">
         <v>0.45</v>
       </c>
       <c r="J88" s="11" t="s">
         <v>304</v>
       </c>
       <c r="K88" s="11" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="L88" s="11" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="M88" s="11" t="s">
         <v>45</v>
@@ -9148,18 +8817,18 @@
       <c r="S88" s="43"/>
       <c r="T88" s="43"/>
       <c r="U88" s="7" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="V88" s="41" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
     </row>
     <row r="89" spans="1:22">
       <c r="A89" s="10" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B89" s="11" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C89" s="12">
         <v>46308</v>
@@ -9174,22 +8843,22 @@
         <v>270</v>
       </c>
       <c r="G89" s="43" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="H89" s="11" t="s">
         <v>52</v>
       </c>
       <c r="I89" s="11" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="J89" s="11" t="s">
         <v>477</v>
       </c>
       <c r="K89" s="11" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="L89" s="11" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="M89" s="11" t="s">
         <v>41</v>
@@ -9214,18 +8883,18 @@
       <c r="S89" s="43"/>
       <c r="T89" s="43"/>
       <c r="U89" s="7" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="V89" s="41" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
     </row>
     <row r="90" spans="1:22">
       <c r="A90" s="10" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="B90" s="11" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C90" s="12">
         <v>46308</v>
@@ -9240,22 +8909,22 @@
         <v>264</v>
       </c>
       <c r="G90" s="43" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="H90" s="11" t="s">
         <v>61</v>
       </c>
       <c r="I90" s="11" t="s">
+        <v>679</v>
+      </c>
+      <c r="J90" s="11" t="s">
         <v>680</v>
       </c>
-      <c r="J90" s="11" t="s">
+      <c r="K90" s="11" t="s">
         <v>681</v>
       </c>
-      <c r="K90" s="11" t="s">
-        <v>682</v>
-      </c>
       <c r="L90" s="11" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="M90" s="11" t="s">
         <v>45</v>
@@ -9280,18 +8949,18 @@
       <c r="S90" s="43"/>
       <c r="T90" s="43"/>
       <c r="U90" s="7" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="V90" s="41" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="91" spans="1:22">
       <c r="A91" s="10" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="B91" s="11" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C91" s="12">
         <v>46308</v>
@@ -9306,22 +8975,22 @@
         <v>264</v>
       </c>
       <c r="G91" s="43" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="H91" s="11" t="s">
         <v>60</v>
       </c>
       <c r="I91" s="11" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="J91" s="11" t="s">
+        <v>685</v>
+      </c>
+      <c r="K91" s="11" t="s">
         <v>686</v>
       </c>
-      <c r="K91" s="11" t="s">
-        <v>687</v>
-      </c>
       <c r="L91" s="11" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="M91" s="11" t="s">
         <v>41</v>
@@ -9346,16 +9015,16 @@
       <c r="S91" s="43"/>
       <c r="T91" s="43"/>
       <c r="U91" s="7" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="V91" s="41"/>
     </row>
     <row r="92" spans="1:22">
       <c r="A92" s="10" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="B92" s="11" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C92" s="12">
         <v>46308</v>
@@ -9367,25 +9036,25 @@
         <v>46308</v>
       </c>
       <c r="F92" s="43" t="s">
+        <v>688</v>
+      </c>
+      <c r="G92" s="43" t="s">
         <v>689</v>
       </c>
-      <c r="G92" s="43" t="s">
+      <c r="H92" s="11" t="s">
         <v>690</v>
       </c>
-      <c r="H92" s="11" t="s">
+      <c r="I92" s="11" t="s">
         <v>691</v>
       </c>
-      <c r="I92" s="11" t="s">
+      <c r="J92" s="11" t="s">
         <v>692</v>
       </c>
-      <c r="J92" s="11" t="s">
+      <c r="K92" s="11" t="s">
         <v>693</v>
       </c>
-      <c r="K92" s="11" t="s">
-        <v>694</v>
-      </c>
       <c r="L92" s="11" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="M92" s="11" t="s">
         <v>41</v>
@@ -9410,18 +9079,18 @@
       <c r="S92" s="43"/>
       <c r="T92" s="43"/>
       <c r="U92" s="7" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="V92" s="41" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="93" spans="1:22">
       <c r="A93" s="10" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="B93" s="11" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C93" s="12">
         <v>46308</v>
@@ -9433,25 +9102,25 @@
         <v>46308</v>
       </c>
       <c r="F93" s="43" t="s">
+        <v>696</v>
+      </c>
+      <c r="G93" s="43" t="s">
         <v>697</v>
-      </c>
-      <c r="G93" s="43" t="s">
-        <v>698</v>
       </c>
       <c r="H93" s="11" t="s">
         <v>62</v>
       </c>
       <c r="I93" s="11" t="s">
+        <v>698</v>
+      </c>
+      <c r="J93" s="11" t="s">
         <v>699</v>
       </c>
-      <c r="J93" s="11" t="s">
+      <c r="K93" s="11" t="s">
         <v>700</v>
       </c>
-      <c r="K93" s="11" t="s">
-        <v>701</v>
-      </c>
       <c r="L93" s="11" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="M93" s="11" t="s">
         <v>45</v>
@@ -9476,18 +9145,18 @@
       <c r="S93" s="43"/>
       <c r="T93" s="43"/>
       <c r="U93" s="7" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="V93" s="41" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
     <row r="94" spans="1:22">
       <c r="A94" s="10" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="B94" s="11" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C94" s="12">
         <v>46308</v>
@@ -9502,22 +9171,22 @@
         <v>272</v>
       </c>
       <c r="G94" s="43" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="H94" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="I94" s="57">
+      <c r="I94" s="50">
         <v>1.1000000000000001</v>
       </c>
       <c r="J94" s="11" t="s">
+        <v>704</v>
+      </c>
+      <c r="K94" s="11" t="s">
         <v>705</v>
       </c>
-      <c r="K94" s="11" t="s">
-        <v>706</v>
-      </c>
       <c r="L94" s="11" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="M94" s="11" t="s">
         <v>45</v>
@@ -9542,18 +9211,18 @@
       <c r="S94" s="43"/>
       <c r="T94" s="43"/>
       <c r="U94" s="7" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="V94" s="41" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
     </row>
     <row r="95" spans="1:22">
       <c r="A95" s="10" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B95" s="11" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C95" s="12">
         <v>46308</v>
@@ -9568,22 +9237,22 @@
         <v>272</v>
       </c>
       <c r="G95" s="43" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="H95" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="I95" s="57">
+      <c r="I95" s="50">
         <v>0.9</v>
       </c>
       <c r="J95" s="11" t="s">
+        <v>709</v>
+      </c>
+      <c r="K95" s="11" t="s">
         <v>710</v>
       </c>
-      <c r="K95" s="11" t="s">
+      <c r="L95" s="11" t="s">
         <v>711</v>
-      </c>
-      <c r="L95" s="11" t="s">
-        <v>712</v>
       </c>
       <c r="M95" s="11" t="s">
         <v>41</v>
@@ -9608,18 +9277,18 @@
       <c r="S95" s="43"/>
       <c r="T95" s="43"/>
       <c r="U95" s="7" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="V95" s="41" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
     </row>
     <row r="96" spans="1:22">
       <c r="A96" s="10" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="B96" s="11" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C96" s="12">
         <v>46308</v>
@@ -9631,25 +9300,25 @@
         <v>46308</v>
       </c>
       <c r="F96" s="43" t="s">
+        <v>714</v>
+      </c>
+      <c r="G96" s="43" t="s">
         <v>715</v>
-      </c>
-      <c r="G96" s="43" t="s">
-        <v>716</v>
       </c>
       <c r="H96" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="I96" s="57">
+      <c r="I96" s="50">
         <v>2.6</v>
       </c>
       <c r="J96" s="11" t="s">
+        <v>716</v>
+      </c>
+      <c r="K96" s="11" t="s">
         <v>717</v>
       </c>
-      <c r="K96" s="11" t="s">
-        <v>718</v>
-      </c>
       <c r="L96" s="11" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="M96" s="11" t="s">
         <v>49</v>
@@ -9674,18 +9343,18 @@
       <c r="S96" s="43"/>
       <c r="T96" s="43"/>
       <c r="U96" s="7" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="V96" s="41" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
     </row>
     <row r="97" spans="1:22">
       <c r="A97" s="10" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="B97" s="11" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C97" s="12">
         <v>46308</v>
@@ -9697,25 +9366,25 @@
         <v>46308</v>
       </c>
       <c r="F97" s="43" t="s">
+        <v>720</v>
+      </c>
+      <c r="G97" s="43" t="s">
         <v>721</v>
-      </c>
-      <c r="G97" s="43" t="s">
-        <v>722</v>
       </c>
       <c r="H97" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="I97" s="57">
+      <c r="I97" s="50">
         <v>1.6</v>
       </c>
       <c r="J97" s="11" t="s">
+        <v>722</v>
+      </c>
+      <c r="K97" s="11" t="s">
         <v>723</v>
       </c>
-      <c r="K97" s="11" t="s">
-        <v>724</v>
-      </c>
       <c r="L97" s="11" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="M97" s="11" t="s">
         <v>49</v>
@@ -9740,18 +9409,18 @@
       <c r="S97" s="43"/>
       <c r="T97" s="43"/>
       <c r="U97" s="7" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="V97" s="41" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
     </row>
     <row r="98" spans="1:22">
       <c r="A98" s="10" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="B98" s="11" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C98" s="12">
         <v>46308</v>
@@ -9763,25 +9432,25 @@
         <v>46308</v>
       </c>
       <c r="F98" s="43" t="s">
+        <v>726</v>
+      </c>
+      <c r="G98" s="43" t="s">
         <v>727</v>
-      </c>
-      <c r="G98" s="43" t="s">
-        <v>728</v>
       </c>
       <c r="H98" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="I98" s="57">
+      <c r="I98" s="50">
         <v>1.2</v>
       </c>
       <c r="J98" s="11" t="s">
+        <v>728</v>
+      </c>
+      <c r="K98" s="11" t="s">
         <v>729</v>
       </c>
-      <c r="K98" s="11" t="s">
-        <v>730</v>
-      </c>
       <c r="L98" s="11" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="M98" s="11" t="s">
         <v>49</v>
@@ -9806,18 +9475,18 @@
       <c r="S98" s="43"/>
       <c r="T98" s="43"/>
       <c r="U98" s="7" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="V98" s="41" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
     </row>
     <row r="99" spans="1:22">
       <c r="A99" s="10" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="B99" s="11" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C99" s="12">
         <v>46308</v>
@@ -9829,25 +9498,25 @@
         <v>46308</v>
       </c>
       <c r="F99" s="43" t="s">
+        <v>732</v>
+      </c>
+      <c r="G99" s="43" t="s">
         <v>733</v>
-      </c>
-      <c r="G99" s="43" t="s">
-        <v>734</v>
       </c>
       <c r="H99" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="I99" s="57">
+      <c r="I99" s="50">
         <v>1.2</v>
       </c>
       <c r="J99" s="11" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="K99" s="11" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="L99" s="11" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="M99" s="11" t="s">
         <v>49</v>
@@ -9872,18 +9541,18 @@
       <c r="S99" s="43"/>
       <c r="T99" s="43"/>
       <c r="U99" s="7" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="V99" s="41" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
     </row>
     <row r="100" spans="1:22">
       <c r="A100" s="10" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="B100" s="11" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C100" s="12">
         <v>46308</v>
@@ -9895,25 +9564,25 @@
         <v>46308</v>
       </c>
       <c r="F100" s="43" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="G100" s="43" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="H100" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="I100" s="57">
+      <c r="I100" s="50">
         <v>1.5</v>
       </c>
       <c r="J100" s="11" t="s">
+        <v>738</v>
+      </c>
+      <c r="K100" s="11" t="s">
         <v>739</v>
       </c>
-      <c r="K100" s="11" t="s">
-        <v>740</v>
-      </c>
       <c r="L100" s="11" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="M100" s="11" t="s">
         <v>49</v>
@@ -9938,18 +9607,18 @@
       <c r="S100" s="43"/>
       <c r="T100" s="43"/>
       <c r="U100" s="7" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="V100" s="41" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="101" spans="1:22">
       <c r="A101" s="10" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="B101" s="11" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C101" s="12">
         <v>46308</v>
@@ -9961,7 +9630,7 @@
         <v>46308</v>
       </c>
       <c r="F101" s="43" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="G101" s="43" t="s">
         <v>116</v>
@@ -9969,17 +9638,17 @@
       <c r="H101" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="I101" s="57">
+      <c r="I101" s="50">
         <v>1.32</v>
       </c>
       <c r="J101" s="11" t="s">
+        <v>743</v>
+      </c>
+      <c r="K101" s="11" t="s">
         <v>744</v>
       </c>
-      <c r="K101" s="11" t="s">
-        <v>745</v>
-      </c>
       <c r="L101" s="11" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="M101" s="11" t="s">
         <v>49</v>
@@ -10004,18 +9673,18 @@
       <c r="S101" s="43"/>
       <c r="T101" s="43"/>
       <c r="U101" s="7" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="V101" s="41" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
     </row>
     <row r="102" spans="1:22">
       <c r="A102" s="10" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="B102" s="11" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C102" s="12">
         <v>46308</v>
@@ -10035,17 +9704,17 @@
       <c r="H102" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="I102" s="58">
+      <c r="I102" s="51">
         <v>40</v>
       </c>
       <c r="J102" s="11" t="s">
+        <v>747</v>
+      </c>
+      <c r="K102" s="11" t="s">
         <v>748</v>
       </c>
-      <c r="K102" s="11" t="s">
-        <v>749</v>
-      </c>
       <c r="L102" s="11" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="M102" s="11" t="s">
         <v>49</v>
@@ -10070,18 +9739,18 @@
       <c r="S102" s="43"/>
       <c r="T102" s="43"/>
       <c r="U102" s="7" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="V102" s="41" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
     </row>
     <row r="103" spans="1:22">
       <c r="A103" s="10" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="B103" s="11" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C103" s="12">
         <v>46308</v>
@@ -10101,17 +9770,17 @@
       <c r="H103" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="I103" s="58">
+      <c r="I103" s="51">
         <v>20</v>
       </c>
       <c r="J103" s="11" t="s">
+        <v>751</v>
+      </c>
+      <c r="K103" s="11" t="s">
         <v>752</v>
       </c>
-      <c r="K103" s="11" t="s">
-        <v>753</v>
-      </c>
       <c r="L103" s="11" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="M103" s="11" t="s">
         <v>49</v>
@@ -10136,18 +9805,18 @@
       <c r="S103" s="43"/>
       <c r="T103" s="43"/>
       <c r="U103" s="7" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="V103" s="41" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
     </row>
     <row r="104" spans="1:22">
       <c r="A104" s="10" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="B104" s="11" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="C104" s="12">
         <v>46308</v>
@@ -10159,25 +9828,25 @@
         <v>46308</v>
       </c>
       <c r="F104" s="43" t="s">
+        <v>755</v>
+      </c>
+      <c r="G104" s="43" t="s">
         <v>756</v>
       </c>
-      <c r="G104" s="43" t="s">
+      <c r="H104" s="11" t="s">
         <v>757</v>
       </c>
-      <c r="H104" s="11" t="s">
+      <c r="I104" s="11" t="s">
         <v>758</v>
       </c>
-      <c r="I104" s="11" t="s">
+      <c r="J104" s="11" t="s">
         <v>759</v>
       </c>
-      <c r="J104" s="11" t="s">
+      <c r="K104" s="11" t="s">
         <v>760</v>
       </c>
-      <c r="K104" s="11" t="s">
-        <v>761</v>
-      </c>
       <c r="L104" s="11" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="M104" s="11" t="s">
         <v>41</v>
@@ -10202,10 +9871,10 @@
       <c r="S104" s="43"/>
       <c r="T104" s="43"/>
       <c r="U104" s="7" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="V104" s="41" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="105" spans="1:22">
@@ -13337,25 +13006,25 @@
     <mergeCell ref="A8:V8"/>
   </mergeCells>
   <conditionalFormatting sqref="P11:P208">
-    <cfRule type="expression" dxfId="41" priority="1">
+    <cfRule type="expression" dxfId="6" priority="1">
       <formula>P11="RECOMENDADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="40" priority="2">
+    <cfRule type="expression" dxfId="5" priority="2">
       <formula>P11="APROVADA - AGUARDANDO EXECUÇÃO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="39" priority="3">
+    <cfRule type="expression" dxfId="4" priority="3">
       <formula>P11="EXECUTADA - EM MATURAÇÃO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="38" priority="4">
+    <cfRule type="expression" dxfId="3" priority="4">
       <formula>P11="EXECUTADA - AVALIADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="37" priority="5">
+    <cfRule type="expression" dxfId="2" priority="5">
       <formula>P11="APROVADA - NÃO EXECUTADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="36" priority="6">
+    <cfRule type="expression" dxfId="1" priority="6">
       <formula>P11="REJEITADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="35" priority="7">
+    <cfRule type="expression" dxfId="0" priority="7">
       <formula>LEFT(P11,9)="BLOQUEADA"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13410,16 +13079,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.95" customHeight="1">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="57" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
+      <c r="B1" s="57"/>
+      <c r="C1" s="57"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="57"/>
+      <c r="F1" s="57"/>
+      <c r="G1" s="57"/>
+      <c r="H1" s="57"/>
     </row>
     <row r="3" spans="1:8" ht="15">
       <c r="A3" s="30" t="s">
@@ -13538,16 +13207,16 @@
       </c>
     </row>
     <row r="18" spans="1:8" ht="15">
-      <c r="A18" s="56" t="s">
+      <c r="A18" s="58" t="s">
         <v>64</v>
       </c>
-      <c r="B18" s="56"/>
-      <c r="C18" s="56"/>
-      <c r="D18" s="56"/>
-      <c r="E18" s="56"/>
-      <c r="F18" s="56"/>
-      <c r="G18" s="56"/>
-      <c r="H18" s="56"/>
+      <c r="B18" s="58"/>
+      <c r="C18" s="58"/>
+      <c r="D18" s="58"/>
+      <c r="E18" s="58"/>
+      <c r="F18" s="58"/>
+      <c r="G18" s="58"/>
+      <c r="H18" s="58"/>
     </row>
     <row r="19" spans="1:8" ht="29.25">
       <c r="A19" s="31" t="s">

</xml_diff>

<commit_message>
[19/10] EC-021 conferida por print; Registro com linha 105 (99 entradas)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1558" uniqueCount="801">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1573" uniqueCount="808">
   <si>
     <t>REGISTRO DE ALTERAÇÕES — AMAZON ADS | WINNET METAIS</t>
   </si>
@@ -2436,6 +2436,27 @@
   </si>
   <si>
     <t>grupo recebe a exata "lixo banheiro" (O7-007)</t>
+  </si>
+  <si>
+    <t>EC-021</t>
+  </si>
+  <si>
+    <t>6B Lixeiras banheiro-O4 25/08</t>
+  </si>
+  <si>
+    <t>exata "lixeira inox para pia de cozinha" (lance 1,50)</t>
+  </si>
+  <si>
+    <t>Ativa, R$ 1,50</t>
+  </si>
+  <si>
+    <t>Gatilho O6-008 disparou: vitalício 32 cliques / R$ 45,69 / 0 venda (régua 15). Termo é de pia de cozinha; a 6B anuncia lixeiras de banheiro. A Geral também gastou 13 cli/30d nele sem venda.</t>
+  </si>
+  <si>
+    <t>ciclos/Monitoramento-19-10.md + relatorios/amazon/monitoramento-19-10/6b_palavras_vitalicio_19-10.csv</t>
+  </si>
+  <si>
+    <t>Alternativa do contrato O6-008: reduzir para 1,20 em vez de pausar. A frase "pia de cozinha" (2 cli / 1,87) fica. Não negativar na Geral por ora (termo próximo converteu L2025-T).</t>
   </si>
 </sst>
 </file>
@@ -3295,15 +3316,15 @@
     <row r="6" spans="1:22" ht="26.1" customHeight="1">
       <c r="A6" s="2">
         <f>COUNTIF(A11:A208,"&lt;&gt;")</f>
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B6" s="3">
         <f>COUNTIF(N11:N208,"SIM")</f>
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C6" s="3">
         <f>COUNTIF(O11:O208,"SIM")</f>
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D6" s="3">
         <f>COUNTIF(P11:P208,"BLOQUEADA*")</f>
@@ -3311,7 +3332,7 @@
       </c>
       <c r="E6" s="3">
         <f>COUNTIF(P11:P208,"EXECUTADA - EM MATURAÇÃO")</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F6" s="4">
         <f>COUNTIF(P11:P208,"EXECUTADA - AVALIADA")</f>
@@ -3480,7 +3501,7 @@
       </c>
       <c r="R11" s="17">
         <f t="shared" ref="R11:R42" ca="1" si="1">IF(E11="","",TODAY()-E11)</f>
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="S11" s="39" t="s">
         <v>362</v>
@@ -3546,7 +3567,7 @@
       </c>
       <c r="R12" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="S12" s="39" t="s">
         <v>363</v>
@@ -3610,7 +3631,7 @@
       </c>
       <c r="R13" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="S13" s="39" t="s">
         <v>364</v>
@@ -3678,7 +3699,7 @@
       </c>
       <c r="R14" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="S14" s="39" t="s">
         <v>365</v>
@@ -3748,7 +3769,7 @@
       </c>
       <c r="R15" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="S15" s="39" t="s">
         <v>366</v>
@@ -3818,7 +3839,7 @@
       </c>
       <c r="R16" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="S16" s="39" t="s">
         <v>367</v>
@@ -3888,7 +3909,7 @@
       </c>
       <c r="R17" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="S17" s="39" t="s">
         <v>368</v>
@@ -3956,7 +3977,7 @@
       </c>
       <c r="R18" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="S18" s="39" t="s">
         <v>369</v>
@@ -4026,7 +4047,7 @@
       </c>
       <c r="R19" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="S19" s="39" t="s">
         <v>370</v>
@@ -4096,7 +4117,7 @@
       </c>
       <c r="R20" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="S20" s="39" t="s">
         <v>371</v>
@@ -4164,7 +4185,7 @@
       </c>
       <c r="R21" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="S21" s="39" t="s">
         <v>372</v>
@@ -4230,7 +4251,7 @@
       </c>
       <c r="R22" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="S22" s="39" t="s">
         <v>373</v>
@@ -4296,7 +4317,7 @@
       </c>
       <c r="R23" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="S23" s="39" t="s">
         <v>372</v>
@@ -4362,7 +4383,7 @@
       </c>
       <c r="R24" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="S24" s="39" t="s">
         <v>374</v>
@@ -4432,7 +4453,7 @@
       </c>
       <c r="R25" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="S25" s="39" t="s">
         <v>375</v>
@@ -4498,7 +4519,7 @@
       </c>
       <c r="R26" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="S26" s="39" t="s">
         <v>376</v>
@@ -4566,7 +4587,7 @@
       </c>
       <c r="R27" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="S27" s="39" t="s">
         <v>377</v>
@@ -4636,7 +4657,7 @@
       </c>
       <c r="R28" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="S28" s="39" t="s">
         <v>378</v>
@@ -4706,7 +4727,7 @@
       </c>
       <c r="R29" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="S29" s="39" t="s">
         <v>379</v>
@@ -4776,7 +4797,7 @@
       </c>
       <c r="R30" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="S30" s="39" t="s">
         <v>380</v>
@@ -4846,7 +4867,7 @@
       </c>
       <c r="R31" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="S31" s="39" t="s">
         <v>381</v>
@@ -4916,7 +4937,7 @@
       </c>
       <c r="R32" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="S32" s="39" t="s">
         <v>401</v>
@@ -4984,7 +5005,7 @@
       </c>
       <c r="R33" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="S33" s="39" t="s">
         <v>402</v>
@@ -5052,7 +5073,7 @@
       </c>
       <c r="R34" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="S34" s="43" t="s">
         <v>459</v>
@@ -5122,7 +5143,7 @@
       </c>
       <c r="R35" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="S35" s="43" t="s">
         <v>460</v>
@@ -5192,7 +5213,7 @@
       </c>
       <c r="R36" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="S36" t="s">
         <v>581</v>
@@ -5262,7 +5283,7 @@
       </c>
       <c r="R37" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="S37" t="s">
         <v>583</v>
@@ -5332,7 +5353,7 @@
       </c>
       <c r="R38" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="S38" t="s">
         <v>585</v>
@@ -5402,7 +5423,7 @@
       </c>
       <c r="R39" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="S39" t="s">
         <v>587</v>
@@ -5472,7 +5493,7 @@
       </c>
       <c r="R40" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="S40" t="s">
         <v>589</v>
@@ -5542,7 +5563,7 @@
       </c>
       <c r="R41" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="S41" t="s">
         <v>590</v>
@@ -5612,7 +5633,7 @@
       </c>
       <c r="R42" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="S42" t="s">
         <v>592</v>
@@ -5682,7 +5703,7 @@
       </c>
       <c r="R43" s="19">
         <f t="shared" ref="R43:R82" ca="1" si="2">IF(E43="","",TODAY()-E43)</f>
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="S43" t="s">
         <v>594</v>
@@ -5752,7 +5773,7 @@
       </c>
       <c r="R44" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="S44" t="s">
         <v>596</v>
@@ -5822,7 +5843,7 @@
       </c>
       <c r="R45" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="S45" t="s">
         <v>598</v>
@@ -5892,7 +5913,7 @@
       </c>
       <c r="R46" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="S46" t="s">
         <v>600</v>
@@ -5962,7 +5983,7 @@
       </c>
       <c r="R47" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="S47" t="s">
         <v>602</v>
@@ -6100,7 +6121,7 @@
       </c>
       <c r="R49" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="S49" t="s">
         <v>606</v>
@@ -6170,7 +6191,7 @@
       </c>
       <c r="R50" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="S50" t="s">
         <v>608</v>
@@ -6240,7 +6261,7 @@
       </c>
       <c r="R51" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="S51" t="s">
         <v>610</v>
@@ -6310,7 +6331,7 @@
       </c>
       <c r="R52" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="S52" t="s">
         <v>612</v>
@@ -6380,7 +6401,7 @@
       </c>
       <c r="R53" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="S53" t="s">
         <v>615</v>
@@ -6450,7 +6471,7 @@
       </c>
       <c r="R54" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="S54" t="s">
         <v>617</v>
@@ -6520,7 +6541,7 @@
       </c>
       <c r="R55" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="S55" t="s">
         <v>619</v>
@@ -6590,7 +6611,7 @@
       </c>
       <c r="R56" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="S56" t="s">
         <v>621</v>
@@ -6660,7 +6681,7 @@
       </c>
       <c r="R57" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="S57" t="s">
         <v>623</v>
@@ -6730,7 +6751,7 @@
       </c>
       <c r="R58" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="S58" t="s">
         <v>625</v>
@@ -6800,7 +6821,7 @@
       </c>
       <c r="R59" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="S59" t="s">
         <v>627</v>
@@ -6870,7 +6891,7 @@
       </c>
       <c r="R60" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="S60" t="s">
         <v>629</v>
@@ -6940,7 +6961,7 @@
       </c>
       <c r="R61" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="S61" t="s">
         <v>629</v>
@@ -7010,7 +7031,7 @@
       </c>
       <c r="R62" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="S62" t="s">
         <v>631</v>
@@ -7080,7 +7101,7 @@
       </c>
       <c r="R63" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="S63" t="s">
         <v>762</v>
@@ -7150,7 +7171,7 @@
       </c>
       <c r="R64" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="S64" t="s">
         <v>764</v>
@@ -7220,7 +7241,7 @@
       </c>
       <c r="R65" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="S65" t="s">
         <v>765</v>
@@ -7290,7 +7311,7 @@
       </c>
       <c r="R66" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="S66" t="s">
         <v>794</v>
@@ -7360,7 +7381,7 @@
       </c>
       <c r="R67" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="S67" t="s">
         <v>792</v>
@@ -7430,7 +7451,7 @@
       </c>
       <c r="R68" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="S68" t="s">
         <v>790</v>
@@ -7500,7 +7521,7 @@
       </c>
       <c r="R69" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="S69" t="s">
         <v>796</v>
@@ -7570,7 +7591,7 @@
       </c>
       <c r="R70" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="S70" t="s">
         <v>788</v>
@@ -7640,7 +7661,7 @@
       </c>
       <c r="R71" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="S71" t="s">
         <v>798</v>
@@ -7710,7 +7731,7 @@
       </c>
       <c r="R72" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="S72" t="s">
         <v>786</v>
@@ -7916,7 +7937,7 @@
       </c>
       <c r="R75" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="S75" t="s">
         <v>781</v>
@@ -8190,7 +8211,7 @@
       </c>
       <c r="R79" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="S79" t="s">
         <v>775</v>
@@ -8260,7 +8281,7 @@
       </c>
       <c r="R80" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="S80" t="s">
         <v>772</v>
@@ -8330,7 +8351,7 @@
       </c>
       <c r="R81" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="S81" t="s">
         <v>771</v>
@@ -8400,7 +8421,7 @@
       </c>
       <c r="R82" s="19">
         <f t="shared" ca="1" si="2"/>
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="S82" t="s">
         <v>769</v>
@@ -8470,7 +8491,7 @@
       </c>
       <c r="R83" s="19">
         <f t="shared" ref="R83:R104" ca="1" si="5">IF(E83="","",TODAY()-E83)</f>
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="S83" s="43" t="s">
         <v>651</v>
@@ -8538,7 +8559,7 @@
       </c>
       <c r="R84" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="S84" s="43" t="s">
         <v>654</v>
@@ -8606,7 +8627,7 @@
       </c>
       <c r="R85" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="S85" s="43" t="s">
         <v>655</v>
@@ -8676,7 +8697,7 @@
       </c>
       <c r="R86" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="S86" s="43" t="s">
         <v>766</v>
@@ -8746,7 +8767,7 @@
       </c>
       <c r="R87" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S87" s="43"/>
       <c r="T87" s="43"/>
@@ -8812,7 +8833,7 @@
       </c>
       <c r="R88" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S88" s="43"/>
       <c r="T88" s="43"/>
@@ -8878,7 +8899,7 @@
       </c>
       <c r="R89" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S89" s="43"/>
       <c r="T89" s="43"/>
@@ -8944,7 +8965,7 @@
       </c>
       <c r="R90" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S90" s="43"/>
       <c r="T90" s="43"/>
@@ -9010,7 +9031,7 @@
       </c>
       <c r="R91" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S91" s="43"/>
       <c r="T91" s="43"/>
@@ -9074,7 +9095,7 @@
       </c>
       <c r="R92" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S92" s="43"/>
       <c r="T92" s="43"/>
@@ -9140,7 +9161,7 @@
       </c>
       <c r="R93" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S93" s="43"/>
       <c r="T93" s="43"/>
@@ -9206,7 +9227,7 @@
       </c>
       <c r="R94" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S94" s="43"/>
       <c r="T94" s="43"/>
@@ -9272,7 +9293,7 @@
       </c>
       <c r="R95" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S95" s="43"/>
       <c r="T95" s="43"/>
@@ -9338,7 +9359,7 @@
       </c>
       <c r="R96" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S96" s="43"/>
       <c r="T96" s="43"/>
@@ -9404,7 +9425,7 @@
       </c>
       <c r="R97" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S97" s="43"/>
       <c r="T97" s="43"/>
@@ -9470,7 +9491,7 @@
       </c>
       <c r="R98" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S98" s="43"/>
       <c r="T98" s="43"/>
@@ -9536,7 +9557,7 @@
       </c>
       <c r="R99" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S99" s="43"/>
       <c r="T99" s="43"/>
@@ -9602,7 +9623,7 @@
       </c>
       <c r="R100" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S100" s="43"/>
       <c r="T100" s="43"/>
@@ -9668,7 +9689,7 @@
       </c>
       <c r="R101" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S101" s="43"/>
       <c r="T101" s="43"/>
@@ -9734,7 +9755,7 @@
       </c>
       <c r="R102" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S102" s="43"/>
       <c r="T102" s="43"/>
@@ -9800,7 +9821,7 @@
       </c>
       <c r="R103" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S103" s="43"/>
       <c r="T103" s="43"/>
@@ -9866,7 +9887,7 @@
       </c>
       <c r="R104" s="19">
         <f t="shared" ca="1" si="5"/>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="S104" s="43"/>
       <c r="T104" s="43"/>
@@ -9878,34 +9899,70 @@
       </c>
     </row>
     <row r="105" spans="1:22">
-      <c r="A105" s="10"/>
-      <c r="B105" s="11"/>
-      <c r="C105" s="12"/>
-      <c r="D105" s="12"/>
-      <c r="E105" s="12"/>
-      <c r="F105" s="43"/>
-      <c r="G105" s="43"/>
-      <c r="H105" s="11"/>
-      <c r="I105" s="11"/>
-      <c r="J105" s="11"/>
-      <c r="K105" s="11"/>
-      <c r="L105" s="11"/>
-      <c r="M105" s="11"/>
-      <c r="N105" s="11"/>
-      <c r="O105" s="11"/>
-      <c r="P105" s="11"/>
-      <c r="Q105" s="18" t="str">
+      <c r="A105" s="10" t="s">
+        <v>801</v>
+      </c>
+      <c r="B105" s="11" t="s">
+        <v>215</v>
+      </c>
+      <c r="C105" s="12">
+        <v>46314</v>
+      </c>
+      <c r="D105" s="12">
+        <v>46314</v>
+      </c>
+      <c r="E105" s="12">
+        <v>46314</v>
+      </c>
+      <c r="F105" s="43" t="s">
+        <v>802</v>
+      </c>
+      <c r="G105" s="43" t="s">
+        <v>803</v>
+      </c>
+      <c r="H105" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="I105" s="11" t="s">
+        <v>804</v>
+      </c>
+      <c r="J105" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="K105" s="11" t="s">
+        <v>805</v>
+      </c>
+      <c r="L105" s="11" t="s">
+        <v>806</v>
+      </c>
+      <c r="M105" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="N105" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O105" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="P105" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q105" s="18">
         <f t="shared" ref="Q105:Q136" si="6">IF(E105="","",E105+1)</f>
-        <v/>
-      </c>
-      <c r="R105" s="19" t="str">
+        <v>46315</v>
+      </c>
+      <c r="R105" s="19">
         <f t="shared" ref="R105:R136" ca="1" si="7">IF(E105="","",TODAY()-E105)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S105" s="43"/>
       <c r="T105" s="43"/>
-      <c r="U105" s="7"/>
-      <c r="V105" s="41"/>
+      <c r="U105" s="7" t="s">
+        <v>666</v>
+      </c>
+      <c r="V105" s="41" t="s">
+        <v>807</v>
+      </c>
     </row>
     <row r="106" spans="1:22">
       <c r="A106" s="10"/>

</xml_diff>

<commit_message>
[21/10] EC-022: titulo e bullets do Q2460-B publicados pelo LEO (Registro linha 106); regra de listing na Memoria (titulo curto, sem marca enquanto generico)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -258,7 +258,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="14"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -441,6 +441,24 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="5" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="5" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -864,7 +882,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
@@ -928,7 +945,6 @@
         <v/>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="21.95" customHeight="1" s="39">
       <c r="A8" s="63" t="inlineStr">
         <is>
@@ -936,7 +952,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="38.1" customHeight="1" s="39">
       <c r="A10" s="5" t="inlineStr">
         <is>
@@ -10562,34 +10577,100 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="10" t="n"/>
-      <c r="B106" s="11" t="n"/>
-      <c r="C106" s="12" t="n"/>
-      <c r="D106" s="12" t="n"/>
-      <c r="E106" s="12" t="n"/>
-      <c r="F106" s="43" t="n"/>
-      <c r="G106" s="43" t="n"/>
-      <c r="H106" s="11" t="n"/>
-      <c r="I106" s="11" t="n"/>
-      <c r="J106" s="11" t="n"/>
-      <c r="K106" s="11" t="n"/>
-      <c r="L106" s="11" t="n"/>
-      <c r="M106" s="11" t="n"/>
-      <c r="N106" s="11" t="n"/>
-      <c r="O106" s="11" t="n"/>
-      <c r="P106" s="11" t="n"/>
-      <c r="Q106" s="18">
+      <c r="A106" s="69" t="inlineStr">
+        <is>
+          <t>EC-022</t>
+        </is>
+      </c>
+      <c r="B106" s="69" t="inlineStr">
+        <is>
+          <t>entre-ciclos</t>
+        </is>
+      </c>
+      <c r="C106" s="70" t="n">
+        <v>46316</v>
+      </c>
+      <c r="D106" s="70" t="n">
+        <v>46316</v>
+      </c>
+      <c r="E106" s="70" t="n">
+        <v>46316</v>
+      </c>
+      <c r="F106" s="71" t="inlineStr">
+        <is>
+          <t>Listing Q2460-B (B0H7YNMBBK)</t>
+        </is>
+      </c>
+      <c r="G106" s="71" t="inlineStr">
+        <is>
+          <t>título + 5 bullets</t>
+        </is>
+      </c>
+      <c r="H106" s="69" t="inlineStr">
+        <is>
+          <t>CORRIGIR PÁGINA</t>
+        </is>
+      </c>
+      <c r="I106" s="69" t="inlineStr">
+        <is>
+          <t>Título 85 car.; bullets genéricos (durável/moderno repetidos, sem medida, uso, peso ou limpeza)</t>
+        </is>
+      </c>
+      <c r="J106" s="69" t="inlineStr">
+        <is>
+          <t>Título "… com Tampa Flip Top Polida para Escritório e Recepção"; bullets: capacidade 30 L 24x24x60 + usos + saco 30 L · flip top uma mão · aço inox 430 polido · 4 kg, base plana · enviada montada</t>
+        </is>
+      </c>
+      <c r="K106" s="69" t="inlineStr">
+        <is>
+          <t>Diagnóstico de página 21/10: 0 vendas desde 07/07, 35 cli/0 na Geral, 0 avaliações, marca Genérico. Bullets eram o único item corrigível sem novo ASIN. Marca não citada nas bullets (ASIN genérico). Título curto por orientação da assessoria.</t>
+        </is>
+      </c>
+      <c r="L106" s="69" t="inlineStr">
+        <is>
+          <t>ciclos/Pagina_Q2460-B_21-10.md + relatorios/amazon/paginas-21-10/</t>
+        </is>
+      </c>
+      <c r="M106" s="69" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="N106" s="69" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="O106" s="69" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="P106" s="69" t="inlineStr">
+        <is>
+          <t>EXECUTADA - EM MATURAÇÃO</t>
+        </is>
+      </c>
+      <c r="Q106" s="72">
         <f>IF(E106="","",E106+1)</f>
         <v/>
       </c>
-      <c r="R106" s="19">
+      <c r="R106" s="73">
         <f>IF(E106="","",TODAY()-E106)</f>
         <v/>
       </c>
-      <c r="S106" s="43" t="n"/>
-      <c r="T106" s="43" t="n"/>
-      <c r="U106" s="7" t="n"/>
-      <c r="V106" s="41" t="n"/>
+      <c r="S106" s="71" t="n"/>
+      <c r="T106" s="71" t="n"/>
+      <c r="U106" s="74" t="inlineStr">
+        <is>
+          <t>24/11/2026</t>
+        </is>
+      </c>
+      <c r="V106" s="71" t="inlineStr">
+        <is>
+          <t>Ler sessões e conversão do Q2460-B no Business Report por 4 semanas. Anúncio na Geral segue pausado (O6-006). Teste de frete embutido proposto, pendente de decisão de Mestra.</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="10" t="n"/>

</xml_diff>

<commit_message>
[21/10] EC-023: teste de frete gratis com preco embutido no Q2460-B (360,97 -> 399,90), aprovado LEO + Dianna, leitura 18/11; regra de diagnostico pela busca na Memoria
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -10673,34 +10673,98 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="10" t="n"/>
-      <c r="B107" s="11" t="n"/>
-      <c r="C107" s="12" t="n"/>
-      <c r="D107" s="12" t="n"/>
-      <c r="E107" s="12" t="n"/>
-      <c r="F107" s="43" t="n"/>
-      <c r="G107" s="43" t="n"/>
-      <c r="H107" s="11" t="n"/>
-      <c r="I107" s="11" t="n"/>
-      <c r="J107" s="11" t="n"/>
-      <c r="K107" s="11" t="n"/>
-      <c r="L107" s="11" t="n"/>
-      <c r="M107" s="11" t="n"/>
-      <c r="N107" s="11" t="n"/>
-      <c r="O107" s="11" t="n"/>
-      <c r="P107" s="11" t="n"/>
-      <c r="Q107" s="18">
+      <c r="A107" s="69" t="inlineStr">
+        <is>
+          <t>EC-023</t>
+        </is>
+      </c>
+      <c r="B107" s="69" t="inlineStr">
+        <is>
+          <t>entre-ciclos</t>
+        </is>
+      </c>
+      <c r="C107" s="70" t="n">
+        <v>46316</v>
+      </c>
+      <c r="D107" s="70" t="n">
+        <v>46316</v>
+      </c>
+      <c r="E107" s="70" t="n"/>
+      <c r="F107" s="71" t="inlineStr">
+        <is>
+          <t>Oferta Q2460-B (B0H7YNMBBK)</t>
+        </is>
+      </c>
+      <c r="G107" s="71" t="inlineStr">
+        <is>
+          <t>preço de tabela + modelo de envio</t>
+        </is>
+      </c>
+      <c r="H107" s="69" t="inlineStr">
+        <is>
+          <t>TESTE DE FRETE GRÁTIS (preço embutido)</t>
+        </is>
+      </c>
+      <c r="I107" s="69" t="inlineStr">
+        <is>
+          <t>R$ 360,97 · modelo de envio padrão (frete cobrado R$ 39,90 SP Interior, 5–7 dias)</t>
+        </is>
+      </c>
+      <c r="J107" s="69" t="inlineStr">
+        <is>
+          <t>R$ 399,90 · modelo "fretegratisteste" (R$ 0,00 em todas as 53 regiões, mesmos prazos)</t>
+        </is>
+      </c>
+      <c r="K107" s="69" t="inlineStr">
+        <is>
+          <t>Busca de 21/10: Winnet em 3º orgânico, único sem "Entrega GRÁTIS" na 1ª tela (Mimo 203 · Tramontina 408 com frete grátis). Frete embutido no preço mantém a margem em SP; frete real de Médios = 71% da tabela (dados/ANALISE_frete_tabela_x_real_20-10.csv). Teste em 1 SKU, reversível. Decisão LEO + Dianna.</t>
+        </is>
+      </c>
+      <c r="L107" s="69" t="inlineStr">
+        <is>
+          <t>ciclos/Pagina_Q2460-B_21-10.md + relatorios/amazon/paginas-21-10/</t>
+        </is>
+      </c>
+      <c r="M107" s="69" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="N107" s="69" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="O107" s="69" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="P107" s="69" t="inlineStr">
+        <is>
+          <t>APROVADA - AGUARDANDO EXECUÇÃO</t>
+        </is>
+      </c>
+      <c r="Q107" s="72">
         <f>IF(E107="","",E107+1)</f>
         <v/>
       </c>
-      <c r="R107" s="19">
+      <c r="R107" s="73">
         <f>IF(E107="","",TODAY()-E107)</f>
         <v/>
       </c>
-      <c r="S107" s="43" t="n"/>
-      <c r="T107" s="43" t="n"/>
-      <c r="U107" s="7" t="n"/>
-      <c r="V107" s="41" t="n"/>
+      <c r="S107" s="71" t="n"/>
+      <c r="T107" s="71" t="n"/>
+      <c r="U107" s="74" t="inlineStr">
+        <is>
+          <t>18/11/2026</t>
+        </is>
+      </c>
+      <c r="V107" s="71" t="inlineStr">
+        <is>
+          <t>Ordem: preço primeiro, modelo depois. Modelo só neste SKU. Leitura: sessões e conversão no Business Report por 4 semanas; se converter, estender a P3070/P3060/P4080 antes da BF. Aprendizado migra para o anúncio novo (oferta ≠ ASIN).</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="10" t="n"/>

</xml_diff>

<commit_message>
[21/10] EC-024: bullets e Included Components do L1618-T publicados pelo LEO (Registro linha 108, 102 entradas); leitura 18/11
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -10672,7 +10672,7 @@
         </is>
       </c>
     </row>
-    <row r="107">
+    <row r="107" s="39">
       <c r="A107" s="69" t="inlineStr">
         <is>
           <t>EC-023</t>
@@ -10766,35 +10766,101 @@
         </is>
       </c>
     </row>
-    <row r="108">
-      <c r="A108" s="10" t="n"/>
-      <c r="B108" s="11" t="n"/>
-      <c r="C108" s="12" t="n"/>
-      <c r="D108" s="12" t="n"/>
-      <c r="E108" s="12" t="n"/>
-      <c r="F108" s="43" t="n"/>
-      <c r="G108" s="43" t="n"/>
-      <c r="H108" s="11" t="n"/>
-      <c r="I108" s="11" t="n"/>
-      <c r="J108" s="11" t="n"/>
-      <c r="K108" s="11" t="n"/>
-      <c r="L108" s="11" t="n"/>
-      <c r="M108" s="11" t="n"/>
-      <c r="N108" s="11" t="n"/>
-      <c r="O108" s="11" t="n"/>
-      <c r="P108" s="11" t="n"/>
-      <c r="Q108" s="18">
+    <row r="108" s="39">
+      <c r="A108" s="69" t="inlineStr">
+        <is>
+          <t>EC-024</t>
+        </is>
+      </c>
+      <c r="B108" s="69" t="inlineStr">
+        <is>
+          <t>entre-ciclos</t>
+        </is>
+      </c>
+      <c r="C108" s="70" t="n">
+        <v>46316</v>
+      </c>
+      <c r="D108" s="70" t="n">
+        <v>46316</v>
+      </c>
+      <c r="E108" s="70" t="n">
+        <v>46316</v>
+      </c>
+      <c r="F108" s="71" t="inlineStr">
+        <is>
+          <t>Listing L1618-T (B0H3QQLFFY)</t>
+        </is>
+      </c>
+      <c r="G108" s="71" t="inlineStr">
+        <is>
+          <t>5 bullets + campo "Included Components"</t>
+        </is>
+      </c>
+      <c r="H108" s="69" t="inlineStr">
+        <is>
+          <t>CORRIGIR PÁGINA (ajuste leve)</t>
+        </is>
+      </c>
+      <c r="I108" s="69" t="inlineStr">
+        <is>
+          <t>Bullets genéricos (COMPACTA E FUNCIONAL / FABRICADA EM AÇO INOX / TAMPA SUPERIOR PRÁTICA / DESIGN ELEGANTE E DISCRETO / FÁCIL LIMPEZA); "Included Components: Lixeira Pitão 03 litros" (nome interno vazado)</t>
+        </is>
+      </c>
+      <c r="J108" s="69" t="inlineStr">
+        <is>
+          <t>Bullets: capacidade 3 L 16x18 + usos + 1,5 kg · tampa solta com puxador · aço inox 430 polido · chapa única sem pedal ou mola · fabricação nacional, enviada montada, aviso de reflexos; "Included Components" = "1 lixeira de 3 litros com tampa". Título mantido (84 car., formato da assessoria)</t>
+        </is>
+      </c>
+      <c r="K108" s="69" t="inlineStr">
+        <is>
+          <t>Diagnóstico de página 21/10: página CONVERTE (10 vendas desde 09/07, nº 258 em Organização para Banheiro) apesar de 0 avaliações e marca Genérico; decisão MANTER com ajuste leve. Bullets sem marca (ASIN genérico). Especificações confirmadas pelo LEO: aço 430, tampa solta, vai montada.</t>
+        </is>
+      </c>
+      <c r="L108" s="69" t="inlineStr">
+        <is>
+          <t>ciclos/Pagina_L1618-T_21-10.md + relatorios/amazon/paginas-21-10/</t>
+        </is>
+      </c>
+      <c r="M108" s="69" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="N108" s="69" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="O108" s="69" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="P108" s="69" t="inlineStr">
+        <is>
+          <t>EXECUTADA - EM MATURAÇÃO</t>
+        </is>
+      </c>
+      <c r="Q108" s="72">
         <f>IF(E108="","",E108+1)</f>
         <v/>
       </c>
-      <c r="R108" s="19">
+      <c r="R108" s="73">
         <f>IF(E108="","",TODAY()-E108)</f>
         <v/>
       </c>
-      <c r="S108" s="43" t="n"/>
-      <c r="T108" s="43" t="n"/>
-      <c r="U108" s="7" t="n"/>
-      <c r="V108" s="41" t="n"/>
+      <c r="S108" s="71" t="n"/>
+      <c r="T108" s="71" t="n"/>
+      <c r="U108" s="74" t="inlineStr">
+        <is>
+          <t>18/11/2026</t>
+        </is>
+      </c>
+      <c r="V108" s="71" t="inlineStr">
+        <is>
+          <t>LEO informou "salvei igual mandou" em 21/10; print da página no ar ainda não conferido (print de edição mostrava o 4º bullet antigo antes do salvamento). Ler sessões e conversão no Business Report por 4 semanas; comparar com a média pré (vendas mensais do SKU). Rotina paralela: "Solicitar avaliação" nos pedidos de 07/10 e 19/10 e em todo pedido novo.</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="10" t="n"/>

</xml_diff>

<commit_message>
[21/10] EC-023 executada e conferida: Q2460-B a R$ 399,90 com Entrega GRATIS no ar (Registro linha 107 em maturacao, leitura 18/11)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -10689,7 +10689,9 @@
       <c r="D107" s="70" t="n">
         <v>46316</v>
       </c>
-      <c r="E107" s="70" t="n"/>
+      <c r="E107" s="70" t="n">
+        <v>46316</v>
+      </c>
       <c r="F107" s="71" t="inlineStr">
         <is>
           <t>Oferta Q2460-B (B0H7YNMBBK)</t>
@@ -10737,12 +10739,12 @@
       </c>
       <c r="O107" s="69" t="inlineStr">
         <is>
-          <t>NÃO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="P107" s="69" t="inlineStr">
         <is>
-          <t>APROVADA - AGUARDANDO EXECUÇÃO</t>
+          <t>EXECUTADA - EM MATURAÇÃO</t>
         </is>
       </c>
       <c r="Q107" s="72">
@@ -10762,7 +10764,7 @@
       </c>
       <c r="V107" s="71" t="inlineStr">
         <is>
-          <t>Ordem: preço primeiro, modelo depois. Modelo só neste SKU. Leitura: sessões e conversão no Business Report por 4 semanas; se converter, estender a P3070/P3060/P4080 antes da BF. Aprendizado migra para o anúncio novo (oferta ≠ ASIN).</t>
+          <t>Ordem: preço primeiro, modelo depois. Modelo só neste SKU. Leitura: sessões e conversão no Business Report por 4 semanas; se converter, estender a P3070/P3060/P4080 antes da BF. Aprendizado migra para o anúncio novo (oferta ≠ ASIN). Executada e conferida por print em 21/10 (navegador anônimo, CEP Bela Vista/SP): página mostra R$ 399,90 (379,90 no Pix) e "Entrega GRÁTIS 26–27 de outubro"; título da EC-022 também no ar. Prazo igual ao do modelo padrão.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[21/10] EC-025: bullets e atributos da ficha do L1618-B publicados pelo LEO (Registro linha 109, 99 entradas); busca 'lixeira basculante inox 3 litros' lida (8 concorrentes 57-90, Brinox 89,99 c/ 638 avaliacoes)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -10864,35 +10864,101 @@
         </is>
       </c>
     </row>
-    <row r="109">
-      <c r="A109" s="10" t="n"/>
-      <c r="B109" s="11" t="n"/>
-      <c r="C109" s="12" t="n"/>
-      <c r="D109" s="12" t="n"/>
-      <c r="E109" s="12" t="n"/>
-      <c r="F109" s="43" t="n"/>
-      <c r="G109" s="43" t="n"/>
-      <c r="H109" s="11" t="n"/>
-      <c r="I109" s="11" t="n"/>
-      <c r="J109" s="11" t="n"/>
-      <c r="K109" s="11" t="n"/>
-      <c r="L109" s="11" t="n"/>
-      <c r="M109" s="11" t="n"/>
-      <c r="N109" s="11" t="n"/>
-      <c r="O109" s="11" t="n"/>
-      <c r="P109" s="11" t="n"/>
-      <c r="Q109" s="18">
+    <row r="109" s="39">
+      <c r="A109" s="69" t="inlineStr">
+        <is>
+          <t>EC-025</t>
+        </is>
+      </c>
+      <c r="B109" s="69" t="inlineStr">
+        <is>
+          <t>entre-ciclos</t>
+        </is>
+      </c>
+      <c r="C109" s="70" t="n">
+        <v>46316</v>
+      </c>
+      <c r="D109" s="70" t="n">
+        <v>46316</v>
+      </c>
+      <c r="E109" s="70" t="n">
+        <v>46316</v>
+      </c>
+      <c r="F109" s="71" t="inlineStr">
+        <is>
+          <t>Listing L1618-B (B0H6KPN1XS)</t>
+        </is>
+      </c>
+      <c r="G109" s="71" t="inlineStr">
+        <is>
+          <t>5 bullets + 4 atributos da ficha</t>
+        </is>
+      </c>
+      <c r="H109" s="69" t="inlineStr">
+        <is>
+          <t>CORRIGIR PÁGINA (ajuste leve)</t>
+        </is>
+      </c>
+      <c r="I109" s="69" t="inlineStr">
+        <is>
+          <t>Bullets genéricos (TAMPA BASCULANTE FLIP TOP / AÇO INOX POLIDO RESISTENTE / CAPACIDADE 3 LITROS COMPACTA / DESIGN MODERNO / USO INTERNO VERSÁTIL); ficha sem Cor, Forma, Mecanismo de abertura e Tipo de acabamento (invisível nos filtros da busca)</t>
+        </is>
+      </c>
+      <c r="J109" s="69" t="inlineStr">
+        <is>
+          <t>Bullets: capacidade 3 L 16x18 + usos + 1,5 kg · tampa basculante flip top de 14 cm · aço inox 430 polido · aro removível para limpeza, sem pedal/mola · fabricação nacional, enviada montada, aviso de reflexos. Ficha: Cor Prata · Forma Cilíndrico · Abertura Basculante · Acabamento Polido. Título mantido (97 car.)</t>
+        </is>
+      </c>
+      <c r="K109" s="69" t="inlineStr">
+        <is>
+          <t>Diagnóstico de página 21/10: 3 pedidos/4 un desde 13/09, 1 devolução por "desempenho ou qualidade" (2 un, sem comentário), 0 avaliações; ficha vazia nos campos que os filtros da busca leem (o irmão L1618-T os tem). Bullets sem marca (ASIN genérico). Especificações confirmadas pelo LEO: disco basculante 14 cm, aro sai, vai montada; aço 430 já na descrição.</t>
+        </is>
+      </c>
+      <c r="L109" s="69" t="inlineStr">
+        <is>
+          <t>ciclos/Pagina_L1618-B_21-10.md + relatorios/amazon/paginas-21-10/</t>
+        </is>
+      </c>
+      <c r="M109" s="69" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="N109" s="69" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="O109" s="69" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="P109" s="69" t="inlineStr">
+        <is>
+          <t>EXECUTADA - EM MATURAÇÃO</t>
+        </is>
+      </c>
+      <c r="Q109" s="72">
         <f>IF(E109="","",E109+1)</f>
         <v/>
       </c>
-      <c r="R109" s="19">
+      <c r="R109" s="73">
         <f>IF(E109="","",TODAY()-E109)</f>
         <v/>
       </c>
-      <c r="S109" s="43" t="n"/>
-      <c r="T109" s="43" t="n"/>
-      <c r="U109" s="7" t="n"/>
-      <c r="V109" s="41" t="n"/>
+      <c r="S109" s="71" t="n"/>
+      <c r="T109" s="71" t="n"/>
+      <c r="U109" s="74" t="inlineStr">
+        <is>
+          <t>18/11/2026</t>
+        </is>
+      </c>
+      <c r="V109" s="71" t="inlineStr">
+        <is>
+          <t>LEO informou "arrumei tudo o que me pediu" em 21/10; print da página no ar ainda não conferido. Ler sessões e conversão no Business Report por 4 semanas; vigiar devoluções do SKU. Rotina paralela: "Solicitar avaliação" nos pedidos de 03/10 e 13/10 e em todo pedido novo. Pergunta aberta para depois: categoria (Lixo e Reciclagem × Banho, onde o L1618-T ranqueia melhor).</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="10" t="n"/>

</xml_diff>

<commit_message>
[21/10] EC-026: bullets do P3060 publicados pelo LEO (Registro linha 110, 100 entradas); busca 'lixeira inox pedal 50 litros': P3060 mais barato entre inox 50 L, SONGMICS 484,49 c/ 2,2 mil avaliacoes no mesmo preco
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -10960,35 +10960,101 @@
         </is>
       </c>
     </row>
-    <row r="110">
-      <c r="A110" s="10" t="n"/>
-      <c r="B110" s="11" t="n"/>
-      <c r="C110" s="12" t="n"/>
-      <c r="D110" s="12" t="n"/>
-      <c r="E110" s="12" t="n"/>
-      <c r="F110" s="43" t="n"/>
-      <c r="G110" s="43" t="n"/>
-      <c r="H110" s="11" t="n"/>
-      <c r="I110" s="11" t="n"/>
-      <c r="J110" s="11" t="n"/>
-      <c r="K110" s="11" t="n"/>
-      <c r="L110" s="11" t="n"/>
-      <c r="M110" s="11" t="n"/>
-      <c r="N110" s="11" t="n"/>
-      <c r="O110" s="11" t="n"/>
-      <c r="P110" s="11" t="n"/>
-      <c r="Q110" s="18">
+    <row r="110" s="39">
+      <c r="A110" s="69" t="inlineStr">
+        <is>
+          <t>EC-026</t>
+        </is>
+      </c>
+      <c r="B110" s="69" t="inlineStr">
+        <is>
+          <t>entre-ciclos</t>
+        </is>
+      </c>
+      <c r="C110" s="70" t="n">
+        <v>46316</v>
+      </c>
+      <c r="D110" s="70" t="n">
+        <v>46316</v>
+      </c>
+      <c r="E110" s="70" t="n">
+        <v>46316</v>
+      </c>
+      <c r="F110" s="71" t="inlineStr">
+        <is>
+          <t>Listing P3060 (B0H4NLBG1Y)</t>
+        </is>
+      </c>
+      <c r="G110" s="71" t="inlineStr">
+        <is>
+          <t>5 bullets</t>
+        </is>
+      </c>
+      <c r="H110" s="69" t="inlineStr">
+        <is>
+          <t>CORRIGIR PÁGINA (ajuste leve)</t>
+        </is>
+      </c>
+      <c r="I110" s="69" t="inlineStr">
+        <is>
+          <t>Bullets do modelo padrão (ABERTURA POR PEDAL / FABRICADA EM AÇO INOX POLIDO / CAPACIDADE DE 50 LITROS / TAMPA FECHADA / ARO REMOVÍVEL INTERNO), sem peso, saco, tipo de aço ou montagem</t>
+        </is>
+      </c>
+      <c r="J110" s="69" t="inlineStr">
+        <is>
+          <t>Bullets: capacidade 50 L 30x60 + usos + saco 50 L · pedal (levanta com o pé, fecha sozinha) · aro interno removível · aço inox 430 polido · fabricação nacional, 5 kg, enviada montada, aviso de reflexos. Título, preço, modelo de envio e ficha NÃO alterados (preço de referência da BF)</t>
+        </is>
+      </c>
+      <c r="K110" s="69" t="inlineStr">
+        <is>
+          <t>Diagnóstico de página 21/10: página completa mas sem classificação, 2 pedidos/4 un; bullets eram o único campo seguro de mexer antes da Melhor Oferta de BF (19–30/11). Sem marca (ASIN genérico). Aço 430 e montagem confirmados pelo LEO.</t>
+        </is>
+      </c>
+      <c r="L110" s="69" t="inlineStr">
+        <is>
+          <t>ciclos/Pagina_P3060_21-10.md + relatorios/amazon/paginas-21-10/</t>
+        </is>
+      </c>
+      <c r="M110" s="69" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="N110" s="69" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="O110" s="69" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="P110" s="69" t="inlineStr">
+        <is>
+          <t>EXECUTADA - EM MATURAÇÃO</t>
+        </is>
+      </c>
+      <c r="Q110" s="72">
         <f>IF(E110="","",E110+1)</f>
         <v/>
       </c>
-      <c r="R110" s="19">
+      <c r="R110" s="73">
         <f>IF(E110="","",TODAY()-E110)</f>
         <v/>
       </c>
-      <c r="S110" s="43" t="n"/>
-      <c r="T110" s="43" t="n"/>
-      <c r="U110" s="7" t="n"/>
-      <c r="V110" s="41" t="n"/>
+      <c r="S110" s="71" t="n"/>
+      <c r="T110" s="71" t="n"/>
+      <c r="U110" s="74" t="inlineStr">
+        <is>
+          <t>18/11/2026</t>
+        </is>
+      </c>
+      <c r="V110" s="71" t="inlineStr">
+        <is>
+          <t>LEO informou "salvei os bullets do P3060" em 21/10; print no ar a conferir. Leitura contaminada pela BF a partir de 19/11: ler 21/10–18/11 pelo Business Report. Preço/envio/título congelados até 30/11. Rotina "Solicitar avaliação" no pedido de 01/10 (se na janela) e novos.</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="10" t="n"/>

</xml_diff>

<commit_message>
[22/10] EC-027: Material Type do P4080 preenchido pelo LEO (Registro linha 111, 101 entradas)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -11056,35 +11056,101 @@
         </is>
       </c>
     </row>
-    <row r="111">
-      <c r="A111" s="10" t="n"/>
-      <c r="B111" s="11" t="n"/>
-      <c r="C111" s="12" t="n"/>
-      <c r="D111" s="12" t="n"/>
-      <c r="E111" s="12" t="n"/>
-      <c r="F111" s="43" t="n"/>
-      <c r="G111" s="43" t="n"/>
-      <c r="H111" s="11" t="n"/>
-      <c r="I111" s="11" t="n"/>
-      <c r="J111" s="11" t="n"/>
-      <c r="K111" s="11" t="n"/>
-      <c r="L111" s="11" t="n"/>
-      <c r="M111" s="11" t="n"/>
-      <c r="N111" s="11" t="n"/>
-      <c r="O111" s="11" t="n"/>
-      <c r="P111" s="11" t="n"/>
-      <c r="Q111" s="18">
+    <row r="111" s="39">
+      <c r="A111" s="69" t="inlineStr">
+        <is>
+          <t>EC-027</t>
+        </is>
+      </c>
+      <c r="B111" s="69" t="inlineStr">
+        <is>
+          <t>entre-ciclos</t>
+        </is>
+      </c>
+      <c r="C111" s="70" t="n">
+        <v>46317</v>
+      </c>
+      <c r="D111" s="70" t="n">
+        <v>46317</v>
+      </c>
+      <c r="E111" s="70" t="n">
+        <v>46317</v>
+      </c>
+      <c r="F111" s="71" t="inlineStr">
+        <is>
+          <t>Listing P4080 (B0H63W8G49)</t>
+        </is>
+      </c>
+      <c r="G111" s="71" t="inlineStr">
+        <is>
+          <t>ficha: campo "Material Type"</t>
+        </is>
+      </c>
+      <c r="H111" s="69" t="inlineStr">
+        <is>
+          <t>CORRIGIR PÁGINA (ajuste leve)</t>
+        </is>
+      </c>
+      <c r="I111" s="69" t="inlineStr">
+        <is>
+          <t>"Material Type" vazio em Materiais e Cuidados (P3070 e P3060 têm "Aço inoxidável")</t>
+        </is>
+      </c>
+      <c r="J111" s="69" t="inlineStr">
+        <is>
+          <t>"Material Type" = Aço inoxidável. Título, preço, modelo de envio e bullets NÃO alterados (preço de referência da BF)</t>
+        </is>
+      </c>
+      <c r="K111" s="69" t="inlineStr">
+        <is>
+          <t>Diagnóstico de página 21/10: único campo de ficha vazio entre os 3 SKUs da BF; os filtros da busca leem os atributos. Sem efeito na Melhor Oferta.</t>
+        </is>
+      </c>
+      <c r="L111" s="69" t="inlineStr">
+        <is>
+          <t>ciclos/Pagina_P4080_21-10.md</t>
+        </is>
+      </c>
+      <c r="M111" s="69" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="N111" s="69" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="O111" s="69" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="P111" s="69" t="inlineStr">
+        <is>
+          <t>EXECUTADA - EM MATURAÇÃO</t>
+        </is>
+      </c>
+      <c r="Q111" s="72">
         <f>IF(E111="","",E111+1)</f>
         <v/>
       </c>
-      <c r="R111" s="19">
+      <c r="R111" s="73">
         <f>IF(E111="","",TODAY()-E111)</f>
         <v/>
       </c>
-      <c r="S111" s="43" t="n"/>
-      <c r="T111" s="43" t="n"/>
-      <c r="U111" s="7" t="n"/>
-      <c r="V111" s="41" t="n"/>
+      <c r="S111" s="71" t="n"/>
+      <c r="T111" s="71" t="n"/>
+      <c r="U111" s="74" t="inlineStr">
+        <is>
+          <t>18/11/2026</t>
+        </is>
+      </c>
+      <c r="V111" s="71" t="inlineStr">
+        <is>
+          <t>LEO informou "preenchi o material do P4080" em 22/10; print a conferir quando a página atualizar. Sem leitura própria (campo de filtro); acompanha a leitura do SKU na O8 e na BF.</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="10" t="n"/>

</xml_diff>

<commit_message>
[22/10] EC-024 conferida por print: 4 bullets novos + 1 antigo mantido, Included Components corrigido; Registro linha 108 com o texto real
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -10810,7 +10810,7 @@
       </c>
       <c r="J108" s="69" t="inlineStr">
         <is>
-          <t>Bullets: capacidade 3 L 16x18 + usos + 1,5 kg · tampa solta com puxador · aço inox 430 polido · chapa única sem pedal ou mola · fabricação nacional, enviada montada, aviso de reflexos; "Included Components" = "1 lixeira de 3 litros com tampa". Título mantido (84 car., formato da assessoria)</t>
+          <t>Bullets publicados: 1 capacidade 3 L 16x18 + usos + 1,5 kg · 2 tampa solta com puxador · 3 aço inox 430 polido · 4 "DESIGN ELEGANTE E DISCRETO" (bullet antigo mantido pelo LEO no lugar do "chapa única sem pedal") · 5 fabricação nacional, enviada montada, aviso de reflexos; "Included Components" = "1 lixeira de 3 litros com tampa". Título mantido (84 car.)</t>
         </is>
       </c>
       <c r="K108" s="69" t="inlineStr">
@@ -10860,7 +10860,7 @@
       </c>
       <c r="V108" s="71" t="inlineStr">
         <is>
-          <t>LEO informou "salvei igual mandou" em 21/10; print da página no ar ainda não conferido (print de edição mostrava o 4º bullet antigo antes do salvamento). Ler sessões e conversão no Business Report por 4 semanas; comparar com a média pré (vendas mensais do SKU). Rotina paralela: "Solicitar avaliação" nos pedidos de 07/10 e 19/10 e em todo pedido novo.</t>
+          <t>Conferida por print em 22/10 (conta da Dianna): 5 bullets e Included Components no ar como descrito. Ler sessões e conversão no Business Report por 4 semanas; comparar com a média pré (vendas mensais do SKU). Rotina paralela: "Solicitar avaliação" nos pedidos de 07/10 e 19/10 e em todo pedido novo.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[22/10] EC-025 conferida por print: 5 bullets e 5 atributos da ficha no ar (Material Type a mais)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
+++ b/dados/Registro_Alteracoes_Amazon_Ads_Winnet.xlsx
@@ -10906,7 +10906,7 @@
       </c>
       <c r="J109" s="69" t="inlineStr">
         <is>
-          <t>Bullets: capacidade 3 L 16x18 + usos + 1,5 kg · tampa basculante flip top de 14 cm · aço inox 430 polido · aro removível para limpeza, sem pedal/mola · fabricação nacional, enviada montada, aviso de reflexos. Ficha: Cor Prata · Forma Cilíndrico · Abertura Basculante · Acabamento Polido. Título mantido (97 car.)</t>
+          <t>Bullets: capacidade 3 L 16x18 + usos + 1,5 kg · tampa basculante flip top de 14 cm · aço inox 430 polido · aro removível para limpeza, sem pedal/mola · fabricação nacional, enviada montada, aviso de reflexos. Ficha: Cor Prata · Forma Cilíndrico · Abertura Basculante · Acabamento Polido · Material Type Aço inoxidável (a mais, por iniciativa do LEO). Título mantido (97 car.)</t>
         </is>
       </c>
       <c r="K109" s="69" t="inlineStr">
@@ -10956,7 +10956,7 @@
       </c>
       <c r="V109" s="71" t="inlineStr">
         <is>
-          <t>LEO informou "arrumei tudo o que me pediu" em 21/10; print da página no ar ainda não conferido. Ler sessões e conversão no Business Report por 4 semanas; vigiar devoluções do SKU. Rotina paralela: "Solicitar avaliação" nos pedidos de 03/10 e 13/10 e em todo pedido novo. Pergunta aberta para depois: categoria (Lixo e Reciclagem × Banho, onde o L1618-T ranqueia melhor).</t>
+          <t>Conferida por print em 22/10 (conta da Dianna): 5 bullets exatamente como propostos; ficha com os 5 atributos preenchidos (incl. Material Type). Ler sessões e conversão no Business Report por 4 semanas; vigiar devoluções do SKU. Rotina paralela: "Solicitar avaliação" nos pedidos de 03/10 e 13/10 e em todo pedido novo. Pergunta aberta para depois: categoria (Lixo e Reciclagem × Banho).</t>
         </is>
       </c>
     </row>

</xml_diff>